<commit_message>
docs: settle change reasons, driver-tracking legal basis and internal roles
History tables get a required change_reason column, generated by the
domain-model tool: typed by the person for administrative decisions, a
fixed text from the app for routine actions (DM-21). Open question 6 is
answered: the company's data processing agreement plus each driver's
acknowledged privacy notice is enough while we sell SaaS (ID-43). D7 is
answered: a role gives internal and customer users the same features,
they differ only in data reach, and each role's feature list is granted
near the end of implementation (ID-44). Feature catalog ACC-14 and
ACC-17 updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -65,12 +65,12 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'organizations'!$A$7:$I$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'organization_history'!$A$7:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'organization_history'!$A$7:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'users'!$A$8:$I$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'user_history'!$A$7:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'user_history'!$A$7:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'user_state'!$A$7:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'memberships'!$A$7:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'membership_history'!$A$7:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'membership_history'!$A$7:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'user_credentials'!$A$6:$I$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'user_sessions'!$A$6:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'one_time_codes'!$A$6:$I$16</definedName>
@@ -606,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I93"/>
+  <dimension ref="A1:I92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="H8" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="H10" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="H13" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
@@ -3671,23 +3671,6 @@
       <c r="C92" s="6" t="inlineStr">
         <is>
           <t>chủ sở hữu telematics</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="108" customHeight="1">
-      <c r="A93" s="6" t="inlineStr">
-        <is>
-          <t>D7</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>Với người dùng nội bộ (xem được mọi tổ chức), mỗi chức danh được những tính năng nào - nhất là dữ liệu cá nhân như lịch sử vị trí và clip camera (ví dụ ACCOUNTANT không được mở clip camera)? vai trò nào chỉ xem một phần?</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="inlineStr">
-        <is>
-          <t>user_role_assignments, feature list in code</t>
         </is>
       </c>
     </row>
@@ -9657,7 +9640,7 @@
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>TRUE với (các) tổ chức của chính chúng ta, đơn vị vận hành nền tảng (nhân sự thuê ngoài làm thay chúng ta, ví dụ một công ty bán hàng thuê ngoài, cũng là thành viên của tổ chức này). Người dùng của tổ chức này xem được dữ liệu của mọi tổ chức và dùng được mọi tính năng (không giới hạn theo gói), vẫn trong phạm vi vai trò (quyết định D7); chỉ tổ chức nội bộ mới được có HEAD_ADMIN và CO_ADMIN. FALSE với mọi tổ chức khác (khách hàng, đối tác): người dùng chỉ thấy dữ liệu liên quan tới tổ chức của mình, tính năng giới hạn theo gói dịch vụ. Đối tác được nhận biết bằng hồ sơ repair_partners, không bằng cờ này. Cột nhạy cảm nhất của bảng: bật cờ này là cấp quyền xem dữ liệu của mọi tổ chức.</t>
+          <t>TRUE với (các) tổ chức của chính chúng ta, đơn vị vận hành nền tảng (nhân sự thuê ngoài làm thay chúng ta, ví dụ một công ty bán hàng thuê ngoài, cũng là thành viên của tổ chức này). Người dùng của tổ chức này xem được dữ liệu của mọi tổ chức và dùng được mọi tính năng (không giới hạn theo gói), vẫn trong phạm vi vai trò (quyết định ID-44); chỉ tổ chức nội bộ mới được có HEAD_ADMIN và CO_ADMIN. FALSE với mọi tổ chức khác (khách hàng, đối tác): người dùng chỉ thấy dữ liệu liên quan tới tổ chức của mình, tính năng giới hạn theo gói dịch vụ. Đối tác được nhận biết bằng hồ sơ repair_partners, không bằng cờ này. Cột nhạy cảm nhất của bảng: bật cờ này là cấp quyền xem dữ liệu của mọi tổ chức.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -16275,7 +16258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -16920,53 +16903,86 @@
       </c>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="inlineStr">
+    <row r="24" ht="40.5" customHeight="1">
+      <c r="A24" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>change_reason</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>varchar(200)</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Customer moved to a new office</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="n"/>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="4" t="n"/>
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="27" customHeight="1">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6" t="inlineStr">
+    <row r="27" ht="27" customHeight="1">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>ix_organization_history_organization_id_time</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>organization_id, changed_at</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="n"/>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A7:I23"/>
+  <autoFilter ref="A7:I24"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'organizations'!A1"/>
@@ -27579,7 +27595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -28125,53 +28141,86 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="inlineStr">
+    <row r="21" ht="40.5" customHeight="1">
+      <c r="A21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>change_reason</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>varchar(200)</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Customer moved to a new office</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="n"/>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="inlineStr">
+    <row r="24" ht="27" customHeight="1">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>ix_user_history_user_id_time</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>user_id, changed_at</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A7:I20"/>
+  <autoFilter ref="A7:I21"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'users'!A1"/>
@@ -31376,7 +31425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -31922,53 +31971,86 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="inlineStr">
+    <row r="21" ht="40.5" customHeight="1">
+      <c r="A21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>change_reason</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>varchar(200)</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Customer moved to a new office</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="n"/>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="inlineStr">
+    <row r="24" ht="27" customHeight="1">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>ix_membership_history_membership_id_time</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>membership_id, changed_at</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A7:I20"/>
+  <autoFilter ref="A7:I21"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'memberships'!A1"/>

</xml_diff>

<commit_message>
docs(decisions): limit who sees a cross-organization driving session
The truck's organization and the driver see it; the driver's own employer
does not (DR-08).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -1852,7 +1852,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="108" customHeight="1">
+    <row r="34" ht="135" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
           <t>19</t>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Ai cầm lái xe nào, trong khoảng thời gian nào (DR-07): tài xế nhận xe bằng cách quét mã QR trên xe hoặc chọn xe ở gần trên ứng dụng, hoặc quản lý nhận xe giúp trên portal. Thay thế driver_vehicle_assignments. Phiên kết thúc khi tài xế trả xe, tài xế khác nhận xe, tài xế nhận xe khác, hoặc xe không di chuyển quá thời gian tự kết thúc của tổ chức (organization_settings). Các sự kiện cần biết tài xế (điểm, chuyến, phiên sạc) lấy tài xế từ đây. Cảnh báo cho tài xế gửi tới tài xế đang nhận xe và portal; xe chạy mà không ai nhận xe sẽ cảnh báo lên portal. Dòng đã đóng không bao giờ bị sửa nên không cần lịch sử thay đổi.</t>
+          <t>Ai cầm lái xe nào, trong khoảng thời gian nào (DR-07): tài xế nhận xe bằng cách quét mã QR trên xe hoặc chọn xe ở gần trên ứng dụng, hoặc quản lý nhận xe giúp trên portal. Thay thế driver_vehicle_assignments. Phiên kết thúc khi tài xế trả xe, tài xế khác nhận xe, tài xế nhận xe khác, hoặc xe không di chuyển quá thời gian tự kết thúc của tổ chức (organization_settings). Các sự kiện cần biết tài xế (điểm, chuyến, phiên sạc) lấy tài xế từ đây. Cảnh báo cho tài xế gửi tới tài xế đang nhận xe và portal; xe chạy mà không ai nhận xe sẽ cảnh báo lên portal. Tổ chức sở hữu xe và chính tài xế (trên ứng dụng) xem được phiên lái; tổ chức tuyển dụng tài xế không xem được phiên lái trên xe của tổ chức khác (DR-08). Dòng đã đóng không bao giờ bị sửa nên không cần lịch sử thay đổi.</t>
         </is>
       </c>
       <c r="H34" s="6" t="n">
@@ -13821,7 +13821,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Ai cầm lái xe nào, trong khoảng thời gian nào (DR-07): tài xế nhận xe bằng cách quét mã QR trên xe hoặc chọn xe ở gần trên ứng dụng, hoặc quản lý nhận xe giúp trên portal. Thay thế driver_vehicle_assignments. Phiên kết thúc khi tài xế trả xe, tài xế khác nhận xe, tài xế nhận xe khác, hoặc xe không di chuyển quá thời gian tự kết thúc của tổ chức (organization_settings). Các sự kiện cần biết tài xế (điểm, chuyến, phiên sạc) lấy tài xế từ đây. Cảnh báo cho tài xế gửi tới tài xế đang nhận xe và portal; xe chạy mà không ai nhận xe sẽ cảnh báo lên portal. Dòng đã đóng không bao giờ bị sửa nên không cần lịch sử thay đổi.</t>
+          <t>Ai cầm lái xe nào, trong khoảng thời gian nào (DR-07): tài xế nhận xe bằng cách quét mã QR trên xe hoặc chọn xe ở gần trên ứng dụng, hoặc quản lý nhận xe giúp trên portal. Thay thế driver_vehicle_assignments. Phiên kết thúc khi tài xế trả xe, tài xế khác nhận xe, tài xế nhận xe khác, hoặc xe không di chuyển quá thời gian tự kết thúc của tổ chức (organization_settings). Các sự kiện cần biết tài xế (điểm, chuyến, phiên sạc) lấy tài xế từ đây. Cảnh báo cho tài xế gửi tới tài xế đang nhận xe và portal; xe chạy mà không ai nhận xe sẽ cảnh báo lên portal. Tổ chức sở hữu xe và chính tài xế (trên ứng dụng) xem được phiên lái; tổ chức tuyển dụng tài xế không xem được phiên lái trên xe của tổ chức khác (DR-08). Dòng đã đóng không bao giờ bị sửa nên không cần lịch sử thay đổi.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(domain-model): drop the spec confirmation time from vehicle models
Figures enter the catalog only once confirmed and may be updated later;
the change history keeps earlier values (VH-15).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -87,8 +87,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'organization_setting_history'!$A$7:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'vehicles'!$A$7:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'vehicle_history'!$A$7:$I$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'vehicle_models'!$A$7:$I$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'vehicle_model_history'!$A$7:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'vehicle_models'!$A$7:$I$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'vehicle_model_history'!$A$7:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'telematics'!$A$6:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'vehicle_telemetry'!$A$6:$I$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'drivers'!$A$6:$I$16</definedName>
@@ -1559,7 +1559,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="67.5" customHeight="1">
+    <row r="26" ht="81" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t>14</t>
@@ -1592,11 +1592,11 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Danh mục dòng xe và thông số kỹ thuật (VEH-03, VH-15), dùng chung cho mọi tổ chức, do bộ phận vận hành của chúng ta quản lý. Chỉ xe điện: không có số liệu diesel (đường cơ sở diesel cho báo cáo carbon là tính năng riêng). Mọi dòng xe hiện tại đều là đầu kéo; cột loại thân xe sẽ được thêm khi có loại khác. Có lưu lịch sử thay đổi vì báo cáo dựa vào các số liệu này.</t>
+          <t>Danh mục dòng xe và thông số kỹ thuật (VEH-03, VH-15), dùng chung cho mọi tổ chức, do bộ phận vận hành của chúng ta quản lý. Số liệu chỉ được nhập khi đã xác nhận và có thể cập nhật sau (lịch sử lưu các giá trị trước). Chỉ xe điện: không có số liệu diesel (đường cơ sở diesel cho báo cáo carbon là tính năng riêng). Mọi dòng xe hiện tại đều là đầu kéo; cột loại thân xe sẽ được thêm khi có loại khác. Có lưu lịch sử thay đổi vì báo cáo dựa vào các số liệu này.</t>
         </is>
       </c>
       <c r="H26" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="H27" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
@@ -10662,7 +10662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10700,7 +10700,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Danh mục dòng xe và thông số kỹ thuật (VEH-03, VH-15), dùng chung cho mọi tổ chức, do bộ phận vận hành của chúng ta quản lý. Chỉ xe điện: không có số liệu diesel (đường cơ sở diesel cho báo cáo carbon là tính năng riêng). Mọi dòng xe hiện tại đều là đầu kéo; cột loại thân xe sẽ được thêm khi có loại khác. Có lưu lịch sử thay đổi vì báo cáo dựa vào các số liệu này.</t>
+          <t>Danh mục dòng xe và thông số kỹ thuật (VEH-03, VH-15), dùng chung cho mọi tổ chức, do bộ phận vận hành của chúng ta quản lý. Số liệu chỉ được nhập khi đã xác nhận và có thể cập nhật sau (lịch sử lưu các giá trị trước). Chỉ xe điện: không có số liệu diesel (đường cơ sở diesel cho báo cáo carbon là tính năng riêng). Mọi dòng xe hiện tại đều là đầu kéo; cột loại thân xe sẽ được thêm khi có loại khác. Có lưu lịch sử thay đổi vì báo cáo dựa vào các số liệu này.</t>
         </is>
       </c>
     </row>
@@ -11018,13 +11018,13 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="27" customHeight="1">
+    <row r="15">
       <c r="A15" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>spec_confirmed_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -11034,19 +11034,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm nhà sản xuất xác nhận bằng văn bản các thông số này; NULL khi còn là ước tính, báo cáo sẽ đánh dấu.</t>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>2026-08-15T00:00:00Z</t>
+          <t>2026-09-01T02:00:00Z</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -11061,7 +11061,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -11078,12 +11078,12 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
+          <t>2026-09-10T07:15:00Z</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -11092,13 +11092,13 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="27" customHeight="1">
       <c r="A17" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>deleted_at</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -11108,19 +11108,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
+          <t>Thời điểm xóa mềm, chỉ dùng cho dòng xe nhập nhầm; NULL khi bản ghi còn hiệu lực.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10T07:15:00Z</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -11129,103 +11129,79 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>deleted_at</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="27" customHeight="1">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>uq_vehicle_models_live_make_model</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>make, model_name</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>có</t>
         </is>
       </c>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm xóa mềm, chỉ dùng cho dòng xe nhập nhầm; NULL khi bản ghi còn hiệu lực.</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="4" t="n"/>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>uq_vehicle_models_live_make_model</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>make, model_name</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>WHERE deleted_at IS NULL</t>
         </is>
       </c>
     </row>
-    <row r="22"/>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
-      <c r="A23" s="4" t="n"/>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>vehicles</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_model_id</t>
         </is>
       </c>
     </row>
@@ -11233,7 +11209,7 @@
       <c r="A24" s="6" t="n"/>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>vehicles</t>
+          <t>vehicle_model_history</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -11242,26 +11218,13 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>vehicle_model_history</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_model_id</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A7:I18"/>
+  <autoFilter ref="A7:I17"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'vehicle_model_history'!A1"/>
-    <hyperlink ref="B24" location="'vehicles'!A1"/>
-    <hyperlink ref="B25" location="'vehicle_model_history'!A1"/>
+    <hyperlink ref="B23" location="'vehicles'!A1"/>
+    <hyperlink ref="B24" location="'vehicle_model_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11273,7 +11236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11646,13 +11609,13 @@
       </c>
       <c r="I15" s="6" t="n"/>
     </row>
-    <row r="16" ht="27" customHeight="1">
+    <row r="16">
       <c r="A16" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>spec_confirmed_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -11669,12 +11632,12 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (vehicle_models.spec_confirmed_at).</t>
+          <t>Giá trị trước khi thay đổi (vehicle_models.created_at).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>2026-08-15T00:00:00Z</t>
+          <t>2026-09-01T02:00:00Z</t>
         </is>
       </c>
       <c r="I16" s="6" t="n"/>
@@ -11685,7 +11648,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -11702,12 +11665,12 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (vehicle_models.created_at).</t>
+          <t>Giá trị trước khi thay đổi (vehicle_models.updated_at).</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
+          <t>2026-09-10T07:15:00Z</t>
         </is>
       </c>
       <c r="I17" s="6" t="n"/>
@@ -11718,7 +11681,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>deleted_at</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -11735,12 +11698,12 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (vehicle_models.updated_at).</t>
+          <t>Giá trị trước khi thay đổi (vehicle_models.deleted_at).</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10T07:15:00Z</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I18" s="6" t="n"/>
@@ -11751,7 +11714,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>deleted_at</t>
+          <t>changed_at</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -11761,182 +11724,149 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (vehicle_models.deleted_at).</t>
+          <t>Thời điểm phiên bản này của dòng bị thay thế.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>2026-09-10T07:15:00Z</t>
         </is>
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20">
+    <row r="20" ht="27" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>changed_at</t>
+          <t>changed_by</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>users.user_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm phiên bản này của dòng bị thay thế.</t>
+          <t>Người dùng đã thực hiện thay đổi; NULL nếu do hệ thống thực hiện.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10T07:15:00Z</t>
+          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
         </is>
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="27" customHeight="1">
+    <row r="21" ht="40.5" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>changed_by</t>
+          <t>change_reason</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>varchar(200)</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>users.user_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Người dùng đã thực hiện thay đổi; NULL nếu do hệ thống thực hiện.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
+          <t>Customer moved to a new office</t>
         </is>
       </c>
       <c r="I21" s="6" t="n"/>
     </row>
-    <row r="22" ht="40.5" customHeight="1">
-      <c r="A22" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>change_reason</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>varchar(200)</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>Customer moved to a new office</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="n"/>
-    </row>
-    <row r="23"/>
-    <row r="24">
-      <c r="A24" s="4" t="n"/>
-      <c r="B24" s="4" t="inlineStr">
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="6" t="inlineStr">
+    <row r="24" ht="27" customHeight="1">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>ix_vehicle_model_history_vehicle_model_id_time</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>vehicle_model_id, changed_at</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A7:I22"/>
+  <autoFilter ref="A7:I21"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'vehicle_models'!A1"/>
     <hyperlink ref="F9" location="'vehicle_models'!A1"/>
-    <hyperlink ref="F21" location="'users'!A1"/>
+    <hyperlink ref="F20" location="'users'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(domain-model): name relationship start columns with _at
owned_since and installed_since become acquired_at and installed_at, so
every timestamp ends in _at as the naming convention requires; DM-22
reworded to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -1471,7 +1471,7 @@
       <c r="G23" s="5" t="inlineStr">
         <is>
           <t>Bản thân chiếc xe tải: định danh (VIN, biển số), thông số và trạng thái kích hoạt.
-• Tại mỗi thời điểm, một xe thuộc một tổ chức (organization_id, owned_since); các chủ trước nằm trong lịch sử thay đổi của xe, và view vehicle_ownership_periods liệt kê mọi giai đoạn sở hữu (VH-10).
+• Tại mỗi thời điểm, một xe thuộc một tổ chức (organization_id, acquired_at); các chủ trước nằm trong lịch sử thay đổi của xe, và view vehicle_ownership_periods liệt kê mọi giai đoạn sở hữu (VH-10).
 • Sau khi bán xe (VH-11): dữ liệu ghi nhận dưới chủ cũ (dữ liệu vận hành và những gì tính từ đó) vẫn thuộc chủ cũ; tình trạng xe (sức khỏe, lỗi, bảo dưỡng, bảo hành) và các tổng tích lũy (quãng đường, năng lượng, chu kỳ sạc) đi theo xe.
 • Chỉ một chủ sở hữu (quyết định ngày 03/10/2026): mỗi xe (và mỗi hồ sơ tài xế) thuộc đúng một tổ chức trong hệ thống. Khi các bên hợp tác (ví dụ chủ xe tự lái hoạt động dưới giấy phép kinh doanh vận tải của một công ty), các bên tự thỏa thuận và khai báo chủ sở hữu cho chúng ta; điều khoản hợp tác của họ nằm ngoài trách nhiệm của chúng ta và không được mô hình hóa.</t>
         </is>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>owned_since</t>
+          <t>acquired_at</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -8123,7 +8123,7 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm chủ hiện tại nhận xe (ngày bàn giao, ngày hiệu lực của lần chuyển quyền). Một giai đoạn kết thúc tại owned_since của chủ kế tiếp. Giá trị của chủ đầu tiên là ngày bàn giao xe.</t>
+          <t>Thời điểm chủ hiện tại nhận xe (ngày bàn giao, ngày hiệu lực của lần chuyển quyền). Một giai đoạn kết thúc tại acquired_at của chủ kế tiếp. Giá trị của chủ đầu tiên là ngày bàn giao xe.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -9199,7 +9199,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>owned_since</t>
+          <t>acquired_at</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -9216,7 +9216,7 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (vehicles.owned_since).</t>
+          <t>Giá trị trước khi thay đổi (vehicles.acquired_at).</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -13505,7 +13505,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>owned_since</t>
+          <t>acquired_at</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -13587,7 +13587,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>installed_since</t>
+          <t>installed_at</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -14240,7 +14240,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>owned_since</t>
+          <t>acquired_at</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -14257,7 +14257,7 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (batteries.owned_since).</t>
+          <t>Giá trị trước khi thay đổi (batteries.acquired_at).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -14306,7 +14306,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>installed_since</t>
+          <t>installed_at</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -14323,7 +14323,7 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (batteries.installed_since).</t>
+          <t>Giá trị trước khi thay đổi (batteries.installed_at).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(decisions): limit extra timestamps on profile tables
A profile table gets a time column only for the start of a relationship
or a contract or schedule date; every other change relies on its history
(DM-23). A vehicle's status may also be switched by a business rule, such
as closing its repair record (VH-17).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -8359,7 +8359,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="94.5" customHeight="1">
+    <row r="17" ht="108" customHeight="1">
       <c r="A17" s="6" t="n">
         <v>10</v>
       </c>
@@ -8382,7 +8382,7 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Trạng thái phục vụ, luôn do con người đặt (VH-05). ACTIVE: đang phục vụ. MAINTENANCE: đang bảo dưỡng hoặc sửa chữa. DECOMMISSIONED: đã rời hệ thống (thanh lý, bán ra ngoài dịch vụ, hoặc ngừng sử dụng vĩnh viễn); giữ lại cho lịch sử và báo cáo, không nhận dữ liệu mới. Xe đang nhàn rỗi hay không gửi dữ liệu thì không lưu: được tính từ dữ liệu vận hành và T-Box.</t>
+          <t>Trạng thái phục vụ, do con người đặt hoặc do quy tắc nghiệp vụ thay mặt công ty, ví dụ trở lại ACTIVE khi hồ sơ sửa chữa được đóng (VH-05, VH-17). ACTIVE: đang phục vụ. MAINTENANCE: đang bảo dưỡng hoặc sửa chữa. DECOMMISSIONED: đã rời hệ thống (thanh lý, bán ra ngoài dịch vụ, hoặc ngừng sử dụng vĩnh viễn); giữ lại cho lịch sử và báo cáo, không nhận dữ liệu mới. Xe đang nhàn rỗi hay không gửi dữ liệu thì không lưu: được tính từ dữ liệu vận hành và T-Box.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): keep the role-assignment tenant copy and own T-Boxes
user_role_assignments keeps organization_id as the one DM-24 exception:
the one-ORG_ADMIN unique index needs it on the same row. The T-Box is an
asset with its own owner, the truck's owner or G3, plus acquired_at; a
device the seller owns moves with the truck (TX-07, answers D6).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -101,7 +101,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'battery_history'!$A$7:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'warranties'!$A$7:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'warranty_history'!$A$7:$I$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'telematics'!$A$6:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'telematics'!$A$6:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'vehicle_telemetry'!$A$6:$I$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'drivers'!$A$6:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'driver_vehicle_assignments'!$A$6:$I$14</definedName>
@@ -628,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I104"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1999,7 +1999,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="27" customHeight="1">
+    <row r="37" ht="40.5" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
           <t>18</t>
@@ -2022,7 +2022,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Chưa quyết định</t>
+          <t>Khách hàng</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -2032,11 +2032,11 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Một thiết bị telematics và chiếc xe nó đang gắn. Thiết bị thuộc khách hàng hay G3 là quyết định D6.</t>
+          <t>Một thiết bị telematics (T-Box) và chiếc xe nó đang gắn. Thiết bị là một tài sản có chủ riêng, là chủ xe hoặc G3 (TX-07); thiết bị thuộc bên bán đi theo xe khi bán xe.</t>
         </is>
       </c>
       <c r="H37" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
@@ -4199,23 +4199,6 @@
       <c r="C103" s="6" t="inlineStr">
         <is>
           <t>wallets, payments</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="40.5" customHeight="1">
-      <c r="A104" s="6" t="inlineStr">
-        <is>
-          <t>D6</t>
-        </is>
-      </c>
-      <c r="B104" s="6" t="inlineStr">
-        <is>
-          <t>Ai sở hữu thiết bị telematics: khách hàng, hay G3 (nằm trong gói thuê bao)?</t>
-        </is>
-      </c>
-      <c r="C104" s="6" t="inlineStr">
-        <is>
-          <t>chủ sở hữu telematics</t>
         </is>
       </c>
     </row>
@@ -9856,7 +9839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10626,7 +10609,7 @@
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>vehicle_telemetry</t>
+          <t>telematics</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -10639,7 +10622,7 @@
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>drivers</t>
+          <t>vehicle_telemetry</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -10648,11 +10631,11 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="27" customHeight="1">
+    <row r="37">
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>driver_vehicle_assignments</t>
+          <t>drivers</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -10661,11 +10644,11 @@
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="27" customHeight="1">
       <c r="A38" s="6" t="n"/>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>driving_sessions</t>
+          <t>driver_vehicle_assignments</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -10678,7 +10661,7 @@
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>charging_credentials</t>
+          <t>driving_sessions</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -10691,7 +10674,7 @@
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>fleets</t>
+          <t>charging_credentials</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -10700,11 +10683,11 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="27" customHeight="1">
+    <row r="41">
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>fleet_vehicle_memberships</t>
+          <t>fleets</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -10713,11 +10696,11 @@
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="27" customHeight="1">
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>fleet_user_assignments</t>
+          <t>fleet_vehicle_memberships</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -10730,7 +10713,7 @@
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>geofences</t>
+          <t>fleet_user_assignments</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -10743,7 +10726,7 @@
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>charging_reservations</t>
+          <t>geofences</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -10756,7 +10739,7 @@
       <c r="A45" s="6" t="n"/>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>charging_sessions</t>
+          <t>charging_reservations</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -10769,7 +10752,7 @@
       <c r="A46" s="6" t="n"/>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>charging_sessions</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -10782,7 +10765,7 @@
       <c r="A47" s="6" t="n"/>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>support_cases</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -10795,7 +10778,7 @@
       <c r="A48" s="6" t="n"/>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>repair_partners</t>
+          <t>support_cases</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -10808,7 +10791,7 @@
       <c r="A49" s="6" t="n"/>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>maintenance_bookings</t>
+          <t>repair_partners</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -10817,11 +10800,11 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="27" customHeight="1">
+    <row r="50">
       <c r="A50" s="6" t="n"/>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>charging_policy_assignments</t>
+          <t>maintenance_bookings</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -10830,11 +10813,11 @@
         </is>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="27" customHeight="1">
       <c r="A51" s="6" t="n"/>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>policy_violations</t>
+          <t>charging_policy_assignments</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -10847,7 +10830,7 @@
       <c r="A52" s="6" t="n"/>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>policy_violations</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -10860,7 +10843,7 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>wallets</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -10873,7 +10856,7 @@
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>wallet_transactions</t>
+          <t>wallets</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -10886,7 +10869,7 @@
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>wallet_transactions</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -10899,7 +10882,7 @@
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>invoice_lines</t>
+          <t>invoices</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -10912,7 +10895,7 @@
       <c r="A57" s="6" t="n"/>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>subscriptions</t>
+          <t>invoice_lines</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -10925,7 +10908,7 @@
       <c r="A58" s="6" t="n"/>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>driver_scores</t>
+          <t>subscriptions</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -10938,7 +10921,7 @@
       <c r="A59" s="6" t="n"/>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>trips</t>
+          <t>driver_scores</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -10951,10 +10934,23 @@
       <c r="A60" s="6" t="n"/>
       <c r="B60" s="7" t="inlineStr">
         <is>
+          <t>trips</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n"/>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
           <t>organization_history</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C61" s="6" t="inlineStr">
         <is>
           <t>organization_id</t>
         </is>
@@ -10975,32 +10971,33 @@
     <hyperlink ref="B32" location="'organization_settings'!A1"/>
     <hyperlink ref="B33" location="'vehicles'!A1"/>
     <hyperlink ref="B34" location="'batteries'!A1"/>
-    <hyperlink ref="B35" location="'vehicle_telemetry'!A1"/>
-    <hyperlink ref="B36" location="'drivers'!A1"/>
-    <hyperlink ref="B37" location="'driver_vehicle_assignments'!A1"/>
-    <hyperlink ref="B38" location="'driving_sessions'!A1"/>
-    <hyperlink ref="B39" location="'charging_credentials'!A1"/>
-    <hyperlink ref="B40" location="'fleets'!A1"/>
-    <hyperlink ref="B41" location="'fleet_vehicle_memberships'!A1"/>
-    <hyperlink ref="B42" location="'fleet_user_assignments'!A1"/>
-    <hyperlink ref="B43" location="'geofences'!A1"/>
-    <hyperlink ref="B44" location="'charging_reservations'!A1"/>
-    <hyperlink ref="B45" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B46" location="'notifications'!A1"/>
-    <hyperlink ref="B47" location="'support_cases'!A1"/>
-    <hyperlink ref="B48" location="'repair_partners'!A1"/>
-    <hyperlink ref="B49" location="'maintenance_bookings'!A1"/>
-    <hyperlink ref="B50" location="'charging_policy_assignments'!A1"/>
-    <hyperlink ref="B51" location="'policy_violations'!A1"/>
-    <hyperlink ref="B52" location="'payments'!A1"/>
-    <hyperlink ref="B53" location="'wallets'!A1"/>
-    <hyperlink ref="B54" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="B55" location="'invoices'!A1"/>
-    <hyperlink ref="B56" location="'invoice_lines'!A1"/>
-    <hyperlink ref="B57" location="'subscriptions'!A1"/>
-    <hyperlink ref="B58" location="'driver_scores'!A1"/>
-    <hyperlink ref="B59" location="'trips'!A1"/>
-    <hyperlink ref="B60" location="'organization_history'!A1"/>
+    <hyperlink ref="B35" location="'telematics'!A1"/>
+    <hyperlink ref="B36" location="'vehicle_telemetry'!A1"/>
+    <hyperlink ref="B37" location="'drivers'!A1"/>
+    <hyperlink ref="B38" location="'driver_vehicle_assignments'!A1"/>
+    <hyperlink ref="B39" location="'driving_sessions'!A1"/>
+    <hyperlink ref="B40" location="'charging_credentials'!A1"/>
+    <hyperlink ref="B41" location="'fleets'!A1"/>
+    <hyperlink ref="B42" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="B43" location="'fleet_user_assignments'!A1"/>
+    <hyperlink ref="B44" location="'geofences'!A1"/>
+    <hyperlink ref="B45" location="'charging_reservations'!A1"/>
+    <hyperlink ref="B46" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B47" location="'notifications'!A1"/>
+    <hyperlink ref="B48" location="'support_cases'!A1"/>
+    <hyperlink ref="B49" location="'repair_partners'!A1"/>
+    <hyperlink ref="B50" location="'maintenance_bookings'!A1"/>
+    <hyperlink ref="B51" location="'charging_policy_assignments'!A1"/>
+    <hyperlink ref="B52" location="'policy_violations'!A1"/>
+    <hyperlink ref="B53" location="'payments'!A1"/>
+    <hyperlink ref="B54" location="'wallets'!A1"/>
+    <hyperlink ref="B55" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="B56" location="'invoices'!A1"/>
+    <hyperlink ref="B57" location="'invoice_lines'!A1"/>
+    <hyperlink ref="B58" location="'subscriptions'!A1"/>
+    <hyperlink ref="B59" location="'driver_scores'!A1"/>
+    <hyperlink ref="B60" location="'trips'!A1"/>
+    <hyperlink ref="B61" location="'organization_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16420,7 +16417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -16451,14 +16448,14 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Miền nghiệp vụ: Thiết bị telematics (telematics)   ·   Chủ sở hữu dữ liệu: Chưa quyết định   ·   Tính năng: F-G1, F-J1, F-J2, F-J3</t>
+          <t>Miền nghiệp vụ: Thiết bị telematics (telematics)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-G1, F-J1, F-J2, F-J3</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một thiết bị telematics và chiếc xe nó đang gắn. Thiết bị thuộc khách hàng hay G3 là quyết định D6.</t>
+          <t>Một thiết bị telematics (T-Box) và chiếc xe nó đang gắn. Thiết bị là một tài sản có chủ riêng, là chủ xe hoặc G3 (TX-07); thiết bị thuộc bên bán đi theo xe khi bán xe.</t>
         </is>
       </c>
     </row>
@@ -16590,7 +16587,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id</t>
+          <t>organization_id</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -16600,7 +16597,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -16610,17 +16607,17 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>vehicles.vehicle_id (khi xóa: đặt về NULL)</t>
+          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Xe mà thiết bị đang gắn; NULL khi đã tháo. Mỗi xe có tối đa một thiết bị còn hiệu lực (chưa xóa mềm).</t>
+          <t>Tổ chức đang sở hữu thiết bị: chủ xe, hoặc G3 khi G3 cung cấp thiết bị (ví dụ kèm gói thuê bao).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
+          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
         </is>
       </c>
       <c r="I9" s="6" t="n"/>
@@ -16631,12 +16628,12 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>acquired_at</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>telematicstatus</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -16648,28 +16645,28 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Trạng thái vận hành của thiết bị.</t>
+          <t>Thời điểm chủ hiện tại nhận thiết bị (DM-22).</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>2026-06-01T00:00:00Z</t>
         </is>
       </c>
       <c r="I10" s="6" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>firmware_version</t>
+          <t>vehicle_id</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -16677,65 +16674,73 @@
           <t>có</t>
         </is>
       </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>vehicles.vehicle_id (khi xóa: đặt về NULL)</t>
+        </is>
+      </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Phiên bản firmware đang chạy trên thiết bị.</t>
+          <t>Xe mà thiết bị đang gắn; NULL khi đã tháo. Mỗi xe có tối đa một thiết bị còn hiệu lực (chưa xóa mềm).</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>1.4.2</t>
+          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
         </is>
       </c>
       <c r="I11" s="6" t="n"/>
     </row>
-    <row r="12" ht="27" customHeight="1">
+    <row r="12">
       <c r="A12" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>telemetry_interval_seconds</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>telematicstatus</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Chu kỳ gửi dữ liệu (giây) đã đẩy xuống thiết bị qua MQTT lần gần nhất (F-J2); NULL trước lần đẩy đầu tiên.</t>
+          <t>Trạng thái vận hành của thiết bị.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13" ht="27" customHeight="1">
+    <row r="13">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>config_pushed_at</t>
+          <t>firmware_version</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -16747,56 +16752,56 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm đẩy chu kỳ đó lần gần nhất; NULL trước lần đẩy đầu tiên.</t>
+          <t>Phiên bản firmware đang chạy trên thiết bị.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>2026-09-12T03:00:00Z</t>
+          <t>1.4.2</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>telemetry_interval_seconds</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
+          <t>Chu kỳ gửi dữ liệu (giây) đã đẩy xuống thiết bị qua MQTT lần gần nhất (F-J2); NULL trước lần đẩy đầu tiên.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>config_pushed_at</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -16806,30 +16811,30 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
+          <t>Thời điểm đẩy chu kỳ đó lần gần nhất; NULL trước lần đẩy đầu tiên.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10T07:15:00Z</t>
+          <t>2026-09-12T03:00:00Z</t>
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
     </row>
-    <row r="16" ht="27" customHeight="1">
+    <row r="16">
       <c r="A16" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>deleted_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -16839,125 +16844,151 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-01T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:15:00Z</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="27" customHeight="1">
+      <c r="A18" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>deleted_at</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
           <t>Thời điểm xóa mềm; NULL khi bản ghi còn hiệu lực. Không bao giờ xóa hẳn.</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>NULL</t>
         </is>
       </c>
-      <c r="I16" s="6" t="n"/>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="I18" s="6" t="n"/>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Kiểu enum</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Giá trị cho phép</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="27" customHeight="1">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="inlineStr">
+    <row r="21" ht="27" customHeight="1">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>telematicstatus</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>ACTIVE, INACTIVE, MAINTENANCE</t>
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="4" t="inlineStr">
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>ix_telematics_status</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-    </row>
-    <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>ix_telematics_telematic_serial</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>telematic_serial</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>ix_telematics_vehicle_id</t>
+          <t>ix_telematics_status</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id</t>
+          <t>status</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -16972,73 +17003,114 @@
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6" t="inlineStr">
         <is>
+          <t>ix_telematics_telematic_serial</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>telematic_serial</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>ix_telematics_vehicle_id</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+    </row>
+    <row r="27" ht="27" customHeight="1">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
           <t>uq_telematics_active_vehicle</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>vehicle_id</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>có</t>
         </is>
       </c>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>WHERE deleted_at IS NULL</t>
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="4" t="n"/>
-      <c r="B27" s="4" t="inlineStr">
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="4" t="n"/>
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Được tham chiếu bởi bảng</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Cột</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="7" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="6" t="n"/>
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>warranties</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>telematic_id</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="7" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="6" t="n"/>
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>vehicle_telemetry</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>telematic_id</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I16"/>
+  <autoFilter ref="A6:I18"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F9" location="'vehicles'!A1"/>
-    <hyperlink ref="B28" location="'warranties'!A1"/>
-    <hyperlink ref="B29" location="'vehicle_telemetry'!A1"/>
+    <hyperlink ref="F9" location="'organizations'!A1"/>
+    <hyperlink ref="F11" location="'vehicles'!A1"/>
+    <hyperlink ref="B30" location="'warranties'!A1"/>
+    <hyperlink ref="B31" location="'vehicle_telemetry'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(domain-model): make the telemetry interval an organization setting
The interval moves from each device to the truck owner's
organization_settings and is pushed to every device on its trucks; the
device reports the interval it uses, so an unapplied push shows. The
T-Box gets an IMEI, and telematic_state holds the latest health report
(SIM, power, signal, storage, GNSS), whose message fields are added to
mqtt-spec.md as provisional (TX-09).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -91,8 +91,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'legal_documents'!$A$6:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'user_role_assignments'!$A$6:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'access_audit_logs'!$A$6:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'organization_settings'!$A$7:$I$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'organization_setting_history'!$A$7:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'organization_settings'!$A$7:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'organization_setting_history'!$A$7:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'vehicles'!$A$7:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'vehicle_history'!$A$7:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'vehicle_models'!$A$7:$I$17</definedName>
@@ -103,9 +103,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'battery_history'!$A$7:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'warranties'!$A$7:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'warranty_history'!$A$7:$I$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'telematics'!$A$8:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'telematics'!$A$8:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'telematic_history'!$A$7:$I$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'telematic_state'!$A$7:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'telematic_state'!$A$7:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'vehicle_telemetry'!$A$6:$I$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'drivers'!$A$6:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="32" hidden="1">'driver_vehicle_assignments'!$A$6:$I$14</definedName>
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="H21" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="H22" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
@@ -2040,7 +2040,7 @@
         </is>
       </c>
       <c r="H37" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
@@ -2093,7 +2093,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="67.5" customHeight="1">
+    <row r="39" ht="94.5" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
           <t>19</t>
@@ -2126,11 +2126,11 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Những gì thiết bị tự báo về mình trên topic trạng thái MQTT (quan sát, không phải quyết định): chỉ giá trị mới nhất, không lưu lịch sử thay đổi (TX-08). Được tạo cùng lúc với thiết bị nên mỗi thiết bị luôn có đúng một dòng trạng thái. Thiết bị có trực tuyến hay không được tính từ dữ liệu vận hành (TX-06), không lưu.</t>
+          <t>Những gì thiết bị tự báo về mình trên topic trạng thái MQTT, khoảng mỗi ngày một lần (quan sát, không phải quyết định): firmware, chu kỳ đang dùng, SIM, nguồn điện, sóng, bộ nhớ, GNSS (TX-08, TX-09; các trường của bản tin là tạm thời cho tới khi nhà cung cấp xác nhận). Chỉ giá trị mới nhất, không lưu lịch sử thay đổi. Được tạo cùng lúc với thiết bị nên mỗi thiết bị luôn có đúng một dòng trạng thái. Thiết bị có trực tuyến hay không được tính từ dữ liệu vận hành (TX-06), không lưu.</t>
         </is>
       </c>
       <c r="H39" s="6" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
@@ -7388,7 +7388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7526,13 +7526,13 @@
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9" ht="27" customHeight="1">
+    <row r="9" ht="54" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>driving_session_auto_end_minutes</t>
+          <t>telemetry_interval_seconds</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -7549,12 +7549,12 @@
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Phiên lái tự kết thúc khi xe không di chuyển trong khoảng thời gian này (DR-07); mặc định 120.</t>
+          <t>Chu kỳ T-Box trên các xe của tổ chức gửi dữ liệu (giây) (TX-09); mặc định 10, trong giới hạn backend cho phép. Được đẩy xuống mọi thiết bị trên xe của tổ chức khi thay đổi, và xuống thiết bị khi được gắn lên xe.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -7563,18 +7563,18 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>driving_session_auto_end_minutes</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -7586,12 +7586,12 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
+          <t>Phiên lái tự kết thúc khi xe không di chuyển trong khoảng thời gian này (DR-07); mặc định 120.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
+          <t>120</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -7606,7 +7606,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -7623,54 +7623,91 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-01T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
           <t>Thời điểm thiết lập được sửa gần nhất (UTC).</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>2026-09-10T07:15:00Z</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>🔍</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="inlineStr">
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Được tham chiếu bởi bảng</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Cột</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="27" customHeight="1">
-      <c r="A14" s="6" t="n"/>
-      <c r="B14" s="7" t="inlineStr">
+    <row r="15" ht="27" customHeight="1">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>organization_setting_history</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>organization_id</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A7:I11"/>
+  <autoFilter ref="A7:I12"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'organization_setting_history'!A1"/>
     <hyperlink ref="F8" location="'organizations'!A1"/>
-    <hyperlink ref="B14" location="'organization_setting_history'!A1"/>
+    <hyperlink ref="B15" location="'organization_setting_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7682,7 +7719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7863,7 +7900,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>driving_session_auto_end_minutes</t>
+          <t>telemetry_interval_seconds</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -7880,12 +7917,12 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (organization_settings.driving_session_auto_end_minutes).</t>
+          <t>Giá trị trước khi thay đổi (organization_settings.telemetry_interval_seconds).</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I10" s="6" t="n"/>
@@ -7896,12 +7933,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>driving_session_auto_end_minutes</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -7913,12 +7950,12 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (organization_settings.created_at).</t>
+          <t>Giá trị trước khi thay đổi (organization_settings.driving_session_auto_end_minutes).</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
+          <t>120</t>
         </is>
       </c>
       <c r="I11" s="6" t="n"/>
@@ -7929,7 +7966,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -7946,23 +7983,23 @@
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (organization_settings.updated_at).</t>
+          <t>Giá trị trước khi thay đổi (organization_settings.created_at).</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10T07:15:00Z</t>
+          <t>2026-09-01T02:00:00Z</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>changed_at</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -7972,14 +8009,14 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm phiên bản này của dòng bị thay thế.</t>
+          <t>Giá trị trước khi thay đổi (organization_settings.updated_at).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -7989,132 +8026,165 @@
       </c>
       <c r="I13" s="6" t="n"/>
     </row>
-    <row r="14" ht="27" customHeight="1">
+    <row r="14">
       <c r="A14" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>changed_by</t>
+          <t>changed_at</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>users.user_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Người dùng đã thực hiện thay đổi; NULL nếu do hệ thống thực hiện.</t>
+          <t>Thời điểm phiên bản này của dòng bị thay thế.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
+          <t>2026-09-10T07:15:00Z</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
     </row>
-    <row r="15" ht="40.5" customHeight="1">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
+          <t>changed_by</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>users.user_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Người dùng đã thực hiện thay đổi; NULL nếu do hệ thống thực hiện.</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n"/>
+    </row>
+    <row r="16" ht="40.5" customHeight="1">
+      <c r="A16" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
           <t>change_reason</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>varchar(200)</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Customer moved to a new office</t>
         </is>
       </c>
-      <c r="I15" s="6" t="n"/>
-    </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="4" t="n"/>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="40.5" customHeight="1">
-      <c r="A18" s="6" t="n"/>
-      <c r="B18" s="6" t="inlineStr">
+    <row r="19" ht="40.5" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>ix_organization_setting_history_organization_id_time</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>organization_id, changed_at</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A7:I15"/>
+  <autoFilter ref="A7:I16"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'organization_settings'!A1"/>
     <hyperlink ref="F9" location="'organization_settings'!A1"/>
-    <hyperlink ref="F14" location="'users'!A1"/>
+    <hyperlink ref="F15" location="'users'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16517,7 +16587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -16658,35 +16728,35 @@
       </c>
       <c r="I9" s="6" t="n"/>
     </row>
-    <row r="10" ht="27" customHeight="1">
+    <row r="10" ht="40.5" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>telematic_serial</t>
+          <t>imei</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>varchar(15)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Số serial in trên thiết bị; cũng là định danh MQTT. Duy nhất trong các thiết bị chưa xóa.</t>
+          <t>Số IMEI của modem thiết bị, nhập khi cấp phát; định danh phần cứng cố định, duy nhất trong các thiết bị chưa xóa. NULL khi chưa nhập.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>TBX-2409-000123</t>
+          <t>356938035643809</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -16701,12 +16771,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
+          <t>telematic_serial</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -16714,24 +16784,16 @@
           <t>không</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức đang sở hữu thiết bị: chủ xe, hoặc G3 khi G3 cung cấp thiết bị (ví dụ kèm gói thuê bao).</t>
+          <t>Số serial in trên thiết bị; cũng là định danh MQTT. Duy nhất trong các thiết bị chưa xóa.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+          <t>TBX-2409-000123</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -16740,18 +16802,18 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="27" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>4</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>acquired_at</t>
+          <t>organization_id</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -16759,16 +16821,24 @@
           <t>không</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm chủ hiện tại nhận thiết bị (DM-22).</t>
+          <t>Tổ chức đang sở hữu thiết bị: chủ xe, hoặc G3 khi G3 cung cấp thiết bị (ví dụ kèm gói thuê bao).</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>2026-06-01T00:00:00Z</t>
+          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -16777,43 +16847,35 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="40.5" customHeight="1">
+    <row r="13">
       <c r="A13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id</t>
+          <t>acquired_at</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>vehicles.vehicle_id (khi xóa: đặt về NULL)</t>
-        </is>
-      </c>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Xe mà thiết bị đang gắn; NULL khi trong kho hoặc đã tháo. Mỗi xe gắn tối đa một thiết bị. Các xe trước lấy từ view telematic_installation_periods (DM-22).</t>
+          <t>Thời điểm chủ hiện tại nhận thiết bị (DM-22).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
+          <t>2026-06-01T00:00:00Z</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -16822,18 +16884,18 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="27" customHeight="1">
+    <row r="14" ht="40.5" customHeight="1">
       <c r="A14" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>installed_at</t>
+          <t>vehicle_id</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -16841,16 +16903,24 @@
           <t>có</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>vehicles.vehicle_id (khi xóa: đặt về NULL)</t>
+        </is>
+      </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm thiết bị được gắn lên xe hiện tại; NULL khi chưa gắn (DM-22).</t>
+          <t>Xe mà thiết bị đang gắn; NULL khi trong kho hoặc đã tháo. Mỗi xe gắn tối đa một thiết bị. Các xe trước lấy từ view telematic_installation_periods (DM-22).</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>2026-06-01T00:00:00Z</t>
+          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -16859,35 +16929,35 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="81" customHeight="1">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>installed_at</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>telematicstatus</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Trạng thái do con người đặt (TX-08). ACTIVE: dùng được. MAINTENANCE: đang sửa chữa hoặc kiểm tra. DECOMMISSIONED: đã rời hệ thống (thanh lý, trả lại). Đang gắn hay trong kho đọc từ vehicle_id; có gửi dữ liệu hay im lặng được tính từ dữ liệu vận hành (TX-06). Chỉ thiết bị đang gắn và ACTIVE mới nhận cấu hình.</t>
+          <t>Thời điểm thiết bị được gắn lên xe hiện tại; NULL khi chưa gắn (DM-22).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>2026-06-01T00:00:00Z</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -16896,35 +16966,35 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="81" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>status_reason</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>varchar(200)</t>
+          <t>telematicstatus</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Lý do của trạng thái hiện tại; NULL khi ACTIVE.</t>
+          <t>Trạng thái do con người đặt (TX-08). ACTIVE: dùng được. MAINTENANCE: đang sửa chữa hoặc kiểm tra. DECOMMISSIONED: đã rời hệ thống (thanh lý, trả lại). Đang gắn hay trong kho đọc từ vehicle_id; có gửi dữ liệu hay im lặng được tính từ dữ liệu vận hành (TX-06). Chỉ thiết bị đang gắn và ACTIVE mới nhận cấu hình.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Antenna replaced at the Hanoi workshop</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -16933,18 +17003,18 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="27" customHeight="1">
+    <row r="17">
       <c r="A17" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>firmware_version</t>
+          <t>status_reason</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>varchar(200)</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -16956,28 +17026,32 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: TX-08] Firmware nhập qua API; thiết bị tự báo nên chuyển sang telematic_state.</t>
+          <t>Lý do của trạng thái hiện tại; NULL khi ACTIVE.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>1.4.2</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="n"/>
-    </row>
-    <row r="18" ht="54" customHeight="1">
+          <t>Antenna replaced at the Hanoi workshop</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="27" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>telemetry_interval_seconds</t>
+          <t>firmware_version</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -16989,32 +17063,28 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Chu kỳ gửi dữ liệu (giây) đã đẩy xuống thiết bị qua MQTT lần gần nhất (F-J2), do con người chọn; NULL trước lần đẩy đầu tiên. Là một quyết định, nên lịch sử thay đổi ghi lại ai đổi, khi nào và vì sao.</t>
+          <t>[Sẽ bỏ: TX-08] Firmware nhập qua API; thiết bị tự báo nên chuyển sang telematic_state.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="40.5" customHeight="1">
+          <t>1.4.2</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="54" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>config_pushed_at</t>
+          <t>telemetry_interval_seconds</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -17026,23 +17096,23 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: TX-08] Thời điểm đẩy chu kỳ lần gần nhất; việc đẩy xảy ra khi lưu thay đổi nên lấy từ changed_at của lịch sử (DM-23).</t>
+          <t>[Sẽ bỏ: TX-09] Chu kỳ gửi đã đẩy xuống thiết bị này; chu kỳ nay là thiết lập của tổ chức (organization_settings), còn chu kỳ thiết bị thực sự dùng được báo trong telematic_state.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>2026-09-12T03:00:00Z</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20">
+    <row r="20" ht="40.5" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>12</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>config_pushed_at</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -17052,26 +17122,22 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
+          <t>[Sẽ bỏ: TX-08] Thời điểm đẩy chu kỳ lần gần nhất; việc đẩy xảy ra khi lưu thay đổi nên lấy từ changed_at của lịch sử (DM-23).</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
+          <t>2026-09-12T03:00:00Z</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
@@ -17079,7 +17145,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -17096,12 +17162,12 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10T07:15:00Z</t>
+          <t>2026-09-01T02:00:00Z</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -17110,13 +17176,13 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="54" customHeight="1">
+    <row r="22">
       <c r="A22" s="6" t="n">
         <v>14</v>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>deleted_at</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -17126,152 +17192,165 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E22" s="6" t="n"/>
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:15:00Z</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1">
+      <c r="A23" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>deleted_at</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
           <t>Thời điểm xóa mềm, chỉ dùng cho thiết bị nhập nhầm; thiết bị thật rời hệ thống được chuyển sang DECOMMISSIONED và tháo khỏi xe, các xe trước được giữ trong lịch sử (TX-08). NULL khi bản ghi còn hiệu lực.</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>NULL</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>🔍</t>
         </is>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24">
-      <c r="A24" s="4" t="n"/>
-      <c r="B24" s="4" t="inlineStr">
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="4" t="n"/>
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Kiểu enum</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Giá trị cho phép</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="54" customHeight="1">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="6" t="inlineStr">
+    <row r="26" ht="54" customHeight="1">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>telematicstatus</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>ACTIVE, INACTIVE (sẽ bỏ), MAINTENANCE, DECOMMISSIONED (dự kiến)</t>
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="4" t="n"/>
-      <c r="B27" s="4" t="inlineStr">
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="4" t="n"/>
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>ix_telematics_status</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="6" t="n"/>
-    </row>
-    <row r="29" ht="40.5" customHeight="1">
+    <row r="29">
       <c r="A29" s="6" t="n"/>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>ix_telematics_telematic_serial</t>
+          <t>ix_telematics_status</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>telematic_serial</t>
+          <t>status</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E29" s="6" t="n"/>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>Planned (TX-08): unique only among devices not deleted (WHERE deleted_at IS NULL)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="27" customHeight="1">
+      <c r="F29" s="6" t="n"/>
+    </row>
+    <row r="30" ht="40.5" customHeight="1">
       <c r="A30" s="6" t="n"/>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>ix_telematics_vehicle_id</t>
+          <t>ix_telematics_telematic_serial</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id</t>
+          <t>telematic_serial</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E30" s="6" t="n"/>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>To be removed (TX-08): the unique index below serves it</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="54" customHeight="1">
+          <t>Planned (TX-08): unique only among devices not deleted (WHERE deleted_at IS NULL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="27" customHeight="1">
       <c r="A31" s="6" t="n"/>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>uq_telematics_active_vehicle</t>
+          <t>ix_telematics_vehicle_id</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -17281,40 +17360,51 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E31" s="6" t="n"/>
       <c r="F31" s="6" t="inlineStr">
         <is>
+          <t>To be removed (TX-08): the unique index below serves it</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="54" customHeight="1">
+      <c r="A32" s="6" t="n"/>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>uq_telematics_active_vehicle</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
           <t>WHERE deleted_at IS NULL; planned (TX-08): WHERE vehicle_id IS NOT NULL AND deleted_at IS NULL, one device per truck</t>
         </is>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33">
-      <c r="A33" s="4" t="n"/>
-      <c r="B33" s="4" t="inlineStr">
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="4" t="n"/>
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>Được tham chiếu bởi bảng</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="n"/>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>warranties</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>telematic_id</t>
         </is>
       </c>
     </row>
@@ -17322,7 +17412,7 @@
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>telematic_state</t>
+          <t>warranties</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -17335,7 +17425,7 @@
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>vehicle_telemetry</t>
+          <t>telematic_state</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -17348,27 +17438,40 @@
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="7" t="inlineStr">
         <is>
+          <t>vehicle_telemetry</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>telematic_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n"/>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
           <t>telematic_history</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>telematic_id</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A8:I22"/>
+  <autoFilter ref="A8:I23"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'telematic_history'!A1"/>
     <hyperlink ref="A6" location="'telematic_state'!A1"/>
-    <hyperlink ref="F11" location="'organizations'!A1"/>
-    <hyperlink ref="F13" location="'vehicles'!A1"/>
-    <hyperlink ref="B34" location="'warranties'!A1"/>
-    <hyperlink ref="B35" location="'telematic_state'!A1"/>
-    <hyperlink ref="B36" location="'vehicle_telemetry'!A1"/>
-    <hyperlink ref="B37" location="'telematic_history'!A1"/>
+    <hyperlink ref="F12" location="'organizations'!A1"/>
+    <hyperlink ref="F14" location="'vehicles'!A1"/>
+    <hyperlink ref="B35" location="'warranties'!A1"/>
+    <hyperlink ref="B36" location="'telematic_state'!A1"/>
+    <hyperlink ref="B37" location="'vehicle_telemetry'!A1"/>
+    <hyperlink ref="B38" location="'telematic_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17561,12 +17664,12 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>telematic_serial</t>
+          <t>imei</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>varchar(15)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -17578,12 +17681,12 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (telematics.telematic_serial).</t>
+          <t>Giá trị trước khi thay đổi (telematics.imei).</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>TBX-2409-000123</t>
+          <t>356938035643809</t>
         </is>
       </c>
       <c r="I10" s="6" t="n"/>
@@ -17594,12 +17697,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
+          <t>telematic_serial</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -17611,12 +17714,12 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (telematics.organization_id).</t>
+          <t>Giá trị trước khi thay đổi (telematics.telematic_serial).</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+          <t>TBX-2409-000123</t>
         </is>
       </c>
       <c r="I11" s="6" t="n"/>
@@ -17627,12 +17730,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>acquired_at</t>
+          <t>organization_id</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -17644,12 +17747,12 @@
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (telematics.acquired_at).</t>
+          <t>Giá trị trước khi thay đổi (telematics.organization_id).</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>2026-06-01T00:00:00Z</t>
+          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
@@ -17660,12 +17763,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id</t>
+          <t>acquired_at</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -17677,12 +17780,12 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (telematics.vehicle_id).</t>
+          <t>Giá trị trước khi thay đổi (telematics.acquired_at).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
+          <t>2026-06-01T00:00:00Z</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
@@ -17693,12 +17796,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>installed_at</t>
+          <t>vehicle_id</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -17710,12 +17813,12 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (telematics.installed_at).</t>
+          <t>Giá trị trước khi thay đổi (telematics.vehicle_id).</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>2026-06-01T00:00:00Z</t>
+          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
@@ -17726,12 +17829,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>installed_at</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>telematicstatus</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -17743,12 +17846,12 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (telematics.status).</t>
+          <t>Giá trị trước khi thay đổi (telematics.installed_at).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>2026-06-01T00:00:00Z</t>
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
@@ -17759,12 +17862,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>status_reason</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>varchar(200)</t>
+          <t>telematicstatus</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -17776,28 +17879,28 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (telematics.status_reason).</t>
+          <t>Giá trị trước khi thay đổi (telematics.status).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Antenna replaced at the Hanoi workshop</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="I16" s="6" t="n"/>
     </row>
-    <row r="17" ht="27" customHeight="1">
+    <row r="17">
       <c r="A17" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>telemetry_interval_seconds</t>
+          <t>status_reason</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>varchar(200)</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -17809,12 +17912,12 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (telematics.telemetry_interval_seconds).</t>
+          <t>Giá trị trước khi thay đổi (telematics.status_reason).</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>Antenna replaced at the Hanoi workshop</t>
         </is>
       </c>
       <c r="I17" s="6" t="n"/>
@@ -18856,7 +18959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -18894,7 +18997,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Những gì thiết bị tự báo về mình trên topic trạng thái MQTT (quan sát, không phải quyết định): chỉ giá trị mới nhất, không lưu lịch sử thay đổi (TX-08). Được tạo cùng lúc với thiết bị nên mỗi thiết bị luôn có đúng một dòng trạng thái. Thiết bị có trực tuyến hay không được tính từ dữ liệu vận hành (TX-06), không lưu.</t>
+          <t>Những gì thiết bị tự báo về mình trên topic trạng thái MQTT, khoảng mỗi ngày một lần (quan sát, không phải quyết định): firmware, chu kỳ đang dùng, SIM, nguồn điện, sóng, bộ nhớ, GNSS (TX-08, TX-09; các trường của bản tin là tạm thời cho tới khi nhà cung cấp xác nhận). Chỉ giá trị mới nhất, không lưu lịch sử thay đổi. Được tạo cùng lúc với thiết bị nên mỗi thiết bị luôn có đúng một dòng trạng thái. Thiết bị có trực tuyến hay không được tính từ dữ liệu vận hành (TX-06), không lưu.</t>
         </is>
       </c>
     </row>
@@ -18994,7 +19097,7 @@
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9" ht="27" customHeight="1">
+    <row r="9">
       <c r="A9" s="6" t="n">
         <v>2</v>
       </c>
@@ -19017,7 +19120,7 @@
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Phiên bản firmware thiết bị báo gần nhất trên topic trạng thái; NULL trước lần báo đầu tiên.</t>
+          <t>Phiên bản firmware thiết bị báo gần nhất.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -19027,18 +19130,18 @@
       </c>
       <c r="I9" s="6" t="n"/>
     </row>
-    <row r="10" ht="27" customHeight="1">
+    <row r="10" ht="40.5" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>firmware_reported_at</t>
+          <t>reported_telemetry_interval_seconds</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -19050,18 +19153,282 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm thiết bị báo phiên bản đó; NULL trước lần báo đầu tiên.</t>
+          <t>Chu kỳ gửi mà thiết bị báo đang dùng; khác với thiết lập của chủ xe nghĩa là lần đẩy gần nhất chưa được áp dụng (TX-09).</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>sim_iccid</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>varchar(22)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Số ICCID của SIM trong thiết bị; đổi khi thay SIM.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>8984049000001234567</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>is_esim</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>TRUE khi SIM là eSIM.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="27" customHeight="1">
+      <c r="A13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>sim_data_status</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Trạng thái dữ liệu di động của SIM theo báo cáo (giá trị tạm: ACTIVE | NO_DATA | SUSPENDED | NO_SIM).</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>supply_voltage_v</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>numeric(5,2)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Điện áp nguồn cấp tại thiết bị (V).</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>24.30</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>signal_dbm</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>smallint</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Cường độ sóng di động (dBm, càng gần 0 càng mạnh).</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>-78</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>storage_used_percent</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>numeric(5,2)</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Tỷ lệ bộ nhớ thiết bị đã dùng, 0-100.</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>41.50</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="17" ht="27" customHeight="1">
+      <c r="A17" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>gnss_status</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Trạng thái định vị vệ tinh theo báo cáo (giá trị tạm: FIX | NO_FIX | ANTENNA_FAULT).</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="27" customHeight="1">
+      <c r="A18" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>reported_at</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm nhận báo cáo trạng thái gần nhất; mọi cột phía trên lấy từ báo cáo đó. NULL trước lần báo đầu tiên.</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
           <t>2026-09-14T00:30:00Z</t>
         </is>
       </c>
-      <c r="I10" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A7:I10"/>
+  <autoFilter ref="A7:I18"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'telematics'!A1"/>

</xml_diff>

<commit_message>
docs(domain-model): give deleted_at one meaning and assets two statuses
deleted_at now means a row is no longer part of the system (it left or
was entered by mistake), with all data kept and the reason in
status_reason; a soft delete also sets the closing status: INACTIVE for
assets, LOCKED for users, CLOSED for organizations, VOIDED for
warranties. Trucks, batteries and T-Boxes keep only ACTIVE and INACTIVE;
maintenance becomes a reason (DM-25, replaces DM-14).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -8435,7 +8435,7 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Biển số đăng ký. Xe chỉ được đăng ký vào hệ thống khi đã có biển số. Sửa được: biển số định danh theo chủ xe (Thông tư 24/2023/TT-BCA), nên xe sang tên sẽ có biển mới và biển cũ có thể xuất hiện lại trên xe khác; lịch sử thay đổi lưu các biển trước đó. Duy nhất trong các xe chưa xóa và chưa DECOMMISSIONED.</t>
+          <t>Biển số đăng ký. Xe chỉ được đăng ký vào hệ thống khi đã có biển số. Sửa được: biển số định danh theo chủ xe (Thông tư 24/2023/TT-BCA), nên xe sang tên sẽ có biển mới và biển cũ có thể xuất hiện lại trên xe khác; lịch sử thay đổi lưu các biển trước đó. Duy nhất trong các xe chưa xóa, nên biển số của xe đã rời hệ thống có thể chuyển sang xe khác.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -8657,7 +8657,7 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Trạng thái phục vụ, do con người đặt hoặc do quy tắc nghiệp vụ thay mặt công ty, ví dụ trở lại ACTIVE khi hồ sơ sửa chữa được đóng (VH-05, VH-17). ACTIVE: đang phục vụ. MAINTENANCE: đang bảo dưỡng hoặc sửa chữa. DECOMMISSIONED: đã rời hệ thống (thanh lý, bán ra ngoài dịch vụ, hoặc ngừng sử dụng vĩnh viễn); giữ lại cho lịch sử và báo cáo, không nhận dữ liệu mới. Xe đang nhàn rỗi hay không gửi dữ liệu thì không lưu: được tính từ dữ liệu vận hành và T-Box.</t>
+          <t>Trạng thái phục vụ, do con người hoặc quy tắc nghiệp vụ thay mặt công ty đặt (DM-25). ACTIVE: đang phục vụ. INACTIVE: không phục vụ, ví dụ đang ở xưởng hoặc chủ xe không dùng; lý do cho biết trường hợp nào (khi có hồ sơ sửa chữa, việc đang bảo dưỡng được đọc từ hồ sơ sửa chữa đang mở). Xe rời hệ thống được chuyển sang INACTIVE và xóa mềm. Xe đang chạy hay gửi dữ liệu được tính từ dữ liệu vận hành, không lưu.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -8694,7 +8694,7 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Lý do của trạng thái hiện tại; NULL khi ACTIVE.</t>
+          <t>Lý do của trạng thái hiện tại, hoặc lý do xe rời hệ thống; NULL khi ACTIVE.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -8848,7 +8848,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="40.5" customHeight="1">
+    <row r="23" ht="54" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>16</v>
       </c>
@@ -8871,7 +8871,7 @@
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm xóa mềm, chỉ dùng cho xe đăng ký nhầm; xe thật rời hệ thống được chuyển sang DECOMMISSIONED, không bao giờ bị xóa. NULL khi bản ghi còn hiệu lực.</t>
+          <t>Thời điểm xóa mềm: bản ghi không còn thuộc hệ thống, do đã rời đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ, lý do nằm trong status_reason. NULL khi còn thuộc hệ thống.</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -8899,7 +8899,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="40.5" customHeight="1">
+    <row r="26" ht="54" customHeight="1">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="6" t="inlineStr">
         <is>
@@ -8908,7 +8908,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE, INACTIVE (sẽ bỏ), MAINTENANCE, DECOMMISSIONED</t>
+          <t>ACTIVE, INACTIVE, MAINTENANCE (sẽ bỏ), DECOMMISSIONED (sẽ bỏ)</t>
         </is>
       </c>
     </row>
@@ -8994,7 +8994,7 @@
       <c r="E31" s="6" t="n"/>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>Planned (VH-07), replaces the full unique constraint: WHERE deleted_at IS NULL AND status &lt;&gt; 'DECOMMISSIONED'</t>
+          <t>Planned (VH-07), replaces the full unique constraint: WHERE deleted_at IS NULL</t>
         </is>
       </c>
     </row>
@@ -9933,7 +9933,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="27" customHeight="1">
+    <row r="26">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="6" t="inlineStr">
         <is>
@@ -9942,7 +9942,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE, MAINTENANCE, DECOMMISSIONED</t>
+          <t>ACTIVE, INACTIVE</t>
         </is>
       </c>
     </row>
@@ -10365,7 +10365,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="81" customHeight="1">
+    <row r="15" ht="94.5" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>8</v>
       </c>
@@ -10388,7 +10388,7 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Vòng đời tổ chức. ACTIVE: đang sử dụng. SUSPENDED: tạm ngừng (ví dụ nợ cước), chặn đăng nhập nhưng vẫn thu dữ liệu xe, có thể mở lại. CLOSED: không còn hợp đồng, chặn đăng nhập, không nhận dữ liệu mới, dữ liệu được giữ theo thời hạn luật định; chỉ mở lại khi ký hợp đồng mới. Giá trị: ACTIVE | SUSPENDED | CLOSED.</t>
+          <t>Vòng đời tổ chức. ACTIVE: đang sử dụng. SUSPENDED: tạm ngừng (ví dụ nợ cước), chặn đăng nhập nhưng vẫn thu dữ liệu xe, có thể mở lại. CLOSED: đã rời đi (không còn hợp đồng), chặn đăng nhập, không nhận dữ liệu mới, dữ liệu được giữ theo thời hạn luật định; luôn đi cùng deleted_at (DM-25); chỉ mở lại khi ký hợp đồng mới. Giá trị: ACTIVE | SUSPENDED | CLOSED.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -10558,7 +10558,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="40.5" customHeight="1">
+    <row r="20" ht="67.5" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
@@ -10581,7 +10581,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm xóa mềm, chỉ dùng cho tổ chức tạo nhầm; khách hàng hay đối tác thật được chuyển sang CLOSED, không bao giờ bị xóa. NULL khi bản ghi còn hiệu lực.</t>
+          <t>Thời điểm xóa mềm: bản ghi không còn thuộc hệ thống, do đã rời đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ, lý do nằm trong status_reason. NULL khi còn thuộc hệ thống. Tổ chức rời đi được chuyển sang CLOSED và xóa mềm; ký hợp đồng mới thì trở lại ACTIVE và xóa giá trị này.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -11609,7 +11609,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="27" customHeight="1">
+    <row r="17" ht="40.5" customHeight="1">
       <c r="A17" s="6" t="n">
         <v>10</v>
       </c>
@@ -11632,7 +11632,7 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm xóa mềm, chỉ dùng cho dòng xe nhập nhầm; NULL khi bản ghi còn hiệu lực.</t>
+          <t>Thời điểm xóa mềm: dòng này không còn được cung cấp, hoặc nhập nhầm (DM-25); các bản ghi đã trỏ tới vẫn giữ. NULL khi còn cung cấp.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -12788,7 +12788,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="27" customHeight="1">
+    <row r="16" ht="40.5" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>9</v>
       </c>
@@ -12811,7 +12811,7 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm xóa mềm, chỉ dùng cho dòng pin nhập nhầm; NULL khi bản ghi còn hiệu lực.</t>
+          <t>Thời điểm xóa mềm: dòng này không còn được cung cấp, hoặc nhập nhầm (DM-25); các bản ghi đã trỏ tới vẫn giữ. NULL khi còn cung cấp.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -13958,7 +13958,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="67.5" customHeight="1">
+    <row r="16" ht="81" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>9</v>
       </c>
@@ -13981,7 +13981,7 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Trạng thái do con người đặt (VH-16). ACTIVE: dùng được. MAINTENANCE: đang sửa chữa hoặc kiểm tra. DECOMMISSIONED: đã rời hệ thống (tái chế, bán cho mục đích tái sử dụng). Đang lắp hay trong kho không phải trạng thái: đọc từ vehicle_id.</t>
+          <t>Trạng thái do con người đặt (DM-25). ACTIVE: dùng được. INACTIVE: hiện không dùng được, ví dụ đang sửa chữa hoặc kiểm tra; lý do cho biết vì sao. Pin rời hệ thống (tái chế, bán cho mục đích tái sử dụng) được chuyển sang INACTIVE và xóa mềm. Đang lắp hay trong kho không phải trạng thái: đọc từ vehicle_id.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -14106,7 +14106,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="40.5" customHeight="1">
+    <row r="20" ht="54" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
@@ -14129,7 +14129,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm xóa mềm, chỉ dùng cho pin nhập nhầm; pin thật rời hệ thống được chuyển sang DECOMMISSIONED. NULL khi bản ghi còn hiệu lực.</t>
+          <t>Thời điểm xóa mềm: bản ghi không còn thuộc hệ thống, do đã rời đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ, lý do nằm trong status_reason. NULL khi còn thuộc hệ thống.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -15620,7 +15620,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="27" customHeight="1">
+    <row r="21" ht="40.5" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
@@ -15643,7 +15643,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm xóa mềm, chỉ dùng cho bảo hành nhập nhầm; NULL khi bản ghi còn hiệu lực.</t>
+          <t>Thời điểm xóa mềm: bảo hành nhập nhầm và không còn thuộc hệ thống (DM-25); đồng thời bị VOIDED, kèm lý do. NULL khi còn thuộc hệ thống.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -16959,7 +16959,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="81" customHeight="1">
+    <row r="15" ht="94.5" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>8</v>
       </c>
@@ -16982,7 +16982,7 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Trạng thái do con người đặt (TX-08). ACTIVE: dùng được. MAINTENANCE: đang sửa chữa hoặc kiểm tra. DECOMMISSIONED: đã rời hệ thống (thanh lý, trả lại). Đang gắn hay trong kho đọc từ vehicle_id; có gửi dữ liệu hay im lặng được tính từ dữ liệu vận hành (TX-06). Chỉ thiết bị đang gắn và ACTIVE mới nhận cấu hình.</t>
+          <t>Trạng thái do con người đặt (DM-25). ACTIVE: dùng được. INACTIVE: hiện không dùng được, ví dụ đang sửa chữa; lý do cho biết vì sao. Thiết bị rời hệ thống (thanh lý, trả lại) được chuyển sang INACTIVE, tháo khỏi xe và xóa mềm. Đang gắn hay trong kho đọc từ vehicle_id; có gửi dữ liệu hay im lặng được tính từ dữ liệu vận hành (TX-06). Chỉ thiết bị đang gắn và ACTIVE mới nhận cấu hình.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -17229,7 +17229,7 @@
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm xóa mềm, chỉ dùng cho thiết bị nhập nhầm; thiết bị thật rời hệ thống được chuyển sang DECOMMISSIONED và tháo khỏi xe, các xe trước được giữ trong lịch sử (TX-08). NULL khi bản ghi còn hiệu lực.</t>
+          <t>Thời điểm xóa mềm: bản ghi không còn thuộc hệ thống, do đã rời đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ, lý do nằm trong status_reason. NULL khi còn thuộc hệ thống. Các xe trước vẫn nằm trong lịch sử.</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -17257,7 +17257,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="54" customHeight="1">
+    <row r="25" ht="27" customHeight="1">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6" t="inlineStr">
         <is>
@@ -17266,7 +17266,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE, INACTIVE (sẽ bỏ), MAINTENANCE, DECOMMISSIONED (dự kiến)</t>
+          <t>ACTIVE, INACTIVE, MAINTENANCE (sẽ bỏ)</t>
         </is>
       </c>
     </row>
@@ -18134,7 +18134,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="27" customHeight="1">
+    <row r="26">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="6" t="inlineStr">
         <is>
@@ -18143,7 +18143,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE, MAINTENANCE, DECOMMISSIONED</t>
+          <t>ACTIVE, INACTIVE</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="27" customHeight="1">
+    <row r="18" ht="67.5" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>10</v>
       </c>
@@ -25226,7 +25226,7 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm xóa mềm; NULL khi bản ghi còn hiệu lực. Không bao giờ xóa hẳn.</t>
+          <t>Thời điểm xóa mềm: bản ghi không còn thuộc hệ thống, do đã rời đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ, lý do nằm trong status_reason. NULL khi còn thuộc hệ thống. Tài khoản bị xóa cũng bị LOCKED, và số điện thoại, e-mail của nó được dùng lại cho tài khoản mới (ID-28).</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): fix primary key names of the reviewed tables
Eight reviewed tables named their primary key after a shortened noun
(session_id, document_id, audit_id...); they now follow <singular>_id,
and user_consents points to legal_documents through legal_document_id.
DM-17 and database.md note that telematics needs no state split.
Adds open question 7 on erasing personal data on request.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -4606,7 +4606,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>session_id</t>
+          <t>user_session_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -5173,7 +5173,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>code_id</t>
+          <t>one_time_code_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -5679,7 +5679,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>consent_id</t>
+          <t>user_consent_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -5798,7 +5798,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>document_id</t>
+          <t>legal_document_id</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -5818,7 +5818,7 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>legal_documents.document_id (khi xóa: chặn xóa)</t>
+          <t>legal_documents.legal_document_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -5961,12 +5961,12 @@
       <c r="A16" s="6" t="n"/>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>uq_user_consents_person_document</t>
+          <t>uq_user_consents_person_legal_document</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>user_id, document_id</t>
+          <t>user_id, legal_document_id</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -5985,12 +5985,12 @@
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>uq_user_consents_organization_document</t>
+          <t>uq_user_consents_organization_legal_document</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>organization_id, document_id</t>
+          <t>organization_id, legal_document_id</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -6119,7 +6119,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>document_id</t>
+          <t>legal_document_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -6424,7 +6424,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>document_id</t>
+          <t>legal_document_id</t>
         </is>
       </c>
     </row>
@@ -6541,7 +6541,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>assignment_id</t>
+          <t>user_role_assignment_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -7023,7 +7023,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>audit_id</t>
+          <t>access_audit_log_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -19041,13 +19041,13 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="27" customHeight="1">
       <c r="A7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>status_report_id</t>
+          <t>telematic_status_report_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -42090,7 +42090,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>credential_id</t>
+          <t>user_credential_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): write check constraints into table notes
Profile tables may carry a date that describes the object itself, and
check constraints, which DBML cannot express, are written in the table
note (DM-26): the DM-25 status invariants and the warranty's single link.
The telematics vehicle link is noted to become ON DELETE RESTRICT, and
warranties may later split into one table per covered object.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -741,7 +741,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="121.5" customHeight="1">
+    <row r="7" ht="135" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>1</t>
@@ -774,7 +774,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Mọi bên mà người dùng đại diện: khách hàng (doanh nghiệp vận tải và chủ xe cá nhân tự lái), (các) tổ chức nội bộ của chính chúng ta, và đối tác sửa chữa/cứu hộ - tất cả được lưu như nhau. Mọi dữ liệu thuộc một tổ chức đều trỏ về đây qua organization_id; xe của chính chúng ta được sở hữu giống hệt xe của khách hàng. Chỉ is_internal phân biệt các tổ chức về quyền truy cập: người dùng nội bộ xem được dữ liệu của mọi tổ chức, còn lại chỉ xem dữ liệu của chính mình. Không có danh sách người liên hệ riêng: ai cần nhận thông tin (hóa đơn, nhắc nhở, cảnh báo) đều là người dùng giữ vai trò tương ứng. Hợp đồng và gói dịch vụ nằm ở bảng riêng.</t>
+          <t>Mọi bên mà người dùng đại diện: khách hàng (doanh nghiệp vận tải và chủ xe cá nhân tự lái), (các) tổ chức nội bộ của chính chúng ta, và đối tác sửa chữa/cứu hộ - tất cả được lưu như nhau. Mọi dữ liệu thuộc một tổ chức đều trỏ về đây qua organization_id; xe của chính chúng ta được sở hữu giống hệt xe của khách hàng. Chỉ is_internal phân biệt các tổ chức về quyền truy cập: người dùng nội bộ xem được dữ liệu của mọi tổ chức, còn lại chỉ xem dữ liệu của chính mình. Không có danh sách người liên hệ riêng: ai cần nhận thông tin (hóa đơn, nhắc nhở, cảnh báo) đều là người dùng giữ vai trò tương ứng. Hợp đồng và gói dịch vụ nằm ở bảng riêng. Ràng buộc kiểm tra: (status = 'CLOSED') = (deleted_at IS NOT NULL) (DM-25).</t>
         </is>
       </c>
       <c r="H7" s="6" t="n">
@@ -831,7 +831,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="67.5" customHeight="1">
+    <row r="9" ht="81" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>2</t>
@@ -864,7 +864,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Một con người - mỗi người một tài khoản, dùng cho mọi tổ chức mà họ làm việc (một người có thể thuộc nhiều tổ chức, qua bảng memberships): nhân viên khách hàng, tài xế, nhân viên nội bộ hoặc kỹ thuật viên đối tác. Quyền của họ đến từ vai trò (chức danh); thông tin riêng của một công việc (ví dụ bằng lái của tài xế) nằm ở hồ sơ, và vai trò DRIVER cần một hồ sơ tài xế còn hiệu lực.</t>
+          <t>Một con người - mỗi người một tài khoản, dùng cho mọi tổ chức mà họ làm việc (một người có thể thuộc nhiều tổ chức, qua bảng memberships): nhân viên khách hàng, tài xế, nhân viên nội bộ hoặc kỹ thuật viên đối tác. Quyền của họ đến từ vai trò (chức danh); thông tin riêng của một công việc (ví dụ bằng lái của tài xế) nằm ở hồ sơ, và vai trò DRIVER cần một hồ sơ tài xế còn hiệu lực. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'LOCKED' (DM-25).</t>
         </is>
       </c>
       <c r="H9" s="6" t="n">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="40.5" customHeight="1">
+    <row r="24" ht="54" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>13</t>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Hồ sơ của một xe tải điện: xe là gì và các quyết định về xe. Không có bảng trạng thái: mọi thứ xe báo về đi qua T-Box và được lưu từng bản tin trong vehicle_telemetry.</t>
+          <t>Hồ sơ của một xe tải điện: xe là gì và các quyết định về xe. Không có bảng trạng thái: mọi thứ xe báo về đi qua T-Box và được lưu từng bản tin trong vehicle_telemetry. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
         </is>
       </c>
       <c r="H24" s="6" t="n">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Một viên pin vật lý, được quản lý như một tài sản (BAT-01, VH-16). Xe đang lắp pin và chủ sở hữu pin là các cột kèm thời điểm bắt đầu (DM-22); các giai đoạn lấy từ view battery_installation_periods và battery_ownership_periods trên battery_history, mã nguồn không bao giờ đọc trực tiếp bảng lịch sử. Lịch sử sức khỏe của pin qua các xe được ghép từ dữ liệu vận hành với các giai đoạn lắp. Khi bán xe mà bên bán sở hữu pin, pin chuyển sang bên mua trong cùng thao tác chuyển quyền (VH-12); pin thuộc bên khác (ví dụ thuê của G3) vẫn thuộc chủ của nó.</t>
+          <t>Một viên pin vật lý, được quản lý như một tài sản (BAT-01, VH-16). Xe đang lắp pin và chủ sở hữu pin là các cột kèm thời điểm bắt đầu (DM-22); các giai đoạn lấy từ view battery_installation_periods và battery_ownership_periods trên battery_history, mã nguồn không bao giờ đọc trực tiếp bảng lịch sử. Lịch sử sức khỏe của pin qua các xe được ghép từ dữ liệu vận hành với các giai đoạn lắp. Khi bán xe mà bên bán sở hữu pin, pin chuyển sang bên mua trong cùng thao tác chuyển quyền (VH-12); pin thuộc bên khác (ví dụ thuê của G3) vẫn thuộc chủ của nó. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
         </is>
       </c>
       <c r="H31" s="6" t="n">
@@ -1890,7 +1890,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="81" customHeight="1">
+    <row r="34" ht="148.5" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
           <t>17</t>
@@ -1923,7 +1923,7 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Một bảo hành của một xe, pin hoặc T-Box (WAR-01, VH-18), đặt riêng cho từng xe. Đối tượng được bảo hành là liên kết duy nhất có giá trị (đúng một, ràng buộc kiểm tra); liên kết đó cũng quyết định các khóa giới hạn áp dụng. Không có organization_id (DM-24): bảo hành đi theo đối tượng, ai đang sở hữu đối tượng thì xem được. Một xe thường có nhiều bảo hành (xe, pin, gia hạn). Có lưu lịch sử thay đổi: việc hủy bảo hành phải cho biết ai và vì sao.</t>
+          <t>Một bảo hành của một xe, pin hoặc T-Box (WAR-01, VH-18), đặt riêng cho từng xe. Đối tượng được bảo hành là liên kết duy nhất có giá trị (đúng một, ràng buộc kiểm tra); liên kết đó cũng quyết định các khóa giới hạn áp dụng. Không có organization_id (DM-24): bảo hành đi theo đối tượng, ai đang sở hữu đối tượng thì xem được. Một xe thường có nhiều bảo hành (xe, pin, gia hạn). Có lưu lịch sử thay đổi: việc hủy bảo hành phải cho biết ai và vì sao. Ràng buộc kiểm tra: num_nonnulls(vehicle_id, battery_id, telematic_id) = 1 (VH-18); deleted_at IS NULL OR status = 'VOIDED' (DM-25). Các khóa limits hợp lệ theo liên kết được đặt do ứng dụng kiểm tra. Có thể sau này: mỗi loại đối tượng một bảng bảo hành, nằm trong miền của đối tượng đó (bảo hành xe, pin, T-Box), nếu quy định của chúng khác nhau nhiều.</t>
         </is>
       </c>
       <c r="H34" s="6" t="n">
@@ -2003,7 +2003,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="94.5" customHeight="1">
+    <row r="37" ht="108" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
           <t>18</t>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Hồ sơ của một thiết bị telematics (T-Box): thiết bị là gì và các quyết định về nó (TX-08). Thiết bị là một tài sản có chủ riêng, là chủ xe hoặc G3 (TX-07); thiết bị thuộc bên bán đi theo xe khi bán xe. Chủ sở hữu và xe đang gắn là các cột kèm thời điểm bắt đầu (DM-22), các giai đoạn đọc qua view telematic_ownership_periods và telematic_installation_periods. Những gì thiết bị tự báo về mình được lưu trong telematic_status_reports; sức khỏe hiện tại là báo cáo mới nhất (TX-11).</t>
+          <t>Hồ sơ của một thiết bị telematics (T-Box): thiết bị là gì và các quyết định về nó (TX-08). Thiết bị là một tài sản có chủ riêng, là chủ xe hoặc G3 (TX-07); thiết bị thuộc bên bán đi theo xe khi bán xe. Chủ sở hữu và xe đang gắn là các cột kèm thời điểm bắt đầu (DM-22), các giai đoạn đọc qua view telematic_ownership_periods và telematic_installation_periods. Những gì thiết bị tự báo về mình được lưu trong telematic_status_reports; sức khỏe hiện tại là báo cáo mới nhất (TX-11). Ràng buộc kiểm tra: deleted_at IS NULL OR (status = 'INACTIVE' AND vehicle_id IS NULL) (DM-25).</t>
         </is>
       </c>
       <c r="H37" s="6" t="n">
@@ -8234,7 +8234,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Hồ sơ của một xe tải điện: xe là gì và các quyết định về xe. Không có bảng trạng thái: mọi thứ xe báo về đi qua T-Box và được lưu từng bản tin trong vehicle_telemetry.</t>
+          <t>Hồ sơ của một xe tải điện: xe là gì và các quyết định về xe. Không có bảng trạng thái: mọi thứ xe báo về đi qua T-Box và được lưu từng bản tin trong vehicle_telemetry. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
         </is>
       </c>
     </row>
@@ -10047,7 +10047,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Mọi bên mà người dùng đại diện: khách hàng (doanh nghiệp vận tải và chủ xe cá nhân tự lái), (các) tổ chức nội bộ của chính chúng ta, và đối tác sửa chữa/cứu hộ - tất cả được lưu như nhau. Mọi dữ liệu thuộc một tổ chức đều trỏ về đây qua organization_id; xe của chính chúng ta được sở hữu giống hệt xe của khách hàng. Chỉ is_internal phân biệt các tổ chức về quyền truy cập: người dùng nội bộ xem được dữ liệu của mọi tổ chức, còn lại chỉ xem dữ liệu của chính mình. Không có danh sách người liên hệ riêng: ai cần nhận thông tin (hóa đơn, nhắc nhở, cảnh báo) đều là người dùng giữ vai trò tương ứng. Hợp đồng và gói dịch vụ nằm ở bảng riêng.</t>
+          <t>Mọi bên mà người dùng đại diện: khách hàng (doanh nghiệp vận tải và chủ xe cá nhân tự lái), (các) tổ chức nội bộ của chính chúng ta, và đối tác sửa chữa/cứu hộ - tất cả được lưu như nhau. Mọi dữ liệu thuộc một tổ chức đều trỏ về đây qua organization_id; xe của chính chúng ta được sở hữu giống hệt xe của khách hàng. Chỉ is_internal phân biệt các tổ chức về quyền truy cập: người dùng nội bộ xem được dữ liệu của mọi tổ chức, còn lại chỉ xem dữ liệu của chính mình. Không có danh sách người liên hệ riêng: ai cần nhận thông tin (hóa đơn, nhắc nhở, cảnh báo) đều là người dùng giữ vai trò tương ứng. Hợp đồng và gói dịch vụ nằm ở bảng riêng. Ràng buộc kiểm tra: (status = 'CLOSED') = (deleted_at IS NOT NULL) (DM-25).</t>
         </is>
       </c>
     </row>
@@ -13579,7 +13579,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một viên pin vật lý, được quản lý như một tài sản (BAT-01, VH-16). Xe đang lắp pin và chủ sở hữu pin là các cột kèm thời điểm bắt đầu (DM-22); các giai đoạn lấy từ view battery_installation_periods và battery_ownership_periods trên battery_history, mã nguồn không bao giờ đọc trực tiếp bảng lịch sử. Lịch sử sức khỏe của pin qua các xe được ghép từ dữ liệu vận hành với các giai đoạn lắp. Khi bán xe mà bên bán sở hữu pin, pin chuyển sang bên mua trong cùng thao tác chuyển quyền (VH-12); pin thuộc bên khác (ví dụ thuê của G3) vẫn thuộc chủ của nó.</t>
+          <t>Một viên pin vật lý, được quản lý như một tài sản (BAT-01, VH-16). Xe đang lắp pin và chủ sở hữu pin là các cột kèm thời điểm bắt đầu (DM-22); các giai đoạn lấy từ view battery_installation_periods và battery_ownership_periods trên battery_history, mã nguồn không bao giờ đọc trực tiếp bảng lịch sử. Lịch sử sức khỏe của pin qua các xe được ghép từ dữ liệu vận hành với các giai đoạn lắp. Khi bán xe mà bên bán sở hữu pin, pin chuyển sang bên mua trong cùng thao tác chuyển quyền (VH-12); pin thuộc bên khác (ví dụ thuê của G3) vẫn thuộc chủ của nó. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
         </is>
       </c>
     </row>
@@ -15056,7 +15056,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một bảo hành của một xe, pin hoặc T-Box (WAR-01, VH-18), đặt riêng cho từng xe. Đối tượng được bảo hành là liên kết duy nhất có giá trị (đúng một, ràng buộc kiểm tra); liên kết đó cũng quyết định các khóa giới hạn áp dụng. Không có organization_id (DM-24): bảo hành đi theo đối tượng, ai đang sở hữu đối tượng thì xem được. Một xe thường có nhiều bảo hành (xe, pin, gia hạn). Có lưu lịch sử thay đổi: việc hủy bảo hành phải cho biết ai và vì sao.</t>
+          <t>Một bảo hành của một xe, pin hoặc T-Box (WAR-01, VH-18), đặt riêng cho từng xe. Đối tượng được bảo hành là liên kết duy nhất có giá trị (đúng một, ràng buộc kiểm tra); liên kết đó cũng quyết định các khóa giới hạn áp dụng. Không có organization_id (DM-24): bảo hành đi theo đối tượng, ai đang sở hữu đối tượng thì xem được. Một xe thường có nhiều bảo hành (xe, pin, gia hạn). Có lưu lịch sử thay đổi: việc hủy bảo hành phải cho biết ai và vì sao. Ràng buộc kiểm tra: num_nonnulls(vehicle_id, battery_id, telematic_id) = 1 (VH-18); deleted_at IS NULL OR status = 'VOIDED' (DM-25). Các khóa limits hợp lệ theo liên kết được đặt do ứng dụng kiểm tra. Có thể sau này: mỗi loại đối tượng một bảng bảo hành, nằm trong miền của đối tượng đó (bảo hành xe, pin, T-Box), nếu quy định của chúng khác nhau nhiều.</t>
         </is>
       </c>
     </row>
@@ -16625,7 +16625,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Hồ sơ của một thiết bị telematics (T-Box): thiết bị là gì và các quyết định về nó (TX-08). Thiết bị là một tài sản có chủ riêng, là chủ xe hoặc G3 (TX-07); thiết bị thuộc bên bán đi theo xe khi bán xe. Chủ sở hữu và xe đang gắn là các cột kèm thời điểm bắt đầu (DM-22), các giai đoạn đọc qua view telematic_ownership_periods và telematic_installation_periods. Những gì thiết bị tự báo về mình được lưu trong telematic_status_reports; sức khỏe hiện tại là báo cáo mới nhất (TX-11).</t>
+          <t>Hồ sơ của một thiết bị telematics (T-Box): thiết bị là gì và các quyết định về nó (TX-08). Thiết bị là một tài sản có chủ riêng, là chủ xe hoặc G3 (TX-07); thiết bị thuộc bên bán đi theo xe khi bán xe. Chủ sở hữu và xe đang gắn là các cột kèm thời điểm bắt đầu (DM-22), các giai đoạn đọc qua view telematic_ownership_periods và telematic_installation_periods. Những gì thiết bị tự báo về mình được lưu trong telematic_status_reports; sức khỏe hiện tại là báo cáo mới nhất (TX-11). Ràng buộc kiểm tra: deleted_at IS NULL OR (status = 'INACTIVE' AND vehicle_id IS NULL) (DM-25).</t>
         </is>
       </c>
     </row>
@@ -16877,7 +16877,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="40.5" customHeight="1">
+    <row r="13" ht="67.5" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>6</v>
       </c>
@@ -16908,7 +16908,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Xe mà thiết bị đang gắn; NULL khi trong kho hoặc đã tháo. Mỗi xe gắn tối đa một thiết bị. Các xe trước lấy từ view telematic_installation_periods (DM-22).</t>
+          <t>Xe mà thiết bị đang gắn; NULL khi trong kho hoặc đã tháo. Mỗi xe gắn tối đa một thiết bị. Các xe trước lấy từ view telematic_installation_periods (DM-22). Dự kiến: khóa ngoại chuyển sang ON DELETE RESTRICT như mọi liên kết khác (hiện là SET NULL).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -24796,7 +24796,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một con người - mỗi người một tài khoản, dùng cho mọi tổ chức mà họ làm việc (một người có thể thuộc nhiều tổ chức, qua bảng memberships): nhân viên khách hàng, tài xế, nhân viên nội bộ hoặc kỹ thuật viên đối tác. Quyền của họ đến từ vai trò (chức danh); thông tin riêng của một công việc (ví dụ bằng lái của tài xế) nằm ở hồ sơ, và vai trò DRIVER cần một hồ sơ tài xế còn hiệu lực.</t>
+          <t>Một con người - mỗi người một tài khoản, dùng cho mọi tổ chức mà họ làm việc (một người có thể thuộc nhiều tổ chức, qua bảng memberships): nhân viên khách hàng, tài xế, nhân viên nội bộ hoặc kỹ thuật viên đối tác. Quyền của họ đến từ vai trò (chức danh); thông tin riêng của một công việc (ví dụ bằng lái của tài xế) nằm ở hồ sơ, và vai trò DRIVER cần một hồ sơ tài xế còn hiệu lực. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'LOCKED' (DM-25).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(domain-model): define the two period views that have a reader
A views note in the DBML defines vehicle_ownership_periods and
battery_installation_periods: their columns, how they are built from
change history and who reads them. The other three period views wait
until a feature needs them (DM-27).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -632,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1778,7 +1778,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="108" customHeight="1">
+    <row r="31" ht="121.5" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
           <t>16</t>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Một viên pin vật lý, được quản lý như một tài sản (BAT-01, VH-16). Xe đang lắp pin và chủ sở hữu pin là các cột kèm thời điểm bắt đầu (DM-22); các giai đoạn lấy từ view battery_installation_periods và battery_ownership_periods trên battery_history, mã nguồn không bao giờ đọc trực tiếp bảng lịch sử. Lịch sử sức khỏe của pin qua các xe được ghép từ dữ liệu vận hành với các giai đoạn lắp. Khi bán xe mà bên bán sở hữu pin, pin chuyển sang bên mua trong cùng thao tác chuyển quyền (VH-12); pin thuộc bên khác (ví dụ thuê của G3) vẫn thuộc chủ của nó. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
+          <t>Một viên pin vật lý, được quản lý như một tài sản (BAT-01, VH-16). Xe đang lắp pin và chủ sở hữu pin là các cột kèm thời điểm bắt đầu (DM-22); các giai đoạn lắp lấy từ view battery_installation_periods (xem ghi chú views); giai đoạn sở hữu có view khi cần lần đầu (DM-27); mã nguồn không bao giờ đọc trực tiếp bảng lịch sử. Lịch sử sức khỏe của pin qua các xe được ghép từ dữ liệu vận hành với các giai đoạn lắp. Khi bán xe mà bên bán sở hữu pin, pin chuyển sang bên mua trong cùng thao tác chuyển quyền (VH-12); pin thuộc bên khác (ví dụ thuê của G3) vẫn thuộc chủ của nó. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
         </is>
       </c>
       <c r="H31" s="6" t="n">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Hồ sơ của một thiết bị telematics (T-Box): thiết bị là gì và các quyết định về nó (TX-08). Thiết bị là một tài sản có chủ riêng, là chủ xe hoặc G3 (TX-07); thiết bị thuộc bên bán đi theo xe khi bán xe. Chủ sở hữu và xe đang gắn là các cột kèm thời điểm bắt đầu (DM-22), các giai đoạn đọc qua view telematic_ownership_periods và telematic_installation_periods. Những gì thiết bị tự báo về mình được lưu trong telematic_status_reports; sức khỏe hiện tại là báo cáo mới nhất (TX-11). Ràng buộc kiểm tra: deleted_at IS NULL OR (status = 'INACTIVE' AND vehicle_id IS NULL) (DM-25).</t>
+          <t>Hồ sơ của một thiết bị telematics (T-Box): thiết bị là gì và các quyết định về nó (TX-08). Thiết bị là một tài sản có chủ riêng, là chủ xe hoặc G3 (TX-07); thiết bị thuộc bên bán đi theo xe khi bán xe. Chủ sở hữu và xe đang gắn là các cột kèm thời điểm bắt đầu (DM-22), các giai đoạn có view khi có tính năng đầu tiên cần (DM-27). Những gì thiết bị tự báo về mình được lưu trong telematic_status_reports; sức khỏe hiện tại là báo cáo mới nhất (TX-11). Ràng buộc kiểm tra: deleted_at IS NULL OR (status = 'INACTIVE' AND vehicle_id IS NULL) (DM-25).</t>
         </is>
       </c>
       <c r="H37" s="6" t="n">
@@ -4258,39 +4258,113 @@
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t>Các quyết định còn mở</t>
+          <t>Các view (giai đoạn đọc từ lịch sử)</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>Mỗi dòng là</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>Được dùng bởi</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="94.5" customHeight="1">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_ownership_periods</t>
+        </is>
+      </c>
+      <c r="B105" s="6" t="inlineStr">
+        <is>
+          <t>một giai đoạn xe thuộc một chủ</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id, organization_id, owned_from, owned_until (NULL với chủ hiện tại)</t>
+        </is>
+      </c>
+      <c r="D105" s="6" t="inlineStr">
+        <is>
+          <t>lịch sử sở hữu và ngày bàn giao đầu tiên (VEH-02), "ngày đó xe của ai"</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="94.5" customHeight="1">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>battery_installation_periods</t>
+        </is>
+      </c>
+      <c r="B106" s="6" t="inlineStr">
+        <is>
+          <t>một lần pin nằm trên một xe</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>battery_id, vehicle_id, installed_from, installed_until (NULL khi đang lắp)</t>
+        </is>
+      </c>
+      <c r="D106" s="6" t="inlineStr">
+        <is>
+          <t>lịch sử sức khỏe pin qua các xe (MON-07), bộ đếm bảo hành pin (WAR-01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107"/>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t>Các quyết định còn mở</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
           <t>Mã</t>
         </is>
       </c>
-      <c r="B104" s="4" t="inlineStr">
+      <c r="B109" s="4" t="inlineStr">
         <is>
           <t>Câu hỏi</t>
         </is>
       </c>
-      <c r="C104" s="4" t="inlineStr">
+      <c r="C109" s="4" t="inlineStr">
         <is>
           <t>Ảnh hưởng tới</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="54" customHeight="1">
-      <c r="A105" s="6" t="inlineStr">
+    <row r="110" ht="54" customHeight="1">
+      <c r="A110" s="6" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B105" s="6" t="inlineStr">
+      <c r="B110" s="6" t="inlineStr">
         <is>
           <t>Ai trả tiền khi tài xế của đội xe sạc: ví của tài xế, ví của đội xe, hay tùy trường hợp?</t>
         </is>
       </c>
-      <c r="C105" s="6" t="inlineStr">
+      <c r="C110" s="6" t="inlineStr">
         <is>
           <t>wallets, payments</t>
         </is>
@@ -13579,7 +13653,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một viên pin vật lý, được quản lý như một tài sản (BAT-01, VH-16). Xe đang lắp pin và chủ sở hữu pin là các cột kèm thời điểm bắt đầu (DM-22); các giai đoạn lấy từ view battery_installation_periods và battery_ownership_periods trên battery_history, mã nguồn không bao giờ đọc trực tiếp bảng lịch sử. Lịch sử sức khỏe của pin qua các xe được ghép từ dữ liệu vận hành với các giai đoạn lắp. Khi bán xe mà bên bán sở hữu pin, pin chuyển sang bên mua trong cùng thao tác chuyển quyền (VH-12); pin thuộc bên khác (ví dụ thuê của G3) vẫn thuộc chủ của nó. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
+          <t>Một viên pin vật lý, được quản lý như một tài sản (BAT-01, VH-16). Xe đang lắp pin và chủ sở hữu pin là các cột kèm thời điểm bắt đầu (DM-22); các giai đoạn lắp lấy từ view battery_installation_periods (xem ghi chú views); giai đoạn sở hữu có view khi cần lần đầu (DM-27); mã nguồn không bao giờ đọc trực tiếp bảng lịch sử. Lịch sử sức khỏe của pin qua các xe được ghép từ dữ liệu vận hành với các giai đoạn lắp. Khi bán xe mà bên bán sở hữu pin, pin chuyển sang bên mua trong cùng thao tác chuyển quyền (VH-12); pin thuộc bên khác (ví dụ thuê của G3) vẫn thuộc chủ của nó. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
         </is>
       </c>
     </row>
@@ -13757,7 +13831,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="40.5" customHeight="1">
+    <row r="11" ht="54" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>4</v>
       </c>
@@ -13788,7 +13862,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức đang sở hữu pin; có thể khác chủ xe (ví dụ G3 cho thuê pin, deferred.md 88). Các chủ trước lấy từ view battery_ownership_periods.</t>
+          <t>Tổ chức đang sở hữu pin; có thể khác chủ xe (ví dụ G3 cho thuê pin, deferred.md 88). Các chủ trước nằm trong battery_history; view được thêm khi có tính năng đầu tiên cần (DM-27).</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -16625,7 +16699,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Hồ sơ của một thiết bị telematics (T-Box): thiết bị là gì và các quyết định về nó (TX-08). Thiết bị là một tài sản có chủ riêng, là chủ xe hoặc G3 (TX-07); thiết bị thuộc bên bán đi theo xe khi bán xe. Chủ sở hữu và xe đang gắn là các cột kèm thời điểm bắt đầu (DM-22), các giai đoạn đọc qua view telematic_ownership_periods và telematic_installation_periods. Những gì thiết bị tự báo về mình được lưu trong telematic_status_reports; sức khỏe hiện tại là báo cáo mới nhất (TX-11). Ràng buộc kiểm tra: deleted_at IS NULL OR (status = 'INACTIVE' AND vehicle_id IS NULL) (DM-25).</t>
+          <t>Hồ sơ của một thiết bị telematics (T-Box): thiết bị là gì và các quyết định về nó (TX-08). Thiết bị là một tài sản có chủ riêng, là chủ xe hoặc G3 (TX-07); thiết bị thuộc bên bán đi theo xe khi bán xe. Chủ sở hữu và xe đang gắn là các cột kèm thời điểm bắt đầu (DM-22), các giai đoạn có view khi có tính năng đầu tiên cần (DM-27). Những gì thiết bị tự báo về mình được lưu trong telematic_status_reports; sức khỏe hiện tại là báo cáo mới nhất (TX-11). Ràng buộc kiểm tra: deleted_at IS NULL OR (status = 'INACTIVE' AND vehicle_id IS NULL) (DM-25).</t>
         </is>
       </c>
     </row>
@@ -16908,7 +16982,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Xe mà thiết bị đang gắn; NULL khi trong kho hoặc đã tháo. Mỗi xe gắn tối đa một thiết bị. Các xe trước lấy từ view telematic_installation_periods (DM-22). Dự kiến: khóa ngoại chuyển sang ON DELETE RESTRICT như mọi liên kết khác (hiện là SET NULL).</t>
+          <t>Xe mà thiết bị đang gắn; NULL khi trong kho hoặc đã tháo. Mỗi xe gắn tối đa một thiết bị. Các xe trước nằm trong telematic_history; view được thêm khi có tính năng đầu tiên cần (DM-27). Dự kiến: khóa ngoại chuyển sang ON DELETE RESTRICT như mọi liên kết khác (hiện là SET NULL).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): rename vehicle_telemetry to telemetry
The telemetry domain's main table takes the domain's name; the code keeps
vehicle_telemetry until the refactor (TM-15).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -37,7 +37,7 @@
     <sheet name="telematics" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="telematic_history" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="telematic_status_reports" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="vehicle_telemetry" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="telemetry" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="drivers" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="driver_vehicle_assignments" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="driving_sessions" sheetId="34" state="visible" r:id="rId34"/>
@@ -106,7 +106,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'telematics'!$A$7:$I$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'telematic_history'!$A$7:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'telematic_status_reports'!$A$6:$I$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'vehicle_telemetry'!$A$6:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'telemetry'!$A$6:$I$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'drivers'!$A$6:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="32" hidden="1">'driver_vehicle_assignments'!$A$6:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="33" hidden="1">'driving_sessions'!$A$6:$I$17</definedName>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="54" customHeight="1">
+    <row r="24" ht="40.5" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>13</t>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Hồ sơ của một xe tải điện: xe là gì và các quyết định về xe. Không có bảng trạng thái: mọi thứ xe báo về đi qua T-Box và được lưu từng bản tin trong vehicle_telemetry. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
+          <t>Hồ sơ của một xe tải điện: xe là gì và các quyết định về xe. Không có bảng trạng thái: mọi thứ xe báo về đi qua T-Box và được lưu từng bản tin trong telemetry. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
         </is>
       </c>
       <c r="H24" s="6" t="n">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>vehicle_telemetry</t>
+          <t>telemetry</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
@@ -4459,9 +4459,9 @@
     <hyperlink ref="C39" location="'telematic_status_reports'!A1"/>
     <hyperlink ref="D39" location="'telematic_status_reports'!A1"/>
     <hyperlink ref="I39" location="'telematic_status_reports'!A1"/>
-    <hyperlink ref="C41" location="'vehicle_telemetry'!A1"/>
-    <hyperlink ref="D41" location="'vehicle_telemetry'!A1"/>
-    <hyperlink ref="I41" location="'vehicle_telemetry'!A1"/>
+    <hyperlink ref="C41" location="'telemetry'!A1"/>
+    <hyperlink ref="D41" location="'telemetry'!A1"/>
+    <hyperlink ref="I41" location="'telemetry'!A1"/>
     <hyperlink ref="C43" location="'drivers'!A1"/>
     <hyperlink ref="D43" location="'drivers'!A1"/>
     <hyperlink ref="I43" location="'drivers'!A1"/>
@@ -8308,7 +8308,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Hồ sơ của một xe tải điện: xe là gì và các quyết định về xe. Không có bảng trạng thái: mọi thứ xe báo về đi qua T-Box và được lưu từng bản tin trong vehicle_telemetry. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
+          <t>Hồ sơ của một xe tải điện: xe là gì và các quyết định về xe. Không có bảng trạng thái: mọi thứ xe báo về đi qua T-Box và được lưu từng bản tin trong telemetry. Ràng buộc kiểm tra: deleted_at IS NULL OR status = 'INACTIVE' (DM-25).</t>
         </is>
       </c>
     </row>
@@ -8805,7 +8805,7 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: VH-06] Tiến độ kích hoạt thiết bị, thang một chiều không phản ánh việc T-Box bị tháo. Thay bằng tính toán: có thiết bị hiện tại từ telematics, đã nhận dữ liệu từ vehicle_telemetry.</t>
+          <t>[Sẽ bỏ: VH-06] Tiến độ kích hoạt thiết bị, thang một chiều không phản ánh việc T-Box bị tháo. Thay bằng tính toán: có thiết bị hiện tại từ telematics, đã nhận dữ liệu từ telemetry.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -9149,7 +9149,7 @@
       <c r="A38" s="6" t="n"/>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>vehicle_telemetry</t>
+          <t>telemetry</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -9324,7 +9324,7 @@
     <hyperlink ref="B35" location="'batteries'!A1"/>
     <hyperlink ref="B36" location="'warranties'!A1"/>
     <hyperlink ref="B37" location="'telematics'!A1"/>
-    <hyperlink ref="B38" location="'vehicle_telemetry'!A1"/>
+    <hyperlink ref="B38" location="'telemetry'!A1"/>
     <hyperlink ref="B39" location="'driver_vehicle_assignments'!A1"/>
     <hyperlink ref="B40" location="'driving_sessions'!A1"/>
     <hyperlink ref="B41" location="'fleet_vehicle_memberships'!A1"/>
@@ -10866,7 +10866,7 @@
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>vehicle_telemetry</t>
+          <t>telemetry</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -11216,7 +11216,7 @@
     <hyperlink ref="B33" location="'vehicles'!A1"/>
     <hyperlink ref="B34" location="'batteries'!A1"/>
     <hyperlink ref="B35" location="'telematics'!A1"/>
-    <hyperlink ref="B36" location="'vehicle_telemetry'!A1"/>
+    <hyperlink ref="B36" location="'telemetry'!A1"/>
     <hyperlink ref="B37" location="'drivers'!A1"/>
     <hyperlink ref="B38" location="'driver_vehicle_assignments'!A1"/>
     <hyperlink ref="B39" location="'driving_sessions'!A1"/>
@@ -17505,7 +17505,7 @@
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>vehicle_telemetry</t>
+          <t>telemetry</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -17536,7 +17536,7 @@
     <hyperlink ref="F13" location="'vehicles'!A1"/>
     <hyperlink ref="B34" location="'warranties'!A1"/>
     <hyperlink ref="B35" location="'telematic_status_reports'!A1"/>
-    <hyperlink ref="B36" location="'vehicle_telemetry'!A1"/>
+    <hyperlink ref="B36" location="'telemetry'!A1"/>
     <hyperlink ref="B37" location="'telematic_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19638,7 +19638,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>20. vehicle_telemetry: Dữ liệu vận hành xe</t>
+          <t>20. telemetry: Dữ liệu vận hành xe</t>
         </is>
       </c>
     </row>
@@ -20531,7 +20531,7 @@
       <c r="A32" s="6" t="n"/>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>ix_vehicle_telemetry_vehicle_time</t>
+          <t>ix_telemetry_vehicle_time</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -20551,7 +20551,7 @@
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>ix_vehicle_telemetry_vehicle_received</t>
+          <t>ix_telemetry_vehicle_received</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -20575,7 +20575,7 @@
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>ix_vehicle_telemetry_message_uuid</t>
+          <t>ix_telemetry_message_uuid</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): review the telemetry table
Measurement columns carry their unit, organization_id (owner at the time)
is required and the telematic_serial copy goes; a signal becomes a column
only when a feature queries it, otherwise it stays in raw_payload (TM-16).
Telemetry is kept in full for now (TM-17). MON-09 notes the missing
ignition and gear signals.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -2161,7 +2161,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="40.5" customHeight="1">
+    <row r="41" ht="54" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
           <t>20</t>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Một bản ghi dữ liệu xe gửi về, mỗi 5-10 giây một bản ghi cho mỗi xe: bảng lớn nhất hệ thống.</t>
+          <t>Một bản ghi dữ liệu xe gửi về, mỗi 5-10 giây một bản ghi cho mỗi xe: bảng lớn nhất hệ thống. Một tín hiệu chỉ trở thành cột riêng khi có tính năng truy vấn nó; trước đó vẫn nằm trong raw_payload, nơi lưu nguyên vẹn mọi bản tin (TM-16). Mọi dòng đều được giữ; hiện chưa xóa hay nén dữ liệu cũ (TM-17).</t>
         </is>
       </c>
       <c r="H41" s="6" t="n">
@@ -19659,7 +19659,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một bản ghi dữ liệu xe gửi về, mỗi 5-10 giây một bản ghi cho mỗi xe: bảng lớn nhất hệ thống.</t>
+          <t>Một bản ghi dữ liệu xe gửi về, mỗi 5-10 giây một bản ghi cho mỗi xe: bảng lớn nhất hệ thống. Một tín hiệu chỉ trở thành cột riêng khi có tính năng truy vấn nó; trước đó vẫn nằm trong raw_payload, nơi lưu nguyên vẹn mọi bản tin (TM-16). Mọi dòng đều được giữ; hiện chưa xóa hay nén dữ liệu cũ (TM-17).</t>
         </is>
       </c>
     </row>
@@ -19801,7 +19801,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -19923,7 +19923,7 @@
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Serial thiết bị, chép vào dòng để phục vụ kiểm tra và gỡ lỗi.</t>
+          <t>[Sẽ bỏ: TM-16] Serial thiết bị, chép vào dòng để phục vụ kiểm tra và gỡ lỗi.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -20046,7 +20046,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>speed</t>
+          <t>speed_kmh</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -20063,7 +20063,7 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Tốc độ (km/h).</t>
+          <t>[Hiện tên là speed, sẽ đổi tên] Tốc độ (km/h).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -20079,7 +20079,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>heading</t>
+          <t>heading_degrees</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -20096,7 +20096,7 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Hướng di chuyển (độ, 0-360, 0 = hướng bắc); NULL nếu không rõ.</t>
+          <t>[Hiện tên là heading, sẽ đổi tên] Hướng di chuyển (độ, 0-360, 0 = hướng bắc); NULL nếu không rõ.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -20106,13 +20106,13 @@
       </c>
       <c r="I17" s="6" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" ht="27" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>12</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>soc</t>
+          <t>soc_percent</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -20129,7 +20129,7 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Mức pin còn lại (SOC), % (0-100).</t>
+          <t>[Hiện tên là soc, sẽ đổi tên] Mức pin còn lại (SOC), % (0-100).</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -20139,13 +20139,13 @@
       </c>
       <c r="I18" s="6" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" ht="27" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>battery_voltage</t>
+          <t>battery_voltage_v</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -20162,7 +20162,7 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Điện áp pack pin (V).</t>
+          <t>[Hiện tên là battery_voltage, sẽ đổi tên] Điện áp pack pin (V).</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -20172,13 +20172,13 @@
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20">
+    <row r="20" ht="27" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>14</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>battery_current</t>
+          <t>battery_current_a</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -20195,7 +20195,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Dòng điện pack pin (A).</t>
+          <t>[Hiện tên là battery_current, sẽ đổi tên] Dòng điện pack pin (A).</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -20205,13 +20205,13 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21">
+    <row r="21" ht="27" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>15</v>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>battery_temperature</t>
+          <t>battery_temperature_celsius</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -20228,7 +20228,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Nhiệt độ pin (°C).</t>
+          <t>[Hiện tên là battery_temperature, sẽ đổi tên] Nhiệt độ pin (°C).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -20304,13 +20304,13 @@
       </c>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24">
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="6" t="n">
         <v>18</v>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>motor_temperature</t>
+          <t>motor_temperature_celsius</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -20327,7 +20327,7 @@
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Nhiệt độ động cơ (°C).</t>
+          <t>[Hiện tên là motor_temperature, sẽ đổi tên] Nhiệt độ động cơ (°C).</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
@@ -20337,13 +20337,13 @@
       </c>
       <c r="I24" s="6" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" ht="27" customHeight="1">
       <c r="A25" s="6" t="n">
         <v>19</v>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>odometer</t>
+          <t>odometer_km</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -20360,7 +20360,7 @@
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Tổng quãng đường đã chạy (km).</t>
+          <t>[Hiện tên là odometer, sẽ đổi tên] Tổng quãng đường đã chạy (km).</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -20370,13 +20370,13 @@
       </c>
       <c r="I25" s="6" t="n"/>
     </row>
-    <row r="26">
+    <row r="26" ht="27" customHeight="1">
       <c r="A26" s="6" t="n">
         <v>20</v>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>signal_strength</t>
+          <t>signal_dbm</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -20393,7 +20393,7 @@
       <c r="F26" s="6" t="n"/>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Cường độ sóng di động (dBm).</t>
+          <t>[Hiện tên là signal_strength, sẽ đổi tên] Cường độ sóng di động (dBm).</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
@@ -20595,7 +20595,7 @@
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>uq_telematic_recorded_at</t>
+          <t>uq_telemetry_telematic_recorded_at</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): note planned RESTRICT on telemetry's links
telemetry's links to vehicles and telematics are CASCADE today, which
would delete samples with their parent; the target is RESTRICT like
every other link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -20547,7 +20547,7 @@
       <c r="E32" s="6" t="n"/>
       <c r="F32" s="6" t="n"/>
     </row>
-    <row r="33" ht="108" customHeight="1">
+    <row r="33" ht="54" customHeight="1">
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6" t="inlineStr">
         <is>
@@ -20567,7 +20567,7 @@
       <c r="E33" s="6" t="n"/>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Last time the backend heard from a vehicle (F-J1/F-J3 device-health monitor); uses the receive clock, which a skewed device clock cannot move. @vi Lần cuối backend nhận dữ liệu từ xe (giám sát thiết bị F-J1/F-J3); dùng đồng hồ nhận của backend, không bị lệch giờ thiết bị làm sai.</t>
+          <t>Lần cuối backend nhận dữ liệu từ xe (giám sát thiết bị F-J1/F-J3); dùng đồng hồ nhận của backend, không bị lệch giờ thiết bị làm sai.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(domain-model): rename telemetry's device message ID
message_uuid becomes device_message_id: the device's own ID for a message
carries its source as a prefix, not its type; our IDs stay _id whatever
their type (TM-18).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -19826,13 +19826,13 @@
       </c>
       <c r="I9" s="6" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>4</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>message_uuid</t>
+          <t>device_message_id</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -19849,7 +19849,7 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Mã thiết bị gán cho mỗi bản tin, dùng để phát hiện trùng.</t>
+          <t>[Hiện tên là message_uuid, sẽ đổi tên] Mã thiết bị gán cho mỗi bản tin, dùng để phát hiện trùng.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -20575,12 +20575,12 @@
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>ix_telemetry_message_uuid</t>
+          <t>ix_telemetry_device_message_id</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>message_uuid</t>
+          <t>device_message_id</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): review the charging sessions table
A session row is now created PENDING at the QR scan, with the paying
organization, the scanning user and the single-use token sent in the remote
start; the charger's start message carrying that token on the same charger
turns it ACTIVE, and any other token is refused (CE-10, CE-11, replacing
CO-06). The truck comes from the driver's open driving session (CE-13). The
session keeps only the meter readings the charger declares; the latest
reading and the energy delivered are derived and dropped (CE-12).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -137,7 +137,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="50" hidden="1">'charging_ocpp_messages'!$A$6:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="51" hidden="1">'charging_station_config_capture'!$A$6:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="52" hidden="1">'charging_station_config_entries'!$A$6:$I$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="53" hidden="1">'charging_sessions'!$A$6:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="53" hidden="1">'charging_sessions'!$A$6:$I$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="54" hidden="1">'charging_session_events'!$A$6:$I$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="55" hidden="1">'charging_session_measurements'!$A$6:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="56" hidden="1">'notifications'!$A$6:$I$16</definedName>
@@ -3303,13 +3303,13 @@
       <c r="G67" s="5" t="inlineStr">
         <is>
           <t>Những gì diễn ra trong mỗi lần sạc: sự kiện, chỉ số công tơ, điện năng đã cấp.
-• Một phiên sạc diễn ra trên một súng sạc của một trạm G3.
-• Khoảng trống hiện nay: phiên sạc chưa gắn với xe, tài xế hay khách hàng nào, chỉ có mã id_tag thô. Lúc ra mắt mọi lần sạc đều bắt đầu bằng quét mã QR (CO-13), nên phiên sạc sẽ ghi người khởi động và tổ chức thanh toán (thiết kế khi rà soát charging_sessions); thanh toán (F-H1/F-H3) và đối soát (NF-10) cần liên kết này.
+• Một phiên sạc diễn ra trên một súng sạc của một trụ. Phiên được tạo khi tài xế quét mã QR trên trụ bằng ứng dụng của chúng ta (CE-10) và ghi người quét, tổ chức trả tiền và, nếu tài xế đang nhận một xe, chiếc xe đó; sau đó bản tin bắt đầu của trụ điền súng sạc và giao dịch (CE-11).
+• Bản đang chạy chưa có liên kết này (chỉ có mã id_tag thô); sẽ có khi tái cấu trúc.
 • Một phiên sạc có nhiều sự kiện và nhiều số đo.</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="67.5" customHeight="1">
+    <row r="68" ht="148.5" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
           <t>38</t>
@@ -3342,11 +3342,11 @@
       </c>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>Một lần sạc trên một súng sạc, từ lúc bắt đầu đến lúc kết thúc. Cần quyết định khi rà soát bảng (CS-18): lần sạc bằng QR (CO-14) cần lưu ngữ cảnh nghiệp vụ ngay khi tài xế quét (ai quét, tổ chức nào trả tiền, mã gửi trong RemoteStartTransaction, câu trả lời của trụ) để ghép với StartTransaction mang mã đó: tạo dòng phiên PENDING khi quét, một bảng các lệnh gửi xuống trụ, hoặc cả hai.</t>
+          <t>Một lần sạc trên một súng của một trụ, từ lúc quét mã QR đến lúc dừng (CE-10). Dòng được tạo ở trạng thái PENDING khi tài xế quét mã QR trong ứng dụng của chúng ta, cùng tổ chức trả tiền, người quét và mã dùng một lần gửi trong lệnh bắt đầu từ xa; bản tin bắt đầu của chính trụ đó mang mã này chuyển phiên sang ACTIVE (CE-11), bản tin dừng chuyển sang COMPLETED; ABANDONED khi lần bắt đầu không xảy ra. Số liệu trực tiếp (kWh đã sạc, % pin, công suất cao nhất) đọc từ charging_session_measurements; đơn giá và số tiền thuộc bản ghi thanh toán (PAY-10). Không có lịch sử thay đổi và không xóa mềm: không ai sửa một phiên sạc. Ràng buộc kiểm tra (CE-10): phiên ACTIVE hoặc COMPLETED phải có mã giao dịch, EVSE, súng, thời điểm bắt đầu và chỉ số công tơ đầu; phiên COMPLETED phải có thời điểm kết thúc; phiên PENDING hoặc ABANDONED không có mã giao dịch.</t>
         </is>
       </c>
       <c r="H68" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I68" s="7" t="inlineStr">
         <is>
@@ -25610,7 +25610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -26391,12 +26391,12 @@
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>charging_policy_versions</t>
+          <t>charging_sessions</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>started_by</t>
         </is>
       </c>
     </row>
@@ -26404,12 +26404,12 @@
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>organization_history</t>
+          <t>charging_policy_versions</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>changed_by</t>
+          <t>created_by</t>
         </is>
       </c>
     </row>
@@ -26417,12 +26417,12 @@
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>user_history</t>
+          <t>organization_history</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>changed_by</t>
         </is>
       </c>
     </row>
@@ -26435,7 +26435,7 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>changed_by</t>
+          <t>user_id</t>
         </is>
       </c>
     </row>
@@ -26443,7 +26443,7 @@
       <c r="A45" s="6" t="n"/>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>membership_history</t>
+          <t>user_history</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -26452,11 +26452,11 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="27" customHeight="1">
+    <row r="46">
       <c r="A46" s="6" t="n"/>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>organization_setting_history</t>
+          <t>membership_history</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -26465,11 +26465,11 @@
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="27" customHeight="1">
       <c r="A47" s="6" t="n"/>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>vehicle_history</t>
+          <t>organization_setting_history</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -26482,7 +26482,7 @@
       <c r="A48" s="6" t="n"/>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>vehicle_model_history</t>
+          <t>vehicle_history</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -26495,7 +26495,7 @@
       <c r="A49" s="6" t="n"/>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>battery_model_history</t>
+          <t>vehicle_model_history</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -26508,7 +26508,7 @@
       <c r="A50" s="6" t="n"/>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>battery_history</t>
+          <t>battery_model_history</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -26521,7 +26521,7 @@
       <c r="A51" s="6" t="n"/>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>warranty_history</t>
+          <t>battery_history</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -26534,7 +26534,7 @@
       <c r="A52" s="6" t="n"/>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>telematic_history</t>
+          <t>warranty_history</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -26547,7 +26547,7 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>driver_history</t>
+          <t>telematic_history</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -26556,11 +26556,11 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="27" customHeight="1">
+    <row r="54">
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>charging_location_history</t>
+          <t>driver_history</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -26569,11 +26569,11 @@
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="27" customHeight="1">
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>charging_station_history</t>
+          <t>charging_location_history</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -26586,7 +26586,7 @@
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>charging_evse_history</t>
+          <t>charging_station_history</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -26595,14 +26595,27 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="27" customHeight="1">
+    <row r="57">
       <c r="A57" s="6" t="n"/>
       <c r="B57" s="7" t="inlineStr">
         <is>
+          <t>charging_evse_history</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>changed_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="27" customHeight="1">
+      <c r="A58" s="6" t="n"/>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
           <t>charging_connector_history</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>changed_by</t>
         </is>
@@ -26631,23 +26644,24 @@
     <hyperlink ref="B38" location="'access_audit_logs'!A1"/>
     <hyperlink ref="B39" location="'charging_location_access'!A1"/>
     <hyperlink ref="B40" location="'charging_location_access'!A1"/>
-    <hyperlink ref="B41" location="'charging_policy_versions'!A1"/>
-    <hyperlink ref="B42" location="'organization_history'!A1"/>
-    <hyperlink ref="B43" location="'user_history'!A1"/>
+    <hyperlink ref="B41" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B42" location="'charging_policy_versions'!A1"/>
+    <hyperlink ref="B43" location="'organization_history'!A1"/>
     <hyperlink ref="B44" location="'user_history'!A1"/>
-    <hyperlink ref="B45" location="'membership_history'!A1"/>
-    <hyperlink ref="B46" location="'organization_setting_history'!A1"/>
-    <hyperlink ref="B47" location="'vehicle_history'!A1"/>
-    <hyperlink ref="B48" location="'vehicle_model_history'!A1"/>
-    <hyperlink ref="B49" location="'battery_model_history'!A1"/>
-    <hyperlink ref="B50" location="'battery_history'!A1"/>
-    <hyperlink ref="B51" location="'warranty_history'!A1"/>
-    <hyperlink ref="B52" location="'telematic_history'!A1"/>
-    <hyperlink ref="B53" location="'driver_history'!A1"/>
-    <hyperlink ref="B54" location="'charging_location_history'!A1"/>
-    <hyperlink ref="B55" location="'charging_station_history'!A1"/>
-    <hyperlink ref="B56" location="'charging_evse_history'!A1"/>
-    <hyperlink ref="B57" location="'charging_connector_history'!A1"/>
+    <hyperlink ref="B45" location="'user_history'!A1"/>
+    <hyperlink ref="B46" location="'membership_history'!A1"/>
+    <hyperlink ref="B47" location="'organization_setting_history'!A1"/>
+    <hyperlink ref="B48" location="'vehicle_history'!A1"/>
+    <hyperlink ref="B49" location="'vehicle_model_history'!A1"/>
+    <hyperlink ref="B50" location="'battery_model_history'!A1"/>
+    <hyperlink ref="B51" location="'battery_history'!A1"/>
+    <hyperlink ref="B52" location="'warranty_history'!A1"/>
+    <hyperlink ref="B53" location="'telematic_history'!A1"/>
+    <hyperlink ref="B54" location="'driver_history'!A1"/>
+    <hyperlink ref="B55" location="'charging_location_history'!A1"/>
+    <hyperlink ref="B56" location="'charging_station_history'!A1"/>
+    <hyperlink ref="B57" location="'charging_evse_history'!A1"/>
+    <hyperlink ref="B58" location="'charging_connector_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -36278,7 +36292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -36316,7 +36330,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một lần sạc trên một súng sạc, từ lúc bắt đầu đến lúc kết thúc. Cần quyết định khi rà soát bảng (CS-18): lần sạc bằng QR (CO-14) cần lưu ngữ cảnh nghiệp vụ ngay khi tài xế quét (ai quét, tổ chức nào trả tiền, mã gửi trong RemoteStartTransaction, câu trả lời của trụ) để ghép với StartTransaction mang mã đó: tạo dòng phiên PENDING khi quét, một bảng các lệnh gửi xuống trụ, hoặc cả hai.</t>
+          <t>Một lần sạc trên một súng của một trụ, từ lúc quét mã QR đến lúc dừng (CE-10). Dòng được tạo ở trạng thái PENDING khi tài xế quét mã QR trong ứng dụng của chúng ta, cùng tổ chức trả tiền, người quét và mã dùng một lần gửi trong lệnh bắt đầu từ xa; bản tin bắt đầu của chính trụ đó mang mã này chuyển phiên sang ACTIVE (CE-11), bản tin dừng chuyển sang COMPLETED; ABANDONED khi lần bắt đầu không xảy ra. Số liệu trực tiếp (kWh đã sạc, % pin, công suất cao nhất) đọc từ charging_session_measurements; đơn giá và số tiền thuộc bản ghi thanh toán (PAY-10). Không có lịch sử thay đổi và không xóa mềm: không ai sửa một phiên sạc. Ràng buộc kiểm tra (CE-10): phiên ACTIVE hoặc COMPLETED phải có mã giao dịch, EVSE, súng, thời điểm bắt đầu và chỉ số công tơ đầu; phiên COMPLETED phải có thời điểm kết thúc; phiên PENDING hoặc ABANDONED không có mã giao dịch.</t>
         </is>
       </c>
     </row>
@@ -36436,7 +36450,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Trạm diễn ra phiên sạc.</t>
+          <t>Trụ sạc nơi diễn ra phiên sạc, biết được từ mã QR khi quét.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -36446,7 +36460,7 @@
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9" ht="27" customHeight="1">
+    <row r="9" ht="54" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
@@ -36477,7 +36491,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>EVSE được dùng.</t>
+          <t>EVSE được dùng, lấy từ bản tin bắt đầu của trụ. Dự kiến (CE-10): cho phép NULL, NULL khi PENDING và với phiên ABANDONED, vì tài xế chọn súng trên màn hình trụ sau khi quét (CO-14).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -36487,7 +36501,7 @@
       </c>
       <c r="I9" s="6" t="n"/>
     </row>
-    <row r="10" ht="27" customHeight="1">
+    <row r="10" ht="40.5" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>4</v>
       </c>
@@ -36518,7 +36532,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Súng sạc được dùng.</t>
+          <t>Súng sạc được dùng, lấy từ bản tin bắt đầu của trụ. Dự kiến (CE-10): cho phép NULL, NULL khi PENDING và với phiên ABANDONED.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -36528,7 +36542,7 @@
       </c>
       <c r="I10" s="6" t="n"/>
     </row>
-    <row r="11" ht="27" customHeight="1">
+    <row r="11" ht="40.5" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
@@ -36544,7 +36558,7 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -36559,7 +36573,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức khách hàng bị tính tiền cho phiên sạc. (xem quyết định D5)</t>
+          <t>Tổ chức trả tiền: tổ chức mà người quét mã đại diện, ghi một lần khi quét và không đổi (DM-24 trường hợp C). Ví nào trong tổ chức trả tiền là câu hỏi mở D5.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -36569,13 +36583,13 @@
       </c>
       <c r="I11" s="6" t="n"/>
     </row>
-    <row r="12" ht="27" customHeight="1">
+    <row r="12" ht="40.5" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id</t>
+          <t>started_by</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -36585,7 +36599,7 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -36595,66 +36609,74 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>vehicles.vehicle_id (khi xóa: chặn xóa)</t>
+          <t>users.user_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Xe được sạc.</t>
+          <t>Người dùng đã quét mã QR trong ứng dụng của chúng ta; mọi lần sạc đều bắt đầu như vậy (CO-13). Lần bắt đầu mang mã không do chúng ta cấp bị từ chối và không tạo dòng (CE-11).</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
+          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="54" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>ocpp_transaction_id</t>
+          <t>vehicle_id</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>varchar(255)</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>vehicles.vehicle_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Mã giao dịch dùng với trụ sạc, duy nhất trong trạm.</t>
+          <t>Xe được sạc, lấy khi quét mã từ phiên lái đang mở của tài xế quét mã (CHG-07); NULL nếu không có (xe khách vãng lai chưa có hồ sơ, hoặc tài xế chưa nhận xe). Sau này có thể lấy từ VIN hoặc địa chỉ MAC do trụ báo (deferred.md 90).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>1042</t>
+          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
     </row>
-    <row r="14" ht="27" customHeight="1">
+    <row r="14" ht="67.5" customHeight="1">
       <c r="A14" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>ocpp_transaction_id</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>chargingsessionstatus</t>
+          <t>varchar(255)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -36666,28 +36688,28 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Phiên sạc còn đang chạy hay đã xong.</t>
+          <t>Mã giao dịch của trụ, duy nhất trong mỗi trụ: trụ OCPP 2.0.1 tự chọn (chuỗi tối đa 36 ký tự); với 1.6J là số thứ tự của chúng ta dạng chữ (CE-03). Dự kiến (CE-10): varchar(36) và cho phép NULL, NULL khi PENDING và với phiên ABANDONED.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>1042</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="94.5" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>started_at</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>chargingsessionstatus</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -36699,23 +36721,23 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm bắt đầu sạc.</t>
+          <t>Vòng đời của phiên; là trạng thái quan sát được nên không có status_reason (DM-19). PENDING: đã nhận lượt quét, chờ trụ. ACTIVE: giao dịch đang chạy. COMPLETED: trụ đã dừng. ABANDONED: lệnh bắt đầu từ xa bị từ chối hoặc hết thời gian chờ, hoặc không có giao dịch nào trong khoảng thời gian cấu hình. Dự kiến (CE-10): giá trị viết hoa; PENDING và ABANDONED là giá trị mới.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>2026-09-15T08:30:00Z</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="40.5" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>ended_at</t>
+          <t>started_at</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -36725,35 +36747,35 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm kết thúc sạc; NULL khi đang sạc.</t>
+          <t>Thời điểm bắt đầu theo đồng hồ của trụ. Dự kiến (CE-10): cho phép NULL, NULL khi PENDING và với phiên ABANDONED; thời điểm quét mã là created_at.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>2026-09-15T09:45:00Z</t>
+          <t>2026-09-15T08:30:00Z</t>
         </is>
       </c>
       <c r="I16" s="6" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" ht="27" customHeight="1">
       <c r="A17" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>meter_start_wh</t>
+          <t>ended_at</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>numeric(24,3)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -36765,23 +36787,23 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Chỉ số công tơ của trụ lúc bắt đầu (Wh).</t>
+          <t>Thời điểm dừng theo đồng hồ của trụ; NULL cho đến khi COMPLETED.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>1520340.000</t>
+          <t>2026-09-15T09:45:00Z</t>
         </is>
       </c>
       <c r="I17" s="6" t="n"/>
     </row>
-    <row r="18" ht="27" customHeight="1">
+    <row r="18">
       <c r="A18" s="6" t="n">
         <v>12</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>meter_end_wh</t>
+          <t>meter_start_wh</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -36798,28 +36820,28 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Chỉ số công tơ mới nhất được chấp nhận (Wh), không bao giờ lùi về thời gian trước.</t>
+          <t>Chỉ số công tơ trụ báo lúc bắt đầu (Wh); NULL khi PENDING.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>1712840.000</t>
+          <t>1520340.000</t>
         </is>
       </c>
       <c r="I18" s="6" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" ht="40.5" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>meter_end_sampled_at</t>
+          <t>meter_end_wh</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>numeric(24,3)</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -36831,28 +36853,28 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm đo meter_end_wh.</t>
+          <t>[Sẽ bỏ: CE-12] Chỉ số công tơ mới nhất được chấp nhận (Wh); là bản sao của số đo điện năng mới nhất trong charging_session_measurements, nay đọc ở đó.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>2026-09-15T09:44:30Z</t>
+          <t>1712840.000</t>
         </is>
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20">
+    <row r="20" ht="27" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>14</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>energy_delivered_wh</t>
+          <t>meter_end_sampled_at</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>numeric(24,3)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -36864,28 +36886,28 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Điện năng đã cấp: chỉ số cuối trừ chỉ số đầu (Wh).</t>
+          <t>[Sẽ bỏ: CE-12] Thời điểm đo meter_end_wh; là sampled_at của số đo mới nhất.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>192500.000</t>
+          <t>2026-09-15T09:44:30Z</t>
         </is>
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="27" customHeight="1">
+    <row r="21" ht="40.5" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>15</v>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>id_tag</t>
+          <t>energy_delivered_wh</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>numeric(24,3)</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -36897,28 +36919,28 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Mã định danh thô (RFID/token) đã bắt đầu phiên, đúng như trụ gửi; chưa được xác thực.</t>
+          <t>[Sẽ bỏ: CE-12] Giá trị suy ra: meter_stop_wh trừ meter_start_wh, tính khi đọc; số kWh tính tiền được chốt trên bản ghi thanh toán (PAY-10).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>04A1B2C3D4E5F6</t>
+          <t>192500.000</t>
         </is>
       </c>
       <c r="I21" s="6" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="108" customHeight="1">
       <c r="A22" s="6" t="n">
         <v>16</v>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>stop_reason</t>
+          <t>id_token</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>varchar(30)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -36930,28 +36952,28 @@
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Lý do dừng sạc, theo trụ sạc báo.</t>
+          <t>[Hiện tên là id_tag, sẽ đổi tên] Mã định danh trụ báo cho giao dịch. Với lần sạc bằng QR, đó là mã dùng một lần chúng ta tạo khi quét và gửi trong lệnh bắt đầu từ xa (tối đa 20 ký tự, giới hạn idTag của OCPP 1.6J); trụ gửi lại mã này trong bản tin bắt đầu, nhờ đó bản tin tìm được dòng này (CE-11). Sau này còn là số thẻ hoặc mã Autocharge (CHG-08); không bao giờ chép vào log ứng dụng (IS-07). Dự kiến (CE-10): varchar(255) (độ dài của OCPP 2.1) và bắt buộc.</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>EVDisconnected</t>
+          <t>G3K7Q2M9X4T1</t>
         </is>
       </c>
       <c r="I22" s="6" t="n"/>
     </row>
-    <row r="23">
+    <row r="23" ht="54" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>17</v>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>meter_stop_wh</t>
+          <t>stop_reason</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>numeric(24,3)</t>
+          <t>varchar(30)</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -36963,56 +36985,56 @@
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Chỉ số công tơ lúc kết thúc do chính trụ sạc báo (Wh).</t>
+          <t>Lý do dừng theo trụ báo, giữ nguyên (reason của 1.6J, stoppedReason của 2.0.1); NULL nếu chưa COMPLETED. Lý do phiên bị ABANDONED không lưu ở đây mà thuộc về bản ghi lệnh bắt đầu từ xa chúng ta đã gửi (CS-18).</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>1712860.000</t>
+          <t>EVDisconnected</t>
         </is>
       </c>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24">
+    <row r="24" ht="54" customHeight="1">
       <c r="A24" s="6" t="n">
         <v>18</v>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>meter_stop_wh</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>numeric(24,3)</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
+          <t>Chỉ số công tơ trụ báo trong bản tin dừng (Wh): con số dùng để tính tiền (CE-12), luôn lưu đúng như trụ gửi (CE-03). NULL cho đến khi COMPLETED, hoặc khi bản tin dừng không có; khi đó tính tiền theo số đo mới nhất.</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>2026-09-15T08:30:00Z</t>
+          <t>1712860.000</t>
         </is>
       </c>
       <c r="I24" s="6" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" ht="27" customHeight="1">
       <c r="A25" s="6" t="n">
         <v>19</v>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -37029,98 +37051,111 @@
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
+          <t>Thời điểm tạo bản ghi (UTC): là thời điểm quét mã với lần sạc bằng QR.</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
+          <t>2026-09-15T08:29:10Z</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="n"/>
+    </row>
+    <row r="26" ht="27" customHeight="1">
+      <c r="A26" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC); thay đổi ở mỗi bước của phiên.</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
           <t>2026-09-15T09:45:00Z</t>
         </is>
       </c>
-      <c r="I25" s="6" t="n"/>
-    </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="4" t="n"/>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="I26" s="6" t="n"/>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="4" t="n"/>
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Kiểu enum</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Giá trị cho phép</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="6" t="inlineStr">
+    <row r="29" ht="81" customHeight="1">
+      <c r="A29" s="6" t="n"/>
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>chargingsessionstatus</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>active, completed</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30" s="4" t="n"/>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>active (sẽ bỏ), completed (sẽ bỏ), PENDING (dự kiến), ACTIVE (dự kiến), COMPLETED (dự kiến), ABANDONED (dự kiến)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="4" t="n"/>
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="27" customHeight="1">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>ix_charging_sessions_ended_at</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>ended_at</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n"/>
     </row>
     <row r="32" ht="27" customHeight="1">
       <c r="A32" s="6" t="n"/>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>ix_charging_sessions_status_updated</t>
+          <t>ix_charging_sessions_ended_at</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>status, updated_at</t>
+          <t>ended_at</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -37135,12 +37170,12 @@
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>ix_charging_sessions_station_status</t>
+          <t>ix_charging_sessions_status_updated</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>station_id, status</t>
+          <t>status, updated_at</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -37155,12 +37190,12 @@
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>ix_charging_sessions_evse_status</t>
+          <t>ix_charging_sessions_station_status</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>evse_id, status</t>
+          <t>station_id, status</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -37175,12 +37210,12 @@
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>ix_charging_sessions_connector_status</t>
+          <t>ix_charging_sessions_evse_status</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>connector_id, status</t>
+          <t>evse_id, status</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -37195,12 +37230,12 @@
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>ix_charging_sessions_started_at</t>
+          <t>ix_charging_sessions_connector_status</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>started_at</t>
+          <t>connector_id, status</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -37215,85 +37250,129 @@
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>uq_charging_sessions_station_transaction</t>
+          <t>ix_charging_sessions_started_at</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>station_id, ocpp_transaction_id</t>
+          <t>started_at</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E37" s="6" t="n"/>
       <c r="F37" s="6" t="n"/>
     </row>
-    <row r="38"/>
-    <row r="39">
-      <c r="A39" s="4" t="n"/>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
+    <row r="38" ht="27" customHeight="1">
+      <c r="A38" s="6" t="n"/>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>uq_charging_sessions_station_transaction</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>station_id, ocpp_transaction_id</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="n"/>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Planned (CE-10): partial, WHERE ocpp_transaction_id IS NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="40.5" customHeight="1">
+      <c r="A39" s="6" t="n"/>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>ix_charging_sessions_pending_token</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>station_id, id_token</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="n"/>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>Planned (CE-11): WHERE status = 'PENDING'; matches a start message to its scan</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="27" customHeight="1">
       <c r="A40" s="6" t="n"/>
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t>charging_session_events</t>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>ix_charging_sessions_organization_started</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>session_id</t>
+          <t>organization_id, started_at</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>Planned (CE-10): a customer's charging history (CHG-04)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="27" customHeight="1">
       <c r="A41" s="6" t="n"/>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>charging_session_measurements</t>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>ix_charging_sessions_vehicle_id</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>session_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="n"/>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>policy_violations</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>session_id</t>
-        </is>
-      </c>
-    </row>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>Planned (CE-13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
     <row r="43">
-      <c r="A43" s="6" t="n"/>
-      <c r="B43" s="7" t="inlineStr">
-        <is>
-          <t>payments</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>session_id</t>
+      <c r="A43" s="4" t="n"/>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
         </is>
       </c>
     </row>
@@ -37301,7 +37380,7 @@
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>wallet_transactions</t>
+          <t>charging_session_events</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -37310,34 +37389,87 @@
         </is>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="27" customHeight="1">
       <c r="A45" s="6" t="n"/>
       <c r="B45" s="7" t="inlineStr">
         <is>
+          <t>charging_session_measurements</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>session_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n"/>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>policy_violations</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>session_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n"/>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>payments</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>session_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n"/>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>wallet_transactions</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>session_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n"/>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
           <t>invoice_lines</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>session_id</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I25"/>
+  <autoFilter ref="A6:I26"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F8" location="'charging_stations'!A1"/>
     <hyperlink ref="F9" location="'charging_evses'!A1"/>
     <hyperlink ref="F10" location="'charging_connectors'!A1"/>
     <hyperlink ref="F11" location="'organizations'!A1"/>
-    <hyperlink ref="F12" location="'vehicles'!A1"/>
-    <hyperlink ref="B40" location="'charging_session_events'!A1"/>
-    <hyperlink ref="B41" location="'charging_session_measurements'!A1"/>
-    <hyperlink ref="B42" location="'policy_violations'!A1"/>
-    <hyperlink ref="B43" location="'payments'!A1"/>
-    <hyperlink ref="B44" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="B45" location="'invoice_lines'!A1"/>
+    <hyperlink ref="F12" location="'users'!A1"/>
+    <hyperlink ref="F13" location="'vehicles'!A1"/>
+    <hyperlink ref="B44" location="'charging_session_events'!A1"/>
+    <hyperlink ref="B45" location="'charging_session_measurements'!A1"/>
+    <hyperlink ref="B46" location="'policy_violations'!A1"/>
+    <hyperlink ref="B47" location="'payments'!A1"/>
+    <hyperlink ref="B48" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="B49" location="'invoice_lines'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(domain-model): review the charging session measurements table
The gateway stores every known measurand in one fixed unit and fills the
OCPP defaults for a missing context (Sample.Periodic) or location (Outlet),
so both become required; location is renamed measurement_location. Readings
outside a session stay in the raw log only (CE-14).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -3399,7 +3399,7 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="27" customHeight="1">
+    <row r="70" ht="67.5" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
           <t>40</t>
@@ -3432,7 +3432,7 @@
       </c>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>Mọi giá trị đo trụ sạc gửi trong phiên (điện năng, công suất, SOC...).</t>
+          <t>Mọi giá trị đo trụ sạc gửi trong phiên (điện năng, công suất, dòng điện, điện áp, SoC, nhiệt độ...), chỉ ghi thêm. Cổng OCPP lưu mỗi đại lượng đã biết theo một đơn vị cố định và điền giá trị mặc định của OCPP khi thiếu context hoặc điểm đo, nên nơi đọc không phải đổi đơn vị hay đoán giá trị mặc định (CE-14). Không có lịch sử thay đổi và không xóa mềm.</t>
         </is>
       </c>
       <c r="H70" s="6" t="n">
@@ -37878,7 +37878,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Mọi giá trị đo trụ sạc gửi trong phiên (điện năng, công suất, SOC...).</t>
+          <t>Mọi giá trị đo trụ sạc gửi trong phiên (điện năng, công suất, dòng điện, điện áp, SoC, nhiệt độ...), chỉ ghi thêm. Cổng OCPP lưu mỗi đại lượng đã biết theo một đơn vị cố định và điền giá trị mặc định của OCPP khi thiếu context hoặc điểm đo, nên nơi đọc không phải đổi đơn vị hay đoán giá trị mặc định (CE-14). Không có lịch sử thay đổi và không xóa mềm.</t>
         </is>
       </c>
     </row>
@@ -37967,7 +37967,7 @@
       </c>
       <c r="I7" s="6" t="n"/>
     </row>
-    <row r="8">
+    <row r="8" ht="27" customHeight="1">
       <c r="A8" s="6" t="n">
         <v>2</v>
       </c>
@@ -37994,7 +37994,7 @@
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm đo; cột thời gian của bảng chuỗi thời gian.</t>
+          <t>Thời điểm đo theo đồng hồ của trụ; cột thời gian của bảng chuỗi thời gian.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -38004,7 +38004,7 @@
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9" ht="27" customHeight="1">
+    <row r="9" ht="40.5" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
@@ -38035,7 +38035,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Phiên sạc chứa số đo.</t>
+          <t>Phiên sạc chứa số đo. Số đo gửi ngoài phiên (lấy mẫu theo đồng hồ) chỉ được giữ trong nhật ký OCPP thô (CE-06, deferred.md 77).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -38045,7 +38045,7 @@
       </c>
       <c r="I9" s="6" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="54" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>4</v>
       </c>
@@ -38068,7 +38068,7 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Đại lượng được đo, theo tên measurand của OCPP.</t>
+          <t>Đại lượng được đo, theo tên của OCPP (Energy.Active.Import.Register, Power.Active.Import, Current.Import, Voltage, SoC, Temperature); tên riêng của hãng được lưu đúng như gửi.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -38078,7 +38078,7 @@
       </c>
       <c r="I10" s="6" t="n"/>
     </row>
-    <row r="11" ht="27" customHeight="1">
+    <row r="11" ht="94.5" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
@@ -38101,7 +38101,7 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Giá trị đo; điện năng luôn lưu bằng Wh, các đại lượng khác theo đơn vị ở cột unit.</t>
+          <t>Giá trị đo. Hiện điện năng được lưu bằng Wh. Dự kiến (CE-14): cổng OCPP đổi mọi đại lượng đã biết sang một đơn vị cố định khi ghi: điện năng Wh (phản kháng varh), công suất W (phản kháng var, biểu kiến VA), dòng điện A, điện áp V, nhiệt độ Celsius, SoC và các tỷ lệ khác Percent; đơn vị kilo nhân 1000, Fahrenheit và K đổi sang Celsius. Đại lượng riêng của hãng được lưu đúng như gửi.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -38111,7 +38111,7 @@
       </c>
       <c r="I11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="40.5" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>6</v>
       </c>
@@ -38134,7 +38134,7 @@
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Đơn vị của giá trị.</t>
+          <t>Đơn vị của giá trị, viết theo OCPP. Dự kiến (CE-14): luôn là đơn vị cố định của đại lượng đã biết; đúng như gửi, hoặc NULL, với đại lượng riêng của hãng.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -38144,7 +38144,7 @@
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="67.5" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
@@ -38167,7 +38167,7 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Lý do trụ sạc gửi số đo.</t>
+          <t>Lý do trụ gửi số đo: Sample.Periodic, Transaction.Begin, Transaction.End, Sample.Clock, Trigger, Interruption.Begin, Interruption.End, Other. Dự kiến (CE-14): bắt buộc; lưu giá trị mặc định của OCPP là Sample.Periodic khi trụ không gửi.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -38177,7 +38177,7 @@
       </c>
       <c r="I13" s="6" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="6" t="n">
         <v>8</v>
       </c>
@@ -38200,7 +38200,7 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Pha điện của giá trị; NULL với sạc DC.</t>
+          <t>Pha điện của giá trị (L1, L2, L3 ...); NULL với sạc DC, là mọi trụ chúng ta đang có.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -38210,13 +38210,13 @@
       </c>
       <c r="I14" s="6" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="135" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>measurement_location</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -38233,7 +38233,7 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Vị trí đo.</t>
+          <t>[Hiện tên là location, sẽ đổi tên] Điểm đo trên đường sạc (OCPP gọi là location): Outlet (đầu ra của trụ về phía xe: tiến trình trực tiếp và số dự phòng khi tính tiền), Inlet (đầu vào từ lưới: tổn thất và chi phí điện của chúng ta), Cable, EV (do xe báo, ví dụ SoC), Body (bên trong tủ trụ). Mọi điểm đo đều được lưu; hiện các tính năng chỉ đọc Outlet, và EV cho SoC (CE-14). Đổi tên vì location dễ hiểu nhầm là địa điểm (charging_locations). Dự kiến (CE-14): bắt buộc; lưu giá trị mặc định của OCPP là Outlet khi trụ không gửi.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): drop charging session events from the target design
For OCPP 1.6J the table only copies the session's start and end, the raw
OCPP log keeps every frame for audit, and no feature reads a session
timeline (CE-15). The 2.0.1 duplicate check and charging-state periods are
designed with 2.0.1 support (deferred.md 78).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -3285,7 +3285,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="108" customHeight="1">
+    <row r="67" ht="121.5" customHeight="1">
       <c r="A67" s="5" t="n"/>
       <c r="B67" s="5" t="inlineStr">
         <is>
@@ -3305,7 +3305,7 @@
           <t>Những gì diễn ra trong mỗi lần sạc: sự kiện, chỉ số công tơ, điện năng đã cấp.
 • Một phiên sạc diễn ra trên một súng sạc của một trụ. Phiên được tạo khi tài xế quét mã QR trên trụ bằng ứng dụng của chúng ta (CE-10) và ghi người quét, tổ chức trả tiền và, nếu tài xế đang nhận một xe, chiếc xe đó; sau đó bản tin bắt đầu của trụ điền súng sạc và giao dịch (CE-11).
 • Bản đang chạy chưa có liên kết này (chỉ có mã id_tag thô); sẽ có khi tái cấu trúc.
-• Một phiên sạc có nhiều sự kiện và nhiều số đo.</t>
+• Một phiên sạc có nhiều số đo. Bảng sự kiện đã được xây dựng nhưng bị bỏ trong thiết kế đích (CE-15).</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="27" customHeight="1">
+    <row r="69" ht="81" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
           <t>39</t>
@@ -3387,7 +3387,7 @@
       </c>
       <c r="G69" s="6" t="inlineStr">
         <is>
-          <t>Từng sự kiện Bắt đầu / Cập nhật / Kết thúc của một phiên sạc.</t>
+          <t>[Sẽ bỏ] Từng sự kiện Bắt đầu / Cập nhật / Kết thúc của một phiên sạc. Bị bỏ trong thiết kế đích (CE-15): với OCPP 1.6J bảng chỉ chép lại thời điểm bắt đầu và kết thúc của phiên, nhật ký OCPP thô đã giữ mọi bản tin để kiểm tra, và chưa tính năng nào đọc dòng thời gian của phiên. Việc loại bản tin trùng của OCPP 2.0.1 (seqNo) và các khoảng trạng thái sạc được thiết kế khi xây dựng hỗ trợ 2.0.1 (deferred.md 78).</t>
         </is>
       </c>
       <c r="H69" s="6" t="n">
@@ -37519,7 +37519,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Từng sự kiện Bắt đầu / Cập nhật / Kết thúc của một phiên sạc.</t>
+          <t>Từng sự kiện Bắt đầu / Cập nhật / Kết thúc của một phiên sạc. Bị bỏ trong thiết kế đích (CE-15): với OCPP 1.6J bảng chỉ chép lại thời điểm bắt đầu và kết thúc của phiên, nhật ký OCPP thô đã giữ mọi bản tin để kiểm tra, và chưa tính năng nào đọc dòng thời gian của phiên. Việc loại bản tin trùng của OCPP 2.0.1 (seqNo) và các khoảng trạng thái sạc được thiết kế khi xây dựng hỗ trợ 2.0.1 (deferred.md 78).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(decisions): review the notifications group last
The notifications table links to every domain that raises alerts, so it is
reviewed after them; the points already raised are kept in NT-08.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -3515,7 +3515,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="27" customHeight="1">
+    <row r="73" ht="40.5" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
           <t>42</t>
@@ -3548,7 +3548,7 @@
       </c>
       <c r="G73" s="6" t="inlineStr">
         <is>
-          <t>Một cảnh báo (pin, bất thường, SOH, thiết bị mất kết nối...). Một bảng chung; mỗi loại cảnh báo là một giá trị enum và một cấu trúc payload.</t>
+          <t>Một cảnh báo (pin, bất thường, SOH, thiết bị mất kết nối...). Một bảng chung; mỗi loại cảnh báo là một giá trị enum và một cấu trúc payload. Được rà soát sau cùng, sau mọi miền phát sinh cảnh báo (NT-08, ghi các điểm cần quyết định).</t>
         </is>
       </c>
       <c r="H73" s="6" t="n">
@@ -39096,7 +39096,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một cảnh báo (pin, bất thường, SOH, thiết bị mất kết nối...). Một bảng chung; mỗi loại cảnh báo là một giá trị enum và một cấu trúc payload.</t>
+          <t>Một cảnh báo (pin, bất thường, SOH, thiết bị mất kết nối...). Một bảng chung; mỗi loại cảnh báo là một giá trị enum và một cấu trúc payload. Được rà soát sau cùng, sau mọi miền phát sinh cảnh báo (NT-08, ghi các điểm cần quyết định).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(domain-model): link configuration snapshots to their command
Every snapshot now comes from one GET_CONFIGURATION command, so captures
get a required command_id and drop the charger and request time they
repeated (CS-21).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -136,7 +136,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="48" hidden="1">'charging_connector_history'!$A$7:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="49" hidden="1">'charging_connector_state'!$A$7:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="50" hidden="1">'charging_ocpp_messages'!$A$6:$I$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="51" hidden="1">'charging_station_config_capture'!$A$6:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="51" hidden="1">'charging_station_config_capture'!$A$6:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="52" hidden="1">'charging_station_config_entries'!$A$6:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="53" hidden="1">'charging_station_commands'!$A$6:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="54" hidden="1">'charging_sessions'!$A$6:$I$26</definedName>
@@ -3198,7 +3198,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="67.5" customHeight="1">
+    <row r="65" ht="94.5" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
           <t>36</t>
@@ -3231,11 +3231,11 @@
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>Một lần chụp cấu hình của trụ sạc: một câu trả lời GetConfiguration (1.6J) hoặc một GetBaseReport được trả lời bằng nhiều phần NotifyReport (2.0.1). Các cấu hình nằm ở charging_station_configuration_entries. Chỉ ghi thêm: cấu hình hiện tại là lần chụp COMPLETE mới nhất, so hai lần chụp cho biết những gì đã đổi (CS-19). Đổi một cấu hình là lệnh gửi xuống trụ, không phải một lần chụp.</t>
+          <t>Một lần chụp cấu hình của trụ sạc: một câu trả lời GetConfiguration (1.6J) hoặc một GetBaseReport được trả lời bằng nhiều phần NotifyReport (2.0.1). Các cấu hình nằm ở charging_station_configuration_entries. Chỉ ghi thêm: cấu hình hiện tại là lần chụp COMPLETE mới nhất, so hai lần chụp cho biết những gì đã đổi (CS-19). Đổi một cấu hình là lệnh gửi xuống trụ, không phải một lần chụp. Mỗi lần chụp đến từ một lệnh GET_CONFIGURATION, nên trụ sạc, thời điểm yêu cầu và người yêu cầu được đọc từ lệnh (CS-21).</t>
         </is>
       </c>
       <c r="H65" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I65" s="7" t="inlineStr">
         <is>
@@ -28582,7 +28582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -29873,7 +29873,7 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>charging_station_configuration_captures</t>
+          <t>charging_station_commands</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -29882,11 +29882,11 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="27" customHeight="1">
+    <row r="54">
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>charging_station_commands</t>
+          <t>charging_sessions</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -29899,7 +29899,7 @@
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>charging_sessions</t>
+          <t>tariffs</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -29912,23 +29912,10 @@
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>tariffs</t>
+          <t>charging_station_history</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>station_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="6" t="n"/>
-      <c r="B57" s="7" t="inlineStr">
-        <is>
-          <t>charging_station_history</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>station_id</t>
         </is>
@@ -29946,11 +29933,10 @@
     <hyperlink ref="B50" location="'charging_evses'!A1"/>
     <hyperlink ref="B51" location="'charging_ocpp_messages'!A1"/>
     <hyperlink ref="B52" location="'charging_station_config_entries'!A1"/>
-    <hyperlink ref="B53" location="'charging_station_config_capture'!A1"/>
-    <hyperlink ref="B54" location="'charging_station_commands'!A1"/>
-    <hyperlink ref="B55" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B56" location="'tariffs'!A1"/>
-    <hyperlink ref="B57" location="'charging_station_history'!A1"/>
+    <hyperlink ref="B53" location="'charging_station_commands'!A1"/>
+    <hyperlink ref="B54" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B55" location="'tariffs'!A1"/>
+    <hyperlink ref="B56" location="'charging_station_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -35301,7 +35287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -35339,7 +35325,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một lần chụp cấu hình của trụ sạc: một câu trả lời GetConfiguration (1.6J) hoặc một GetBaseReport được trả lời bằng nhiều phần NotifyReport (2.0.1). Các cấu hình nằm ở charging_station_configuration_entries. Chỉ ghi thêm: cấu hình hiện tại là lần chụp COMPLETE mới nhất, so hai lần chụp cho biết những gì đã đổi (CS-19). Đổi một cấu hình là lệnh gửi xuống trụ, không phải một lần chụp.</t>
+          <t>Một lần chụp cấu hình của trụ sạc: một câu trả lời GetConfiguration (1.6J) hoặc một GetBaseReport được trả lời bằng nhiều phần NotifyReport (2.0.1). Các cấu hình nằm ở charging_station_configuration_entries. Chỉ ghi thêm: cấu hình hiện tại là lần chụp COMPLETE mới nhất, so hai lần chụp cho biết những gì đã đổi (CS-19). Đổi một cấu hình là lệnh gửi xuống trụ, không phải một lần chụp. Mỗi lần chụp đến từ một lệnh GET_CONFIGURATION, nên trụ sạc, thời điểm yêu cầu và người yêu cầu được đọc từ lệnh (CS-21).</t>
         </is>
       </c>
     </row>
@@ -35428,13 +35414,13 @@
       </c>
       <c r="I7" s="6" t="n"/>
     </row>
-    <row r="8" ht="27" customHeight="1">
+    <row r="8" ht="54" customHeight="1">
       <c r="A8" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>station_id</t>
+          <t>command_id</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -35449,22 +35435,22 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>FK</t>
+          <t>FK UQ</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>charging_stations.station_id (khi xóa: chặn xóa)</t>
+          <t>charging_station_commands.command_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Trụ sạc.</t>
+          <t>Lệnh GET_CONFIGURATION đã yêu cầu lần chụp này (CS-21), kể cả lệnh tự động sau khi khởi động; mỗi lệnh cho một lần chụp. Trụ sạc, thời điểm yêu cầu và người yêu cầu được đọc từ lệnh.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>4b9d6f3a-2e8c-4a1b-9d5e-7f0c3a8b2d88</t>
+          <t>0000000c-5a6b-4c7d-8e9f-0a1b2c3d4e5f</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
@@ -35568,13 +35554,13 @@
       </c>
       <c r="I11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="27" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>requested_at</t>
+          <t>captured_at</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -35584,143 +35570,110 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm cổng OCPP hỏi trụ.</t>
+          <t>Thời điểm nhận câu trả lời (2.0.1: phần cuối cùng); NULL khi đang chờ hoặc thất bại.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>2026-09-14T22:00:06Z</t>
+          <t>2026-09-14T22:00:10Z</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13" ht="27" customHeight="1">
+    <row r="13" ht="40.5" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>captured_at</t>
+          <t>outcome</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm nhận câu trả lời (2.0.1: phần cuối cùng); NULL khi đang chờ hoặc thất bại.</t>
+          <t>Kết quả quan sát được. PENDING: đã hỏi, chưa đủ. COMPLETE: đã nhận đủ. FAILED: không trả lời kịp, trả lời lỗi, hoặc thiếu phần.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>2026-09-14T22:00:10Z</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
     </row>
-    <row r="14" ht="40.5" customHeight="1">
-      <c r="A14" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>outcome</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>varchar(20)</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40.5" customHeight="1">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>ix_charging_config_captures_ocpp_request_id</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>ocpp_request_id</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>không</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Kết quả quan sát được. PENDING: đã hỏi, chưa đủ. COMPLETE: đã nhận đủ. FAILED: không trả lời kịp, trả lời lỗi, hoặc thiếu phần.</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>COMPLETE</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="n"/>
-    </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>ix_charging_config_captures_station_captured</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>station_id, captured_at</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>The latest complete snapshot of a charger</t>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Finds the snapshot when a 2.0.1 NotifyReport part arrives, together with the command's charger</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I14"/>
+  <autoFilter ref="A6:I13"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F8" location="'charging_stations'!A1"/>
+    <hyperlink ref="F8" location="'charging_station_commands'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -35890,7 +35843,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: CS-19] Trụ sạc; nay nằm ở lần chụp.</t>
+          <t>[Sẽ bỏ: CS-19] Trụ sạc; nay đọc qua lệnh của lần chụp (CS-21).</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -36385,7 +36338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -37013,6 +36966,33 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="4" t="n"/>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="27" customHeight="1">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>charging_station_configuration_captures</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>command_id</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A6:I19"/>
   <hyperlinks>
@@ -37021,6 +37001,7 @@
     <hyperlink ref="F9" location="'charging_evses'!A1"/>
     <hyperlink ref="F10" location="'charging_sessions'!A1"/>
     <hyperlink ref="F13" location="'users'!A1"/>
+    <hyperlink ref="B26" location="'charging_station_config_capture'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(domain-model): review the fleet vehicle memberships table
Rename the key and the period columns to added_at / removed_at, add who
added or removed a truck, and read the organization through the fleet
(FL-09).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -123,7 +123,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="34" hidden="1">'driving_sessions'!$A$6:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="35" hidden="1">'fleets'!$A$7:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="36" hidden="1">'fleet_history'!$A$7:$I$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="37" hidden="1">'fleet_vehicle_memberships'!$A$6:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="37" hidden="1">'fleet_vehicle_memberships'!$A$6:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="38" hidden="1">'geofences'!$A$6:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="39" hidden="1">'fleet_user_assignments'!$A$6:$I$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="40" hidden="1">'charging_locations'!$A$7:$I$18</definedName>
@@ -2545,7 +2545,7 @@
         </is>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="81" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
           <t>25</t>
@@ -2578,11 +2578,11 @@
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>Xe nào thuộc đội nào, trong khoảng thời gian nào (lịch sử mở/đóng).</t>
+          <t>Xe nào thuộc đội nào, trong khoảng thời gian nào (lịch sử mở/đóng). Mỗi xe chỉ thuộc tối đa một đội tại một thời điểm và giai đoạn không có dữ liệu riêng, nên theo DM-22 lẽ ra đặt fleet_id trên vehicles; bảng được giữ vì miền xe không được phụ thuộc miền đội xe (FL-01, FL-09). Không có lịch sử thay đổi: dòng chỉ bị đóng (DM-20); added_by / removed_by cho biết ai thực hiện. Không có cột lý do: lý do xe rời đội rõ từ sự việc (chuyển đội, bán xe, đội bị xóa).</t>
         </is>
       </c>
       <c r="H50" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
@@ -10584,7 +10584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11415,11 +11415,11 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="27" customHeight="1">
+    <row r="40">
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>fleet_vehicle_memberships</t>
+          <t>fleet_user_assignments</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -11432,7 +11432,7 @@
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>fleet_user_assignments</t>
+          <t>geofences</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -11445,7 +11445,7 @@
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>geofences</t>
+          <t>charging_locations</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -11454,29 +11454,29 @@
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="27" customHeight="1">
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>charging_locations</t>
+          <t>charging_location_access</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="27" customHeight="1">
+          <t>allowed_organization_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>charging_location_access</t>
+          <t>charging_sessions</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>allowed_organization_id</t>
+          <t>organization_id</t>
         </is>
       </c>
     </row>
@@ -11484,7 +11484,7 @@
       <c r="A45" s="6" t="n"/>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>charging_sessions</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -11497,7 +11497,7 @@
       <c r="A46" s="6" t="n"/>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>support_cases</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -11510,7 +11510,7 @@
       <c r="A47" s="6" t="n"/>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>support_cases</t>
+          <t>repair_partners</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -11523,7 +11523,7 @@
       <c r="A48" s="6" t="n"/>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>repair_partners</t>
+          <t>maintenance_bookings</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -11532,11 +11532,11 @@
         </is>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="27" customHeight="1">
       <c r="A49" s="6" t="n"/>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>maintenance_bookings</t>
+          <t>charging_policy_assignments</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -11545,11 +11545,11 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="27" customHeight="1">
+    <row r="50">
       <c r="A50" s="6" t="n"/>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>charging_policy_assignments</t>
+          <t>policy_violations</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -11562,7 +11562,7 @@
       <c r="A51" s="6" t="n"/>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>policy_violations</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -11575,7 +11575,7 @@
       <c r="A52" s="6" t="n"/>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>wallets</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -11588,7 +11588,7 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>wallets</t>
+          <t>wallet_transactions</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -11601,7 +11601,7 @@
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>wallet_transactions</t>
+          <t>invoices</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -11614,7 +11614,7 @@
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>invoice_lines</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -11627,7 +11627,7 @@
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>invoice_lines</t>
+          <t>subscriptions</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -11640,7 +11640,7 @@
       <c r="A57" s="6" t="n"/>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>subscriptions</t>
+          <t>driver_scores</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -11653,7 +11653,7 @@
       <c r="A58" s="6" t="n"/>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>driver_scores</t>
+          <t>trips</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -11666,23 +11666,10 @@
       <c r="A59" s="6" t="n"/>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>trips</t>
+          <t>organization_history</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
-        <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="n"/>
-      <c r="B60" s="7" t="inlineStr">
-        <is>
-          <t>organization_history</t>
-        </is>
-      </c>
-      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>organization_id</t>
         </is>
@@ -11708,27 +11695,26 @@
     <hyperlink ref="B37" location="'driver_vehicle_assignments'!A1"/>
     <hyperlink ref="B38" location="'driving_sessions'!A1"/>
     <hyperlink ref="B39" location="'fleets'!A1"/>
-    <hyperlink ref="B40" location="'fleet_vehicle_memberships'!A1"/>
-    <hyperlink ref="B41" location="'fleet_user_assignments'!A1"/>
-    <hyperlink ref="B42" location="'geofences'!A1"/>
-    <hyperlink ref="B43" location="'charging_locations'!A1"/>
-    <hyperlink ref="B44" location="'charging_location_access'!A1"/>
-    <hyperlink ref="B45" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B46" location="'notifications'!A1"/>
-    <hyperlink ref="B47" location="'support_cases'!A1"/>
-    <hyperlink ref="B48" location="'repair_partners'!A1"/>
-    <hyperlink ref="B49" location="'maintenance_bookings'!A1"/>
-    <hyperlink ref="B50" location="'charging_policy_assignments'!A1"/>
-    <hyperlink ref="B51" location="'policy_violations'!A1"/>
-    <hyperlink ref="B52" location="'payments'!A1"/>
-    <hyperlink ref="B53" location="'wallets'!A1"/>
-    <hyperlink ref="B54" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="B55" location="'invoices'!A1"/>
-    <hyperlink ref="B56" location="'invoice_lines'!A1"/>
-    <hyperlink ref="B57" location="'subscriptions'!A1"/>
-    <hyperlink ref="B58" location="'driver_scores'!A1"/>
-    <hyperlink ref="B59" location="'trips'!A1"/>
-    <hyperlink ref="B60" location="'organization_history'!A1"/>
+    <hyperlink ref="B40" location="'fleet_user_assignments'!A1"/>
+    <hyperlink ref="B41" location="'geofences'!A1"/>
+    <hyperlink ref="B42" location="'charging_locations'!A1"/>
+    <hyperlink ref="B43" location="'charging_location_access'!A1"/>
+    <hyperlink ref="B44" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B45" location="'notifications'!A1"/>
+    <hyperlink ref="B46" location="'support_cases'!A1"/>
+    <hyperlink ref="B47" location="'repair_partners'!A1"/>
+    <hyperlink ref="B48" location="'maintenance_bookings'!A1"/>
+    <hyperlink ref="B49" location="'charging_policy_assignments'!A1"/>
+    <hyperlink ref="B50" location="'policy_violations'!A1"/>
+    <hyperlink ref="B51" location="'payments'!A1"/>
+    <hyperlink ref="B52" location="'wallets'!A1"/>
+    <hyperlink ref="B53" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="B54" location="'invoices'!A1"/>
+    <hyperlink ref="B55" location="'invoice_lines'!A1"/>
+    <hyperlink ref="B56" location="'subscriptions'!A1"/>
+    <hyperlink ref="B57" location="'driver_scores'!A1"/>
+    <hyperlink ref="B58" location="'trips'!A1"/>
+    <hyperlink ref="B59" location="'organization_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -25089,7 +25075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -25127,7 +25113,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Xe nào thuộc đội nào, trong khoảng thời gian nào (lịch sử mở/đóng).</t>
+          <t>Xe nào thuộc đội nào, trong khoảng thời gian nào (lịch sử mở/đóng). Mỗi xe chỉ thuộc tối đa một đội tại một thời điểm và giai đoạn không có dữ liệu riêng, nên theo DM-22 lẽ ra đặt fleet_id trên vehicles; bảng được giữ vì miền xe không được phụ thuộc miền đội xe (FL-01, FL-09). Không có lịch sử thay đổi: dòng chỉ bị đóng (DM-20); added_by / removed_by cho biết ai thực hiện. Không có cột lý do: lý do xe rời đội rõ từ sự việc (chuyển đội, bán xe, đội bị xóa).</t>
         </is>
       </c>
     </row>
@@ -25179,13 +25165,13 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="54" customHeight="1">
       <c r="A7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>membership_id</t>
+          <t>fleet_vehicle_membership_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -25206,7 +25192,7 @@
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Mã nội bộ của giai đoạn thành viên.</t>
+          <t>[Hiện tên là membership_id, sẽ đổi tên] Mã nội bộ của một giai đoạn thành viên. Đổi tên vì memberships.membership_id (miền danh tính) là một người trong một tổ chức, một khái niệm khác (FL-09).</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -25222,7 +25208,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
+          <t>fleet_id</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -25232,7 +25218,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -25242,28 +25228,28 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+          <t>fleets.fleet_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức khách hàng của giai đoạn thành viên.</t>
+          <t>Đội xe chứa xe; dòng đọc tổ chức qua đội xe (DM-24), vì đội xe không bao giờ chuyển sang tổ chức khác.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+          <t>8d5f2b7e-1a9c-4f3d-b8e2-6c0a4d9f1e77</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>fleet_id</t>
+          <t>vehicle_id</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -25283,17 +25269,17 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>fleets.fleet_id (khi xóa: chặn xóa)</t>
+          <t>vehicles.vehicle_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Đội xe chứa xe.</t>
+          <t>Xe thuộc đội; xe phải thuộc tổ chức của đội khi được thêm vào.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>8d5f2b7e-1a9c-4f3d-b8e2-6c0a4d9f1e77</t>
+          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
         </is>
       </c>
       <c r="I9" s="6" t="n"/>
@@ -25304,12 +25290,12 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id</t>
+          <t>added_at</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -25317,35 +25303,27 @@
           <t>không</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>vehicles.vehicle_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Xe thuộc đội.</t>
+          <t>[Hiện tên là joined_at, sẽ đổi tên] Thời điểm xe được thêm vào đội (FL-09).</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
+          <t>2026-09-01T00:00:00Z</t>
         </is>
       </c>
       <c r="I10" s="6" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>joined_at</t>
+          <t>removed_at</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -25355,19 +25333,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm xe vào đội.</t>
+          <t>[Hiện tên là left_at, sẽ đổi tên] Thời điểm xe bị đưa ra khỏi đội; NULL khi vẫn còn trong đội (FL-09).</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00Z</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I11" s="6" t="n"/>
@@ -25378,12 +25356,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>left_at</t>
+          <t>added_by</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -25391,60 +25369,76 @@
           <t>có</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>users.user_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm xe rời đội; NULL khi vẫn còn trong đội.</t>
+          <t>Người dùng đã thêm xe vào đội.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="40.5" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>removed_by</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>users.user_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
+          <t>Người dùng đã đưa xe ra khỏi đội; NULL khi vẫn là thành viên, hoặc khi hệ thống tự đóng (xe được bán, VH-12, hoặc đội bị xóa, FL-06).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
     </row>
-    <row r="14" ht="27" customHeight="1">
+    <row r="14">
       <c r="A14" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -25461,71 +25455,84 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-01T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n"/>
+    </row>
+    <row r="15" ht="27" customHeight="1">
+      <c r="A15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
           <t>Thời điểm bản ghi được sửa gần nhất (thay đổi khi xe rời đội).</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>2026-09-10T07:15:00Z</t>
         </is>
       </c>
-      <c r="I14" s="6" t="n"/>
-    </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="I15" s="6" t="n"/>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="E17" s="4" t="n"/>
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>ix_fleet_vehicle_memberships_fleet_id</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>fleet_id</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
     </row>
     <row r="18" ht="27" customHeight="1">
       <c r="A18" s="6" t="n"/>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>ix_fleet_vehicle_memberships_fleet_time</t>
+          <t>ix_fleet_vehicle_memberships_fleet_id</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>fleet_id, joined_at</t>
+          <t>fleet_id</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -25534,18 +25541,22 @@
         </is>
       </c>
       <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Dropped: covered by ix_fleet_vehicle_memberships_fleet_time (FL-09)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="27" customHeight="1">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>ix_fleet_vehicle_memberships_vehicle_id</t>
+          <t>ix_fleet_vehicle_memberships_fleet_time</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id</t>
+          <t>fleet_id, added_at</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -25560,33 +25571,54 @@
       <c r="A20" s="6" t="n"/>
       <c r="B20" s="6" t="inlineStr">
         <is>
+          <t>ix_fleet_vehicle_memberships_vehicle_id</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="27" customHeight="1">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
           <t>uq_fleet_vehicle_memberships_active_vehicle</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>vehicle_id</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>có</t>
         </is>
       </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>WHERE left_at IS NULL</t>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>WHERE removed_at IS NULL (built as left_at)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I14"/>
+  <autoFilter ref="A6:I15"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F8" location="'organizations'!A1"/>
-    <hyperlink ref="F9" location="'fleets'!A1"/>
-    <hyperlink ref="F10" location="'vehicles'!A1"/>
+    <hyperlink ref="F8" location="'fleets'!A1"/>
+    <hyperlink ref="F9" location="'vehicles'!A1"/>
+    <hyperlink ref="F12" location="'users'!A1"/>
+    <hyperlink ref="F13" location="'users'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26034,7 +26066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -26785,42 +26817,42 @@
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="27" customHeight="1">
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>charging_location_access</t>
+          <t>fleet_vehicle_memberships</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>granted_by</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
+          <t>added_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="27" customHeight="1">
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>charging_location_access</t>
+          <t>fleet_vehicle_memberships</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>revoked_by</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="27" customHeight="1">
+          <t>removed_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>charging_station_commands</t>
+          <t>charging_location_access</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>requested_by</t>
+          <t>granted_by</t>
         </is>
       </c>
     </row>
@@ -26828,25 +26860,25 @@
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>charging_sessions</t>
+          <t>charging_location_access</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>started_by</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
+          <t>revoked_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="27" customHeight="1">
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>charging_policy_versions</t>
+          <t>charging_station_commands</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>requested_by</t>
         </is>
       </c>
     </row>
@@ -26854,12 +26886,12 @@
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>organization_history</t>
+          <t>charging_sessions</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>changed_by</t>
+          <t>started_by</t>
         </is>
       </c>
     </row>
@@ -26867,12 +26899,12 @@
       <c r="A45" s="6" t="n"/>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>user_history</t>
+          <t>charging_policy_versions</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>created_by</t>
         </is>
       </c>
     </row>
@@ -26880,7 +26912,7 @@
       <c r="A46" s="6" t="n"/>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>user_history</t>
+          <t>organization_history</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -26893,20 +26925,20 @@
       <c r="A47" s="6" t="n"/>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>membership_history</t>
+          <t>user_history</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>changed_by</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="27" customHeight="1">
+          <t>user_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
       <c r="A48" s="6" t="n"/>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>organization_setting_history</t>
+          <t>user_history</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -26919,7 +26951,7 @@
       <c r="A49" s="6" t="n"/>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>vehicle_history</t>
+          <t>membership_history</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -26928,11 +26960,11 @@
         </is>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="27" customHeight="1">
       <c r="A50" s="6" t="n"/>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>vehicle_model_history</t>
+          <t>organization_setting_history</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -26945,7 +26977,7 @@
       <c r="A51" s="6" t="n"/>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>battery_model_history</t>
+          <t>vehicle_history</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -26958,7 +26990,7 @@
       <c r="A52" s="6" t="n"/>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>battery_history</t>
+          <t>vehicle_model_history</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -26971,7 +27003,7 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>warranty_history</t>
+          <t>battery_model_history</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -26984,7 +27016,7 @@
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>telematic_history</t>
+          <t>battery_history</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -26997,7 +27029,7 @@
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>driver_history</t>
+          <t>warranty_history</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -27010,7 +27042,7 @@
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>fleet_history</t>
+          <t>telematic_history</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -27019,11 +27051,11 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="27" customHeight="1">
+    <row r="57">
       <c r="A57" s="6" t="n"/>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>charging_location_history</t>
+          <t>driver_history</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -27036,7 +27068,7 @@
       <c r="A58" s="6" t="n"/>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>charging_station_history</t>
+          <t>fleet_history</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -27045,11 +27077,11 @@
         </is>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="27" customHeight="1">
       <c r="A59" s="6" t="n"/>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>charging_evse_history</t>
+          <t>charging_location_history</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -27058,14 +27090,40 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="27" customHeight="1">
+    <row r="60">
       <c r="A60" s="6" t="n"/>
       <c r="B60" s="7" t="inlineStr">
         <is>
+          <t>charging_station_history</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>changed_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n"/>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>charging_evse_history</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>changed_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="27" customHeight="1">
+      <c r="A62" s="6" t="n"/>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
           <t>charging_connector_history</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C62" s="6" t="inlineStr">
         <is>
           <t>changed_by</t>
         </is>
@@ -27092,28 +27150,30 @@
     <hyperlink ref="B36" location="'user_role_assignments'!A1"/>
     <hyperlink ref="B37" location="'user_role_assignments'!A1"/>
     <hyperlink ref="B38" location="'access_audit_logs'!A1"/>
-    <hyperlink ref="B39" location="'charging_location_access'!A1"/>
-    <hyperlink ref="B40" location="'charging_location_access'!A1"/>
-    <hyperlink ref="B41" location="'charging_station_commands'!A1"/>
-    <hyperlink ref="B42" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B43" location="'charging_policy_versions'!A1"/>
-    <hyperlink ref="B44" location="'organization_history'!A1"/>
-    <hyperlink ref="B45" location="'user_history'!A1"/>
-    <hyperlink ref="B46" location="'user_history'!A1"/>
-    <hyperlink ref="B47" location="'membership_history'!A1"/>
-    <hyperlink ref="B48" location="'organization_setting_history'!A1"/>
-    <hyperlink ref="B49" location="'vehicle_history'!A1"/>
-    <hyperlink ref="B50" location="'vehicle_model_history'!A1"/>
-    <hyperlink ref="B51" location="'battery_model_history'!A1"/>
-    <hyperlink ref="B52" location="'battery_history'!A1"/>
-    <hyperlink ref="B53" location="'warranty_history'!A1"/>
-    <hyperlink ref="B54" location="'telematic_history'!A1"/>
-    <hyperlink ref="B55" location="'driver_history'!A1"/>
-    <hyperlink ref="B56" location="'fleet_history'!A1"/>
-    <hyperlink ref="B57" location="'charging_location_history'!A1"/>
-    <hyperlink ref="B58" location="'charging_station_history'!A1"/>
-    <hyperlink ref="B59" location="'charging_evse_history'!A1"/>
-    <hyperlink ref="B60" location="'charging_connector_history'!A1"/>
+    <hyperlink ref="B39" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="B40" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="B41" location="'charging_location_access'!A1"/>
+    <hyperlink ref="B42" location="'charging_location_access'!A1"/>
+    <hyperlink ref="B43" location="'charging_station_commands'!A1"/>
+    <hyperlink ref="B44" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B45" location="'charging_policy_versions'!A1"/>
+    <hyperlink ref="B46" location="'organization_history'!A1"/>
+    <hyperlink ref="B47" location="'user_history'!A1"/>
+    <hyperlink ref="B48" location="'user_history'!A1"/>
+    <hyperlink ref="B49" location="'membership_history'!A1"/>
+    <hyperlink ref="B50" location="'organization_setting_history'!A1"/>
+    <hyperlink ref="B51" location="'vehicle_history'!A1"/>
+    <hyperlink ref="B52" location="'vehicle_model_history'!A1"/>
+    <hyperlink ref="B53" location="'battery_model_history'!A1"/>
+    <hyperlink ref="B54" location="'battery_history'!A1"/>
+    <hyperlink ref="B55" location="'warranty_history'!A1"/>
+    <hyperlink ref="B56" location="'telematic_history'!A1"/>
+    <hyperlink ref="B57" location="'driver_history'!A1"/>
+    <hyperlink ref="B58" location="'fleet_history'!A1"/>
+    <hyperlink ref="B59" location="'charging_location_history'!A1"/>
+    <hyperlink ref="B60" location="'charging_station_history'!A1"/>
+    <hyperlink ref="B61" location="'charging_evse_history'!A1"/>
+    <hyperlink ref="B62" location="'charging_connector_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(domain-model): review the fleet user assignments table
Rename the key, read the organization through the fleet and membership,
record who granted or removed fleet access, and define the visible set as
the union of the assigned fleets and their subtrees (FL-10).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -125,7 +125,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="36" hidden="1">'fleet_history'!$A$7:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="37" hidden="1">'fleet_vehicle_memberships'!$A$6:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="38" hidden="1">'geofences'!$A$6:$I$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="39" hidden="1">'fleet_user_assignments'!$A$6:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="39" hidden="1">'fleet_user_assignments'!$A$6:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="40" hidden="1">'charging_locations'!$A$7:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="41" hidden="1">'charging_location_history'!$A$7:$I$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="42" hidden="1">'charging_location_access'!$A$6:$I$15</definedName>
@@ -2635,7 +2635,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="67.5" customHeight="1">
+    <row r="52" ht="121.5" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
           <t>27</t>
@@ -2668,11 +2668,11 @@
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>Giới hạn vai trò cấp đội xe của một người dùng trong một số đội xe của tổ chức lớn (ví dụ một quản lý cho đội Hà Nội, một quản lý khác cho đội TP.HCM). Người dùng không có dòng nào đang hiệu lực ở đây thì quản lý mọi đội xe của tổ chức. Nằm ở miền Đội xe, không ở miền Danh tính, để miền Danh tính không phụ thuộc miền nào.</t>
+          <t>Giới hạn vai trò cấp đội xe của một người dùng trong một số đội xe của tổ chức lớn (ví dụ một quản lý cho đội Hà Nội, một quản lý khác cho đội TP.HCM). Người dùng không có dòng nào đang hiệu lực ở đây thì quản lý mọi đội xe của tổ chức. Phạm vi xem là hợp của các đội được giao và mọi đội bên dưới, mỗi xe một lần, gồm các xe đang thuộc các đội đó (FL-10). Được phép giao một đội đã nằm dưới một đội cha được giao (giữ quyền khi cây thay đổi); portal sẽ cảnh báo. Nằm ở miền Đội xe, không ở miền Danh tính, để miền Danh tính không phụ thuộc miền nào. Không có lịch sử thay đổi: dòng chỉ bị đóng (DM-20); assigned_by / unassigned_by cho biết ai thực hiện.</t>
         </is>
       </c>
       <c r="H52" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
@@ -10584,7 +10584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11419,7 +11419,7 @@
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>fleet_user_assignments</t>
+          <t>geofences</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -11432,7 +11432,7 @@
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>geofences</t>
+          <t>charging_locations</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -11441,29 +11441,29 @@
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="27" customHeight="1">
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>charging_locations</t>
+          <t>charging_location_access</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="27" customHeight="1">
+          <t>allowed_organization_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>charging_location_access</t>
+          <t>charging_sessions</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>allowed_organization_id</t>
+          <t>organization_id</t>
         </is>
       </c>
     </row>
@@ -11471,7 +11471,7 @@
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>charging_sessions</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -11484,7 +11484,7 @@
       <c r="A45" s="6" t="n"/>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>support_cases</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -11497,7 +11497,7 @@
       <c r="A46" s="6" t="n"/>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>support_cases</t>
+          <t>repair_partners</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -11510,7 +11510,7 @@
       <c r="A47" s="6" t="n"/>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>repair_partners</t>
+          <t>maintenance_bookings</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -11519,11 +11519,11 @@
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="27" customHeight="1">
       <c r="A48" s="6" t="n"/>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>maintenance_bookings</t>
+          <t>charging_policy_assignments</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -11532,11 +11532,11 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="27" customHeight="1">
+    <row r="49">
       <c r="A49" s="6" t="n"/>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>charging_policy_assignments</t>
+          <t>policy_violations</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -11549,7 +11549,7 @@
       <c r="A50" s="6" t="n"/>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>policy_violations</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -11562,7 +11562,7 @@
       <c r="A51" s="6" t="n"/>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>wallets</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -11575,7 +11575,7 @@
       <c r="A52" s="6" t="n"/>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>wallets</t>
+          <t>wallet_transactions</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -11588,7 +11588,7 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>wallet_transactions</t>
+          <t>invoices</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -11601,7 +11601,7 @@
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>invoice_lines</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -11614,7 +11614,7 @@
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>invoice_lines</t>
+          <t>subscriptions</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -11627,7 +11627,7 @@
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>subscriptions</t>
+          <t>driver_scores</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -11640,7 +11640,7 @@
       <c r="A57" s="6" t="n"/>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>driver_scores</t>
+          <t>trips</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -11653,23 +11653,10 @@
       <c r="A58" s="6" t="n"/>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>trips</t>
+          <t>organization_history</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
-        <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="6" t="n"/>
-      <c r="B59" s="7" t="inlineStr">
-        <is>
-          <t>organization_history</t>
-        </is>
-      </c>
-      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>organization_id</t>
         </is>
@@ -11695,26 +11682,25 @@
     <hyperlink ref="B37" location="'driver_vehicle_assignments'!A1"/>
     <hyperlink ref="B38" location="'driving_sessions'!A1"/>
     <hyperlink ref="B39" location="'fleets'!A1"/>
-    <hyperlink ref="B40" location="'fleet_user_assignments'!A1"/>
-    <hyperlink ref="B41" location="'geofences'!A1"/>
-    <hyperlink ref="B42" location="'charging_locations'!A1"/>
-    <hyperlink ref="B43" location="'charging_location_access'!A1"/>
-    <hyperlink ref="B44" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B45" location="'notifications'!A1"/>
-    <hyperlink ref="B46" location="'support_cases'!A1"/>
-    <hyperlink ref="B47" location="'repair_partners'!A1"/>
-    <hyperlink ref="B48" location="'maintenance_bookings'!A1"/>
-    <hyperlink ref="B49" location="'charging_policy_assignments'!A1"/>
-    <hyperlink ref="B50" location="'policy_violations'!A1"/>
-    <hyperlink ref="B51" location="'payments'!A1"/>
-    <hyperlink ref="B52" location="'wallets'!A1"/>
-    <hyperlink ref="B53" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="B54" location="'invoices'!A1"/>
-    <hyperlink ref="B55" location="'invoice_lines'!A1"/>
-    <hyperlink ref="B56" location="'subscriptions'!A1"/>
-    <hyperlink ref="B57" location="'driver_scores'!A1"/>
-    <hyperlink ref="B58" location="'trips'!A1"/>
-    <hyperlink ref="B59" location="'organization_history'!A1"/>
+    <hyperlink ref="B40" location="'geofences'!A1"/>
+    <hyperlink ref="B41" location="'charging_locations'!A1"/>
+    <hyperlink ref="B42" location="'charging_location_access'!A1"/>
+    <hyperlink ref="B43" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B44" location="'notifications'!A1"/>
+    <hyperlink ref="B45" location="'support_cases'!A1"/>
+    <hyperlink ref="B46" location="'repair_partners'!A1"/>
+    <hyperlink ref="B47" location="'maintenance_bookings'!A1"/>
+    <hyperlink ref="B48" location="'charging_policy_assignments'!A1"/>
+    <hyperlink ref="B49" location="'policy_violations'!A1"/>
+    <hyperlink ref="B50" location="'payments'!A1"/>
+    <hyperlink ref="B51" location="'wallets'!A1"/>
+    <hyperlink ref="B52" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="B53" location="'invoices'!A1"/>
+    <hyperlink ref="B54" location="'invoice_lines'!A1"/>
+    <hyperlink ref="B55" location="'subscriptions'!A1"/>
+    <hyperlink ref="B56" location="'driver_scores'!A1"/>
+    <hyperlink ref="B57" location="'trips'!A1"/>
+    <hyperlink ref="B58" location="'organization_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26066,7 +26052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -26847,12 +26833,12 @@
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>charging_location_access</t>
+          <t>fleet_user_assignments</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>granted_by</t>
+          <t>assigned_by</t>
         </is>
       </c>
     </row>
@@ -26860,25 +26846,25 @@
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>charging_location_access</t>
+          <t>fleet_user_assignments</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>revoked_by</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="27" customHeight="1">
+          <t>unassigned_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>charging_station_commands</t>
+          <t>charging_location_access</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>requested_by</t>
+          <t>granted_by</t>
         </is>
       </c>
     </row>
@@ -26886,25 +26872,25 @@
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>charging_sessions</t>
+          <t>charging_location_access</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>started_by</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
+          <t>revoked_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="27" customHeight="1">
       <c r="A45" s="6" t="n"/>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>charging_policy_versions</t>
+          <t>charging_station_commands</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>requested_by</t>
         </is>
       </c>
     </row>
@@ -26912,12 +26898,12 @@
       <c r="A46" s="6" t="n"/>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>organization_history</t>
+          <t>charging_sessions</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>changed_by</t>
+          <t>started_by</t>
         </is>
       </c>
     </row>
@@ -26925,12 +26911,12 @@
       <c r="A47" s="6" t="n"/>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>user_history</t>
+          <t>charging_policy_versions</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>created_by</t>
         </is>
       </c>
     </row>
@@ -26938,7 +26924,7 @@
       <c r="A48" s="6" t="n"/>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>user_history</t>
+          <t>organization_history</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -26951,20 +26937,20 @@
       <c r="A49" s="6" t="n"/>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>membership_history</t>
+          <t>user_history</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>changed_by</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="27" customHeight="1">
+          <t>user_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
       <c r="A50" s="6" t="n"/>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>organization_setting_history</t>
+          <t>user_history</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -26977,7 +26963,7 @@
       <c r="A51" s="6" t="n"/>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>vehicle_history</t>
+          <t>membership_history</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -26986,11 +26972,11 @@
         </is>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="27" customHeight="1">
       <c r="A52" s="6" t="n"/>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>vehicle_model_history</t>
+          <t>organization_setting_history</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -27003,7 +26989,7 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>battery_model_history</t>
+          <t>vehicle_history</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -27016,7 +27002,7 @@
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>battery_history</t>
+          <t>vehicle_model_history</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -27029,7 +27015,7 @@
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>warranty_history</t>
+          <t>battery_model_history</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -27042,7 +27028,7 @@
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>telematic_history</t>
+          <t>battery_history</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -27055,7 +27041,7 @@
       <c r="A57" s="6" t="n"/>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>driver_history</t>
+          <t>warranty_history</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -27068,7 +27054,7 @@
       <c r="A58" s="6" t="n"/>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>fleet_history</t>
+          <t>telematic_history</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -27077,11 +27063,11 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="27" customHeight="1">
+    <row r="59">
       <c r="A59" s="6" t="n"/>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>charging_location_history</t>
+          <t>driver_history</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -27094,7 +27080,7 @@
       <c r="A60" s="6" t="n"/>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>charging_station_history</t>
+          <t>fleet_history</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -27103,11 +27089,11 @@
         </is>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="27" customHeight="1">
       <c r="A61" s="6" t="n"/>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>charging_evse_history</t>
+          <t>charging_location_history</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -27116,14 +27102,40 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="27" customHeight="1">
+    <row r="62">
       <c r="A62" s="6" t="n"/>
       <c r="B62" s="7" t="inlineStr">
         <is>
+          <t>charging_station_history</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>changed_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n"/>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>charging_evse_history</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>changed_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="27" customHeight="1">
+      <c r="A64" s="6" t="n"/>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
           <t>charging_connector_history</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C64" s="6" t="inlineStr">
         <is>
           <t>changed_by</t>
         </is>
@@ -27152,28 +27164,30 @@
     <hyperlink ref="B38" location="'access_audit_logs'!A1"/>
     <hyperlink ref="B39" location="'fleet_vehicle_memberships'!A1"/>
     <hyperlink ref="B40" location="'fleet_vehicle_memberships'!A1"/>
-    <hyperlink ref="B41" location="'charging_location_access'!A1"/>
-    <hyperlink ref="B42" location="'charging_location_access'!A1"/>
-    <hyperlink ref="B43" location="'charging_station_commands'!A1"/>
-    <hyperlink ref="B44" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B45" location="'charging_policy_versions'!A1"/>
-    <hyperlink ref="B46" location="'organization_history'!A1"/>
-    <hyperlink ref="B47" location="'user_history'!A1"/>
-    <hyperlink ref="B48" location="'user_history'!A1"/>
-    <hyperlink ref="B49" location="'membership_history'!A1"/>
-    <hyperlink ref="B50" location="'organization_setting_history'!A1"/>
-    <hyperlink ref="B51" location="'vehicle_history'!A1"/>
-    <hyperlink ref="B52" location="'vehicle_model_history'!A1"/>
-    <hyperlink ref="B53" location="'battery_model_history'!A1"/>
-    <hyperlink ref="B54" location="'battery_history'!A1"/>
-    <hyperlink ref="B55" location="'warranty_history'!A1"/>
-    <hyperlink ref="B56" location="'telematic_history'!A1"/>
-    <hyperlink ref="B57" location="'driver_history'!A1"/>
-    <hyperlink ref="B58" location="'fleet_history'!A1"/>
-    <hyperlink ref="B59" location="'charging_location_history'!A1"/>
-    <hyperlink ref="B60" location="'charging_station_history'!A1"/>
-    <hyperlink ref="B61" location="'charging_evse_history'!A1"/>
-    <hyperlink ref="B62" location="'charging_connector_history'!A1"/>
+    <hyperlink ref="B41" location="'fleet_user_assignments'!A1"/>
+    <hyperlink ref="B42" location="'fleet_user_assignments'!A1"/>
+    <hyperlink ref="B43" location="'charging_location_access'!A1"/>
+    <hyperlink ref="B44" location="'charging_location_access'!A1"/>
+    <hyperlink ref="B45" location="'charging_station_commands'!A1"/>
+    <hyperlink ref="B46" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B47" location="'charging_policy_versions'!A1"/>
+    <hyperlink ref="B48" location="'organization_history'!A1"/>
+    <hyperlink ref="B49" location="'user_history'!A1"/>
+    <hyperlink ref="B50" location="'user_history'!A1"/>
+    <hyperlink ref="B51" location="'membership_history'!A1"/>
+    <hyperlink ref="B52" location="'organization_setting_history'!A1"/>
+    <hyperlink ref="B53" location="'vehicle_history'!A1"/>
+    <hyperlink ref="B54" location="'vehicle_model_history'!A1"/>
+    <hyperlink ref="B55" location="'battery_model_history'!A1"/>
+    <hyperlink ref="B56" location="'battery_history'!A1"/>
+    <hyperlink ref="B57" location="'warranty_history'!A1"/>
+    <hyperlink ref="B58" location="'telematic_history'!A1"/>
+    <hyperlink ref="B59" location="'driver_history'!A1"/>
+    <hyperlink ref="B60" location="'fleet_history'!A1"/>
+    <hyperlink ref="B61" location="'charging_location_history'!A1"/>
+    <hyperlink ref="B62" location="'charging_station_history'!A1"/>
+    <hyperlink ref="B63" location="'charging_evse_history'!A1"/>
+    <hyperlink ref="B64" location="'charging_connector_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27185,7 +27199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -27223,7 +27237,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Giới hạn vai trò cấp đội xe của một người dùng trong một số đội xe của tổ chức lớn (ví dụ một quản lý cho đội Hà Nội, một quản lý khác cho đội TP.HCM). Người dùng không có dòng nào đang hiệu lực ở đây thì quản lý mọi đội xe của tổ chức. Nằm ở miền Đội xe, không ở miền Danh tính, để miền Danh tính không phụ thuộc miền nào.</t>
+          <t>Giới hạn vai trò cấp đội xe của một người dùng trong một số đội xe của tổ chức lớn (ví dụ một quản lý cho đội Hà Nội, một quản lý khác cho đội TP.HCM). Người dùng không có dòng nào đang hiệu lực ở đây thì quản lý mọi đội xe của tổ chức. Phạm vi xem là hợp của các đội được giao và mọi đội bên dưới, mỗi xe một lần, gồm các xe đang thuộc các đội đó (FL-10). Được phép giao một đội đã nằm dưới một đội cha được giao (giữ quyền khi cây thay đổi); portal sẽ cảnh báo. Nằm ở miền Đội xe, không ở miền Danh tính, để miền Danh tính không phụ thuộc miền nào. Không có lịch sử thay đổi: dòng chỉ bị đóng (DM-20); assigned_by / unassigned_by cho biết ai thực hiện.</t>
         </is>
       </c>
     </row>
@@ -27281,7 +27295,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>assignment_id</t>
+          <t>fleet_user_assignment_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -27312,13 +27326,13 @@
       </c>
       <c r="I7" s="6" t="n"/>
     </row>
-    <row r="8" ht="27" customHeight="1">
+    <row r="8" ht="40.5" customHeight="1">
       <c r="A8" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
+          <t>fleet_id</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -27338,28 +27352,28 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+          <t>fleets.fleet_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức của đội xe và người dùng.</t>
+          <t>Đội xe mà người dùng được giới hạn trong đó, cùng mọi đội xe nằm dưới. Phải thuộc tổ chức của thành viên (dịch vụ kiểm tra; dòng đọc tổ chức qua một trong hai, DM-24).</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+          <t>8d5f2b7e-1a9c-4f3d-b8e2-6c0a4d9f1e77</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9" ht="27" customHeight="1">
+    <row r="9" ht="40.5" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>fleet_id</t>
+          <t>membership_id</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -27379,33 +27393,33 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>fleets.fleet_id (khi xóa: chặn xóa)</t>
+          <t>memberships.membership_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Đội xe mà người dùng được giới hạn trong đó, cùng mọi đội xe nằm dưới.</t>
+          <t>Thành viên (người trong tổ chức này) có các vai trò cấp đội xe (FLEET_MANAGER, DISPATCHER) chỉ áp dụng cho các đội xe được liệt kê.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>8d5f2b7e-1a9c-4f3d-b8e2-6c0a4d9f1e77</t>
+          <t>00000022-5a6b-4c7d-8e9f-0a1b2c3d4e5f</t>
         </is>
       </c>
       <c r="I9" s="6" t="n"/>
     </row>
-    <row r="10" ht="40.5" customHeight="1">
+    <row r="10">
       <c r="A10" s="6" t="n">
         <v>4</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>membership_id</t>
+          <t>assigned_at</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -27413,57 +27427,57 @@
           <t>không</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>memberships.membership_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Thành viên (người trong tổ chức này) có các vai trò cấp đội xe (FLEET_MANAGER, DISPATCHER) chỉ áp dụng cho các đội xe được liệt kê.</t>
+          <t>Thời điểm người dùng được giao đội xe này.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>00000022-5a6b-4c7d-8e9f-0a1b2c3d4e5f</t>
+          <t>2026-09-01T02:00:00Z</t>
         </is>
       </c>
       <c r="I10" s="6" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>assigned_at</t>
+          <t>assigned_by</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>users.user_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm người dùng được giao đội xe này.</t>
+          <t>Ai đã giao (thường là ORG_ADMIN); NULL khi hệ thống tự giao.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
+          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
         </is>
       </c>
       <c r="I11" s="6" t="n"/>
@@ -27501,62 +27515,104 @@
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="inlineStr">
+    <row r="13" ht="27" customHeight="1">
+      <c r="A13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>unassigned_by</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>users.user_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Ai đã thu lại; NULL khi còn hiệu lực, hoặc khi hệ thống tự kết thúc (thành viên rời tổ chức hoặc đội bị xóa).</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n"/>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="27" customHeight="1">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6" t="inlineStr">
+    <row r="16" ht="27" customHeight="1">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>uq_fleet_user_assignments_active</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>fleet_id, membership_id</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>có</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>WHERE unassigned_at IS NULL</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I12"/>
+  <autoFilter ref="A6:I13"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F8" location="'organizations'!A1"/>
-    <hyperlink ref="F9" location="'fleets'!A1"/>
-    <hyperlink ref="F10" location="'memberships'!A1"/>
+    <hyperlink ref="F8" location="'fleets'!A1"/>
+    <hyperlink ref="F9" location="'memberships'!A1"/>
+    <hyperlink ref="F11" location="'users'!A1"/>
+    <hyperlink ref="F13" location="'users'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(domain-model): review the tariffs table
A tariff belongs to the organization owning the locations it prices, as
the owner's default or for one location; its prices move to immutable
versions (BL-08).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -74,17 +74,18 @@
     <sheet name="charging_policy_assignments" sheetId="65" state="visible" r:id="rId65"/>
     <sheet name="policy_violations" sheetId="66" state="visible" r:id="rId66"/>
     <sheet name="tariffs" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="payments" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="wallets" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="wallet_transactions" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="invoices" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet name="invoice_lines" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet name="subscription_plans" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet name="plan_features" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet name="subscriptions" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet name="driver_scores" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet name="promotion_campaigns" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet name="trips" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="tariff_history" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="payments" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="wallets" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="wallet_transactions" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="invoices" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="invoice_lines" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="subscription_plans" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="plan_features" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="subscriptions" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="driver_scores" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="promotion_campaigns" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="trips" sheetId="79" state="visible" r:id="rId79"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'organizations'!$A$7:$I$20</definedName>
@@ -152,18 +153,19 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="63" hidden="1">'charging_policy_versions'!$A$6:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="64" hidden="1">'charging_policy_assignments'!$A$6:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="65" hidden="1">'policy_violations'!$A$6:$I$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="66" hidden="1">'tariffs'!$A$6:$I$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="67" hidden="1">'payments'!$A$6:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="68" hidden="1">'wallets'!$A$6:$I$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="69" hidden="1">'wallet_transactions'!$A$6:$I$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="70" hidden="1">'invoices'!$A$6:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="71" hidden="1">'invoice_lines'!$A$6:$I$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="72" hidden="1">'subscription_plans'!$A$6:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="73" hidden="1">'plan_features'!$A$6:$I$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="74" hidden="1">'subscriptions'!$A$6:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="75" hidden="1">'driver_scores'!$A$6:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="76" hidden="1">'promotion_campaigns'!$A$6:$I$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="77" hidden="1">'trips'!$A$6:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="66" hidden="1">'tariffs'!$A$7:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="67" hidden="1">'tariff_history'!$A$7:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="68" hidden="1">'payments'!$A$6:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="69" hidden="1">'wallets'!$A$6:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="70" hidden="1">'wallet_transactions'!$A$6:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="71" hidden="1">'invoices'!$A$6:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="72" hidden="1">'invoice_lines'!$A$6:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="73" hidden="1">'subscription_plans'!$A$6:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="74" hidden="1">'plan_features'!$A$6:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="75" hidden="1">'subscriptions'!$A$6:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="76" hidden="1">'driver_scores'!$A$6:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="77" hidden="1">'promotion_campaigns'!$A$6:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="78" hidden="1">'trips'!$A$6:$I$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -652,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I120"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -683,7 +685,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>77 bảng trong 16 miền nghiệp vụ: 58 bảng chính, 16 bảng lịch sử (N.h), 3 bảng trạng thái. Bấm vào tên bảng hoặc «→ Mở» để mở sheet chi tiết của bảng; chú giải và các quyết định còn mở nằm ở cuối trang.</t>
+          <t>78 bảng trong 16 miền nghiệp vụ: 58 bảng chính, 17 bảng lịch sử (N.h), 3 bảng trạng thái. Bấm vào tên bảng hoặc «→ Mở» để mở sheet chi tiết của bảng; chú giải và các quyết định còn mở nằm ở cuối trang.</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3981,7 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>9 bảng</t>
+          <t>10 bảng</t>
         </is>
       </c>
       <c r="D84" s="5" t="n"/>
@@ -3997,7 +3999,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="27" customHeight="1">
+    <row r="85" ht="81" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
           <t>50</t>
@@ -4015,12 +4017,12 @@
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>Biểu giá điện</t>
+          <t>Biểu giá</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>Nội bộ</t>
+          <t>Khách hàng</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
@@ -4030,11 +4032,11 @@
       </c>
       <c r="G85" s="6" t="inlineStr">
         <is>
-          <t>Giá điện. Ai sở hữu biểu giá (G3 Energy hay G3 Network) là mục 5 của feature-list.</t>
+          <t>Giá của ai và áp dụng ở đâu (BL-08); giá cụ thể là các phiên bản không sửa được trong tariff_versions, nên biên nhận luôn hiện đúng giá đã tính. Giá tại một trạm là biểu giá ACTIVE của chính trạm đó, nếu không có thì là biểu giá mặc định của chủ sở hữu. Bật lịch sử thay đổi; không xóa mềm. Sau này: giá riêng theo hợp đồng của một khách hàng, và giá khác nhau theo từng trụ trong cùng một trạm.</t>
         </is>
       </c>
       <c r="H85" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
@@ -4042,10 +4044,10 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="27" customHeight="1">
+    <row r="86" ht="40.5" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>50.h</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
@@ -4055,12 +4057,12 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>tariff_history</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Thanh toán</t>
+          <t>Lịch sử biểu giá</t>
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr">
@@ -4070,16 +4072,16 @@
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
-          <t>F-H1</t>
+          <t>F-C8, F-H1</t>
         </is>
       </c>
       <c r="G86" s="6" t="inlineStr">
         <is>
-          <t>Một lần thanh toán qua cổng thanh toán hoặc ví, thường cho một phiên sạc.</t>
+          <t>Mọi phiên bản trước đây của một dòng trong bảng tariffs: bản sao toàn bộ dòng, chụp ngay trước khi thay đổi và được trigger ghi trong cùng giao dịch. Do công cụ domain-model tự sinh từ @tracked *, không bao giờ viết tay.</t>
         </is>
       </c>
       <c r="H86" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I86" s="7" t="inlineStr">
         <is>
@@ -4090,7 +4092,7 @@
     <row r="87" ht="27" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
@@ -4100,12 +4102,12 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>wallets</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>Ví</t>
+          <t>Thanh toán</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr">
@@ -4115,16 +4117,16 @@
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>F-H2</t>
+          <t>F-H1</t>
         </is>
       </c>
       <c r="G87" s="6" t="inlineStr">
         <is>
-          <t>Số dư trả trước của một tài xế hoặc của cả tổ chức.</t>
+          <t>Một lần thanh toán qua cổng thanh toán hoặc ví, thường cho một phiên sạc.</t>
         </is>
       </c>
       <c r="H87" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I87" s="7" t="inlineStr">
         <is>
@@ -4135,7 +4137,7 @@
     <row r="88" ht="27" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
@@ -4145,12 +4147,12 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>wallet_transactions</t>
+          <t>wallets</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>Giao dịch ví</t>
+          <t>Ví</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr">
@@ -4165,11 +4167,11 @@
       </c>
       <c r="G88" s="6" t="inlineStr">
         <is>
-          <t>Biến động tiền vào/ra khỏi ví, chỉ ghi thêm.</t>
+          <t>Số dư trả trước của một tài xế hoặc của cả tổ chức.</t>
         </is>
       </c>
       <c r="H88" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I88" s="7" t="inlineStr">
         <is>
@@ -4180,7 +4182,7 @@
     <row r="89" ht="27" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>53</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
@@ -4190,12 +4192,12 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>wallet_transactions</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>Hóa đơn</t>
+          <t>Giao dịch ví</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
@@ -4205,16 +4207,16 @@
       </c>
       <c r="F89" s="6" t="inlineStr">
         <is>
-          <t>F-H3, F-H4</t>
+          <t>F-H2</t>
         </is>
       </c>
       <c r="G89" s="6" t="inlineStr">
         <is>
-          <t>Một hóa đơn điện tử hợp lệ. Khi đã PHÁT HÀNH thì không sửa, chỉ điều chỉnh hoặc hủy bằng hóa đơn mới.</t>
+          <t>Biến động tiền vào/ra khỏi ví, chỉ ghi thêm.</t>
         </is>
       </c>
       <c r="H89" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I89" s="7" t="inlineStr">
         <is>
@@ -4225,617 +4227,662 @@
     <row r="90" ht="27" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>Thanh toán &amp; hóa đơn (billing)</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr">
+        <is>
+          <t>Hóa đơn</t>
+        </is>
+      </c>
+      <c r="E90" s="6" t="inlineStr">
+        <is>
+          <t>Khách hàng</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="inlineStr">
+        <is>
+          <t>F-H3, F-H4</t>
+        </is>
+      </c>
+      <c r="G90" s="6" t="inlineStr">
+        <is>
+          <t>Một hóa đơn điện tử hợp lệ. Khi đã PHÁT HÀNH thì không sửa, chỉ điều chỉnh hoặc hủy bằng hóa đơn mới.</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I90" s="7" t="inlineStr">
+        <is>
+          <t>→ Mở</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="27" customHeight="1">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
           <t>55</t>
         </is>
       </c>
-      <c r="B90" s="6" t="inlineStr">
+      <c r="B91" s="6" t="inlineStr">
         <is>
           <t>Thanh toán &amp; hóa đơn (billing)</t>
         </is>
       </c>
-      <c r="C90" s="7" t="inlineStr">
+      <c r="C91" s="7" t="inlineStr">
         <is>
           <t>invoice_lines</t>
         </is>
       </c>
-      <c r="D90" s="7" t="inlineStr">
+      <c r="D91" s="7" t="inlineStr">
         <is>
           <t>Dòng hóa đơn</t>
         </is>
       </c>
-      <c r="E90" s="6" t="inlineStr">
+      <c r="E91" s="6" t="inlineStr">
         <is>
           <t>Khách hàng</t>
         </is>
       </c>
-      <c r="F90" s="6" t="inlineStr">
+      <c r="F91" s="6" t="inlineStr">
         <is>
           <t>F-H3, F-H4</t>
         </is>
       </c>
-      <c r="G90" s="6" t="inlineStr">
+      <c r="G91" s="6" t="inlineStr">
         <is>
           <t>Một dòng của hóa đơn: một phiên sạc hoặc một kỳ thuê bao.</t>
         </is>
       </c>
-      <c r="H90" s="6" t="n">
+      <c r="H91" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="I90" s="7" t="inlineStr">
+      <c r="I91" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="54" customHeight="1">
-      <c r="A91" s="6" t="inlineStr">
+    <row r="92" ht="54" customHeight="1">
+      <c r="A92" s="6" t="inlineStr">
         <is>
           <t>56</t>
         </is>
       </c>
-      <c r="B91" s="6" t="inlineStr">
+      <c r="B92" s="6" t="inlineStr">
         <is>
           <t>Thanh toán &amp; hóa đơn (billing)</t>
         </is>
       </c>
-      <c r="C91" s="7" t="inlineStr">
+      <c r="C92" s="7" t="inlineStr">
         <is>
           <t>subscription_plans</t>
         </is>
       </c>
-      <c r="D91" s="7" t="inlineStr">
+      <c r="D92" s="7" t="inlineStr">
         <is>
           <t>Gói dịch vụ</t>
         </is>
       </c>
-      <c r="E91" s="6" t="inlineStr">
+      <c r="E92" s="6" t="inlineStr">
         <is>
           <t>Nội bộ</t>
         </is>
       </c>
-      <c r="F91" s="6" t="inlineStr">
+      <c r="F92" s="6" t="inlineStr">
         <is>
           <t>F-H4</t>
         </is>
       </c>
-      <c r="G91" s="6" t="inlineStr">
+      <c r="G92" s="6" t="inlineStr">
         <is>
           <t>Một gói dịch vụ: mỗi gói là một dòng (GUEST là gói mặc định miễn phí, STANDARD, ADVANCED, PRO, ..., hoặc gói riêng cho một khách hàng); tính năng của gói nằm ở plan_features. Giá được tính theo từng tính năng (xem ghi chú của miền thanh toán).</t>
         </is>
       </c>
-      <c r="H91" s="6" t="n">
+      <c r="H92" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="I91" s="7" t="inlineStr">
+      <c r="I92" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="40.5" customHeight="1">
-      <c r="A92" s="6" t="inlineStr">
+    <row r="93" ht="40.5" customHeight="1">
+      <c r="A93" s="6" t="inlineStr">
         <is>
           <t>57</t>
         </is>
       </c>
-      <c r="B92" s="6" t="inlineStr">
+      <c r="B93" s="6" t="inlineStr">
         <is>
           <t>Thanh toán &amp; hóa đơn (billing)</t>
         </is>
       </c>
-      <c r="C92" s="7" t="inlineStr">
+      <c r="C93" s="7" t="inlineStr">
         <is>
           <t>plan_features</t>
         </is>
       </c>
-      <c r="D92" s="7" t="inlineStr">
+      <c r="D93" s="7" t="inlineStr">
         <is>
           <t>Tính năng của gói dịch vụ</t>
         </is>
       </c>
-      <c r="E92" s="6" t="inlineStr">
+      <c r="E93" s="6" t="inlineStr">
         <is>
           <t>Nội bộ</t>
         </is>
       </c>
-      <c r="F92" s="6" t="inlineStr">
+      <c r="F93" s="6" t="inlineStr">
         <is>
           <t>F-H4</t>
         </is>
       </c>
-      <c r="G92" s="6" t="inlineStr">
+      <c r="G93" s="6" t="inlineStr">
         <is>
           <t>Mỗi gói dịch vụ gồm những tính năng nào. Gói dịch vụ là dữ liệu, nên G3 có thể tạo gói mới (Pro, Max, gói riêng cho một khách hàng) trên portal mà không cần lập trình viên; chỉ tính năng hoàn toàn mới mới cần viết mã.</t>
         </is>
       </c>
-      <c r="H92" s="6" t="n">
+      <c r="H93" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="I92" s="7" t="inlineStr">
+      <c r="I93" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="27" customHeight="1">
-      <c r="A93" s="6" t="inlineStr">
+    <row r="94" ht="27" customHeight="1">
+      <c r="A94" s="6" t="inlineStr">
         <is>
           <t>58</t>
         </is>
       </c>
-      <c r="B93" s="6" t="inlineStr">
+      <c r="B94" s="6" t="inlineStr">
         <is>
           <t>Thanh toán &amp; hóa đơn (billing)</t>
         </is>
       </c>
-      <c r="C93" s="7" t="inlineStr">
+      <c r="C94" s="7" t="inlineStr">
         <is>
           <t>subscriptions</t>
         </is>
       </c>
-      <c r="D93" s="7" t="inlineStr">
+      <c r="D94" s="7" t="inlineStr">
         <is>
           <t>Thuê bao</t>
         </is>
       </c>
-      <c r="E93" s="6" t="inlineStr">
+      <c r="E94" s="6" t="inlineStr">
         <is>
           <t>Khách hàng</t>
         </is>
       </c>
-      <c r="F93" s="6" t="inlineStr">
+      <c r="F94" s="6" t="inlineStr">
         <is>
           <t>F-H4</t>
         </is>
       </c>
-      <c r="G93" s="6" t="inlineStr">
+      <c r="G94" s="6" t="inlineStr">
         <is>
           <t>Một xe đăng ký một gói; quá hạn thanh toán sẽ khóa tính năng.</t>
         </is>
       </c>
-      <c r="H93" s="6" t="n">
+      <c r="H94" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="I93" s="7" t="inlineStr">
+      <c r="I94" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="27" customHeight="1">
-      <c r="A94" s="5" t="n"/>
-      <c r="B94" s="5" t="inlineStr">
+    <row r="95" ht="27" customHeight="1">
+      <c r="A95" s="5" t="n"/>
+      <c r="B95" s="5" t="inlineStr">
         <is>
           <t>Chấm điểm tài xế (scoring)</t>
         </is>
       </c>
-      <c r="C94" s="5" t="inlineStr">
+      <c r="C95" s="5" t="inlineStr">
         <is>
           <t>1 bảng</t>
         </is>
       </c>
-      <c r="D94" s="5" t="n"/>
-      <c r="E94" s="5" t="n"/>
-      <c r="F94" s="5" t="n"/>
-      <c r="G94" s="5" t="inlineStr">
+      <c r="D95" s="5" t="n"/>
+      <c r="E95" s="5" t="n"/>
+      <c r="F95" s="5" t="n"/>
+      <c r="G95" s="5" t="inlineStr">
         <is>
           <t>Chấm điểm an toàn cho tài xế từ hành vi lái xe.
 • Mỗi tuần, mỗi tài xế có một điểm, tính từ dữ liệu vận hành của xe họ lái.</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="6" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="6" t="inlineStr">
         <is>
           <t>59</t>
         </is>
       </c>
-      <c r="B95" s="6" t="inlineStr">
+      <c r="B96" s="6" t="inlineStr">
         <is>
           <t>Chấm điểm tài xế (scoring)</t>
         </is>
       </c>
-      <c r="C95" s="7" t="inlineStr">
+      <c r="C96" s="7" t="inlineStr">
         <is>
           <t>driver_scores</t>
         </is>
       </c>
-      <c r="D95" s="7" t="inlineStr">
+      <c r="D96" s="7" t="inlineStr">
         <is>
           <t>Điểm tài xế</t>
         </is>
       </c>
-      <c r="E95" s="6" t="inlineStr">
+      <c r="E96" s="6" t="inlineStr">
         <is>
           <t>Khách hàng</t>
         </is>
       </c>
-      <c r="F95" s="6" t="inlineStr">
+      <c r="F96" s="6" t="inlineStr">
         <is>
           <t>F-K1</t>
         </is>
       </c>
-      <c r="G95" s="6" t="inlineStr">
+      <c r="G96" s="6" t="inlineStr">
         <is>
           <t>Điểm an toàn hằng tuần của tài xế, tính từ dữ liệu vận hành xe.</t>
         </is>
       </c>
-      <c r="H95" s="6" t="n">
+      <c r="H96" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="I95" s="7" t="inlineStr">
+      <c r="I96" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="27" customHeight="1">
-      <c r="A96" s="5" t="n"/>
-      <c r="B96" s="5" t="inlineStr">
+    <row r="97" ht="27" customHeight="1">
+      <c r="A97" s="5" t="n"/>
+      <c r="B97" s="5" t="inlineStr">
         <is>
           <t>Chưa phân miền (unassigned)</t>
         </is>
       </c>
-      <c r="C96" s="5" t="inlineStr">
+      <c r="C97" s="5" t="inlineStr">
         <is>
           <t>2 bảng</t>
         </is>
       </c>
-      <c r="D96" s="5" t="n"/>
-      <c r="E96" s="5" t="n"/>
-      <c r="F96" s="5" t="n"/>
-      <c r="G96" s="5" t="inlineStr">
+      <c r="D97" s="5" t="n"/>
+      <c r="E97" s="5" t="n"/>
+      <c r="F97" s="5" t="n"/>
+      <c r="G97" s="5" t="inlineStr">
         <is>
           <t>Các tính năng chưa được quyết định thuộc miền nghiệp vụ nào (xem feature-list.md).</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="6" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>Chưa phân miền (unassigned)</t>
-        </is>
-      </c>
-      <c r="C97" s="7" t="inlineStr">
-        <is>
-          <t>promotion_campaigns</t>
-        </is>
-      </c>
-      <c r="D97" s="7" t="inlineStr">
-        <is>
-          <t>Chiến dịch khuyến mãi</t>
-        </is>
-      </c>
-      <c r="E97" s="6" t="inlineStr">
-        <is>
-          <t>Nội bộ</t>
-        </is>
-      </c>
-      <c r="F97" s="6" t="inlineStr">
-        <is>
-          <t>F-F4</t>
-        </is>
-      </c>
-      <c r="G97" s="6" t="inlineStr">
-        <is>
-          <t>Một chiến dịch nhắc bảo dưỡng hoặc khuyến mãi.</t>
-        </is>
-      </c>
-      <c r="H97" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="I97" s="7" t="inlineStr">
-        <is>
-          <t>→ Mở</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>Chưa phân miền (unassigned)</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>promotion_campaigns</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr">
+        <is>
+          <t>Chiến dịch khuyến mãi</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>Nội bộ</t>
+        </is>
+      </c>
+      <c r="F98" s="6" t="inlineStr">
+        <is>
+          <t>F-F4</t>
+        </is>
+      </c>
+      <c r="G98" s="6" t="inlineStr">
+        <is>
+          <t>Một chiến dịch nhắc bảo dưỡng hoặc khuyến mãi.</t>
+        </is>
+      </c>
+      <c r="H98" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I98" s="7" t="inlineStr">
+        <is>
+          <t>→ Mở</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
           <t>61</t>
         </is>
       </c>
-      <c r="B98" s="6" t="inlineStr">
+      <c r="B99" s="6" t="inlineStr">
         <is>
           <t>Chưa phân miền (unassigned)</t>
         </is>
       </c>
-      <c r="C98" s="7" t="inlineStr">
+      <c r="C99" s="7" t="inlineStr">
         <is>
           <t>trips</t>
         </is>
       </c>
-      <c r="D98" s="7" t="inlineStr">
+      <c r="D99" s="7" t="inlineStr">
         <is>
           <t>Chuyến đi</t>
         </is>
       </c>
-      <c r="E98" s="6" t="inlineStr">
+      <c r="E99" s="6" t="inlineStr">
         <is>
           <t>Khách hàng</t>
         </is>
       </c>
-      <c r="F98" s="6" t="inlineStr">
+      <c r="F99" s="6" t="inlineStr">
         <is>
           <t>F-A9</t>
         </is>
       </c>
-      <c r="G98" s="6" t="inlineStr">
+      <c r="G99" s="6" t="inlineStr">
         <is>
           <t>Một chuyến đi của xe. F-A9 đang tạm dừng: chưa có khái niệm chuyến đi.</t>
         </is>
       </c>
-      <c r="H98" s="6" t="n">
+      <c r="H99" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="I98" s="7" t="inlineStr">
+      <c r="I99" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="99"/>
-    <row r="100" ht="27" customHeight="1">
-      <c r="A100" s="4" t="inlineStr">
+    <row r="100"/>
+    <row r="101" ht="27" customHeight="1">
+      <c r="A101" s="4" t="inlineStr">
         <is>
           <t>Chú giải</t>
         </is>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B101" s="4" t="inlineStr">
         <is>
           <t>Ý nghĩa</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="108" customHeight="1">
-      <c r="A101" s="6" t="inlineStr">
+    <row r="102" ht="108" customHeight="1">
+      <c r="A102" s="6" t="inlineStr">
         <is>
           <t>Chủ sở hữu dữ liệu: Khách hàng</t>
         </is>
       </c>
-      <c r="B101" s="6" t="inlineStr">
+      <c r="B102" s="6" t="inlineStr">
         <is>
           <t>Thuộc về một tổ chức (thường là khách hàng; công ty G3 cũng có thể sở hữu); có cột organization_id hoặc lấy qua bảng cha (DM-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="94.5" customHeight="1">
-      <c r="A102" s="6" t="inlineStr">
-        <is>
-          <t>Chủ sở hữu dữ liệu: Nội bộ</t>
-        </is>
-      </c>
-      <c r="B102" s="6" t="inlineStr">
-        <is>
-          <t>Dữ liệu của chính chúng ta (đơn vị vận hành nền tảng), dùng chung cho mọi tổ chức.</t>
         </is>
       </c>
     </row>
     <row r="103" ht="94.5" customHeight="1">
       <c r="A103" s="6" t="inlineStr">
         <is>
+          <t>Chủ sở hữu dữ liệu: Nội bộ</t>
+        </is>
+      </c>
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>Dữ liệu của chính chúng ta (đơn vị vận hành nền tảng), dùng chung cho mọi tổ chức.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="94.5" customHeight="1">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
           <t>Chủ sở hữu dữ liệu: Hai bên</t>
         </is>
       </c>
-      <c r="B103" s="6" t="inlineStr">
+      <c r="B104" s="6" t="inlineStr">
         <is>
           <t>Tài sản của G3 được khách hàng sử dụng; cả hai bên cùng liên quan.</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="121.5" customHeight="1">
-      <c r="A104" s="6" t="inlineStr">
+    <row r="105" ht="121.5" customHeight="1">
+      <c r="A105" s="6" t="inlineStr">
         <is>
           <t>Chủ sở hữu dữ liệu: Chưa quyết định</t>
         </is>
       </c>
-      <c r="B104" s="6" t="inlineStr">
+      <c r="B105" s="6" t="inlineStr">
         <is>
           <t>Đang chờ một quyết định còn mở (xem cuối trang).</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="81" customHeight="1">
-      <c r="A105" s="6" t="inlineStr">
+    <row r="106" ht="81" customHeight="1">
+      <c r="A106" s="6" t="inlineStr">
         <is>
           <t>Miền nghiệp vụ (domain)</t>
         </is>
       </c>
-      <c r="B105" s="6" t="inlineStr">
+      <c r="B106" s="6" t="inlineStr">
         <is>
           <t>Một phần của hệ thống sở hữu dữ liệu riêng, ví dụ Xe, Trạm sạc, Thanh toán. Mỗi miền gồm một hoặc nhiều bảng.</t>
         </is>
       </c>
     </row>
-    <row r="106" ht="54" customHeight="1">
-      <c r="A106" s="6" t="inlineStr">
+    <row r="107" ht="54" customHeight="1">
+      <c r="A107" s="6" t="inlineStr">
         <is>
           <t>Bảng</t>
         </is>
       </c>
-      <c r="B106" s="6" t="inlineStr">
+      <c r="B107" s="6" t="inlineStr">
         <is>
           <t>Một loại dữ liệu được lưu, ví dụ Xe hoặc Phiên sạc. Mỗi bảng có một sheet riêng liệt kê từng cột.</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="40.5" customHeight="1">
-      <c r="A107" s="6" t="inlineStr">
+    <row r="108" ht="40.5" customHeight="1">
+      <c r="A108" s="6" t="inlineStr">
         <is>
           <t>Tính năng</t>
         </is>
       </c>
-      <c r="B107" s="6" t="inlineStr">
+      <c r="B108" s="6" t="inlineStr">
         <is>
           <t>Mã tính năng trong danh sách tính năng (feature-list.md), ví dụ F-B2.</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="67.5" customHeight="1">
-      <c r="A108" s="6" t="inlineStr">
+    <row r="109" ht="67.5" customHeight="1">
+      <c r="A109" s="6" t="inlineStr">
         <is>
           <t>PK / FK / UQ</t>
         </is>
       </c>
-      <c r="B108" s="6" t="inlineStr">
+      <c r="B109" s="6" t="inlineStr">
         <is>
           <t>PK: khóa chính (định danh duy nhất của dòng). FK: khóa ngoại (trỏ tới dòng của bảng khác). UQ: giá trị không được trùng.</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="54" customHeight="1">
-      <c r="A109" s="6" t="inlineStr">
+    <row r="110" ht="54" customHeight="1">
+      <c r="A110" s="6" t="inlineStr">
         <is>
           <t>Ví dụ</t>
         </is>
       </c>
-      <c r="B109" s="6" t="inlineStr">
+      <c r="B110" s="6" t="inlineStr">
         <is>
           <t>Giá trị mẫu. Các mã ví dụ khớp nhau giữa các bảng, nên có thể lần theo một bản ghi mẫu qua nhiều sheet.</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="40.5" customHeight="1">
-      <c r="A110" s="6" t="inlineStr">
+    <row r="111" ht="40.5" customHeight="1">
+      <c r="A111" s="6" t="inlineStr">
         <is>
           <t>NULL</t>
         </is>
       </c>
-      <c r="B110" s="6" t="inlineStr">
+      <c r="B111" s="6" t="inlineStr">
         <is>
           <t>Ô không có giá trị. Ý nghĩa của NULL được giải thích trong cột Ý nghĩa.</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="81" customHeight="1">
-      <c r="A111" s="6" t="inlineStr">
+    <row r="112" ht="81" customHeight="1">
+      <c r="A112" s="6" t="inlineStr">
         <is>
           <t>🔍 Lưu lịch sử</t>
         </is>
       </c>
-      <c r="B111" s="6" t="inlineStr">
+      <c r="B112" s="6" t="inlineStr">
         <is>
           <t>Cột được theo dõi: khi cột này thay đổi, toàn bộ dòng cũ được chép sang bảng lịch sử (tên kết thúc bằng _history) kèm thời điểm và người thay đổi.</t>
         </is>
       </c>
     </row>
-    <row r="112"/>
-    <row r="113">
-      <c r="A113" s="8" t="inlineStr">
+    <row r="113"/>
+    <row r="114">
+      <c r="A114" s="8" t="inlineStr">
         <is>
           <t>Các view (giai đoạn đọc từ lịch sử)</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="4" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
         <is>
           <t>View</t>
         </is>
       </c>
-      <c r="B114" s="4" t="inlineStr">
+      <c r="B115" s="4" t="inlineStr">
         <is>
           <t>Mỗi dòng là</t>
         </is>
       </c>
-      <c r="C114" s="4" t="inlineStr">
+      <c r="C115" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D114" s="4" t="inlineStr">
+      <c r="D115" s="4" t="inlineStr">
         <is>
           <t>Được dùng bởi</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="94.5" customHeight="1">
-      <c r="A115" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_ownership_periods</t>
-        </is>
-      </c>
-      <c r="B115" s="6" t="inlineStr">
-        <is>
-          <t>một giai đoạn xe thuộc một chủ</t>
-        </is>
-      </c>
-      <c r="C115" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id, organization_id, owned_from, owned_until (NULL với chủ hiện tại)</t>
-        </is>
-      </c>
-      <c r="D115" s="6" t="inlineStr">
-        <is>
-          <t>lịch sử sở hữu và ngày bàn giao đầu tiên (VEH-02), "ngày đó xe của ai"</t>
         </is>
       </c>
     </row>
     <row r="116" ht="94.5" customHeight="1">
       <c r="A116" s="6" t="inlineStr">
         <is>
+          <t>vehicle_ownership_periods</t>
+        </is>
+      </c>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
+          <t>một giai đoạn xe thuộc một chủ</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id, organization_id, owned_from, owned_until (NULL với chủ hiện tại)</t>
+        </is>
+      </c>
+      <c r="D116" s="6" t="inlineStr">
+        <is>
+          <t>lịch sử sở hữu và ngày bàn giao đầu tiên (VEH-02), "ngày đó xe của ai"</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="94.5" customHeight="1">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
           <t>battery_installation_periods</t>
         </is>
       </c>
-      <c r="B116" s="6" t="inlineStr">
+      <c r="B117" s="6" t="inlineStr">
         <is>
           <t>một lần pin nằm trên một xe</t>
         </is>
       </c>
-      <c r="C116" s="6" t="inlineStr">
+      <c r="C117" s="6" t="inlineStr">
         <is>
           <t>battery_id, vehicle_id, installed_from, installed_until (NULL khi đang lắp)</t>
         </is>
       </c>
-      <c r="D116" s="6" t="inlineStr">
+      <c r="D117" s="6" t="inlineStr">
         <is>
           <t>lịch sử sức khỏe pin qua các xe (MON-07), bộ đếm bảo hành pin (WAR-01)</t>
         </is>
       </c>
     </row>
-    <row r="117"/>
-    <row r="118">
-      <c r="A118" s="8" t="inlineStr">
+    <row r="118"/>
+    <row r="119">
+      <c r="A119" s="8" t="inlineStr">
         <is>
           <t>Các quyết định còn mở</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="4" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="4" t="inlineStr">
         <is>
           <t>Mã</t>
         </is>
       </c>
-      <c r="B119" s="4" t="inlineStr">
+      <c r="B120" s="4" t="inlineStr">
         <is>
           <t>Câu hỏi</t>
         </is>
       </c>
-      <c r="C119" s="4" t="inlineStr">
+      <c r="C120" s="4" t="inlineStr">
         <is>
           <t>Ảnh hưởng tới</t>
         </is>
       </c>
     </row>
-    <row r="120" ht="54" customHeight="1">
-      <c r="A120" s="6" t="inlineStr">
+    <row r="121" ht="54" customHeight="1">
+      <c r="A121" s="6" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B120" s="6" t="inlineStr">
+      <c r="B121" s="6" t="inlineStr">
         <is>
           <t>Ai trả tiền khi tài xế của đội xe sạc: ví của tài xế, ví của đội xe, hay tùy trường hợp?</t>
         </is>
       </c>
-      <c r="C120" s="6" t="inlineStr">
+      <c r="C121" s="6" t="inlineStr">
         <is>
           <t>wallets, payments</t>
         </is>
@@ -5041,39 +5088,42 @@
     <hyperlink ref="C85" location="'tariffs'!A1"/>
     <hyperlink ref="D85" location="'tariffs'!A1"/>
     <hyperlink ref="I85" location="'tariffs'!A1"/>
-    <hyperlink ref="C86" location="'payments'!A1"/>
-    <hyperlink ref="D86" location="'payments'!A1"/>
-    <hyperlink ref="I86" location="'payments'!A1"/>
-    <hyperlink ref="C87" location="'wallets'!A1"/>
-    <hyperlink ref="D87" location="'wallets'!A1"/>
-    <hyperlink ref="I87" location="'wallets'!A1"/>
-    <hyperlink ref="C88" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="D88" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="I88" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="C89" location="'invoices'!A1"/>
-    <hyperlink ref="D89" location="'invoices'!A1"/>
-    <hyperlink ref="I89" location="'invoices'!A1"/>
-    <hyperlink ref="C90" location="'invoice_lines'!A1"/>
-    <hyperlink ref="D90" location="'invoice_lines'!A1"/>
-    <hyperlink ref="I90" location="'invoice_lines'!A1"/>
-    <hyperlink ref="C91" location="'subscription_plans'!A1"/>
-    <hyperlink ref="D91" location="'subscription_plans'!A1"/>
-    <hyperlink ref="I91" location="'subscription_plans'!A1"/>
-    <hyperlink ref="C92" location="'plan_features'!A1"/>
-    <hyperlink ref="D92" location="'plan_features'!A1"/>
-    <hyperlink ref="I92" location="'plan_features'!A1"/>
-    <hyperlink ref="C93" location="'subscriptions'!A1"/>
-    <hyperlink ref="D93" location="'subscriptions'!A1"/>
-    <hyperlink ref="I93" location="'subscriptions'!A1"/>
-    <hyperlink ref="C95" location="'driver_scores'!A1"/>
-    <hyperlink ref="D95" location="'driver_scores'!A1"/>
-    <hyperlink ref="I95" location="'driver_scores'!A1"/>
-    <hyperlink ref="C97" location="'promotion_campaigns'!A1"/>
-    <hyperlink ref="D97" location="'promotion_campaigns'!A1"/>
-    <hyperlink ref="I97" location="'promotion_campaigns'!A1"/>
-    <hyperlink ref="C98" location="'trips'!A1"/>
-    <hyperlink ref="D98" location="'trips'!A1"/>
-    <hyperlink ref="I98" location="'trips'!A1"/>
+    <hyperlink ref="C86" location="'tariff_history'!A1"/>
+    <hyperlink ref="D86" location="'tariff_history'!A1"/>
+    <hyperlink ref="I86" location="'tariff_history'!A1"/>
+    <hyperlink ref="C87" location="'payments'!A1"/>
+    <hyperlink ref="D87" location="'payments'!A1"/>
+    <hyperlink ref="I87" location="'payments'!A1"/>
+    <hyperlink ref="C88" location="'wallets'!A1"/>
+    <hyperlink ref="D88" location="'wallets'!A1"/>
+    <hyperlink ref="I88" location="'wallets'!A1"/>
+    <hyperlink ref="C89" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="D89" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="I89" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="C90" location="'invoices'!A1"/>
+    <hyperlink ref="D90" location="'invoices'!A1"/>
+    <hyperlink ref="I90" location="'invoices'!A1"/>
+    <hyperlink ref="C91" location="'invoice_lines'!A1"/>
+    <hyperlink ref="D91" location="'invoice_lines'!A1"/>
+    <hyperlink ref="I91" location="'invoice_lines'!A1"/>
+    <hyperlink ref="C92" location="'subscription_plans'!A1"/>
+    <hyperlink ref="D92" location="'subscription_plans'!A1"/>
+    <hyperlink ref="I92" location="'subscription_plans'!A1"/>
+    <hyperlink ref="C93" location="'plan_features'!A1"/>
+    <hyperlink ref="D93" location="'plan_features'!A1"/>
+    <hyperlink ref="I93" location="'plan_features'!A1"/>
+    <hyperlink ref="C94" location="'subscriptions'!A1"/>
+    <hyperlink ref="D94" location="'subscriptions'!A1"/>
+    <hyperlink ref="I94" location="'subscriptions'!A1"/>
+    <hyperlink ref="C96" location="'driver_scores'!A1"/>
+    <hyperlink ref="D96" location="'driver_scores'!A1"/>
+    <hyperlink ref="I96" location="'driver_scores'!A1"/>
+    <hyperlink ref="C98" location="'promotion_campaigns'!A1"/>
+    <hyperlink ref="D98" location="'promotion_campaigns'!A1"/>
+    <hyperlink ref="I98" location="'promotion_campaigns'!A1"/>
+    <hyperlink ref="C99" location="'trips'!A1"/>
+    <hyperlink ref="D99" location="'trips'!A1"/>
+    <hyperlink ref="I99" location="'trips'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10584,7 +10634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11549,7 +11599,7 @@
       <c r="A50" s="6" t="n"/>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>tariffs</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -11562,7 +11612,7 @@
       <c r="A51" s="6" t="n"/>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>wallets</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -11575,7 +11625,7 @@
       <c r="A52" s="6" t="n"/>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>wallet_transactions</t>
+          <t>wallets</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -11588,7 +11638,7 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>wallet_transactions</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -11601,7 +11651,7 @@
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>invoice_lines</t>
+          <t>invoices</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -11614,7 +11664,7 @@
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>subscriptions</t>
+          <t>invoice_lines</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -11627,7 +11677,7 @@
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>driver_scores</t>
+          <t>subscriptions</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -11640,7 +11690,7 @@
       <c r="A57" s="6" t="n"/>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>trips</t>
+          <t>driver_scores</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -11653,10 +11703,23 @@
       <c r="A58" s="6" t="n"/>
       <c r="B58" s="7" t="inlineStr">
         <is>
+          <t>trips</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n"/>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
           <t>organization_history</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>organization_id</t>
         </is>
@@ -11692,15 +11755,16 @@
     <hyperlink ref="B47" location="'maintenance_bookings'!A1"/>
     <hyperlink ref="B48" location="'charging_policy_assignments'!A1"/>
     <hyperlink ref="B49" location="'policy_violations'!A1"/>
-    <hyperlink ref="B50" location="'payments'!A1"/>
-    <hyperlink ref="B51" location="'wallets'!A1"/>
-    <hyperlink ref="B52" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="B53" location="'invoices'!A1"/>
-    <hyperlink ref="B54" location="'invoice_lines'!A1"/>
-    <hyperlink ref="B55" location="'subscriptions'!A1"/>
-    <hyperlink ref="B56" location="'driver_scores'!A1"/>
-    <hyperlink ref="B57" location="'trips'!A1"/>
-    <hyperlink ref="B58" location="'organization_history'!A1"/>
+    <hyperlink ref="B50" location="'tariffs'!A1"/>
+    <hyperlink ref="B51" location="'payments'!A1"/>
+    <hyperlink ref="B52" location="'wallets'!A1"/>
+    <hyperlink ref="B53" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="B54" location="'invoices'!A1"/>
+    <hyperlink ref="B55" location="'invoice_lines'!A1"/>
+    <hyperlink ref="B56" location="'subscriptions'!A1"/>
+    <hyperlink ref="B57" location="'driver_scores'!A1"/>
+    <hyperlink ref="B58" location="'trips'!A1"/>
+    <hyperlink ref="B59" location="'organization_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26052,7 +26116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -27136,6 +27200,19 @@
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>changed_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="n"/>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>tariff_history</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
         <is>
           <t>changed_by</t>
         </is>
@@ -27188,6 +27265,7 @@
     <hyperlink ref="B62" location="'charging_station_history'!A1"/>
     <hyperlink ref="B63" location="'charging_evse_history'!A1"/>
     <hyperlink ref="B64" location="'charging_connector_history'!A1"/>
+    <hyperlink ref="B65" location="'tariff_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27624,7 +27702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -28245,14 +28323,27 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="27" customHeight="1">
+    <row r="27">
       <c r="A27" s="6" t="n"/>
       <c r="B27" s="7" t="inlineStr">
         <is>
+          <t>tariffs</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>location_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="27" customHeight="1">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
           <t>charging_location_history</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>location_id</t>
         </is>
@@ -28266,7 +28357,8 @@
     <hyperlink ref="F9" location="'organizations'!A1"/>
     <hyperlink ref="B25" location="'charging_location_access'!A1"/>
     <hyperlink ref="B26" location="'charging_stations'!A1"/>
-    <hyperlink ref="B27" location="'charging_location_history'!A1"/>
+    <hyperlink ref="B27" location="'tariffs'!A1"/>
+    <hyperlink ref="B28" location="'charging_location_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -29468,7 +29560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -30785,23 +30877,10 @@
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>tariffs</t>
+          <t>charging_station_history</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>station_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="n"/>
-      <c r="B56" s="7" t="inlineStr">
-        <is>
-          <t>charging_station_history</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>station_id</t>
         </is>
@@ -30821,8 +30900,7 @@
     <hyperlink ref="B52" location="'charging_station_config_entries'!A1"/>
     <hyperlink ref="B53" location="'charging_station_commands'!A1"/>
     <hyperlink ref="B54" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B55" location="'tariffs'!A1"/>
-    <hyperlink ref="B56" location="'charging_station_history'!A1"/>
+    <hyperlink ref="B55" location="'charging_station_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -44328,7 +44406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -44345,7 +44423,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>50. tariffs: Biểu giá điện</t>
+          <t>50. tariffs: Biểu giá</t>
         </is>
       </c>
     </row>
@@ -44359,114 +44437,84 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Nội bộ   ·   Tính năng: F-C8, F-H1</t>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-C8, F-H1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Giá điện. Ai sở hữu biểu giá (G3 Energy hay G3 Network) là mục 5 của feature-list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
-    <row r="6" ht="27" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+          <t>Giá của ai và áp dụng ở đâu (BL-08); giá cụ thể là các phiên bản không sửa được trong tariff_versions, nên biên nhận luôn hiện đúng giá đã tính. Giá tại một trạm là biểu giá ACTIVE của chính trạm đó, nếu không có thì là biểu giá mặc định của chủ sở hữu. Bật lịch sử thay đổi; không xóa mềm. Sau này: giá riêng theo hợp đồng của một khách hàng, và giá khác nhau theo từng trụ trong cùng một trạm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>🔍 Lưu lịch sử: khi một cột có dấu 🔍 thay đổi, toàn bộ dòng cũ được chép sang bảng tariff_history.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7" ht="27" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Cột</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Kiểu dữ liệu</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Cho phép rỗng</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Khóa</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Tham chiếu tới</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Ý nghĩa</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Ví dụ</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Lưu lịch sử</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>tariff_id</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Mã nội bộ của biểu giá.</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>f2b9e6c3-1d8a-4f5b-a3c7-9e0d4b1f8a10</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>tariff_code</t>
+          <t>tariff_id</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -44474,106 +44522,126 @@
           <t>không</t>
         </is>
       </c>
-      <c r="E8" s="6" t="n"/>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Mã biểu giá in trên biên nhận.</t>
+          <t>Mã nội bộ của biểu giá.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>TOU-2026-Q4</t>
+          <t>f2b9e6c3-1d8a-4f5b-a3c7-9e0d4b1f8a10</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9" ht="27" customHeight="1">
+    <row r="9" ht="67.5" customHeight="1">
       <c r="A9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Chủ sở hữu: tổ chức có các trạm được định giá bởi biểu giá này (BL-08): tổ chức nội bộ của chúng ta với mạng công cộng, hoặc khách hàng với các trụ riêng của mình (CS-10). Tổ chức nội bộ nào sở hữu mạng công cộng (G3 Energy hay G3 Network, PAY-09) là dữ liệu, không phải thiết kế.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40.5" customHeight="1">
+      <c r="A10" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>station_id</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>location_id</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>uuid</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>có</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>FK</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>charging_stations.station_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Trạm áp dụng; NULL nếu áp dụng toàn mạng.</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>charging_locations.location_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Trạm được định giá; NULL là biểu giá mặc định của chủ sở hữu cho mọi trạm của mình. Trạm phải thuộc chủ sở hữu. Tài xế thấy một giá cho mỗi địa điểm.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>NULL</t>
         </is>
       </c>
-      <c r="I9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="27" customHeight="1">
-      <c r="A10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>price_per_kwh</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>numeric(12,2)</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Đơn giá điện cơ bản cho mỗi kWh, theo đơn vị tiền tệ của biểu giá.</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>4500.00</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="n"/>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>char(3)</t>
+          <t>varchar(100)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -44585,61 +44653,69 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Mã tiền tệ ISO 4217.</t>
+          <t>Tên hiển thị trên ứng dụng và biên nhận.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>VND</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="n"/>
-    </row>
-    <row r="12" ht="27" customHeight="1">
+          <t>Giá chuẩn 2026</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>schedule</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>jsonb</t>
+          <t>char(3)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Các khung giờ giá theo thời điểm trong ngày, dạng JSON.</t>
+          <t>Mã tiền tệ ISO 4217.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>[{"from": "22:00", "to": "04:00", "price_per_kwh": 3200}]</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="n"/>
-    </row>
-    <row r="13">
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>valid_from</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -44651,28 +44727,32 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm biểu giá có hiệu lực.</t>
+          <t>Do chủ sở hữu quyết định. ACTIVE: đang dùng. INACTIVE: đã ngừng.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>2026-10-01T00:00:00Z</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="n"/>
-    </row>
-    <row r="14">
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>valid_to</t>
+          <t>status_reason</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>varchar(200)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -44684,7 +44764,7 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm hết hiệu lực; NULL nếu không thời hạn.</t>
+          <t>Lý do biểu giá có trạng thái hiện tại, ví dụ vì sao ngừng dùng (DM-19); NULL nếu không cần giải thích.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -44692,19 +44772,805 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="I14" s="6" t="n"/>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-01T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:15:00Z</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40.5" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>uq_tariffs_active_owner_location</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>organization_id, location_id</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>WHERE status = ACTIVE, NULLS NOT DISTINCT: one active tariff per location and one default per owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>ix_tariffs_location_id</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>location_id</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>tariff_history</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>tariff_id</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I14"/>
+  <autoFilter ref="A7:I16"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F9" location="'charging_stations'!A1"/>
+    <hyperlink ref="A5" location="'tariff_history'!A1"/>
+    <hyperlink ref="F9" location="'organizations'!A1"/>
+    <hyperlink ref="F10" location="'charging_locations'!A1"/>
+    <hyperlink ref="B23" location="'tariff_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>50.h. tariff_history: Lịch sử biểu giá</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>← Tổng quan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-C8, F-H1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Mọi phiên bản trước đây của một dòng trong bảng tariffs: bản sao toàn bộ dòng, chụp ngay trước khi thay đổi và được trigger ghi trong cùng giao dịch. Do công cụ domain-model tự sinh từ @tracked *, không bao giờ viết tay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Bảng lịch sử của: tariffs</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7" ht="27" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Kiểu dữ liệu</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Cho phép rỗng</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Khóa</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Tham chiếu tới</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Ý nghĩa</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Ví dụ</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Lưu lịch sử</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>history_id</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Mã tự tăng của dòng lịch sử.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>1024</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>tariff_id</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>tariffs.tariff_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Giá trị trước khi thay đổi (tariffs.tariff_id).</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>f2b9e6c3-1d8a-4f5b-a3c7-9e0d4b1f8a10</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Giá trị trước khi thay đổi (tariffs.organization_id).</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>location_id</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Giá trị trước khi thay đổi (tariffs.location_id).</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>varchar(100)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Giá trị trước khi thay đổi (tariffs.name).</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Giá chuẩn 2026</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>char(3)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Giá trị trước khi thay đổi (tariffs.currency).</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Giá trị trước khi thay đổi (tariffs.status).</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>status_reason</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>varchar(200)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Giá trị trước khi thay đổi (tariffs.status_reason).</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Giá trị trước khi thay đổi (tariffs.created_at).</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-01T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Giá trị trước khi thay đổi (tariffs.updated_at).</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:15:00Z</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>changed_at</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm phiên bản này của dòng bị thay thế.</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:15:00Z</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="27" customHeight="1">
+      <c r="A19" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>changed_by</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>users.user_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Người dùng đã thực hiện thay đổi; NULL nếu do hệ thống thực hiện.</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="40.5" customHeight="1">
+      <c r="A20" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>change_reason</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>varchar(200)</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Customer moved to a new office</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="n"/>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="27" customHeight="1">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>ix_tariff_history_tariff_id_time</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>tariff_id, changed_at</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I20"/>
+  <hyperlinks>
+    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
+    <hyperlink ref="A5" location="'tariffs'!A1"/>
+    <hyperlink ref="F9" location="'tariffs'!A1"/>
+    <hyperlink ref="F19" location="'users'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -45184,359 +46050,6 @@
     <hyperlink ref="F8" location="'organizations'!A1"/>
     <hyperlink ref="F9" location="'charging_sessions'!A1"/>
     <hyperlink ref="B19" location="'wallet_transactions'!A1"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>52. wallets: Ví</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>← Tổng quan</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H2</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>Số dư trả trước của một tài xế hoặc của cả tổ chức.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
-    <row r="6" ht="27" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Kiểu dữ liệu</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Cho phép rỗng</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Khóa</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Tham chiếu tới</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Ý nghĩa</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Ví dụ</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Lưu lịch sử</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>wallet_id</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Mã nội bộ của ví.</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>5c3a0e7d-2f9b-4c1e-a8d3-7b6f0c2e9a32</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="27" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Tổ chức khách hàng sở hữu ví.</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>driver_id</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>drivers.driver_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Tài xế sở hữu ví; NULL với ví cấp tổ chức (quyết định D5).</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>balance</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>numeric(14,2)</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Số dư hiện tại; phải bằng tổng các giao dịch của ví.</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>12500000.00</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>currency</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>char(3)</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Mã tiền tệ ISO 4217.</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>VND</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>varchar(20)</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Ví có dùng được không.</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="n"/>
-    </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>wallet_transactions</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>wallet_id</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A6:I12"/>
-  <hyperlinks>
-    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F8" location="'organizations'!A1"/>
-    <hyperlink ref="F9" location="'drivers'!A1"/>
-    <hyperlink ref="B15" location="'wallet_transactions'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -46238,6 +46751,359 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
+          <t>52. wallets: Ví</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>← Tổng quan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Số dư trả trước của một tài xế hoặc của cả tổ chức.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6" ht="27" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Kiểu dữ liệu</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Cho phép rỗng</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Khóa</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Tham chiếu tới</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Ý nghĩa</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Ví dụ</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Lưu lịch sử</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>wallet_id</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Mã nội bộ của ví.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>5c3a0e7d-2f9b-4c1e-a8d3-7b6f0c2e9a32</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="27" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Tổ chức khách hàng sở hữu ví.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>driver_id</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>drivers.driver_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Tài xế sở hữu ví; NULL với ví cấp tổ chức (quyết định D5).</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>numeric(14,2)</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Số dư hiện tại; phải bằng tổng các giao dịch của ví.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>12500000.00</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>char(3)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Mã tiền tệ ISO 4217.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Ví có dùng được không.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n"/>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>wallet_transactions</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>wallet_id</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:I12"/>
+  <hyperlinks>
+    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
+    <hyperlink ref="F8" location="'organizations'!A1"/>
+    <hyperlink ref="F9" location="'drivers'!A1"/>
+    <hyperlink ref="B15" location="'wallet_transactions'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
           <t>53. wallet_transactions: Giao dịch ví</t>
         </is>
       </c>
@@ -46657,7 +47523,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47133,7 +47999,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47575,7 +48441,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47961,7 +48827,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -48251,401 +49117,6 @@
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F8" location="'subscription_plans'!A1"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>58. subscriptions: Thuê bao</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>← Tổng quan</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H4</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>Một xe đăng ký một gói; quá hạn thanh toán sẽ khóa tính năng.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
-    <row r="6" ht="27" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Kiểu dữ liệu</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Cho phép rỗng</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Khóa</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Tham chiếu tới</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Ý nghĩa</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Ví dụ</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Lưu lịch sử</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>subscription_id</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Mã nội bộ của thuê bao.</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>9a7e4c1b-6d3f-4a5c-b0e8-2f1d7c9b3e54</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="27" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Tổ chức khách hàng đăng ký.</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="27" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>plan_id</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>subscription_plans.plan_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Gói được đăng ký.</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>0c9a6e3d-8f5b-4c7e-a2d1-4b3f9e6c0a65</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="27" customHeight="1">
-      <c r="A10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>vehicles.vehicle_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Xe được áp dụng.</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>started_at</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm bắt đầu thuê bao.</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-01T00:00:00Z</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>ends_at</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm kết thúc; NULL nếu tự gia hạn cho tới khi hủy.</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="n"/>
-    </row>
-    <row r="13" ht="27" customHeight="1">
-      <c r="A13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>varchar(20)</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Trạng thái thuê bao; OVERDUE sẽ khóa các tính năng trả phí. Giá trị: ACTIVE | OVERDUE | EXPIRED | CANCELLED.</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="n"/>
-    </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>invoice_lines</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>subscription_id</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A6:I13"/>
-  <hyperlinks>
-    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F8" location="'organizations'!A1"/>
-    <hyperlink ref="F9" location="'subscription_plans'!A1"/>
-    <hyperlink ref="F10" location="'vehicles'!A1"/>
-    <hyperlink ref="B16" location="'invoice_lines'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -48674,6 +49145,401 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
+          <t>58. subscriptions: Thuê bao</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>← Tổng quan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Một xe đăng ký một gói; quá hạn thanh toán sẽ khóa tính năng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6" ht="27" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Kiểu dữ liệu</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Cho phép rỗng</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Khóa</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Tham chiếu tới</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Ý nghĩa</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Ví dụ</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Lưu lịch sử</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>subscription_id</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Mã nội bộ của thuê bao.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>9a7e4c1b-6d3f-4a5c-b0e8-2f1d7c9b3e54</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="27" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Tổ chức khách hàng đăng ký.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="27" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>plan_id</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>subscription_plans.plan_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Gói được đăng ký.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>0c9a6e3d-8f5b-4c7e-a2d1-4b3f9e6c0a65</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="27" customHeight="1">
+      <c r="A10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>vehicles.vehicle_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Xe được áp dụng.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>started_at</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm bắt đầu thuê bao.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-01T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>ends_at</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm kết thúc; NULL nếu tự gia hạn cho tới khi hủy.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="27" customHeight="1">
+      <c r="A13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Trạng thái thuê bao; OVERDUE sẽ khóa các tính năng trả phí. Giá trị: ACTIVE | OVERDUE | EXPIRED | CANCELLED.</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n"/>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>invoice_lines</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>subscription_id</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:I13"/>
+  <hyperlinks>
+    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
+    <hyperlink ref="F8" location="'organizations'!A1"/>
+    <hyperlink ref="F9" location="'subscription_plans'!A1"/>
+    <hyperlink ref="F10" location="'vehicles'!A1"/>
+    <hyperlink ref="B16" location="'invoice_lines'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
           <t>59. driver_scores: Điểm tài xế</t>
         </is>
       </c>
@@ -49054,7 +49920,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -49361,7 +50227,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs(domain-model): design the tariff versions table
Immutable price sets per tariff version; the price shown at the scan is
frozen for the whole session on its billing record (BL-09).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -75,17 +75,18 @@
     <sheet name="policy_violations" sheetId="66" state="visible" r:id="rId66"/>
     <sheet name="tariffs" sheetId="67" state="visible" r:id="rId67"/>
     <sheet name="tariff_history" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="payments" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="wallets" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="wallet_transactions" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet name="invoices" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet name="invoice_lines" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet name="subscription_plans" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet name="plan_features" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet name="subscriptions" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet name="driver_scores" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet name="promotion_campaigns" sheetId="78" state="visible" r:id="rId78"/>
-    <sheet name="trips" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet name="tariff_versions" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="payments" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="wallets" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="wallet_transactions" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="invoices" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="invoice_lines" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="subscription_plans" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="plan_features" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="subscriptions" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="driver_scores" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="promotion_campaigns" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet name="trips" sheetId="80" state="visible" r:id="rId80"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'organizations'!$A$7:$I$20</definedName>
@@ -155,17 +156,18 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="65" hidden="1">'policy_violations'!$A$6:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="66" hidden="1">'tariffs'!$A$7:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="67" hidden="1">'tariff_history'!$A$7:$I$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="68" hidden="1">'payments'!$A$6:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="69" hidden="1">'wallets'!$A$6:$I$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="70" hidden="1">'wallet_transactions'!$A$6:$I$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="71" hidden="1">'invoices'!$A$6:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="72" hidden="1">'invoice_lines'!$A$6:$I$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="73" hidden="1">'subscription_plans'!$A$6:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="74" hidden="1">'plan_features'!$A$6:$I$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="75" hidden="1">'subscriptions'!$A$6:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="76" hidden="1">'driver_scores'!$A$6:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="77" hidden="1">'promotion_campaigns'!$A$6:$I$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="78" hidden="1">'trips'!$A$6:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="68" hidden="1">'tariff_versions'!$A$6:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="69" hidden="1">'payments'!$A$6:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="70" hidden="1">'wallets'!$A$6:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="71" hidden="1">'wallet_transactions'!$A$6:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="72" hidden="1">'invoices'!$A$6:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="73" hidden="1">'invoice_lines'!$A$6:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="74" hidden="1">'subscription_plans'!$A$6:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="75" hidden="1">'plan_features'!$A$6:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="76" hidden="1">'subscriptions'!$A$6:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="77" hidden="1">'driver_scores'!$A$6:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="78" hidden="1">'promotion_campaigns'!$A$6:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="79" hidden="1">'trips'!$A$6:$I$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -654,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I121"/>
+  <dimension ref="A1:I122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -685,7 +687,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>78 bảng trong 16 miền nghiệp vụ: 58 bảng chính, 17 bảng lịch sử (N.h), 3 bảng trạng thái. Bấm vào tên bảng hoặc «→ Mở» để mở sheet chi tiết của bảng; chú giải và các quyết định còn mở nằm ở cuối trang.</t>
+          <t>79 bảng trong 16 miền nghiệp vụ: 59 bảng chính, 17 bảng lịch sử (N.h), 3 bảng trạng thái. Bấm vào tên bảng hoặc «→ Mở» để mở sheet chi tiết của bảng; chú giải và các quyết định còn mở nằm ở cuối trang.</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3983,7 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>10 bảng</t>
+          <t>11 bảng</t>
         </is>
       </c>
       <c r="D84" s="5" t="n"/>
@@ -4089,7 +4091,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="27" customHeight="1">
+    <row r="87" ht="81" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
           <t>51</t>
@@ -4102,12 +4104,12 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>tariff_versions</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>Thanh toán</t>
+          <t>Phiên bản biểu giá</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr">
@@ -4117,12 +4119,12 @@
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>F-H1</t>
+          <t>F-C8, F-H1</t>
         </is>
       </c>
       <c r="G87" s="6" t="inlineStr">
         <is>
-          <t>Một lần thanh toán qua cổng thanh toán hoặc ví, thường cho một phiên sạc.</t>
+          <t>Một bộ giá không sửa được của biểu giá (BL-09); đổi giá là tạo phiên bản mới. Phiên bản hiện hành là phiên bản mới nhất có effective_from đã tới. Khi quét mã, ứng dụng hiện giá của khung giờ đó, và giá này được chốt cho cả phiên (PAY-09) trên bản ghi tính tiền của phiên, không ghi trên charging_sessions. Không có lịch sử thay đổi: phiên bản không bao giờ bị sửa. Ràng buộc kiểm tra (BL-09): giá không âm; thuế suất từ 0 đến 100.</t>
         </is>
       </c>
       <c r="H87" s="6" t="n">
@@ -4147,12 +4149,12 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>wallets</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>Ví</t>
+          <t>Thanh toán</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr">
@@ -4162,16 +4164,16 @@
       </c>
       <c r="F88" s="6" t="inlineStr">
         <is>
-          <t>F-H2</t>
+          <t>F-H1</t>
         </is>
       </c>
       <c r="G88" s="6" t="inlineStr">
         <is>
-          <t>Số dư trả trước của một tài xế hoặc của cả tổ chức.</t>
+          <t>Một lần thanh toán qua cổng thanh toán hoặc ví, thường cho một phiên sạc.</t>
         </is>
       </c>
       <c r="H88" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I88" s="7" t="inlineStr">
         <is>
@@ -4192,12 +4194,12 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>wallet_transactions</t>
+          <t>wallets</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>Giao dịch ví</t>
+          <t>Ví</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
@@ -4212,11 +4214,11 @@
       </c>
       <c r="G89" s="6" t="inlineStr">
         <is>
-          <t>Biến động tiền vào/ra khỏi ví, chỉ ghi thêm.</t>
+          <t>Số dư trả trước của một tài xế hoặc của cả tổ chức.</t>
         </is>
       </c>
       <c r="H89" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I89" s="7" t="inlineStr">
         <is>
@@ -4237,12 +4239,12 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>wallet_transactions</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>Hóa đơn</t>
+          <t>Giao dịch ví</t>
         </is>
       </c>
       <c r="E90" s="6" t="inlineStr">
@@ -4252,16 +4254,16 @@
       </c>
       <c r="F90" s="6" t="inlineStr">
         <is>
-          <t>F-H3, F-H4</t>
+          <t>F-H2</t>
         </is>
       </c>
       <c r="G90" s="6" t="inlineStr">
         <is>
-          <t>Một hóa đơn điện tử hợp lệ. Khi đã PHÁT HÀNH thì không sửa, chỉ điều chỉnh hoặc hủy bằng hóa đơn mới.</t>
+          <t>Biến động tiền vào/ra khỏi ví, chỉ ghi thêm.</t>
         </is>
       </c>
       <c r="H90" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I90" s="7" t="inlineStr">
         <is>
@@ -4282,303 +4284,303 @@
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>Hóa đơn</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>Khách hàng</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr">
+        <is>
+          <t>F-H3, F-H4</t>
+        </is>
+      </c>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t>Một hóa đơn điện tử hợp lệ. Khi đã PHÁT HÀNH thì không sửa, chỉ điều chỉnh hoặc hủy bằng hóa đơn mới.</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I91" s="7" t="inlineStr">
+        <is>
+          <t>→ Mở</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="27" customHeight="1">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>Thanh toán &amp; hóa đơn (billing)</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
           <t>invoice_lines</t>
         </is>
       </c>
-      <c r="D91" s="7" t="inlineStr">
+      <c r="D92" s="7" t="inlineStr">
         <is>
           <t>Dòng hóa đơn</t>
         </is>
       </c>
-      <c r="E91" s="6" t="inlineStr">
+      <c r="E92" s="6" t="inlineStr">
         <is>
           <t>Khách hàng</t>
         </is>
       </c>
-      <c r="F91" s="6" t="inlineStr">
+      <c r="F92" s="6" t="inlineStr">
         <is>
           <t>F-H3, F-H4</t>
         </is>
       </c>
-      <c r="G91" s="6" t="inlineStr">
+      <c r="G92" s="6" t="inlineStr">
         <is>
           <t>Một dòng của hóa đơn: một phiên sạc hoặc một kỳ thuê bao.</t>
         </is>
       </c>
-      <c r="H91" s="6" t="n">
+      <c r="H92" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="I91" s="7" t="inlineStr">
+      <c r="I92" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="54" customHeight="1">
-      <c r="A92" s="6" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-      <c r="B92" s="6" t="inlineStr">
+    <row r="93" ht="54" customHeight="1">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
         <is>
           <t>Thanh toán &amp; hóa đơn (billing)</t>
         </is>
       </c>
-      <c r="C92" s="7" t="inlineStr">
+      <c r="C93" s="7" t="inlineStr">
         <is>
           <t>subscription_plans</t>
         </is>
       </c>
-      <c r="D92" s="7" t="inlineStr">
+      <c r="D93" s="7" t="inlineStr">
         <is>
           <t>Gói dịch vụ</t>
         </is>
       </c>
-      <c r="E92" s="6" t="inlineStr">
+      <c r="E93" s="6" t="inlineStr">
         <is>
           <t>Nội bộ</t>
         </is>
       </c>
-      <c r="F92" s="6" t="inlineStr">
+      <c r="F93" s="6" t="inlineStr">
         <is>
           <t>F-H4</t>
         </is>
       </c>
-      <c r="G92" s="6" t="inlineStr">
+      <c r="G93" s="6" t="inlineStr">
         <is>
           <t>Một gói dịch vụ: mỗi gói là một dòng (GUEST là gói mặc định miễn phí, STANDARD, ADVANCED, PRO, ..., hoặc gói riêng cho một khách hàng); tính năng của gói nằm ở plan_features. Giá được tính theo từng tính năng (xem ghi chú của miền thanh toán).</t>
         </is>
       </c>
-      <c r="H92" s="6" t="n">
+      <c r="H93" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="I92" s="7" t="inlineStr">
+      <c r="I93" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="40.5" customHeight="1">
-      <c r="A93" s="6" t="inlineStr">
-        <is>
-          <t>57</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
+    <row r="94" ht="40.5" customHeight="1">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
         <is>
           <t>Thanh toán &amp; hóa đơn (billing)</t>
         </is>
       </c>
-      <c r="C93" s="7" t="inlineStr">
+      <c r="C94" s="7" t="inlineStr">
         <is>
           <t>plan_features</t>
         </is>
       </c>
-      <c r="D93" s="7" t="inlineStr">
+      <c r="D94" s="7" t="inlineStr">
         <is>
           <t>Tính năng của gói dịch vụ</t>
         </is>
       </c>
-      <c r="E93" s="6" t="inlineStr">
+      <c r="E94" s="6" t="inlineStr">
         <is>
           <t>Nội bộ</t>
         </is>
       </c>
-      <c r="F93" s="6" t="inlineStr">
+      <c r="F94" s="6" t="inlineStr">
         <is>
           <t>F-H4</t>
         </is>
       </c>
-      <c r="G93" s="6" t="inlineStr">
+      <c r="G94" s="6" t="inlineStr">
         <is>
           <t>Mỗi gói dịch vụ gồm những tính năng nào. Gói dịch vụ là dữ liệu, nên G3 có thể tạo gói mới (Pro, Max, gói riêng cho một khách hàng) trên portal mà không cần lập trình viên; chỉ tính năng hoàn toàn mới mới cần viết mã.</t>
         </is>
       </c>
-      <c r="H93" s="6" t="n">
+      <c r="H94" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="I93" s="7" t="inlineStr">
+      <c r="I94" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="27" customHeight="1">
-      <c r="A94" s="6" t="inlineStr">
-        <is>
-          <t>58</t>
-        </is>
-      </c>
-      <c r="B94" s="6" t="inlineStr">
+    <row r="95" ht="27" customHeight="1">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
         <is>
           <t>Thanh toán &amp; hóa đơn (billing)</t>
         </is>
       </c>
-      <c r="C94" s="7" t="inlineStr">
+      <c r="C95" s="7" t="inlineStr">
         <is>
           <t>subscriptions</t>
         </is>
       </c>
-      <c r="D94" s="7" t="inlineStr">
+      <c r="D95" s="7" t="inlineStr">
         <is>
           <t>Thuê bao</t>
         </is>
       </c>
-      <c r="E94" s="6" t="inlineStr">
+      <c r="E95" s="6" t="inlineStr">
         <is>
           <t>Khách hàng</t>
         </is>
       </c>
-      <c r="F94" s="6" t="inlineStr">
+      <c r="F95" s="6" t="inlineStr">
         <is>
           <t>F-H4</t>
         </is>
       </c>
-      <c r="G94" s="6" t="inlineStr">
+      <c r="G95" s="6" t="inlineStr">
         <is>
           <t>Một xe đăng ký một gói; quá hạn thanh toán sẽ khóa tính năng.</t>
         </is>
       </c>
-      <c r="H94" s="6" t="n">
+      <c r="H95" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="I94" s="7" t="inlineStr">
+      <c r="I95" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="27" customHeight="1">
-      <c r="A95" s="5" t="n"/>
-      <c r="B95" s="5" t="inlineStr">
+    <row r="96" ht="27" customHeight="1">
+      <c r="A96" s="5" t="n"/>
+      <c r="B96" s="5" t="inlineStr">
         <is>
           <t>Chấm điểm tài xế (scoring)</t>
         </is>
       </c>
-      <c r="C95" s="5" t="inlineStr">
+      <c r="C96" s="5" t="inlineStr">
         <is>
           <t>1 bảng</t>
         </is>
       </c>
-      <c r="D95" s="5" t="n"/>
-      <c r="E95" s="5" t="n"/>
-      <c r="F95" s="5" t="n"/>
-      <c r="G95" s="5" t="inlineStr">
+      <c r="D96" s="5" t="n"/>
+      <c r="E96" s="5" t="n"/>
+      <c r="F96" s="5" t="n"/>
+      <c r="G96" s="5" t="inlineStr">
         <is>
           <t>Chấm điểm an toàn cho tài xế từ hành vi lái xe.
 • Mỗi tuần, mỗi tài xế có một điểm, tính từ dữ liệu vận hành của xe họ lái.</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="6" t="inlineStr">
-        <is>
-          <t>59</t>
-        </is>
-      </c>
-      <c r="B96" s="6" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
         <is>
           <t>Chấm điểm tài xế (scoring)</t>
         </is>
       </c>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="C97" s="7" t="inlineStr">
         <is>
           <t>driver_scores</t>
         </is>
       </c>
-      <c r="D96" s="7" t="inlineStr">
+      <c r="D97" s="7" t="inlineStr">
         <is>
           <t>Điểm tài xế</t>
         </is>
       </c>
-      <c r="E96" s="6" t="inlineStr">
+      <c r="E97" s="6" t="inlineStr">
         <is>
           <t>Khách hàng</t>
         </is>
       </c>
-      <c r="F96" s="6" t="inlineStr">
+      <c r="F97" s="6" t="inlineStr">
         <is>
           <t>F-K1</t>
         </is>
       </c>
-      <c r="G96" s="6" t="inlineStr">
+      <c r="G97" s="6" t="inlineStr">
         <is>
           <t>Điểm an toàn hằng tuần của tài xế, tính từ dữ liệu vận hành xe.</t>
         </is>
       </c>
-      <c r="H96" s="6" t="n">
+      <c r="H97" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="I96" s="7" t="inlineStr">
+      <c r="I97" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="27" customHeight="1">
-      <c r="A97" s="5" t="n"/>
-      <c r="B97" s="5" t="inlineStr">
+    <row r="98" ht="27" customHeight="1">
+      <c r="A98" s="5" t="n"/>
+      <c r="B98" s="5" t="inlineStr">
         <is>
           <t>Chưa phân miền (unassigned)</t>
         </is>
       </c>
-      <c r="C97" s="5" t="inlineStr">
+      <c r="C98" s="5" t="inlineStr">
         <is>
           <t>2 bảng</t>
         </is>
       </c>
-      <c r="D97" s="5" t="n"/>
-      <c r="E97" s="5" t="n"/>
-      <c r="F97" s="5" t="n"/>
-      <c r="G97" s="5" t="inlineStr">
+      <c r="D98" s="5" t="n"/>
+      <c r="E98" s="5" t="n"/>
+      <c r="F98" s="5" t="n"/>
+      <c r="G98" s="5" t="inlineStr">
         <is>
           <t>Các tính năng chưa được quyết định thuộc miền nghiệp vụ nào (xem feature-list.md).</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="6" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>Chưa phân miền (unassigned)</t>
-        </is>
-      </c>
-      <c r="C98" s="7" t="inlineStr">
-        <is>
-          <t>promotion_campaigns</t>
-        </is>
-      </c>
-      <c r="D98" s="7" t="inlineStr">
-        <is>
-          <t>Chiến dịch khuyến mãi</t>
-        </is>
-      </c>
-      <c r="E98" s="6" t="inlineStr">
-        <is>
-          <t>Nội bộ</t>
-        </is>
-      </c>
-      <c r="F98" s="6" t="inlineStr">
-        <is>
-          <t>F-F4</t>
-        </is>
-      </c>
-      <c r="G98" s="6" t="inlineStr">
-        <is>
-          <t>Một chiến dịch nhắc bảo dưỡng hoặc khuyến mãi.</t>
-        </is>
-      </c>
-      <c r="H98" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="I98" s="7" t="inlineStr">
-        <is>
-          <t>→ Mở</t>
         </is>
       </c>
     </row>
@@ -4595,294 +4597,339 @@
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
+          <t>promotion_campaigns</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>Chiến dịch khuyến mãi</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>Nội bộ</t>
+        </is>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
+        <is>
+          <t>F-F4</t>
+        </is>
+      </c>
+      <c r="G99" s="6" t="inlineStr">
+        <is>
+          <t>Một chiến dịch nhắc bảo dưỡng hoặc khuyến mãi.</t>
+        </is>
+      </c>
+      <c r="H99" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I99" s="7" t="inlineStr">
+        <is>
+          <t>→ Mở</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>Chưa phân miền (unassigned)</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
           <t>trips</t>
         </is>
       </c>
-      <c r="D99" s="7" t="inlineStr">
+      <c r="D100" s="7" t="inlineStr">
         <is>
           <t>Chuyến đi</t>
         </is>
       </c>
-      <c r="E99" s="6" t="inlineStr">
+      <c r="E100" s="6" t="inlineStr">
         <is>
           <t>Khách hàng</t>
         </is>
       </c>
-      <c r="F99" s="6" t="inlineStr">
+      <c r="F100" s="6" t="inlineStr">
         <is>
           <t>F-A9</t>
         </is>
       </c>
-      <c r="G99" s="6" t="inlineStr">
+      <c r="G100" s="6" t="inlineStr">
         <is>
           <t>Một chuyến đi của xe. F-A9 đang tạm dừng: chưa có khái niệm chuyến đi.</t>
         </is>
       </c>
-      <c r="H99" s="6" t="n">
+      <c r="H100" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="I99" s="7" t="inlineStr">
+      <c r="I100" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="100"/>
-    <row r="101" ht="27" customHeight="1">
-      <c r="A101" s="4" t="inlineStr">
+    <row r="101"/>
+    <row r="102" ht="27" customHeight="1">
+      <c r="A102" s="4" t="inlineStr">
         <is>
           <t>Chú giải</t>
         </is>
       </c>
-      <c r="B101" s="4" t="inlineStr">
+      <c r="B102" s="4" t="inlineStr">
         <is>
           <t>Ý nghĩa</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="108" customHeight="1">
-      <c r="A102" s="6" t="inlineStr">
+    <row r="103" ht="108" customHeight="1">
+      <c r="A103" s="6" t="inlineStr">
         <is>
           <t>Chủ sở hữu dữ liệu: Khách hàng</t>
         </is>
       </c>
-      <c r="B102" s="6" t="inlineStr">
+      <c r="B103" s="6" t="inlineStr">
         <is>
           <t>Thuộc về một tổ chức (thường là khách hàng; công ty G3 cũng có thể sở hữu); có cột organization_id hoặc lấy qua bảng cha (DM-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="94.5" customHeight="1">
-      <c r="A103" s="6" t="inlineStr">
-        <is>
-          <t>Chủ sở hữu dữ liệu: Nội bộ</t>
-        </is>
-      </c>
-      <c r="B103" s="6" t="inlineStr">
-        <is>
-          <t>Dữ liệu của chính chúng ta (đơn vị vận hành nền tảng), dùng chung cho mọi tổ chức.</t>
         </is>
       </c>
     </row>
     <row r="104" ht="94.5" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
         <is>
+          <t>Chủ sở hữu dữ liệu: Nội bộ</t>
+        </is>
+      </c>
+      <c r="B104" s="6" t="inlineStr">
+        <is>
+          <t>Dữ liệu của chính chúng ta (đơn vị vận hành nền tảng), dùng chung cho mọi tổ chức.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="94.5" customHeight="1">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
           <t>Chủ sở hữu dữ liệu: Hai bên</t>
         </is>
       </c>
-      <c r="B104" s="6" t="inlineStr">
+      <c r="B105" s="6" t="inlineStr">
         <is>
           <t>Tài sản của G3 được khách hàng sử dụng; cả hai bên cùng liên quan.</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="121.5" customHeight="1">
-      <c r="A105" s="6" t="inlineStr">
+    <row r="106" ht="121.5" customHeight="1">
+      <c r="A106" s="6" t="inlineStr">
         <is>
           <t>Chủ sở hữu dữ liệu: Chưa quyết định</t>
         </is>
       </c>
-      <c r="B105" s="6" t="inlineStr">
+      <c r="B106" s="6" t="inlineStr">
         <is>
           <t>Đang chờ một quyết định còn mở (xem cuối trang).</t>
         </is>
       </c>
     </row>
-    <row r="106" ht="81" customHeight="1">
-      <c r="A106" s="6" t="inlineStr">
+    <row r="107" ht="81" customHeight="1">
+      <c r="A107" s="6" t="inlineStr">
         <is>
           <t>Miền nghiệp vụ (domain)</t>
         </is>
       </c>
-      <c r="B106" s="6" t="inlineStr">
+      <c r="B107" s="6" t="inlineStr">
         <is>
           <t>Một phần của hệ thống sở hữu dữ liệu riêng, ví dụ Xe, Trạm sạc, Thanh toán. Mỗi miền gồm một hoặc nhiều bảng.</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="54" customHeight="1">
-      <c r="A107" s="6" t="inlineStr">
+    <row r="108" ht="54" customHeight="1">
+      <c r="A108" s="6" t="inlineStr">
         <is>
           <t>Bảng</t>
         </is>
       </c>
-      <c r="B107" s="6" t="inlineStr">
+      <c r="B108" s="6" t="inlineStr">
         <is>
           <t>Một loại dữ liệu được lưu, ví dụ Xe hoặc Phiên sạc. Mỗi bảng có một sheet riêng liệt kê từng cột.</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="40.5" customHeight="1">
-      <c r="A108" s="6" t="inlineStr">
+    <row r="109" ht="40.5" customHeight="1">
+      <c r="A109" s="6" t="inlineStr">
         <is>
           <t>Tính năng</t>
         </is>
       </c>
-      <c r="B108" s="6" t="inlineStr">
+      <c r="B109" s="6" t="inlineStr">
         <is>
           <t>Mã tính năng trong danh sách tính năng (feature-list.md), ví dụ F-B2.</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="67.5" customHeight="1">
-      <c r="A109" s="6" t="inlineStr">
+    <row r="110" ht="67.5" customHeight="1">
+      <c r="A110" s="6" t="inlineStr">
         <is>
           <t>PK / FK / UQ</t>
         </is>
       </c>
-      <c r="B109" s="6" t="inlineStr">
+      <c r="B110" s="6" t="inlineStr">
         <is>
           <t>PK: khóa chính (định danh duy nhất của dòng). FK: khóa ngoại (trỏ tới dòng của bảng khác). UQ: giá trị không được trùng.</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="54" customHeight="1">
-      <c r="A110" s="6" t="inlineStr">
+    <row r="111" ht="54" customHeight="1">
+      <c r="A111" s="6" t="inlineStr">
         <is>
           <t>Ví dụ</t>
         </is>
       </c>
-      <c r="B110" s="6" t="inlineStr">
+      <c r="B111" s="6" t="inlineStr">
         <is>
           <t>Giá trị mẫu. Các mã ví dụ khớp nhau giữa các bảng, nên có thể lần theo một bản ghi mẫu qua nhiều sheet.</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="40.5" customHeight="1">
-      <c r="A111" s="6" t="inlineStr">
+    <row r="112" ht="40.5" customHeight="1">
+      <c r="A112" s="6" t="inlineStr">
         <is>
           <t>NULL</t>
         </is>
       </c>
-      <c r="B111" s="6" t="inlineStr">
+      <c r="B112" s="6" t="inlineStr">
         <is>
           <t>Ô không có giá trị. Ý nghĩa của NULL được giải thích trong cột Ý nghĩa.</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="81" customHeight="1">
-      <c r="A112" s="6" t="inlineStr">
+    <row r="113" ht="81" customHeight="1">
+      <c r="A113" s="6" t="inlineStr">
         <is>
           <t>🔍 Lưu lịch sử</t>
         </is>
       </c>
-      <c r="B112" s="6" t="inlineStr">
+      <c r="B113" s="6" t="inlineStr">
         <is>
           <t>Cột được theo dõi: khi cột này thay đổi, toàn bộ dòng cũ được chép sang bảng lịch sử (tên kết thúc bằng _history) kèm thời điểm và người thay đổi.</t>
         </is>
       </c>
     </row>
-    <row r="113"/>
-    <row r="114">
-      <c r="A114" s="8" t="inlineStr">
+    <row r="114"/>
+    <row r="115">
+      <c r="A115" s="8" t="inlineStr">
         <is>
           <t>Các view (giai đoạn đọc từ lịch sử)</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="4" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
         <is>
           <t>View</t>
         </is>
       </c>
-      <c r="B115" s="4" t="inlineStr">
+      <c r="B116" s="4" t="inlineStr">
         <is>
           <t>Mỗi dòng là</t>
         </is>
       </c>
-      <c r="C115" s="4" t="inlineStr">
+      <c r="C116" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D115" s="4" t="inlineStr">
+      <c r="D116" s="4" t="inlineStr">
         <is>
           <t>Được dùng bởi</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="94.5" customHeight="1">
-      <c r="A116" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_ownership_periods</t>
-        </is>
-      </c>
-      <c r="B116" s="6" t="inlineStr">
-        <is>
-          <t>một giai đoạn xe thuộc một chủ</t>
-        </is>
-      </c>
-      <c r="C116" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id, organization_id, owned_from, owned_until (NULL với chủ hiện tại)</t>
-        </is>
-      </c>
-      <c r="D116" s="6" t="inlineStr">
-        <is>
-          <t>lịch sử sở hữu và ngày bàn giao đầu tiên (VEH-02), "ngày đó xe của ai"</t>
         </is>
       </c>
     </row>
     <row r="117" ht="94.5" customHeight="1">
       <c r="A117" s="6" t="inlineStr">
         <is>
+          <t>vehicle_ownership_periods</t>
+        </is>
+      </c>
+      <c r="B117" s="6" t="inlineStr">
+        <is>
+          <t>một giai đoạn xe thuộc một chủ</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id, organization_id, owned_from, owned_until (NULL với chủ hiện tại)</t>
+        </is>
+      </c>
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>lịch sử sở hữu và ngày bàn giao đầu tiên (VEH-02), "ngày đó xe của ai"</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="94.5" customHeight="1">
+      <c r="A118" s="6" t="inlineStr">
+        <is>
           <t>battery_installation_periods</t>
         </is>
       </c>
-      <c r="B117" s="6" t="inlineStr">
+      <c r="B118" s="6" t="inlineStr">
         <is>
           <t>một lần pin nằm trên một xe</t>
         </is>
       </c>
-      <c r="C117" s="6" t="inlineStr">
+      <c r="C118" s="6" t="inlineStr">
         <is>
           <t>battery_id, vehicle_id, installed_from, installed_until (NULL khi đang lắp)</t>
         </is>
       </c>
-      <c r="D117" s="6" t="inlineStr">
+      <c r="D118" s="6" t="inlineStr">
         <is>
           <t>lịch sử sức khỏe pin qua các xe (MON-07), bộ đếm bảo hành pin (WAR-01)</t>
         </is>
       </c>
     </row>
-    <row r="118"/>
-    <row r="119">
-      <c r="A119" s="8" t="inlineStr">
+    <row r="119"/>
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
         <is>
           <t>Các quyết định còn mở</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="4" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
         <is>
           <t>Mã</t>
         </is>
       </c>
-      <c r="B120" s="4" t="inlineStr">
+      <c r="B121" s="4" t="inlineStr">
         <is>
           <t>Câu hỏi</t>
         </is>
       </c>
-      <c r="C120" s="4" t="inlineStr">
+      <c r="C121" s="4" t="inlineStr">
         <is>
           <t>Ảnh hưởng tới</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="54" customHeight="1">
-      <c r="A121" s="6" t="inlineStr">
+    <row r="122" ht="54" customHeight="1">
+      <c r="A122" s="6" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B121" s="6" t="inlineStr">
+      <c r="B122" s="6" t="inlineStr">
         <is>
           <t>Ai trả tiền khi tài xế của đội xe sạc: ví của tài xế, ví của đội xe, hay tùy trường hợp?</t>
         </is>
       </c>
-      <c r="C121" s="6" t="inlineStr">
+      <c r="C122" s="6" t="inlineStr">
         <is>
           <t>wallets, payments</t>
         </is>
@@ -5091,39 +5138,42 @@
     <hyperlink ref="C86" location="'tariff_history'!A1"/>
     <hyperlink ref="D86" location="'tariff_history'!A1"/>
     <hyperlink ref="I86" location="'tariff_history'!A1"/>
-    <hyperlink ref="C87" location="'payments'!A1"/>
-    <hyperlink ref="D87" location="'payments'!A1"/>
-    <hyperlink ref="I87" location="'payments'!A1"/>
-    <hyperlink ref="C88" location="'wallets'!A1"/>
-    <hyperlink ref="D88" location="'wallets'!A1"/>
-    <hyperlink ref="I88" location="'wallets'!A1"/>
-    <hyperlink ref="C89" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="D89" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="I89" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="C90" location="'invoices'!A1"/>
-    <hyperlink ref="D90" location="'invoices'!A1"/>
-    <hyperlink ref="I90" location="'invoices'!A1"/>
-    <hyperlink ref="C91" location="'invoice_lines'!A1"/>
-    <hyperlink ref="D91" location="'invoice_lines'!A1"/>
-    <hyperlink ref="I91" location="'invoice_lines'!A1"/>
-    <hyperlink ref="C92" location="'subscription_plans'!A1"/>
-    <hyperlink ref="D92" location="'subscription_plans'!A1"/>
-    <hyperlink ref="I92" location="'subscription_plans'!A1"/>
-    <hyperlink ref="C93" location="'plan_features'!A1"/>
-    <hyperlink ref="D93" location="'plan_features'!A1"/>
-    <hyperlink ref="I93" location="'plan_features'!A1"/>
-    <hyperlink ref="C94" location="'subscriptions'!A1"/>
-    <hyperlink ref="D94" location="'subscriptions'!A1"/>
-    <hyperlink ref="I94" location="'subscriptions'!A1"/>
-    <hyperlink ref="C96" location="'driver_scores'!A1"/>
-    <hyperlink ref="D96" location="'driver_scores'!A1"/>
-    <hyperlink ref="I96" location="'driver_scores'!A1"/>
-    <hyperlink ref="C98" location="'promotion_campaigns'!A1"/>
-    <hyperlink ref="D98" location="'promotion_campaigns'!A1"/>
-    <hyperlink ref="I98" location="'promotion_campaigns'!A1"/>
-    <hyperlink ref="C99" location="'trips'!A1"/>
-    <hyperlink ref="D99" location="'trips'!A1"/>
-    <hyperlink ref="I99" location="'trips'!A1"/>
+    <hyperlink ref="C87" location="'tariff_versions'!A1"/>
+    <hyperlink ref="D87" location="'tariff_versions'!A1"/>
+    <hyperlink ref="I87" location="'tariff_versions'!A1"/>
+    <hyperlink ref="C88" location="'payments'!A1"/>
+    <hyperlink ref="D88" location="'payments'!A1"/>
+    <hyperlink ref="I88" location="'payments'!A1"/>
+    <hyperlink ref="C89" location="'wallets'!A1"/>
+    <hyperlink ref="D89" location="'wallets'!A1"/>
+    <hyperlink ref="I89" location="'wallets'!A1"/>
+    <hyperlink ref="C90" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="D90" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="I90" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="C91" location="'invoices'!A1"/>
+    <hyperlink ref="D91" location="'invoices'!A1"/>
+    <hyperlink ref="I91" location="'invoices'!A1"/>
+    <hyperlink ref="C92" location="'invoice_lines'!A1"/>
+    <hyperlink ref="D92" location="'invoice_lines'!A1"/>
+    <hyperlink ref="I92" location="'invoice_lines'!A1"/>
+    <hyperlink ref="C93" location="'subscription_plans'!A1"/>
+    <hyperlink ref="D93" location="'subscription_plans'!A1"/>
+    <hyperlink ref="I93" location="'subscription_plans'!A1"/>
+    <hyperlink ref="C94" location="'plan_features'!A1"/>
+    <hyperlink ref="D94" location="'plan_features'!A1"/>
+    <hyperlink ref="I94" location="'plan_features'!A1"/>
+    <hyperlink ref="C95" location="'subscriptions'!A1"/>
+    <hyperlink ref="D95" location="'subscriptions'!A1"/>
+    <hyperlink ref="I95" location="'subscriptions'!A1"/>
+    <hyperlink ref="C97" location="'driver_scores'!A1"/>
+    <hyperlink ref="D97" location="'driver_scores'!A1"/>
+    <hyperlink ref="I97" location="'driver_scores'!A1"/>
+    <hyperlink ref="C99" location="'promotion_campaigns'!A1"/>
+    <hyperlink ref="D99" location="'promotion_campaigns'!A1"/>
+    <hyperlink ref="I99" location="'promotion_campaigns'!A1"/>
+    <hyperlink ref="C100" location="'trips'!A1"/>
+    <hyperlink ref="D100" location="'trips'!A1"/>
+    <hyperlink ref="I100" location="'trips'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26116,7 +26166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -26988,12 +27038,12 @@
       <c r="A48" s="6" t="n"/>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>organization_history</t>
+          <t>tariff_versions</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>changed_by</t>
+          <t>created_by</t>
         </is>
       </c>
     </row>
@@ -27001,12 +27051,12 @@
       <c r="A49" s="6" t="n"/>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>user_history</t>
+          <t>organization_history</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>changed_by</t>
         </is>
       </c>
     </row>
@@ -27019,7 +27069,7 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>changed_by</t>
+          <t>user_id</t>
         </is>
       </c>
     </row>
@@ -27027,7 +27077,7 @@
       <c r="A51" s="6" t="n"/>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>membership_history</t>
+          <t>user_history</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -27036,11 +27086,11 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="27" customHeight="1">
+    <row r="52">
       <c r="A52" s="6" t="n"/>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>organization_setting_history</t>
+          <t>membership_history</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -27049,11 +27099,11 @@
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="27" customHeight="1">
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>vehicle_history</t>
+          <t>organization_setting_history</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -27066,7 +27116,7 @@
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>vehicle_model_history</t>
+          <t>vehicle_history</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -27079,7 +27129,7 @@
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>battery_model_history</t>
+          <t>vehicle_model_history</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -27092,7 +27142,7 @@
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>battery_history</t>
+          <t>battery_model_history</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -27105,7 +27155,7 @@
       <c r="A57" s="6" t="n"/>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>warranty_history</t>
+          <t>battery_history</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -27118,7 +27168,7 @@
       <c r="A58" s="6" t="n"/>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>telematic_history</t>
+          <t>warranty_history</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -27131,7 +27181,7 @@
       <c r="A59" s="6" t="n"/>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>driver_history</t>
+          <t>telematic_history</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -27144,7 +27194,7 @@
       <c r="A60" s="6" t="n"/>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>fleet_history</t>
+          <t>driver_history</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -27153,11 +27203,11 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="27" customHeight="1">
+    <row r="61">
       <c r="A61" s="6" t="n"/>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>charging_location_history</t>
+          <t>fleet_history</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -27166,11 +27216,11 @@
         </is>
       </c>
     </row>
-    <row r="62">
+    <row r="62" ht="27" customHeight="1">
       <c r="A62" s="6" t="n"/>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>charging_station_history</t>
+          <t>charging_location_history</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -27183,7 +27233,7 @@
       <c r="A63" s="6" t="n"/>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>charging_evse_history</t>
+          <t>charging_station_history</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -27192,11 +27242,11 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="27" customHeight="1">
+    <row r="64">
       <c r="A64" s="6" t="n"/>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>charging_connector_history</t>
+          <t>charging_evse_history</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -27205,14 +27255,27 @@
         </is>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="27" customHeight="1">
       <c r="A65" s="6" t="n"/>
       <c r="B65" s="7" t="inlineStr">
         <is>
+          <t>charging_connector_history</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>changed_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="n"/>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
           <t>tariff_history</t>
         </is>
       </c>
-      <c r="C65" s="6" t="inlineStr">
+      <c r="C66" s="6" t="inlineStr">
         <is>
           <t>changed_by</t>
         </is>
@@ -27248,24 +27311,25 @@
     <hyperlink ref="B45" location="'charging_station_commands'!A1"/>
     <hyperlink ref="B46" location="'charging_sessions'!A1"/>
     <hyperlink ref="B47" location="'charging_policy_versions'!A1"/>
-    <hyperlink ref="B48" location="'organization_history'!A1"/>
-    <hyperlink ref="B49" location="'user_history'!A1"/>
+    <hyperlink ref="B48" location="'tariff_versions'!A1"/>
+    <hyperlink ref="B49" location="'organization_history'!A1"/>
     <hyperlink ref="B50" location="'user_history'!A1"/>
-    <hyperlink ref="B51" location="'membership_history'!A1"/>
-    <hyperlink ref="B52" location="'organization_setting_history'!A1"/>
-    <hyperlink ref="B53" location="'vehicle_history'!A1"/>
-    <hyperlink ref="B54" location="'vehicle_model_history'!A1"/>
-    <hyperlink ref="B55" location="'battery_model_history'!A1"/>
-    <hyperlink ref="B56" location="'battery_history'!A1"/>
-    <hyperlink ref="B57" location="'warranty_history'!A1"/>
-    <hyperlink ref="B58" location="'telematic_history'!A1"/>
-    <hyperlink ref="B59" location="'driver_history'!A1"/>
-    <hyperlink ref="B60" location="'fleet_history'!A1"/>
-    <hyperlink ref="B61" location="'charging_location_history'!A1"/>
-    <hyperlink ref="B62" location="'charging_station_history'!A1"/>
-    <hyperlink ref="B63" location="'charging_evse_history'!A1"/>
-    <hyperlink ref="B64" location="'charging_connector_history'!A1"/>
-    <hyperlink ref="B65" location="'tariff_history'!A1"/>
+    <hyperlink ref="B51" location="'user_history'!A1"/>
+    <hyperlink ref="B52" location="'membership_history'!A1"/>
+    <hyperlink ref="B53" location="'organization_setting_history'!A1"/>
+    <hyperlink ref="B54" location="'vehicle_history'!A1"/>
+    <hyperlink ref="B55" location="'vehicle_model_history'!A1"/>
+    <hyperlink ref="B56" location="'battery_model_history'!A1"/>
+    <hyperlink ref="B57" location="'battery_history'!A1"/>
+    <hyperlink ref="B58" location="'warranty_history'!A1"/>
+    <hyperlink ref="B59" location="'telematic_history'!A1"/>
+    <hyperlink ref="B60" location="'driver_history'!A1"/>
+    <hyperlink ref="B61" location="'fleet_history'!A1"/>
+    <hyperlink ref="B62" location="'charging_location_history'!A1"/>
+    <hyperlink ref="B63" location="'charging_station_history'!A1"/>
+    <hyperlink ref="B64" location="'charging_evse_history'!A1"/>
+    <hyperlink ref="B65" location="'charging_connector_history'!A1"/>
+    <hyperlink ref="B66" location="'tariff_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -44406,7 +44470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -44939,10 +45003,23 @@
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="7" t="inlineStr">
         <is>
+          <t>tariff_versions</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>tariff_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
           <t>tariff_history</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>tariff_id</t>
         </is>
@@ -44955,7 +45032,8 @@
     <hyperlink ref="A5" location="'tariff_history'!A1"/>
     <hyperlink ref="F9" location="'organizations'!A1"/>
     <hyperlink ref="F10" location="'charging_locations'!A1"/>
-    <hyperlink ref="B23" location="'tariff_history'!A1"/>
+    <hyperlink ref="B23" location="'tariff_versions'!A1"/>
+    <hyperlink ref="B24" location="'tariff_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -45576,7 +45654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -45593,7 +45671,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>51. payments: Thanh toán</t>
+          <t>51. tariff_versions: Phiên bản biểu giá</t>
         </is>
       </c>
     </row>
@@ -45607,14 +45685,14 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H1</t>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-C8, F-H1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một lần thanh toán qua cổng thanh toán hoặc ví, thường cho một phiên sạc.</t>
+          <t>Một bộ giá không sửa được của biểu giá (BL-09); đổi giá là tạo phiên bản mới. Phiên bản hiện hành là phiên bản mới nhất có effective_from đã tới. Khi quét mã, ứng dụng hiện giá của khung giờ đó, và giá này được chốt cho cả phiên (PAY-09) trên bản ghi tính tiền của phiên, không ghi trên charging_sessions. Không có lịch sử thay đổi: phiên bản không bao giờ bị sửa. Ràng buộc kiểm tra (BL-09): giá không âm; thuế suất từ 0 đến 100.</t>
         </is>
       </c>
     </row>
@@ -45672,7 +45750,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>payment_id</t>
+          <t>tariff_version_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -45693,23 +45771,23 @@
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Mã nội bộ của thanh toán.</t>
+          <t>Mã nội bộ của phiên bản biểu giá.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>3e1c8b5f-9a2d-4e7b-b4f1-6c0a9e3d2b21</t>
+          <t>1a7c3e9f-5b2d-4f8a-9c6e-0d3b8f1a7c55</t>
         </is>
       </c>
       <c r="I7" s="6" t="n"/>
     </row>
-    <row r="8" ht="27" customHeight="1">
+    <row r="8">
       <c r="A8" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
+          <t>tariff_id</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -45729,74 +45807,66 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+          <t>tariffs.tariff_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức khách hàng đã thanh toán.</t>
+          <t>Biểu giá chứa phiên bản này.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+          <t>f2b9e6c3-1d8a-4f5b-a3c7-9e0d4b1f8a10</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9" ht="27" customHeight="1">
+    <row r="9">
       <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>session_id</t>
+          <t>version_no</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>charging_sessions.session_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Phiên sạc được thanh toán; NULL với các khoản khác.</t>
+          <t>Số phiên bản trong biểu giá, bắt đầu từ 1.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>e5a2d8f1-4b7c-4e9a-b3d6-2c1f0e9a8dbb</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" s="6" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>4</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>effective_from</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>numeric(14,2)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -45808,28 +45878,28 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Số tiền đã thanh toán.</t>
+          <t>Thời điểm phiên bản này thay phiên bản trước: lúc ban hành hoặc muộn hơn, không bao giờ sớm hơn.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>866250.00</t>
+          <t>2026-10-15T00:00:00Z</t>
         </is>
       </c>
       <c r="I10" s="6" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>price_per_kwh</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>char(3)</t>
+          <t>numeric(12,2)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -45841,78 +45911,78 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Mã tiền tệ ISO 4217.</t>
+          <t>Đơn giá thường cho mỗi kWh, chưa gồm VAT, theo tiền tệ của biểu giá.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>VND</t>
+          <t>4500.00</t>
         </is>
       </c>
       <c r="I11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="54" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>method</t>
+          <t>time_periods</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>jsonb</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Phương thức thanh toán. Giá trị: VNPAY | MOMO | WALLET.</t>
+          <t>Giá theo khung giờ thay cho giá thường trong một số giờ, theo giờ Việt Nam: danh sách {days, from, to, price_per_kwh}; NULL nếu một giá cả ngày. Ghi một lần và đọc cả khối nên dùng JSON thay vì nhiều dòng.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>VNPAY</t>
+          <t>[{"days": ["MON", "TUE", "WED", "THU", "FRI", "SAT"], "from": "22:00", "to": "04:00", "price_per_kwh": 3200}]</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13" ht="27" customHeight="1">
+    <row r="13" ht="40.5" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>gateway_reference</t>
+          <t>vat_rate_percent</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>varchar(100)</t>
+          <t>numeric(4,2)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Mã tham chiếu/token của cổng thanh toán (không bao giờ lưu dữ liệu thẻ) (NF-05).</t>
+          <t>Thuế suất VAT áp dụng cho phiên bản này; giá lưu chưa gồm VAT và hiển thị đã gồm VAT; hóa đơn điện tử cần tách riêng (PAY-11).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>VNP14592873</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
@@ -45923,12 +45993,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>change_reason</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>varchar(200)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -45940,12 +46010,12 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Trạng thái thanh toán.</t>
+          <t>Lý do ban hành phiên bản này.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>SUCCEEDED</t>
+          <t>Theo khung giờ cao điểm mới của EVN</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
@@ -45956,29 +46026,37 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>paid_at</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>users.user_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm cổng thanh toán xác nhận; NULL cho tới lúc đó.</t>
+          <t>Người dùng đã ban hành.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>2026-09-15T09:46:12Z</t>
+          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
@@ -46006,12 +46084,12 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
+          <t>Thời điểm ban hành (UTC).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>2026-09-15T09:45:00Z</t>
+          <t>2026-10-10T03:00:00Z</t>
         </is>
       </c>
       <c r="I16" s="6" t="n"/>
@@ -46021,25 +46099,67 @@
       <c r="A18" s="4" t="n"/>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Được tham chiếu bởi bảng</t>
+          <t>Chỉ mục (index)</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="27" customHeight="1">
       <c r="A19" s="6" t="n"/>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>wallet_transactions</t>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>uq_tariff_versions_tariff_version_no</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>payment_id</t>
+          <t>tariff_id, version_no</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="27" customHeight="1">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>ix_tariff_versions_tariff_effective</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>tariff_id, effective_from</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>The current version: the newest whose effective_from has passed</t>
         </is>
       </c>
     </row>
@@ -46047,9 +46167,8 @@
   <autoFilter ref="A6:I16"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F8" location="'organizations'!A1"/>
-    <hyperlink ref="F9" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B19" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="F8" location="'tariffs'!A1"/>
+    <hyperlink ref="F15" location="'users'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -46734,7 +46853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -46751,7 +46870,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>52. wallets: Ví</t>
+          <t>52. payments: Thanh toán</t>
         </is>
       </c>
     </row>
@@ -46765,14 +46884,14 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H2</t>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Số dư trả trước của một tài xế hoặc của cả tổ chức.</t>
+          <t>Một lần thanh toán qua cổng thanh toán hoặc ví, thường cho một phiên sạc.</t>
         </is>
       </c>
     </row>
@@ -46830,7 +46949,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>wallet_id</t>
+          <t>payment_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -46851,12 +46970,12 @@
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Mã nội bộ của ví.</t>
+          <t>Mã nội bộ của thanh toán.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>5c3a0e7d-2f9b-4c1e-a8d3-7b6f0c2e9a32</t>
+          <t>3e1c8b5f-9a2d-4e7b-b4f1-6c0a9e3d2b21</t>
         </is>
       </c>
       <c r="I7" s="6" t="n"/>
@@ -46892,7 +47011,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức khách hàng sở hữu ví.</t>
+          <t>Tổ chức khách hàng đã thanh toán.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -46902,13 +47021,13 @@
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>driver_id</t>
+          <t>session_id</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -46928,17 +47047,17 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>drivers.driver_id (khi xóa: chặn xóa)</t>
+          <t>charging_sessions.session_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Tài xế sở hữu ví; NULL với ví cấp tổ chức (quyết định D5).</t>
+          <t>Phiên sạc được thanh toán; NULL với các khoản khác.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>e5a2d8f1-4b7c-4e9a-b3d6-2c1f0e9a8dbb</t>
         </is>
       </c>
       <c r="I9" s="6" t="n"/>
@@ -46949,7 +47068,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>balance</t>
+          <t>amount</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -46966,12 +47085,12 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Số dư hiện tại; phải bằng tổng các giao dịch của ví.</t>
+          <t>Số tiền đã thanh toán.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>12500000.00</t>
+          <t>866250.00</t>
         </is>
       </c>
       <c r="I10" s="6" t="n"/>
@@ -47015,7 +47134,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>method</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -47032,50 +47151,182 @@
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Ví có dùng được không.</t>
+          <t>Phương thức thanh toán. Giá trị: VNPAY | MOMO | WALLET.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>VNPAY</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13"/>
+    <row r="13" ht="27" customHeight="1">
+      <c r="A13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>gateway_reference</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>varchar(100)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Mã tham chiếu/token của cổng thanh toán (không bao giờ lưu dữ liệu thẻ) (NF-05).</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>VNP14592873</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n"/>
+    </row>
     <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="A14" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Trạng thái thanh toán.</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>SUCCEEDED</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>paid_at</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm cổng thanh toán xác nhận; NULL cho tới lúc đó.</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-15T09:46:12Z</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-15T09:45:00Z</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Được tham chiếu bởi bảng</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Cột</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>wallet_transactions</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>wallet_id</t>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>payment_id</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I12"/>
+  <autoFilter ref="A6:I16"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F8" location="'organizations'!A1"/>
-    <hyperlink ref="F9" location="'drivers'!A1"/>
-    <hyperlink ref="B15" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="F9" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B19" location="'wallet_transactions'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -47104,7 +47355,360 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>53. wallet_transactions: Giao dịch ví</t>
+          <t>53. wallets: Ví</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>← Tổng quan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Số dư trả trước của một tài xế hoặc của cả tổ chức.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6" ht="27" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Kiểu dữ liệu</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Cho phép rỗng</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Khóa</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Tham chiếu tới</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Ý nghĩa</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Ví dụ</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Lưu lịch sử</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>wallet_id</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Mã nội bộ của ví.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>5c3a0e7d-2f9b-4c1e-a8d3-7b6f0c2e9a32</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="27" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Tổ chức khách hàng sở hữu ví.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>driver_id</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>drivers.driver_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Tài xế sở hữu ví; NULL với ví cấp tổ chức (quyết định D5).</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>numeric(14,2)</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Số dư hiện tại; phải bằng tổng các giao dịch của ví.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>12500000.00</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>char(3)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Mã tiền tệ ISO 4217.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Ví có dùng được không.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n"/>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>wallet_transactions</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>wallet_id</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:I12"/>
+  <hyperlinks>
+    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
+    <hyperlink ref="F8" location="'organizations'!A1"/>
+    <hyperlink ref="F9" location="'drivers'!A1"/>
+    <hyperlink ref="B15" location="'wallet_transactions'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>54. wallet_transactions: Giao dịch ví</t>
         </is>
       </c>
     </row>
@@ -47523,7 +48127,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47546,7 +48150,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>54. invoices: Hóa đơn</t>
+          <t>55. invoices: Hóa đơn</t>
         </is>
       </c>
     </row>
@@ -47999,7 +48603,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -48022,7 +48626,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>55. invoice_lines: Dòng hóa đơn</t>
+          <t>56. invoice_lines: Dòng hóa đơn</t>
         </is>
       </c>
     </row>
@@ -48441,7 +49045,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -48464,7 +49068,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>56. subscription_plans: Gói dịch vụ</t>
+          <t>57. subscription_plans: Gói dịch vụ</t>
         </is>
       </c>
     </row>
@@ -48827,7 +49431,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -48850,7 +49454,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>57. plan_features: Tính năng của gói dịch vụ</t>
+          <t>58. plan_features: Tính năng của gói dịch vụ</t>
         </is>
       </c>
     </row>
@@ -49117,401 +49721,6 @@
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F8" location="'subscription_plans'!A1"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>58. subscriptions: Thuê bao</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>← Tổng quan</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H4</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>Một xe đăng ký một gói; quá hạn thanh toán sẽ khóa tính năng.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
-    <row r="6" ht="27" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Kiểu dữ liệu</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Cho phép rỗng</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Khóa</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Tham chiếu tới</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Ý nghĩa</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Ví dụ</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Lưu lịch sử</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>subscription_id</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Mã nội bộ của thuê bao.</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>9a7e4c1b-6d3f-4a5c-b0e8-2f1d7c9b3e54</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="27" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Tổ chức khách hàng đăng ký.</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="27" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>plan_id</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>subscription_plans.plan_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Gói được đăng ký.</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>0c9a6e3d-8f5b-4c7e-a2d1-4b3f9e6c0a65</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="27" customHeight="1">
-      <c r="A10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>vehicles.vehicle_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Xe được áp dụng.</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>started_at</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm bắt đầu thuê bao.</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-01T00:00:00Z</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>ends_at</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm kết thúc; NULL nếu tự gia hạn cho tới khi hủy.</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="n"/>
-    </row>
-    <row r="13" ht="27" customHeight="1">
-      <c r="A13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>varchar(20)</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Trạng thái thuê bao; OVERDUE sẽ khóa các tính năng trả phí. Giá trị: ACTIVE | OVERDUE | EXPIRED | CANCELLED.</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="n"/>
-    </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>invoice_lines</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>subscription_id</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A6:I13"/>
-  <hyperlinks>
-    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F8" location="'organizations'!A1"/>
-    <hyperlink ref="F9" location="'subscription_plans'!A1"/>
-    <hyperlink ref="F10" location="'vehicles'!A1"/>
-    <hyperlink ref="B16" location="'invoice_lines'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -49540,7 +49749,402 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>59. driver_scores: Điểm tài xế</t>
+          <t>59. subscriptions: Thuê bao</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>← Tổng quan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Một xe đăng ký một gói; quá hạn thanh toán sẽ khóa tính năng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6" ht="27" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Kiểu dữ liệu</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Cho phép rỗng</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Khóa</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Tham chiếu tới</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Ý nghĩa</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Ví dụ</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Lưu lịch sử</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>subscription_id</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Mã nội bộ của thuê bao.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>9a7e4c1b-6d3f-4a5c-b0e8-2f1d7c9b3e54</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="27" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Tổ chức khách hàng đăng ký.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="27" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>plan_id</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>subscription_plans.plan_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Gói được đăng ký.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>0c9a6e3d-8f5b-4c7e-a2d1-4b3f9e6c0a65</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="27" customHeight="1">
+      <c r="A10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>vehicles.vehicle_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Xe được áp dụng.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>started_at</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm bắt đầu thuê bao.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-01T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>ends_at</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm kết thúc; NULL nếu tự gia hạn cho tới khi hủy.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="27" customHeight="1">
+      <c r="A13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Trạng thái thuê bao; OVERDUE sẽ khóa các tính năng trả phí. Giá trị: ACTIVE | OVERDUE | EXPIRED | CANCELLED.</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n"/>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>invoice_lines</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>subscription_id</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:I13"/>
+  <hyperlinks>
+    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
+    <hyperlink ref="F8" location="'organizations'!A1"/>
+    <hyperlink ref="F9" location="'subscription_plans'!A1"/>
+    <hyperlink ref="F10" location="'vehicles'!A1"/>
+    <hyperlink ref="B16" location="'invoice_lines'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>60. driver_scores: Điểm tài xế</t>
         </is>
       </c>
     </row>
@@ -49920,7 +50524,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -49943,7 +50547,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>60. promotion_campaigns: Chiến dịch khuyến mãi</t>
+          <t>61. promotion_campaigns: Chiến dịch khuyến mãi</t>
         </is>
       </c>
     </row>
@@ -50222,406 +50826,6 @@
   <autoFilter ref="A6:I12"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>61. trips: Chuyến đi</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>← Tổng quan</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>Miền nghiệp vụ: Chưa phân miền (unassigned)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-A9</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>Một chuyến đi của xe. F-A9 đang tạm dừng: chưa có khái niệm chuyến đi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
-    <row r="6" ht="27" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Kiểu dữ liệu</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Cho phép rỗng</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Khóa</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Tham chiếu tới</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Ý nghĩa</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Ví dụ</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Lưu lịch sử</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>trip_id</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Mã nội bộ của chuyến đi.</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>2e1c8a5f-0b7d-4e9c-b4a3-6d5f1e8c2b76</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="27" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Tổ chức khách hàng sở hữu xe.</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="27" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>vehicles.vehicle_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Xe thực hiện chuyến.</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>driver_id</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>drivers.driver_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Tài xế của chuyến, nếu biết.</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>6e3b9d2a-4c1f-4e8b-9a7d-0c2e5f1b8d66</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>started_at</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm bắt đầu chuyến.</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-15T00:30:00Z</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>ended_at</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm kết thúc; NULL khi đang chạy.</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-15T06:10:00Z</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="n"/>
-    </row>
-    <row r="13" ht="27" customHeight="1">
-      <c r="A13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>declared_load_status</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>varchar(20)</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Trạng thái tải do tài xế khai báo. Giá trị: LOADED | EMPTY.</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>LOADED</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="n"/>
-    </row>
-    <row r="14" ht="27" customHeight="1">
-      <c r="A14" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>inferred_load_status</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>varchar(20)</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Trạng thái tải suy ra từ dữ liệu vận hành. Giá trị: LOADED | EMPTY.</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>LOADED</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="n"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A6:I14"/>
-  <hyperlinks>
-    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F8" location="'organizations'!A1"/>
-    <hyperlink ref="F9" location="'vehicles'!A1"/>
-    <hyperlink ref="F10" location="'drivers'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -51269,6 +51473,406 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>62. trips: Chuyến đi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>← Tổng quan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Miền nghiệp vụ: Chưa phân miền (unassigned)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Một chuyến đi của xe. F-A9 đang tạm dừng: chưa có khái niệm chuyến đi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6" ht="27" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Kiểu dữ liệu</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Cho phép rỗng</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Khóa</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Tham chiếu tới</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Ý nghĩa</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Ví dụ</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Lưu lịch sử</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>trip_id</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Mã nội bộ của chuyến đi.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>2e1c8a5f-0b7d-4e9c-b4a3-6d5f1e8c2b76</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="27" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Tổ chức khách hàng sở hữu xe.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="27" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>vehicles.vehicle_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Xe thực hiện chuyến.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>driver_id</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>drivers.driver_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Tài xế của chuyến, nếu biết.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>6e3b9d2a-4c1f-4e8b-9a7d-0c2e5f1b8d66</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>started_at</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm bắt đầu chuyến.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-15T00:30:00Z</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>ended_at</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm kết thúc; NULL khi đang chạy.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-15T06:10:00Z</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="27" customHeight="1">
+      <c r="A13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>declared_load_status</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Trạng thái tải do tài xế khai báo. Giá trị: LOADED | EMPTY.</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>LOADED</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n"/>
+    </row>
+    <row r="14" ht="27" customHeight="1">
+      <c r="A14" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>inferred_load_status</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Trạng thái tải suy ra từ dữ liệu vận hành. Giá trị: LOADED | EMPTY.</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>LOADED</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:I14"/>
+  <hyperlinks>
+    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
+    <hyperlink ref="F8" location="'organizations'!A1"/>
+    <hyperlink ref="F9" location="'vehicles'!A1"/>
+    <hyperlink ref="F10" location="'drivers'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
docs(domain-model): rename the session billing record to charging_session_bills
One bill per charging session; 'charge' read as a charging session and
'fee' as a price (BL-11).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -76,8 +76,8 @@
     <sheet name="tariffs" sheetId="67" state="visible" r:id="rId67"/>
     <sheet name="tariff_history" sheetId="68" state="visible" r:id="rId68"/>
     <sheet name="tariff_versions" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="charging_session_charges" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="charging_session_charge_history" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="charging_session_bills" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="charging_session_bill_history" sheetId="71" state="visible" r:id="rId71"/>
     <sheet name="payments" sheetId="72" state="visible" r:id="rId72"/>
     <sheet name="wallets" sheetId="73" state="visible" r:id="rId73"/>
     <sheet name="wallet_transactions" sheetId="74" state="visible" r:id="rId74"/>
@@ -159,8 +159,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="66" hidden="1">'tariffs'!$A$7:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="67" hidden="1">'tariff_history'!$A$7:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="68" hidden="1">'tariff_versions'!$A$6:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="69" hidden="1">'charging_session_charges'!$A$7:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="70" hidden="1">'charging_session_charge_history'!$A$7:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="69" hidden="1">'charging_session_bills'!$A$7:$I$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="70" hidden="1">'charging_session_bill_history'!$A$7:$I$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="71" hidden="1">'payments'!$A$6:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="72" hidden="1">'wallets'!$A$6:$I$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="73" hidden="1">'wallet_transactions'!$A$6:$I$15</definedName>
@@ -4153,12 +4153,12 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>charging_session_charges</t>
+          <t>charging_session_bills</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>Phí phiên sạc</t>
+          <t>Phiếu tính tiền phiên sạc</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr">
@@ -4173,7 +4173,7 @@
       </c>
       <c r="G88" s="6" t="inlineStr">
         <is>
-          <t>Chi phí của một lần sạc (BL-10, CE-12, PAY-10): đơn giá chốt khi quét mã, số kWh tính tiền và số tiền. Thuộc miền thanh toán, trỏ tới phiên sạc, không bao giờ ngược lại. Số tiền là số đã thu sau làm tròn nên được lưu cố định, giống nhau trên biên nhận, thanh toán và hóa đơn điện tử. Bật lịch sử thay đổi: cho tính tiền một khoản bị giữ là quyết định của con người. Không sửa sau khi BILLED; sai sót được điều chỉnh bằng hoàn tiền hoặc hóa đơn điều chỉnh. Ràng buộc kiểm tra (BL-10): khoản BILLED phải đủ điện năng, nguồn, số tiền và thời điểm; khoản QUOTED hoặc VOID không có các giá trị đó.</t>
+          <t>Phiếu tính tiền của một phiên sạc (BL-10, BL-11, CE-12, PAY-10): đơn giá chốt khi quét mã, số kWh tính tiền và số tiền. Thuộc miền thanh toán, trỏ tới phiên sạc, không bao giờ ngược lại. Số tiền là số đã thu sau làm tròn nên được lưu cố định, giống nhau trên biên nhận, thanh toán và hóa đơn điện tử. Bật lịch sử thay đổi: cho tính tiền một phiếu bị giữ là quyết định của con người. Không sửa sau khi BILLED; sai sót được điều chỉnh bằng hoàn tiền hoặc hóa đơn điều chỉnh. Ràng buộc kiểm tra (BL-10): khoản BILLED phải đủ điện năng, nguồn, số tiền và thời điểm; khoản QUOTED hoặc VOID không có các giá trị đó.</t>
         </is>
       </c>
       <c r="H88" s="6" t="n">
@@ -4198,12 +4198,12 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>charging_session_charge_history</t>
+          <t>charging_session_bill_history</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>Lịch sử phí phiên sạc</t>
+          <t>Lịch sử phiếu tính tiền phiên sạc</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="G89" s="6" t="inlineStr">
         <is>
-          <t>Mọi phiên bản trước đây của một dòng trong bảng charging_session_charges: bản sao toàn bộ dòng, chụp ngay trước khi thay đổi và được trigger ghi trong cùng giao dịch. Do công cụ domain-model tự sinh từ @tracked *, không bao giờ viết tay.</t>
+          <t>Mọi phiên bản trước đây của một dòng trong bảng charging_session_bills: bản sao toàn bộ dòng, chụp ngay trước khi thay đổi và được trigger ghi trong cùng giao dịch. Do công cụ domain-model tự sinh từ @tracked *, không bao giờ viết tay.</t>
         </is>
       </c>
       <c r="H89" s="6" t="n">
@@ -5235,12 +5235,12 @@
     <hyperlink ref="C87" location="'tariff_versions'!A1"/>
     <hyperlink ref="D87" location="'tariff_versions'!A1"/>
     <hyperlink ref="I87" location="'tariff_versions'!A1"/>
-    <hyperlink ref="C88" location="'charging_session_charges'!A1"/>
-    <hyperlink ref="D88" location="'charging_session_charges'!A1"/>
-    <hyperlink ref="I88" location="'charging_session_charges'!A1"/>
-    <hyperlink ref="C89" location="'charging_session_charge_history'!A1"/>
-    <hyperlink ref="D89" location="'charging_session_charge_history'!A1"/>
-    <hyperlink ref="I89" location="'charging_session_charge_history'!A1"/>
+    <hyperlink ref="C88" location="'charging_session_bills'!A1"/>
+    <hyperlink ref="D88" location="'charging_session_bills'!A1"/>
+    <hyperlink ref="I88" location="'charging_session_bills'!A1"/>
+    <hyperlink ref="C89" location="'charging_session_bill_history'!A1"/>
+    <hyperlink ref="D89" location="'charging_session_bill_history'!A1"/>
+    <hyperlink ref="I89" location="'charging_session_bill_history'!A1"/>
     <hyperlink ref="C90" location="'payments'!A1"/>
     <hyperlink ref="D90" location="'payments'!A1"/>
     <hyperlink ref="I90" location="'payments'!A1"/>
@@ -27385,7 +27385,7 @@
       <c r="A67" s="6" t="n"/>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>charging_session_charge_history</t>
+          <t>charging_session_bill_history</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -27443,7 +27443,7 @@
     <hyperlink ref="B64" location="'charging_evse_history'!A1"/>
     <hyperlink ref="B65" location="'charging_connector_history'!A1"/>
     <hyperlink ref="B66" location="'tariff_history'!A1"/>
-    <hyperlink ref="B67" location="'charging_session_charge_history'!A1"/>
+    <hyperlink ref="B67" location="'charging_session_bill_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -39295,7 +39295,7 @@
       <c r="A48" s="6" t="n"/>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>charging_session_charges</t>
+          <t>charging_session_bills</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -39357,7 +39357,7 @@
     <hyperlink ref="B45" location="'charging_session_events'!A1"/>
     <hyperlink ref="B46" location="'charging_session_measurements'!A1"/>
     <hyperlink ref="B47" location="'policy_violations'!A1"/>
-    <hyperlink ref="B48" location="'charging_session_charges'!A1"/>
+    <hyperlink ref="B48" location="'charging_session_bills'!A1"/>
     <hyperlink ref="B49" location="'payments'!A1"/>
     <hyperlink ref="B50" location="'wallet_transactions'!A1"/>
     <hyperlink ref="B51" location="'invoice_lines'!A1"/>
@@ -46309,7 +46309,7 @@
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>charging_session_charges</t>
+          <t>charging_session_bills</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -46324,7 +46324,7 @@
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F8" location="'tariffs'!A1"/>
     <hyperlink ref="F15" location="'users'!A1"/>
-    <hyperlink ref="B23" location="'charging_session_charges'!A1"/>
+    <hyperlink ref="B23" location="'charging_session_bills'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -47026,7 +47026,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>52. charging_session_charges: Phí phiên sạc</t>
+          <t>52. charging_session_bills: Phiếu tính tiền phiên sạc</t>
         </is>
       </c>
     </row>
@@ -47047,14 +47047,14 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Chi phí của một lần sạc (BL-10, CE-12, PAY-10): đơn giá chốt khi quét mã, số kWh tính tiền và số tiền. Thuộc miền thanh toán, trỏ tới phiên sạc, không bao giờ ngược lại. Số tiền là số đã thu sau làm tròn nên được lưu cố định, giống nhau trên biên nhận, thanh toán và hóa đơn điện tử. Bật lịch sử thay đổi: cho tính tiền một khoản bị giữ là quyết định của con người. Không sửa sau khi BILLED; sai sót được điều chỉnh bằng hoàn tiền hoặc hóa đơn điều chỉnh. Ràng buộc kiểm tra (BL-10): khoản BILLED phải đủ điện năng, nguồn, số tiền và thời điểm; khoản QUOTED hoặc VOID không có các giá trị đó.</t>
+          <t>Phiếu tính tiền của một phiên sạc (BL-10, BL-11, CE-12, PAY-10): đơn giá chốt khi quét mã, số kWh tính tiền và số tiền. Thuộc miền thanh toán, trỏ tới phiên sạc, không bao giờ ngược lại. Số tiền là số đã thu sau làm tròn nên được lưu cố định, giống nhau trên biên nhận, thanh toán và hóa đơn điện tử. Bật lịch sử thay đổi: cho tính tiền một phiếu bị giữ là quyết định của con người. Không sửa sau khi BILLED; sai sót được điều chỉnh bằng hoàn tiền hoặc hóa đơn điều chỉnh. Ràng buộc kiểm tra (BL-10): khoản BILLED phải đủ điện năng, nguồn, số tiền và thời điểm; khoản QUOTED hoặc VOID không có các giá trị đó.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>🔍 Lưu lịch sử: khi một cột có dấu 🔍 thay đổi, toàn bộ dòng cũ được chép sang bảng charging_session_charge_history.</t>
+          <t>🔍 Lưu lịch sử: khi một cột có dấu 🔍 thay đổi, toàn bộ dòng cũ được chép sang bảng charging_session_bill_history.</t>
         </is>
       </c>
     </row>
@@ -47106,13 +47106,13 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="27" customHeight="1">
+    <row r="8">
       <c r="A8" s="6" t="n">
         <v>1</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>charging_session_charge_id</t>
+          <t>charging_session_bill_id</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -47133,7 +47133,7 @@
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Mã nội bộ của khoản phí sạc.</t>
+          <t>Mã nội bộ của phiếu tính tiền.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -47174,7 +47174,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Phiên sạc; mỗi phiên một khoản phí. Bên trả tiền đọc từ phiên (charging_sessions.organization_id, DM-24).</t>
+          <t>Phiên sạc; mỗi phiên một phiếu tính tiền. Bên trả tiền đọc từ phiên (charging_sessions.organization_id, DM-24).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -47669,7 +47669,7 @@
       <c r="A24" s="6" t="n"/>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>ix_charging_session_charges_tariff_version_id</t>
+          <t>ix_charging_session_bills_tariff_version_id</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -47689,7 +47689,7 @@
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>ix_charging_session_charges_status_created</t>
+          <t>ix_charging_session_bills_status_created</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -47727,12 +47727,12 @@
       <c r="A28" s="6" t="n"/>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>charging_session_charge_history</t>
+          <t>charging_session_bill_history</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>charging_session_charge_id</t>
+          <t>charging_session_bill_id</t>
         </is>
       </c>
     </row>
@@ -47740,10 +47740,10 @@
   <autoFilter ref="A7:I21"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="A5" location="'charging_session_charge_history'!A1"/>
+    <hyperlink ref="A5" location="'charging_session_bill_history'!A1"/>
     <hyperlink ref="F9" location="'charging_sessions'!A1"/>
     <hyperlink ref="F10" location="'tariff_versions'!A1"/>
-    <hyperlink ref="B28" location="'charging_session_charge_history'!A1"/>
+    <hyperlink ref="B28" location="'charging_session_bill_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -47772,7 +47772,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>52.h. charging_session_charge_history: Lịch sử phí phiên sạc</t>
+          <t>52.h. charging_session_bill_history: Lịch sử phiếu tính tiền phiên sạc</t>
         </is>
       </c>
     </row>
@@ -47793,14 +47793,14 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Mọi phiên bản trước đây của một dòng trong bảng charging_session_charges: bản sao toàn bộ dòng, chụp ngay trước khi thay đổi và được trigger ghi trong cùng giao dịch. Do công cụ domain-model tự sinh từ @tracked *, không bao giờ viết tay.</t>
+          <t>Mọi phiên bản trước đây của một dòng trong bảng charging_session_bills: bản sao toàn bộ dòng, chụp ngay trước khi thay đổi và được trigger ghi trong cùng giao dịch. Do công cụ domain-model tự sinh từ @tracked *, không bao giờ viết tay.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Bảng lịch sử của: charging_session_charges</t>
+          <t>Bảng lịch sử của: charging_session_bills</t>
         </is>
       </c>
     </row>
@@ -47895,7 +47895,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>charging_session_charge_id</t>
+          <t>charging_session_bill_id</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -47915,12 +47915,12 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>charging_session_charges.charging_session_charge_id (khi xóa: chặn xóa)</t>
+          <t>charging_session_bills.charging_session_bill_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.charging_session_charge_id).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.charging_session_bill_id).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -47953,7 +47953,7 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.session_id).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.session_id).</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -47986,7 +47986,7 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.tariff_version_id).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.tariff_version_id).</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -48019,7 +48019,7 @@
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.price_per_kwh).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.price_per_kwh).</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -48052,7 +48052,7 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.vat_rate_percent).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.vat_rate_percent).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -48085,7 +48085,7 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.status).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.status).</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -48118,7 +48118,7 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.status_reason).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.status_reason).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -48151,7 +48151,7 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.energy_wh).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.energy_wh).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -48184,7 +48184,7 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.energy_source).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.energy_source).</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -48217,7 +48217,7 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.amount_before_vat).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.amount_before_vat).</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -48250,7 +48250,7 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.vat_amount).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.vat_amount).</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -48283,7 +48283,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.billed_at).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.billed_at).</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -48316,7 +48316,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.created_at).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.created_at).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -48349,7 +48349,7 @@
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (charging_session_charges.updated_at).</t>
+          <t>Giá trị trước khi thay đổi (charging_session_bills.updated_at).</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -48495,12 +48495,12 @@
       <c r="A28" s="6" t="n"/>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>ix_charging_session_charge_history_charging_session_charge_id_time</t>
+          <t>ix_charging_session_bill_history_charging_session_bill_id_time</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>charging_session_charge_id, changed_at</t>
+          <t>charging_session_bill_id, changed_at</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -48515,8 +48515,8 @@
   <autoFilter ref="A7:I25"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="A5" location="'charging_session_charges'!A1"/>
-    <hyperlink ref="F9" location="'charging_session_charges'!A1"/>
+    <hyperlink ref="A5" location="'charging_session_bills'!A1"/>
+    <hyperlink ref="F9" location="'charging_session_bills'!A1"/>
     <hyperlink ref="F24" location="'users'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(domain-model): trim wallets and payments to a driver's balance
Wallets and payments belong to a person only, payments are top-ups and
refunds, and launch top-ups use a VietQR bank transfer matched by a unique
transfer code; MoMo, ZaloPay and cards come later as new methods (BL-15).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -162,9 +162,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="68" hidden="1">'tariff_versions'!$A$6:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="69" hidden="1">'charging_session_bills'!$A$7:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="70" hidden="1">'charging_session_bill_history'!$A$7:$I$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="71" hidden="1">'payments'!$A$6:$I$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="72" hidden="1">'wallets'!$A$7:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="73" hidden="1">'wallet_history'!$A$7:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="71" hidden="1">'payments'!$A$6:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="72" hidden="1">'wallets'!$A$7:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="73" hidden="1">'wallet_history'!$A$7:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="74" hidden="1">'wallet_transactions'!$A$6:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="75" hidden="1">'invoices'!$A$6:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="76" hidden="1">'invoice_lines'!$A$6:$I$15</definedName>
@@ -3999,7 +3999,7 @@
         <is>
           <t>Tiền: giá điện, thanh toán, ví trả trước, hóa đơn điện tử và thuê bao SaaS.
 • Biểu giá định giá điện cho toàn mạng hoặc từng trạm, theo khung giờ.
-• Một ví là số dư trả trước của một người (khi ra mắt) hoặc một tổ chức (sau này); giao dịch ví là sổ chỉ ghi thêm. Một thanh toán là tiền thật qua cổng: nạp tiền hoặc hoàn tiền khi ra mắt (BL-12 đến BL-14).
+• Một ví là số dư trả trước để sạc của một người; giao dịch ví là sổ chỉ ghi thêm. Một thanh toán là tiền thật vào hoặc ra: nạp bằng chuyển khoản VietQR, hoặc hoàn tiền (BL-12 đến BL-15).
 • Một hóa đơn thuộc một tổ chức và có các dòng hóa đơn cho phiên sạc hoặc kỳ thuê bao.
 • Một thuê bao đưa một xe vào một gói dịch vụ.
 • Muốn tính tiền một phiên sạc phải biết phiên đó của ai.
@@ -4232,7 +4232,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="81" customHeight="1">
+    <row r="90" ht="94.5" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
           <t>53</t>
@@ -4255,21 +4255,21 @@
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>Khách hàng</t>
+          <t>Nội bộ</t>
         </is>
       </c>
       <c r="F90" s="6" t="inlineStr">
         <is>
-          <t>F-H1</t>
+          <t>F-H1, F-H2</t>
         </is>
       </c>
       <c r="G90" s="6" t="inlineStr">
         <is>
-          <t>Tiền đi qua cổng thanh toán hoặc ngân hàng (BL-12): chỉ tiền thật vào hoặc ra. Trả tiền phiên sạc bằng ví là giao dịch ví, không phải thanh toán. Khi ra mắt chỉ có TOP_UP và REFUND; SESSION_BILL và INVOICE đến cùng các phương thức sau. Không có lịch sử thay đổi (trạng thái do cổng báo); không xóa mềm (chứng từ tài chính). Thẻ đã lưu (mã hóa token) là bảng sau này. Ràng buộc kiểm tra (BL-12): liên kết có giá trị khớp với mục đích.</t>
+          <t>Tiền thật vào hoặc ra khỏi ví của một người (BL-12, BL-15): chỉ nạp tiền và hoàn tiền. Khi ra mắt, tài xế nạp bằng chuyển khoản qua mã VietQR mang nội dung chuyển khoản duy nhất; dịch vụ nhận thông báo ngân hàng ghép giao dịch đến và ví được cộng đúng số tiền thực nhận. MoMo, ZaloPay và thẻ đến sau như giá trị mới. Trả tiền phiên sạc bằng ví là giao dịch ví, không phải thanh toán. Không có lịch sử thay đổi; không xóa mềm. Ràng buộc kiểm tra (BL-15): chỉ REFUND mới có refund_of_payment_id.</t>
         </is>
       </c>
       <c r="H90" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I90" s="7" t="inlineStr">
         <is>
@@ -4277,7 +4277,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="135" customHeight="1">
+    <row r="91" ht="121.5" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
           <t>54</t>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>Khách hàng</t>
+          <t>Nội bộ</t>
         </is>
       </c>
       <c r="F91" s="6" t="inlineStr">
@@ -4310,11 +4310,11 @@
       </c>
       <c r="G91" s="6" t="inlineStr">
         <is>
-          <t>Số dư trả trước chỉ dùng cho dịch vụ của chính chúng ta (BL-13). Khi ra mắt, mỗi người tự nạp tiền vào ví của mình và trả từng phiên sạc từ đó; ví của tổ chức được chuẩn bị cho các phương thức sau. Để bắt đầu sạc, số dư phải bằng hoặc cao hơn mức tối thiểu đặt trong backend (BL-14); kiểm tra khi quét mã, không bằng ràng buộc cơ sở dữ liệu, vì lần trừ tiền cuối phiên có thể làm số dư âm, sau đó người dùng không thể sạc tiếp cho tới khi nạp lại trên mức tối thiểu. Bật lịch sử thay đổi cho các quyết định (khóa ví), trừ cột balance vì mọi giao dịch đều làm thay đổi nó. Không xóa mềm. Không gọi là ví điện tử khi giới thiệu ra bên ngoài (câu hỏi mở 11). Ràng buộc kiểm tra (BL-13): chỉ đúng một chủ sở hữu.</t>
+          <t>Số dư trả trước để sạc của một người, chỉ dùng cho dịch vụ của chính chúng ta (BL-13, BL-15): người đó nạp tiền và trả từng phiên sạc từ ví. Ví của tổ chức chỉ được thêm cùng các phương thức thanh toán doanh nghiệp. Để bắt đầu sạc, số dư phải bằng hoặc cao hơn mức tối thiểu đặt trong backend (BL-14); kiểm tra khi quét mã, không bằng ràng buộc cơ sở dữ liệu, vì lần trừ tiền cuối phiên có thể làm số dư âm, sau đó người dùng không thể sạc tiếp cho tới khi nạp lại trên mức tối thiểu. Bật lịch sử thay đổi cho các quyết định (khóa ví), trừ cột balance vì mọi giao dịch đều làm thay đổi nó. Không xóa mềm. Không gọi là ví điện tử khi giới thiệu ra bên ngoài (câu hỏi mở 11).</t>
         </is>
       </c>
       <c r="H91" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I91" s="7" t="inlineStr">
         <is>
@@ -4345,7 +4345,7 @@
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>Khách hàng</t>
+          <t>Nội bộ</t>
         </is>
       </c>
       <c r="F92" s="6" t="inlineStr">
@@ -4359,7 +4359,7 @@
         </is>
       </c>
       <c r="H92" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I92" s="7" t="inlineStr">
         <is>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t>Khách hàng</t>
+          <t>Nội bộ</t>
         </is>
       </c>
       <c r="F93" s="6" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11834,7 +11834,7 @@
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>driver_scores</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -11847,7 +11847,7 @@
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>wallets</t>
+          <t>trips</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -11860,36 +11860,10 @@
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>driver_scores</t>
+          <t>organization_history</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="6" t="n"/>
-      <c r="B57" s="7" t="inlineStr">
-        <is>
-          <t>trips</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="6" t="n"/>
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>organization_history</t>
-        </is>
-      </c>
-      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>organization_id</t>
         </is>
@@ -11929,11 +11903,9 @@
     <hyperlink ref="B51" location="'invoices'!A1"/>
     <hyperlink ref="B52" location="'invoice_lines'!A1"/>
     <hyperlink ref="B53" location="'subscriptions'!A1"/>
-    <hyperlink ref="B54" location="'payments'!A1"/>
-    <hyperlink ref="B55" location="'wallets'!A1"/>
-    <hyperlink ref="B56" location="'driver_scores'!A1"/>
-    <hyperlink ref="B57" location="'trips'!A1"/>
-    <hyperlink ref="B58" location="'organization_history'!A1"/>
+    <hyperlink ref="B54" location="'driver_scores'!A1"/>
+    <hyperlink ref="B55" location="'trips'!A1"/>
+    <hyperlink ref="B56" location="'organization_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27161,7 +27133,7 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>paid_by</t>
+          <t>user_id</t>
         </is>
       </c>
     </row>
@@ -47042,7 +47014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -47760,7 +47732,7 @@
       <c r="A28" s="6" t="n"/>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>wallet_transactions</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -47773,23 +47745,10 @@
       <c r="A29" s="6" t="n"/>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>wallet_transactions</t>
+          <t>charging_session_bill_history</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>charging_session_bill_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="27" customHeight="1">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>charging_session_bill_history</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>charging_session_bill_id</t>
         </is>
@@ -47802,9 +47761,8 @@
     <hyperlink ref="A5" location="'charging_session_bill_history'!A1"/>
     <hyperlink ref="F9" location="'charging_sessions'!A1"/>
     <hyperlink ref="F10" location="'tariff_versions'!A1"/>
-    <hyperlink ref="B28" location="'payments'!A1"/>
-    <hyperlink ref="B29" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="B30" location="'charging_session_bill_history'!A1"/>
+    <hyperlink ref="B28" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="B29" location="'charging_session_bill_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -48590,7 +48548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -48621,14 +48579,14 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H1</t>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Nội bộ   ·   Tính năng: F-H1, F-H2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Tiền đi qua cổng thanh toán hoặc ngân hàng (BL-12): chỉ tiền thật vào hoặc ra. Trả tiền phiên sạc bằng ví là giao dịch ví, không phải thanh toán. Khi ra mắt chỉ có TOP_UP và REFUND; SESSION_BILL và INVOICE đến cùng các phương thức sau. Không có lịch sử thay đổi (trạng thái do cổng báo); không xóa mềm (chứng từ tài chính). Thẻ đã lưu (mã hóa token) là bảng sau này. Ràng buộc kiểm tra (BL-12): liên kết có giá trị khớp với mục đích.</t>
+          <t>Tiền thật vào hoặc ra khỏi ví của một người (BL-12, BL-15): chỉ nạp tiền và hoàn tiền. Khi ra mắt, tài xế nạp bằng chuyển khoản qua mã VietQR mang nội dung chuyển khoản duy nhất; dịch vụ nhận thông báo ngân hàng ghép giao dịch đến và ví được cộng đúng số tiền thực nhận. MoMo, ZaloPay và thẻ đến sau như giá trị mới. Trả tiền phiên sạc bằng ví là giao dịch ví, không phải thanh toán. Không có lịch sử thay đổi; không xóa mềm. Ràng buộc kiểm tra (BL-15): chỉ REFUND mới có refund_of_payment_id.</t>
         </is>
       </c>
     </row>
@@ -48723,7 +48681,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -48743,280 +48701,256 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+          <t>users.user_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức thanh toán hoặc nhận hoàn tiền, ghi một lần (DM-24 trường hợp C).</t>
+          <t>Người nạp tiền vào ví của mình, hoặc nhận hoàn tiền (BL-15).</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9" ht="27" customHeight="1">
+    <row r="9" ht="40.5" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>paid_by</t>
+          <t>purpose</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>users.user_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Người dùng đã thanh toán trên ứng dụng; NULL với chuyển khoản ngân hàng.</t>
+          <t>TOP_UP: nạp tiền vào ví của người đó. REFUND: hoàn lại số dư chưa dùng (BL-15). Trả trực tiếp phiếu tính tiền hay hóa đơn đến cùng các phương thức sau.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
+          <t>TOP_UP</t>
         </is>
       </c>
       <c r="I9" s="6" t="n"/>
     </row>
-    <row r="10" ht="67.5" customHeight="1">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>4</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>purpose</t>
+          <t>refund_of_payment_id</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>payments.payment_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Tiền dùng cho việc gì (BL-12). TOP_UP: nạp tiền vào ví (khi ra mắt). REFUND: hoàn tiền, ví dụ số dư ví chưa dùng (khi ra mắt). SESSION_BILL: trả trực tiếp một phiếu tính tiền phiên sạc (sau này). INVOICE: trả một hóa đơn (sau này, thanh toán doanh nghiệp).</t>
+          <t>Lần nạp mà khoản hoàn tiền trả lại qua; chỉ có giá trị với REFUND (hoàn tiền qua đúng kênh đã nạp, câu hỏi mở 11).</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>TOP_UP</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I10" s="6" t="n"/>
     </row>
-    <row r="11" ht="27" customHeight="1">
+    <row r="11" ht="40.5" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>charging_session_bill_id</t>
+          <t>amount</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>numeric(14,2)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>charging_session_bills.charging_session_bill_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Phiếu tính tiền được trả; chỉ có giá trị với SESSION_BILL.</t>
+          <t>Số tiền, luôn dương; mục đích cho biết chiều tiền. Với chuyển khoản là số tiền thực nhận, có thể khác số tài xế định nạp.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>500000.00</t>
         </is>
       </c>
       <c r="I11" s="6" t="n"/>
     </row>
-    <row r="12" ht="27" customHeight="1">
+    <row r="12">
       <c r="A12" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>invoice_id</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>char(3)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>invoices.invoice_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Hóa đơn được trả; chỉ có giá trị với INVOICE.</t>
+          <t>Mã tiền tệ ISO 4217.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>VND</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13" ht="27" customHeight="1">
+    <row r="13" ht="54" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>refund_of_payment_id</t>
+          <t>method</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>payments.payment_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Thanh toán mà lần hoàn tiền này trả lại; chỉ có giá trị với REFUND.</t>
+          <t>Cách chuyển tiền. Khi ra mắt: BANK_TRANSFER qua mã VietQR (BL-15). Sau này: MOMO, ZALOPAY, CARD là giá trị mới, không đổi bảng. Trả bằng ví không phải thanh toán mà là giao dịch ví.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>BANK_TRANSFER</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="40.5" customHeight="1">
       <c r="A14" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>transfer_code</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>numeric(14,2)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Số tiền, luôn dương; mục đích cho biết chiều tiền.</t>
+          <t>Nội dung chuyển khoản duy nhất mà giao dịch của tài xế phải có, nằm trong mã VietQR; dùng để ghép giao dịch đến với dòng này. Có giá trị với lần nạp BANK_TRANSFER.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>500000.00</t>
+          <t>G3NAP7K2Q9</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>gateway_reference</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>char(3)</t>
+          <t>varchar(100)</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Mã tiền tệ ISO 4217.</t>
+          <t>Mã giao dịch của ngân hàng hoặc cổng thanh toán, dùng để đối soát; không bao giờ là dữ liệu thẻ (NF-05).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>VND</t>
+          <t>FT26283912345</t>
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
@@ -49027,78 +48961,78 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>method</t>
+          <t>gateway_result_code</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>varchar(30)</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Cách chuyển tiền. Trả bằng ví không phải là thanh toán (không có tiền vào) mà là giao dịch ví.</t>
+          <t>Mã kết quả của ngân hàng hoặc cổng, đúng như gửi về; NULL nếu không có.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>VNPAY</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I16" s="6" t="n"/>
     </row>
-    <row r="17" ht="27" customHeight="1">
+    <row r="17" ht="40.5" customHeight="1">
       <c r="A17" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>gateway_reference</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>varchar(100)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Mã giao dịch của cổng thanh toán, dùng để đối soát; không bao giờ là dữ liệu thẻ (NF-05).</t>
+          <t>PENDING: đã hiện mã QR, chưa nhận tiền. SUCCEEDED: đã nhận tiền (hoặc đã chuyển hoàn). FAILED: thất bại hoặc hết hạn chưa trả. Là trạng thái quan sát nên không có cột lý do.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>VNP14592873</t>
+          <t>SUCCEEDED</t>
         </is>
       </c>
       <c r="I17" s="6" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" ht="27" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>12</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>gateway_result_code</t>
+          <t>completed_at</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>varchar(30)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -49110,28 +49044,28 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Mã kết quả của cổng thanh toán, đúng như gửi về (PAY-06).</t>
+          <t>Thời điểm xác nhận đã nhận hoặc đã chuyển tiền, hoặc yêu cầu thất bại; NULL khi PENDING.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>00</t>
+          <t>2026-09-15T09:46:12Z</t>
         </is>
       </c>
       <c r="I18" s="6" t="n"/>
     </row>
-    <row r="19" ht="27" customHeight="1">
+    <row r="19">
       <c r="A19" s="6" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -49143,23 +49077,23 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Theo cổng thanh toán báo về; là trạng thái quan sát nên không có cột lý do.</t>
+          <t>Thời điểm tạo bản ghi (UTC): lúc hiện mã QR.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>SUCCEEDED</t>
+          <t>2026-09-15T09:45:00Z</t>
         </is>
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20" ht="27" customHeight="1">
+    <row r="20">
       <c r="A20" s="6" t="n">
         <v>14</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>completed_at</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -49169,14 +49103,14 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm cổng xác nhận thành công hay thất bại; NULL khi PENDING.</t>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -49186,152 +49120,123 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-15T09:45:00Z</t>
-        </is>
-      </c>
-      <c r="I21" s="6" t="n"/>
-    </row>
+    <row r="21"/>
     <row r="22">
-      <c r="A22" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-15T09:46:12Z</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="n"/>
-    </row>
-    <row r="23"/>
-    <row r="24">
-      <c r="A24" s="4" t="n"/>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="40.5" customHeight="1">
+    <row r="23" ht="27" customHeight="1">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>uq_payments_transfer_code</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>transfer_code</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>WHERE transfer_code IS NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40.5" customHeight="1">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>uq_payments_method_gateway_reference</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>method, gateway_reference</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>WHERE gateway_reference IS NOT NULL: the same bank notification is never recorded twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>uq_payments_method_gateway_reference</t>
+          <t>ix_payments_user_created</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>method, gateway_reference</t>
+          <t>user_id, created_at</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>WHERE gateway_reference IS NOT NULL: the same gateway callback is never recorded twice</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="27" customHeight="1">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>ix_payments_organization_created</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>organization_id, created_at</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="n"/>
-    </row>
-    <row r="27"/>
+      <c r="F25" s="6" t="n"/>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="4" t="n"/>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
     <row r="28">
-      <c r="A28" s="4" t="n"/>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>payments</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>refund_of_payment_id</t>
         </is>
       </c>
     </row>
@@ -49339,39 +49244,23 @@
       <c r="A29" s="6" t="n"/>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>wallet_transactions</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>refund_of_payment_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>wallet_transactions</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
           <t>payment_id</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I22"/>
+  <autoFilter ref="A6:I20"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F8" location="'organizations'!A1"/>
-    <hyperlink ref="F9" location="'users'!A1"/>
-    <hyperlink ref="F11" location="'charging_session_bills'!A1"/>
-    <hyperlink ref="F12" location="'invoices'!A1"/>
-    <hyperlink ref="F13" location="'payments'!A1"/>
-    <hyperlink ref="B29" location="'payments'!A1"/>
-    <hyperlink ref="B30" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="F8" location="'users'!A1"/>
+    <hyperlink ref="F10" location="'payments'!A1"/>
+    <hyperlink ref="B28" location="'payments'!A1"/>
+    <hyperlink ref="B29" location="'wallet_transactions'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -49383,7 +49272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -49414,14 +49303,14 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H2</t>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Nội bộ   ·   Tính năng: F-H2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Số dư trả trước chỉ dùng cho dịch vụ của chính chúng ta (BL-13). Khi ra mắt, mỗi người tự nạp tiền vào ví của mình và trả từng phiên sạc từ đó; ví của tổ chức được chuẩn bị cho các phương thức sau. Để bắt đầu sạc, số dư phải bằng hoặc cao hơn mức tối thiểu đặt trong backend (BL-14); kiểm tra khi quét mã, không bằng ràng buộc cơ sở dữ liệu, vì lần trừ tiền cuối phiên có thể làm số dư âm, sau đó người dùng không thể sạc tiếp cho tới khi nạp lại trên mức tối thiểu. Bật lịch sử thay đổi cho các quyết định (khóa ví), trừ cột balance vì mọi giao dịch đều làm thay đổi nó. Không xóa mềm. Không gọi là ví điện tử khi giới thiệu ra bên ngoài (câu hỏi mở 11). Ràng buộc kiểm tra (BL-13): chỉ đúng một chủ sở hữu.</t>
+          <t>Số dư trả trước để sạc của một người, chỉ dùng cho dịch vụ của chính chúng ta (BL-13, BL-15): người đó nạp tiền và trả từng phiên sạc từ ví. Ví của tổ chức chỉ được thêm cùng các phương thức thanh toán doanh nghiệp. Để bắt đầu sạc, số dư phải bằng hoặc cao hơn mức tối thiểu đặt trong backend (BL-14); kiểm tra khi quét mã, không bằng ràng buộc cơ sở dữ liệu, vì lần trừ tiền cuối phiên có thể làm số dư âm, sau đó người dùng không thể sạc tiếp cho tới khi nạp lại trên mức tối thiểu. Bật lịch sử thay đổi cho các quyết định (khóa ví), trừ cột balance vì mọi giao dịch đều làm thay đổi nó. Không xóa mềm. Không gọi là ví điện tử khi giới thiệu ra bên ngoài (câu hỏi mở 11).</t>
         </is>
       </c>
     </row>
@@ -49533,7 +49422,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -49548,7 +49437,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Người sở hữu ví (phương thức khi ra mắt, BL-13): ví đi theo người đó sang mọi tổ chức họ lái xe cho. Chỉ đúng một trong user_id và organization_id có giá trị.</t>
+          <t>Người sở hữu ví (BL-13, BL-15): ví đi theo người đó sang mọi tổ chức họ lái xe cho. Ví của tổ chức chỉ được thêm cùng các phương thức thanh toán doanh nghiệp.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -49562,63 +49451,51 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="40.5" customHeight="1">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>numeric(14,2)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức sở hữu ví (phương thức sau này: tổ chức trả trước và tài xế dùng, hoặc tổ chức phân bổ cho tài xế); NULL với ví cá nhân.</t>
+          <t>Số dư hiện tại, luôn bằng tổng các giao dịch. Có thể âm khi một phiên sạc tốn nhiều hơn số dư (BL-14).</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="27" customHeight="1">
+          <t>1250000.00</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
       <c r="A11" s="6" t="n">
         <v>4</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>balance</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>numeric(14,2)</t>
+          <t>char(3)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -49630,28 +49507,32 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Số dư hiện tại, luôn bằng tổng các giao dịch. Có thể âm khi một phiên sạc tốn nhiều hơn số dư (BL-14).</t>
+          <t>Mã tiền tệ ISO 4217.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>1250000.00</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="n"/>
-    </row>
-    <row r="12">
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40.5" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>char(3)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -49663,12 +49544,12 @@
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Mã tiền tệ ISO 4217.</t>
+          <t>Do chúng ta quyết định. ACTIVE: dùng được. BLOCKED: không nạp tiền và không bắt đầu sạc, ví dụ khi đang kiểm tra gian lận.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>VND</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -49677,35 +49558,35 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="40.5" customHeight="1">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>status_reason</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>varchar(200)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Do chúng ta quyết định. ACTIVE: dùng được. BLOCKED: không nạp tiền và không bắt đầu sạc, ví dụ khi đang kiểm tra gian lận.</t>
+          <t>Lý do ví có trạng thái hiện tại, ví dụ vì sao bị khóa (DM-19); NULL nếu không cần giải thích.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -49714,35 +49595,35 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="27" customHeight="1">
+    <row r="14">
       <c r="A14" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>status_reason</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>varchar(200)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Lý do ví có trạng thái hiện tại, ví dụ vì sao bị khóa (DM-19); NULL nếu không cần giải thích.</t>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>2026-09-01T02:00:00Z</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -49757,7 +49638,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -49774,12 +49655,12 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
+          <t>2026-09-15T09:46:12Z</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -49788,165 +49669,103 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-15T09:46:12Z</t>
-        </is>
-      </c>
-      <c r="I16" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="27" customHeight="1">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>uq_wallets_user_id</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>user_id</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>có</t>
         </is>
       </c>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>WHERE user_id IS NOT NULL: one wallet per person</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>uq_wallets_organization_id</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>WHERE organization_id IS NOT NULL: one wallet per organization</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>One wallet per person</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>wallet_transactions</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>wallet_id</t>
+        </is>
+      </c>
+    </row>
     <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>wallet_transactions</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>wallet_history</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>wallet_id</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>wallet_history</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>wallet_id</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A7:I16"/>
+  <autoFilter ref="A7:I15"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'wallet_history'!A1"/>
     <hyperlink ref="F9" location="'users'!A1"/>
-    <hyperlink ref="F10" location="'organizations'!A1"/>
-    <hyperlink ref="B23" location="'wallet_transactions'!A1"/>
-    <hyperlink ref="B24" location="'wallet_history'!A1"/>
+    <hyperlink ref="B21" location="'wallet_transactions'!A1"/>
+    <hyperlink ref="B22" location="'wallet_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -49958,7 +49777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -49989,7 +49808,7 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H2</t>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Nội bộ   ·   Tính năng: F-H2</t>
         </is>
       </c>
     </row>
@@ -50172,12 +49991,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>numeric(14,2)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -50189,12 +50008,12 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (wallets.organization_id).</t>
+          <t>Giá trị trước khi thay đổi (wallets.balance).</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>1250000.00</t>
         </is>
       </c>
       <c r="I11" s="6" t="n"/>
@@ -50205,12 +50024,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>balance</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>numeric(14,2)</t>
+          <t>char(3)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -50222,12 +50041,12 @@
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (wallets.balance).</t>
+          <t>Giá trị trước khi thay đổi (wallets.currency).</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>1250000.00</t>
+          <t>VND</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
@@ -50238,12 +50057,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>char(3)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -50255,12 +50074,12 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (wallets.currency).</t>
+          <t>Giá trị trước khi thay đổi (wallets.status).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>VND</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
@@ -50271,12 +50090,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>status_reason</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>varchar(200)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -50288,12 +50107,12 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (wallets.status).</t>
+          <t>Giá trị trước khi thay đổi (wallets.status_reason).</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
@@ -50304,12 +50123,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>status_reason</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>varchar(200)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -50321,12 +50140,12 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (wallets.status_reason).</t>
+          <t>Giá trị trước khi thay đổi (wallets.created_at).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>2026-09-01T02:00:00Z</t>
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
@@ -50337,7 +50156,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -50354,12 +50173,12 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (wallets.created_at).</t>
+          <t>Giá trị trước khi thay đổi (wallets.updated_at).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
+          <t>2026-09-15T09:46:12Z</t>
         </is>
       </c>
       <c r="I16" s="6" t="n"/>
@@ -50370,7 +50189,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>changed_at</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -50380,182 +50199,149 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Giá trị trước khi thay đổi (wallets.updated_at).</t>
+          <t>Thời điểm phiên bản này của dòng bị thay thế.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-15T09:46:12Z</t>
+          <t>2026-09-10T07:15:00Z</t>
         </is>
       </c>
       <c r="I17" s="6" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" ht="27" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>changed_at</t>
+          <t>changed_by</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>users.user_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm phiên bản này của dòng bị thay thế.</t>
+          <t>Người dùng đã thực hiện thay đổi; NULL nếu do hệ thống thực hiện.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10T07:15:00Z</t>
+          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
         </is>
       </c>
       <c r="I18" s="6" t="n"/>
     </row>
-    <row r="19" ht="27" customHeight="1">
+    <row r="19" ht="40.5" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>12</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>changed_by</t>
+          <t>change_reason</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>varchar(200)</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>users.user_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Người dùng đã thực hiện thay đổi; NULL nếu do hệ thống thực hiện.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>9b2e7d4a-1c3f-4a8e-b6d2-5e0f1a9c3d22</t>
+          <t>Customer moved to a new office</t>
         </is>
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20" ht="40.5" customHeight="1">
-      <c r="A20" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>change_reason</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>varchar(200)</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="27" customHeight="1">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>ix_wallet_history_wallet_id_time</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>wallet_id, changed_at</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>không</t>
         </is>
       </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>Customer moved to a new office</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="n"/>
-    </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>ix_wallet_history_wallet_id_time</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>wallet_id, changed_at</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A7:I20"/>
+  <autoFilter ref="A7:I19"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'wallets'!A1"/>
     <hyperlink ref="F9" location="'wallets'!A1"/>
-    <hyperlink ref="F19" location="'users'!A1"/>
+    <hyperlink ref="F18" location="'users'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -50598,7 +50384,7 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-H2</t>
+          <t>Miền nghiệp vụ: Thanh toán &amp; hóa đơn (billing)   ·   Chủ sở hữu dữ liệu: Nội bộ   ·   Tính năng: F-H2</t>
         </is>
       </c>
     </row>
@@ -51135,7 +50921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -51594,26 +51380,12 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>payments</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>invoice_id</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A6:I16"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F8" location="'organizations'!A1"/>
     <hyperlink ref="B19" location="'invoice_lines'!A1"/>
-    <hyperlink ref="B20" location="'payments'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(domain-model): review the notifications table
Organization required, the truck link kept for filtering with RESTRICT, a
generic subject link that opens the right screen, read state moved to a
per-person recipients table, and four new planned alert kinds from this
review (NT-09).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -152,7 +152,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="57" hidden="1">'charging_sessions'!$A$6:$I$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="58" hidden="1">'charging_session_events'!$A$6:$I$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="59" hidden="1">'charging_session_measurements'!$A$6:$I$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="60" hidden="1">'notifications'!$A$6:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="60" hidden="1">'notifications'!$A$6:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="61" hidden="1">'support_cases'!$A$6:$I$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="62" hidden="1">'repair_partners'!$A$6:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="63" hidden="1">'maintenance_bookings'!$A$6:$I$13</definedName>
@@ -3665,7 +3665,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="40.5" customHeight="1">
+    <row r="76" ht="81" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
           <t>43</t>
@@ -3698,11 +3698,11 @@
       </c>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>Một cảnh báo (pin, bất thường, SOH, thiết bị mất kết nối...). Một bảng chung; mỗi loại cảnh báo là một giá trị enum và một cấu trúc payload. Được rà soát sau cùng, sau mọi miền phát sinh cảnh báo (NT-08, ghi các điểm cần quyết định).</t>
+          <t>Một cảnh báo (pin, bất thường, SOH, thiết bị mất kết nối...). Một bảng chung; mỗi loại cảnh báo là một giá trị enum và một cấu trúc payload. Được rà soát sau cùng (NT-08) và chốt ở NT-09: bắt buộc có tổ chức, liên kết chung tới đối tượng để mở đúng màn hình, trạng thái đã đọc theo từng người ở bảng người nhận. Chỉ ghi thêm; không lịch sử thay đổi, không xóa mềm. Ràng buộc kiểm tra (NT-09): subject_type và subject_id cùng có hoặc cùng không.</t>
         </is>
       </c>
       <c r="H76" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I76" s="7" t="inlineStr">
         <is>
@@ -42861,7 +42861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -42899,7 +42899,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một cảnh báo (pin, bất thường, SOH, thiết bị mất kết nối...). Một bảng chung; mỗi loại cảnh báo là một giá trị enum và một cấu trúc payload. Được rà soát sau cùng, sau mọi miền phát sinh cảnh báo (NT-08, ghi các điểm cần quyết định).</t>
+          <t>Một cảnh báo (pin, bất thường, SOH, thiết bị mất kết nối...). Một bảng chung; mỗi loại cảnh báo là một giá trị enum và một cấu trúc payload. Được rà soát sau cùng (NT-08) và chốt ở NT-09: bắt buộc có tổ chức, liên kết chung tới đối tượng để mở đúng màn hình, trạng thái đã đọc theo từng người ở bảng người nhận. Chỉ ghi thêm; không lịch sử thay đổi, không xóa mềm. Ràng buộc kiểm tra (NT-09): subject_type và subject_id cùng có hoặc cùng không.</t>
         </is>
       </c>
     </row>
@@ -43004,7 +43004,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -43019,7 +43019,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức khách hàng được xem thông báo.</t>
+          <t>Tổ chức sở hữu cảnh báo, ghi một lần: chủ xe tại thời điểm đó (DM-24 trường hợp C).</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -43136,35 +43136,35 @@
       </c>
       <c r="I11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="94.5" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>subject_type</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>varchar(200)</t>
+          <t>varchar(30)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Tóm tắt ngắn.</t>
+          <t>Cảnh báo nói về đối tượng nào, và do đó ứng dụng mở màn hình nào (NTF-02): VEHICLE, TELEMATIC, CHARGING_SESSION, SUPPORT_CASE, TRIP, GEOFENCE, WALLET... Loại mới chỉ thêm giá trị, không thêm cột. Không có khóa ngoại (trỏ tới nhiều bảng khác nhau); đối tượng luôn tồn tại vì không bao giờ xóa hẳn (DM-25). Khi mở vẫn áp dụng kiểm tra quyền của màn hình đó.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Pin còn 20%</t>
+          <t>TRIP</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
@@ -43175,45 +43175,45 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>body</t>
+          <t>subject_id</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>varchar(500)</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Mô tả chi tiết.</t>
+          <t>Mã của đối tượng đó; có giá trị đúng khi subject_type có giá trị.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Xe 51D-123.45 còn 20% pin. Trạm gần nhất: Trạm sạc G3 Bình Dương (8.4 km).</t>
+          <t>2e1c8a5f-0b7d-4e9c-b4a3-6d5f1e8c2b76</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
     </row>
-    <row r="14" ht="40.5" customHeight="1">
+    <row r="14">
       <c r="A14" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>payload</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>jsonb</t>
+          <t>varchar(200)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -43225,28 +43225,28 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Chi tiết riêng theo loại thông báo, dạng JSON.</t>
+          <t>Tóm tắt ngắn.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>{"threshold": 20, "soc": 19.8, "nearest_station_id": "4b9d6f3a-2e8c-4a1b-9d5e-7f0c3a8b2d88", "distance_m": 8400}</t>
+          <t>Pin còn 20%</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>body</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>varchar(500)</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -43258,136 +43258,226 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm phát sinh thông báo.</t>
+          <t>Mô tả chi tiết.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>2026-09-15T08:30:00Z</t>
+          <t>Xe 51D-123.45 còn 20% pin. Trạm gần nhất: Trạm sạc G3 Bình Dương (8.4 km).</t>
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
     </row>
-    <row r="16" ht="27" customHeight="1">
+    <row r="16" ht="40.5" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>read_at</t>
+          <t>payload</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>jsonb</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm người vận hành đánh dấu đã đọc; NULL nếu chưa đọc.</t>
+          <t>Chi tiết riêng theo loại thông báo, dạng JSON.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
+          <t>{"threshold": 20, "soc": 19.8, "nearest_station_id": "4b9d6f3a-2e8c-4a1b-9d5e-7f0c3a8b2d88", "distance_m": 8400}</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm phát sinh thông báo.</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-15T08:30:00Z</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="27" customHeight="1">
+      <c r="A18" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>read_at</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>[Sẽ bỏ: NT-09] Thời điểm người vận hành đánh dấu đã đọc; NULL nếu chưa đọc.</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
           <t>NULL</t>
         </is>
       </c>
-      <c r="I16" s="6" t="n"/>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="I18" s="6" t="n"/>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Kiểu enum</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Giá trị cho phép</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="108" customHeight="1">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="inlineStr">
+    <row r="21" ht="189" customHeight="1">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>notificationtype</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>BATTERY_ALERT, ANOMALY_ALERT, SOH_ALERT, DEVICE_OFFLINE_ALERT, SOS_ALERT, GEOFENCE_ALERT, NO_DRIVER_CHECK_IN_ALERT (dự kiến), OUTSIDE_DRIVER_CHECK_IN (dự kiến)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>BATTERY_ALERT, ANOMALY_ALERT, SOH_ALERT, DEVICE_OFFLINE_ALERT, SOS_ALERT, GEOFENCE_ALERT, NO_DRIVER_CHECK_IN_ALERT (dự kiến), OUTSIDE_DRIVER_CHECK_IN (dự kiến), NO_TRIP_STARTED (dự kiến), LOW_WALLET_BALANCE (dự kiến), TOP_UP_RECEIVED (dự kiến), CHARGING_RECEIPT (dự kiến)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="27" customHeight="1">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>notificationseverity</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>INFO, WARNING, CRITICAL</t>
         </is>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="4" t="n"/>
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="inlineStr">
+    <row r="25" ht="27" customHeight="1">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>ix_notifications_vehicle_id</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>vehicle_id</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>không</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+    </row>
+    <row r="26" ht="27" customHeight="1">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>ix_notifications_organization_cursor</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>organization_id, notification_id</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Planned (NT-09): an organization's alerts after a cursor</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I16"/>
+  <autoFilter ref="A6:I18"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F8" location="'organizations'!A1"/>

</xml_diff>

<commit_message>
refactor(fleet): build the target fleets and memberships design (FL-08, FL-09)
fleets: drop status and its enum; name and fleet_code are optional with
ck_fleets_name_or_code (at least one); new parent_fleet_id (self-FK) so
fleets nest (FL-02). The service refuses an unknown parent (404), a move
under the fleet itself or its own sub-fleets (400), and deleting a fleet
that still has live sub-fleets (409).

fleet_vehicle_memberships: membership_id -> fleet_vehicle_membership_id,
joined_at/left_at -> added_at/removed_at (API fields and path follow);
the plain fleet_id index is dropped (covered by the fleet/time index).

organization_id, per-organization code uniqueness, added_by/removed_by
and the fleet change history wait for the identity tables and stay
@planned in the DBML.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01URvQGCMdGQH5axXbsyq4p6
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -132,7 +132,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="34" hidden="1">'driving_sessions'!$A$6:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="35" hidden="1">'trips'!$A$7:$I$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="36" hidden="1">'trip_history'!$A$7:$I$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="37" hidden="1">'fleets'!$A$7:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="37" hidden="1">'fleets'!$A$7:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="38" hidden="1">'fleet_history'!$A$7:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="39" hidden="1">'fleet_vehicle_memberships'!$A$6:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="40" hidden="1">'geofences'!$A$6:$I$14</definedName>
@@ -2601,7 +2601,7 @@
         </is>
       </c>
       <c r="H50" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
@@ -26411,7 +26411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -26545,7 +26545,7 @@
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9" ht="27" customHeight="1">
+    <row r="9" ht="40.5" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>2</v>
       </c>
@@ -26576,7 +26576,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức sở hữu đội xe, là chủ sở hữu trực tiếp (DM-24 trường hợp A).</t>
+          <t>Tổ chức sở hữu đội xe, là chủ sở hữu trực tiếp (DM-24 trường hợp A). Sẽ được thêm cùng với bảng organizations (miền danh tính).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -26635,7 +26635,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="40.5" customHeight="1">
+    <row r="11" ht="81" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>4</v>
       </c>
@@ -26651,7 +26651,7 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -26662,7 +26662,7 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Mã ngắn do khách hàng chọn, dùng khi nhập dữ liệu và trong báo cáo. Dự kiến (FL-08): không bắt buộc, và chỉ duy nhất trong tổ chức giữa các đội chưa bị xóa.</t>
+          <t>Mã ngắn do khách hàng chọn, dùng khi nhập dữ liệu và trong báo cáo; không bắt buộc, nhưng đội phải có ít nhất tên hoặc mã (ràng buộc kiểm tra, FL-08). Hiện tại là duy nhất trên toàn hệ thống; khi có organization_id thì chỉ cần duy nhất trong tổ chức, giữa các đội chưa bị xóa (FL-08). NULL khi đội chỉ có tên.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -26692,14 +26692,14 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Tên do khách hàng chọn, hiển thị trên portal. Dự kiến (FL-08): không bắt buộc; một đội có ít nhất tên hoặc mã (ràng buộc kiểm tra).</t>
+          <t>Tên do khách hàng chọn, hiển thị trên portal; không bắt buộc, nhưng đội phải có ít nhất tên hoặc mã (ràng buộc kiểm tra, FL-08). NULL khi đội chỉ có mã.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -26713,18 +26713,18 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="27" customHeight="1">
+    <row r="13">
       <c r="A13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>fleetstatus</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -26736,15 +26736,19 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: FL-08] Trạng thái của đội xe; đội xe chỉ là một nhóm nên chỉ có tồn tại hoặc đã xóa.</t>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="n"/>
+          <t>2026-09-01T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
@@ -26752,7 +26756,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -26769,12 +26773,12 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
+          <t>2026-09-10T07:15:00Z</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -26783,13 +26787,13 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="54" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>deleted_at</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -26799,19 +26803,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
+          <t>Thời điểm xóa mềm: đội xe không còn tồn tại (DM-25); các xe thành viên rời đội (FL-06) và lịch sử được giữ lại. Lý do xóa là lý do thay đổi trong lịch sử. NULL khi đội còn tồn tại.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10T07:15:00Z</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -26820,226 +26824,203 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="54" customHeight="1">
-      <c r="A16" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>deleted_at</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="27" customHeight="1">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>ix_fleets_fleet_code</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>fleet_code</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>có</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm xóa mềm: đội xe không còn tồn tại (DM-25); các xe thành viên rời đội (FL-06) và lịch sử được giữ lại. Lý do xóa là lý do thay đổi trong lịch sử. NULL khi đội còn tồn tại.</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="I16" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Kiểu enum</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Giá trị cho phép</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="27" customHeight="1">
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Replaced by uq_fleets_live_organization_code (FL-08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40.5" customHeight="1">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>fleetstatus</t>
+          <t>uq_fleets_live_organization_code</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE (sẽ bỏ), INACTIVE (sẽ bỏ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>ix_fleets_status</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
+          <t>organization_id, fleet_code</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Planned (FL-08): WHERE deleted_at IS NULL AND fleet_code IS NOT NULL. Added with organization_id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="27" customHeight="1">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>ix_fleets_organization_id</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>không</t>
         </is>
       </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>Dropped with status (FL-08)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>ix_fleets_fleet_code</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>fleet_code</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>Replaced by uq_fleets_live_organization_code (FL-08)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="27" customHeight="1">
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Planned (FL-08): added with organization_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="27" customHeight="1">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>ix_fleets_parent_fleet_id</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>parent_fleet_id</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Walking the tree</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
       <c r="A24" s="6" t="n"/>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>uq_fleets_live_organization_code</t>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>fleets</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>organization_id, fleet_code</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Planned (FL-08): WHERE deleted_at IS NULL AND fleet_code IS NOT NULL</t>
+          <t>parent_fleet_id</t>
         </is>
       </c>
     </row>
     <row r="25" ht="27" customHeight="1">
       <c r="A25" s="6" t="n"/>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>ix_fleets_organization_id</t>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>fleet_vehicle_memberships</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>Planned (FL-08)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="27" customHeight="1">
+          <t>fleet_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
       <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>ix_fleets_parent_fleet_id</t>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>fleet_user_assignments</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>parent_fleet_id</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>Planned (FL-08): walking the tree</t>
-        </is>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="4" t="n"/>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
+          <t>fleet_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>geofences</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>fleet_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="27" customHeight="1">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>charging_policy_assignments</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>fleet_id</t>
         </is>
       </c>
     </row>
@@ -27047,93 +27028,28 @@
       <c r="A29" s="6" t="n"/>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>fleets</t>
+          <t>fleet_history</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>parent_fleet_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="27" customHeight="1">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>fleet_vehicle_memberships</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
           <t>fleet_id</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>fleet_user_assignments</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>fleet_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>geofences</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>fleet_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="27" customHeight="1">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>charging_policy_assignments</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>fleet_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="n"/>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>fleet_history</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>fleet_id</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A7:I16"/>
+  <autoFilter ref="A7:I15"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'fleet_history'!A1"/>
     <hyperlink ref="F9" location="'organizations'!A1"/>
     <hyperlink ref="F10" location="'fleets'!A1"/>
-    <hyperlink ref="B29" location="'fleets'!A1"/>
-    <hyperlink ref="B30" location="'fleet_vehicle_memberships'!A1"/>
-    <hyperlink ref="B31" location="'fleet_user_assignments'!A1"/>
-    <hyperlink ref="B32" location="'geofences'!A1"/>
-    <hyperlink ref="B33" location="'charging_policy_assignments'!A1"/>
-    <hyperlink ref="B34" location="'fleet_history'!A1"/>
+    <hyperlink ref="B24" location="'fleets'!A1"/>
+    <hyperlink ref="B25" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="B26" location="'fleet_user_assignments'!A1"/>
+    <hyperlink ref="B27" location="'geofences'!A1"/>
+    <hyperlink ref="B28" location="'charging_policy_assignments'!A1"/>
+    <hyperlink ref="B29" location="'fleet_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -29022,7 +28938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -29112,7 +29028,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1">
+    <row r="7" ht="40.5" customHeight="1">
       <c r="A7" s="6" t="n">
         <v>1</v>
       </c>
@@ -29139,7 +29055,7 @@
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là membership_id, sẽ đổi tên] Mã nội bộ của một giai đoạn thành viên. Đổi tên vì memberships.membership_id (miền danh tính) là một người trong một tổ chức, một khái niệm khác (FL-09).</t>
+          <t>Mã nội bộ của một giai đoạn thành viên. Đổi tên vì memberships.membership_id (miền danh tính) là một người trong một tổ chức, một khái niệm khác (FL-09).</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -29231,7 +29147,7 @@
       </c>
       <c r="I9" s="6" t="n"/>
     </row>
-    <row r="10" ht="27" customHeight="1">
+    <row r="10">
       <c r="A10" s="6" t="n">
         <v>4</v>
       </c>
@@ -29254,7 +29170,7 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là joined_at, sẽ đổi tên] Thời điểm xe được thêm vào đội (FL-09).</t>
+          <t>Thời điểm xe được thêm vào đội (FL-09).</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -29287,7 +29203,7 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là left_at, sẽ đổi tên] Thời điểm xe bị đưa ra khỏi đội; NULL khi vẫn còn trong đội (FL-09).</t>
+          <t>Thời điểm xe bị đưa ra khỏi đội; NULL khi vẫn còn trong đội (FL-09).</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -29297,7 +29213,7 @@
       </c>
       <c r="I11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="27" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>6</v>
       </c>
@@ -29328,7 +29244,7 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Người dùng đã thêm xe vào đội.</t>
+          <t>Người dùng đã thêm xe vào đội. Sẽ được thêm cùng với bảng users (miền danh tính).</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -29338,7 +29254,7 @@
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13" ht="40.5" customHeight="1">
+    <row r="13" ht="54" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
@@ -29369,7 +29285,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Người dùng đã đưa xe ra khỏi đội; NULL khi vẫn là thành viên, hoặc khi hệ thống tự đóng (xe được bán, VH-12, hoặc đội bị xóa, FL-06).</t>
+          <t>Người dùng đã đưa xe ra khỏi đội; NULL khi vẫn là thành viên, hoặc khi hệ thống tự đóng (xe được bán, VH-12, hoặc đội bị xóa, FL-06). Sẽ được thêm cùng với bảng users (miền danh tính).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -29474,12 +29390,12 @@
       <c r="A18" s="6" t="n"/>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>ix_fleet_vehicle_memberships_fleet_id</t>
+          <t>ix_fleet_vehicle_memberships_fleet_time</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>fleet_id</t>
+          <t>fleet_id, added_at</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -29488,22 +29404,18 @@
         </is>
       </c>
       <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>Dropped: covered by ix_fleet_vehicle_memberships_fleet_time (FL-09)</t>
-        </is>
-      </c>
+      <c r="F18" s="6" t="n"/>
     </row>
     <row r="19" ht="27" customHeight="1">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>ix_fleet_vehicle_memberships_fleet_time</t>
+          <t>ix_fleet_vehicle_memberships_vehicle_id</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>fleet_id, added_at</t>
+          <t>vehicle_id</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -29518,7 +29430,7 @@
       <c r="A20" s="6" t="n"/>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>ix_fleet_vehicle_memberships_vehicle_id</t>
+          <t>uq_fleet_vehicle_memberships_active_vehicle</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -29528,33 +29440,13 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-    </row>
-    <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>uq_fleet_vehicle_memberships_active_vehicle</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>WHERE removed_at IS NULL (built as left_at)</t>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>WHERE removed_at IS NULL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(identity): build the identity tables and the change history (WP1)
Identity models (organizations, users, memberships, credentials, sessions,
one-time codes, consents, role assignments, audit log, settings), the
shared history tables and triggers for tracked tables (DM-29: a missing
reason is recorded as "Unspecified change"), and fleets now carry
organization_id with per-organization fleet codes.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01URvQGCMdGQH5axXbsyq4p6
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -9110,7 +9110,7 @@
       </c>
       <c r="I15" s="6" t="n"/>
     </row>
-    <row r="16" ht="40.5" customHeight="1">
+    <row r="16" ht="54" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>9</v>
       </c>
@@ -9133,7 +9133,7 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="I22" s="6" t="n"/>
     </row>
-    <row r="23" ht="40.5" customHeight="1">
+    <row r="23" ht="54" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>16</v>
       </c>
@@ -10919,7 +10919,7 @@
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -13253,7 +13253,7 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="40.5" customHeight="1">
+    <row r="21" ht="54" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
@@ -13276,7 +13276,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -14399,7 +14399,7 @@
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20" ht="40.5" customHeight="1">
+    <row r="20" ht="54" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
@@ -14422,7 +14422,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -15876,7 +15876,7 @@
       </c>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24" ht="40.5" customHeight="1">
+    <row r="24" ht="54" customHeight="1">
       <c r="A24" s="6" t="n">
         <v>17</v>
       </c>
@@ -15899,7 +15899,7 @@
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
@@ -17544,7 +17544,7 @@
       </c>
       <c r="I25" s="6" t="n"/>
     </row>
-    <row r="26" ht="40.5" customHeight="1">
+    <row r="26" ht="54" customHeight="1">
       <c r="A26" s="6" t="n">
         <v>19</v>
       </c>
@@ -17567,7 +17567,7 @@
       <c r="F26" s="6" t="n"/>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
@@ -19140,7 +19140,7 @@
       </c>
       <c r="I22" s="6" t="n"/>
     </row>
-    <row r="23" ht="40.5" customHeight="1">
+    <row r="23" ht="54" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>16</v>
       </c>
@@ -19163,7 +19163,7 @@
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -19908,7 +19908,7 @@
       </c>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24" ht="40.5" customHeight="1">
+    <row r="24" ht="54" customHeight="1">
       <c r="A24" s="6" t="n">
         <v>17</v>
       </c>
@@ -19931,7 +19931,7 @@
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
@@ -22890,7 +22890,7 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="40.5" customHeight="1">
+    <row r="21" ht="54" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
@@ -22913,7 +22913,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -26315,7 +26315,7 @@
       </c>
       <c r="I33" s="6" t="n"/>
     </row>
-    <row r="34" ht="40.5" customHeight="1">
+    <row r="34" ht="54" customHeight="1">
       <c r="A34" s="6" t="n">
         <v>27</v>
       </c>
@@ -26338,7 +26338,7 @@
       <c r="F34" s="6" t="n"/>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
@@ -26411,7 +26411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -26545,7 +26545,7 @@
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9" ht="40.5" customHeight="1">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>2</v>
       </c>
@@ -26576,7 +26576,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Tổ chức sở hữu đội xe, là chủ sở hữu trực tiếp (DM-24 trường hợp A). Sẽ được thêm cùng với bảng organizations (miền danh tính).</t>
+          <t>Tổ chức sở hữu đội xe, là chủ sở hữu trực tiếp (DM-24 trường hợp A).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -26635,7 +26635,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="81" customHeight="1">
+    <row r="11" ht="67.5" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>4</v>
       </c>
@@ -26654,15 +26654,11 @@
           <t>có</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>UQ</t>
-        </is>
-      </c>
+      <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Mã ngắn do khách hàng chọn, dùng khi nhập dữ liệu và trong báo cáo; không bắt buộc, nhưng đội phải có ít nhất tên hoặc mã (ràng buộc kiểm tra, FL-08). Hiện tại là duy nhất trên toàn hệ thống; khi có organization_id thì chỉ cần duy nhất trong tổ chức, giữa các đội chưa bị xóa (FL-08). NULL khi đội chỉ có tên.</t>
+          <t>Mã ngắn do khách hàng chọn, dùng khi nhập dữ liệu và trong báo cáo; không bắt buộc, nhưng đội phải có ít nhất tên hoặc mã (ràng buộc kiểm tra, FL-08). Chỉ cần duy nhất trong tổ chức, giữa các đội chưa bị xóa (FL-08). NULL khi đội chỉ có tên.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -26849,16 +26845,16 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="27" customHeight="1">
+    <row r="18" ht="40.5" customHeight="1">
       <c r="A18" s="6" t="n"/>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>ix_fleets_fleet_code</t>
+          <t>uq_fleets_live_organization_code</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>fleet_code</t>
+          <t>organization_id, fleet_code</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -26869,31 +26865,31 @@
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Replaced by uq_fleets_live_organization_code (FL-08)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="40.5" customHeight="1">
+          <t>WHERE deleted_at IS NULL AND fleet_code IS NOT NULL: a code names one live fleet inside its organization (FL-08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="27" customHeight="1">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>uq_fleets_live_organization_code</t>
+          <t>ix_fleets_organization_id</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>organization_id, fleet_code</t>
+          <t>organization_id</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Planned (FL-08): WHERE deleted_at IS NULL AND fleet_code IS NOT NULL. Added with organization_id.</t>
+          <t>Fleets of one organization (FL-08)</t>
         </is>
       </c>
     </row>
@@ -26901,12 +26897,12 @@
       <c r="A20" s="6" t="n"/>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>ix_fleets_organization_id</t>
+          <t>ix_fleets_parent_fleet_id</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
+          <t>parent_fleet_id</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -26917,66 +26913,55 @@
       <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Planned (FL-08): added with organization_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>ix_fleets_parent_fleet_id</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
+          <t>Walking the tree</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>fleets</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>parent_fleet_id</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>Walking the tree</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="4" t="n"/>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
+    </row>
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="6" t="n"/>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>fleets</t>
+          <t>fleet_vehicle_memberships</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>parent_fleet_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="27" customHeight="1">
+          <t>fleet_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>fleet_vehicle_memberships</t>
+          <t>fleet_user_assignments</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -26989,7 +26974,7 @@
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>fleet_user_assignments</t>
+          <t>geofences</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -26998,11 +26983,11 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="27" customHeight="1">
       <c r="A27" s="6" t="n"/>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>geofences</t>
+          <t>charging_policy_assignments</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -27011,27 +26996,14 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="27" customHeight="1">
+    <row r="28">
       <c r="A28" s="6" t="n"/>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>charging_policy_assignments</t>
+          <t>fleet_history</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>fleet_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>fleet_history</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>fleet_id</t>
         </is>
@@ -27044,12 +27016,12 @@
     <hyperlink ref="A5" location="'fleet_history'!A1"/>
     <hyperlink ref="F9" location="'organizations'!A1"/>
     <hyperlink ref="F10" location="'fleets'!A1"/>
-    <hyperlink ref="B24" location="'fleets'!A1"/>
-    <hyperlink ref="B25" location="'fleet_vehicle_memberships'!A1"/>
-    <hyperlink ref="B26" location="'fleet_user_assignments'!A1"/>
-    <hyperlink ref="B27" location="'geofences'!A1"/>
-    <hyperlink ref="B28" location="'charging_policy_assignments'!A1"/>
-    <hyperlink ref="B29" location="'fleet_history'!A1"/>
+    <hyperlink ref="B23" location="'fleets'!A1"/>
+    <hyperlink ref="B24" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="B25" location="'fleet_user_assignments'!A1"/>
+    <hyperlink ref="B26" location="'geofences'!A1"/>
+    <hyperlink ref="B27" location="'charging_policy_assignments'!A1"/>
+    <hyperlink ref="B28" location="'fleet_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27541,7 +27513,7 @@
       </c>
       <c r="I18" s="6" t="n"/>
     </row>
-    <row r="19" ht="40.5" customHeight="1">
+    <row r="19" ht="54" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>12</v>
       </c>
@@ -27564,7 +27536,7 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -29244,7 +29216,7 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Người dùng đã thêm xe vào đội. Sẽ được thêm cùng với bảng users (miền danh tính).</t>
+          <t>Người dùng đã thêm xe vào đội; NULL khi không rõ hoặc do hệ thống thực hiện.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -29254,7 +29226,7 @@
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13" ht="54" customHeight="1">
+    <row r="13" ht="40.5" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
@@ -29285,7 +29257,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Người dùng đã đưa xe ra khỏi đội; NULL khi vẫn là thành viên, hoặc khi hệ thống tự đóng (xe được bán, VH-12, hoặc đội bị xóa, FL-06). Sẽ được thêm cùng với bảng users (miền danh tính).</t>
+          <t>Người dùng đã đưa xe ra khỏi đội; NULL khi vẫn là thành viên, hoặc khi hệ thống tự đóng (xe được bán, VH-12, hoặc đội bị xóa, FL-06).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -31577,7 +31549,7 @@
       </c>
       <c r="I21" s="6" t="n"/>
     </row>
-    <row r="22" ht="40.5" customHeight="1">
+    <row r="22" ht="54" customHeight="1">
       <c r="A22" s="6" t="n">
         <v>15</v>
       </c>
@@ -31600,7 +31572,7 @@
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -34119,7 +34091,7 @@
       </c>
       <c r="I21" s="6" t="n"/>
     </row>
-    <row r="22" ht="40.5" customHeight="1">
+    <row r="22" ht="54" customHeight="1">
       <c r="A22" s="6" t="n">
         <v>15</v>
       </c>
@@ -34142,7 +34114,7 @@
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -35893,7 +35865,7 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="40.5" customHeight="1">
+    <row r="21" ht="54" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
@@ -35916,7 +35888,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -36502,7 +36474,7 @@
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20" ht="40.5" customHeight="1">
+    <row r="20" ht="54" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
@@ -36525,7 +36497,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -37957,7 +37929,7 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="40.5" customHeight="1">
+    <row r="21" ht="54" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
@@ -37980,7 +37952,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -44925,7 +44897,7 @@
       </c>
       <c r="I17" s="6" t="n"/>
     </row>
-    <row r="18" ht="40.5" customHeight="1">
+    <row r="18" ht="54" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>11</v>
       </c>
@@ -44948,7 +44920,7 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -50314,7 +50286,7 @@
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20" ht="40.5" customHeight="1">
+    <row r="20" ht="54" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
@@ -50337,7 +50309,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -52402,7 +52374,7 @@
       </c>
       <c r="I24" s="6" t="n"/>
     </row>
-    <row r="25" ht="40.5" customHeight="1">
+    <row r="25" ht="54" customHeight="1">
       <c r="A25" s="6" t="n">
         <v>18</v>
       </c>
@@ -52425,7 +52397,7 @@
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -54207,7 +54179,7 @@
       </c>
       <c r="I18" s="6" t="n"/>
     </row>
-    <row r="19" ht="40.5" customHeight="1">
+    <row r="19" ht="54" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>12</v>
       </c>
@@ -54230,7 +54202,7 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -54849,7 +54821,7 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="40.5" customHeight="1">
+    <row r="21" ht="54" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
@@ -54872,7 +54844,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Thay đổi không có lý do sẽ bị từ chối.</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">

</xml_diff>

<commit_message>
feat(vehicles): build vehicles, models, batteries and warranties (WP1)
vehicles take organization_id, acquired_at and a vehicle model, with
change history; vehicle_models, battery_models, batteries and warranties
are new (VH-20); fleet checks the vehicle belongs to the fleet's
organization (FL-09).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01URvQGCMdGQH5axXbsyq4p6
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -112,7 +112,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'access_audit_logs'!$A$6:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'organization_settings'!$A$7:$I$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'organization_setting_history'!$A$7:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'vehicles'!$A$7:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'vehicles'!$A$7:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'vehicle_history'!$A$7:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'vehicle_models'!$A$7:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'vehicle_model_history'!$A$7:$I$21</definedName>
@@ -1516,7 +1516,7 @@
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Bản thân chiếc xe tải: định danh (VIN, biển số), thông số và trạng thái kích hoạt.
+          <t>Bản thân chiếc xe tải: chủ sở hữu, định danh (VIN, biển số), dòng xe và trạng thái phục vụ.
 • Tại mỗi thời điểm, một xe thuộc một tổ chức (organization_id, acquired_at); các chủ trước nằm trong lịch sử thay đổi của xe, và view vehicle_ownership_periods liệt kê mọi giai đoạn sở hữu (VH-10).
 • Sau khi bán xe (VH-11): dữ liệu ghi nhận dưới chủ cũ (dữ liệu vận hành và những gì tính từ đó) vẫn thuộc chủ cũ; tình trạng xe (sức khỏe, lỗi, bảo dưỡng, bảo hành) và các tổng tích lũy (quãng đường, năng lượng, chu kỳ sạc) đi theo xe.
 • Chỉ một chủ sở hữu (quyết định ngày 03/10/2026): mỗi xe (và mỗi hồ sơ tài xế) thuộc đúng một tổ chức trong hệ thống. Khi các bên hợp tác (ví dụ chủ xe tự lái hoạt động dưới giấy phép kinh doanh vận tải của một công ty), các bên tự thỏa thuận và khai báo chủ sở hữu cho chúng ta; điều khoản hợp tác của họ nằm ngoài trách nhiệm của chúng ta và không được mô hình hóa.</t>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="H24" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
@@ -1613,7 +1613,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="81" customHeight="1">
+    <row r="26" ht="108" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t>14</t>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Danh mục dòng xe và thông số kỹ thuật (VEH-03, VH-15), dùng chung cho mọi tổ chức, do bộ phận vận hành của chúng ta quản lý. Số liệu chỉ được nhập khi đã xác nhận và có thể cập nhật sau (lịch sử lưu các giá trị trước). Chỉ xe điện: không có số liệu diesel (đường cơ sở diesel cho báo cáo carbon là tính năng riêng). Mọi dòng xe hiện tại đều là đầu kéo; cột loại thân xe sẽ được thêm khi có loại khác. Có lưu lịch sử thay đổi vì báo cáo dựa vào các số liệu này.</t>
+          <t>Danh mục dòng xe và thông số kỹ thuật (VEH-03, VH-15), dùng chung cho mọi tổ chức, do bộ phận vận hành của chúng ta quản lý. Số liệu chỉ được nhập khi đã xác nhận và có thể cập nhật sau (lịch sử lưu các giá trị trước). Chỉ xe điện: không có số liệu diesel (đường cơ sở diesel cho báo cáo carbon là tính năng riêng). Mọi dòng xe hiện tại đều là đầu kéo; cột loại thân xe sẽ được thêm khi có loại khác. Có lưu lịch sử thay đổi vì báo cáo dựa vào các số liệu này. Cho đến khi miền pin đọc được, dung lượng pin danh định của dòng xe là dung lượng pack mà báo cáo dùng (VH-20).</t>
         </is>
       </c>
       <c r="H26" s="6" t="n">
@@ -1720,7 +1720,7 @@
       <c r="F28" s="5" t="n"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Quản lý từng pin xe như một tài sản riêng: pin có thể chuyển giữa các xe và có thể thuộc một tổ chức khác với chủ xe. Phụ thuộc miền xe và miền định danh; miền xe không phụ thuộc miền này. Chưa được xây dựng.
+          <t>Quản lý từng pin xe như một tài sản riêng: pin có thể chuyển giữa các xe và có thể thuộc một tổ chức khác với chủ xe. Phụ thuộc miền xe và miền định danh; miền xe không phụ thuộc miền này.
 • Một dòng pin là một loại pin kèm thông số kỹ thuật.
 • Một pin là một khối pin vật lý: chủ sở hữu và xe đang lắp là các cột kèm lịch sử (mỗi xe một pin).</t>
         </is>
@@ -1923,7 +1923,7 @@
       <c r="F33" s="5" t="n"/>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Bảo hành của xe, pin, T-Box và trụ sạc: thời hạn, giới hạn và lý do một bảo hành bị hủy. Phụ thuộc miền xe, pin, telematics và trạm sạc; không miền nào phụ thuộc miền này. Chưa được xây dựng.
+          <t>Bảo hành của xe, pin, T-Box và trụ sạc: thời hạn, giới hạn và lý do một bảo hành bị hủy. Phụ thuộc miền xe, pin, telematics và trạm sạc; không miền nào phụ thuộc miền này.
 • Một bảo hành áp dụng cho đúng một xe, pin, T-Box hoặc trụ sạc và đi theo đối tượng sang chủ kế tiếp.</t>
         </is>
       </c>
@@ -9206,7 +9206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9547,12 +9547,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>make</t>
+          <t>year</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -9564,28 +9564,32 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: VH-15] Hãng sản xuất; nay là vehicle_models.make.</t>
+          <t>Năm sản xuất.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Tri-Ring</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="n"/>
-    </row>
-    <row r="15">
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="108" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>vehiclestatus</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -9597,45 +9601,49 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: VH-15] Dòng xe; nay là vehicle_models.model_name.</t>
+          <t>Trạng thái phục vụ, do con người hoặc quy tắc nghiệp vụ thay mặt công ty đặt (DM-25). ACTIVE: đang phục vụ. INACTIVE: không phục vụ, ví dụ đang ở xưởng hoặc chủ xe không dùng; lý do cho biết trường hợp nào (khi có hồ sơ sửa chữa, việc đang bảo dưỡng được đọc từ hồ sơ sửa chữa đang mở). Xe rời hệ thống được chuyển sang INACTIVE và xóa mềm. Xe đang chạy hay gửi dữ liệu được tính từ dữ liệu vận hành, không lưu.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>EVT-400</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="n"/>
-    </row>
-    <row r="16">
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="27" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>year</t>
+          <t>status_reason</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>varchar(200)</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Năm sản xuất.</t>
+          <t>Lý do của trạng thái hiện tại, hoặc lý do xe rời hệ thống; NULL khi ACTIVE.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Brake system repair at the Binh Duong workshop</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -9644,18 +9652,18 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="108" customHeight="1">
+    <row r="17">
       <c r="A17" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>vehiclestatus</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -9667,12 +9675,12 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Trạng thái phục vụ, do con người hoặc quy tắc nghiệp vụ thay mặt công ty đặt (DM-25). ACTIVE: đang phục vụ. INACTIVE: không phục vụ, ví dụ đang ở xưởng hoặc chủ xe không dùng; lý do cho biết trường hợp nào (khi có hồ sơ sửa chữa, việc đang bảo dưỡng được đọc từ hồ sơ sửa chữa đang mở). Xe rời hệ thống được chuyển sang INACTIVE và xóa mềm. Xe đang chạy hay gửi dữ liệu được tính từ dữ liệu vận hành, không lưu.</t>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>2026-09-01T02:00:00Z</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -9681,35 +9689,35 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="27" customHeight="1">
+    <row r="18">
       <c r="A18" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>status_reason</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>varchar(200)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Lý do của trạng thái hiện tại, hoặc lý do xe rời hệ thống; NULL khi ACTIVE.</t>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Brake system repair at the Binh Duong workshop</t>
+          <t>2026-09-10T07:15:00Z</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -9724,329 +9732,252 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>activation_status</t>
+          <t>deleted_at</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>vehicleactivationstatus</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: VH-06] Tiến độ kích hoạt thiết bị, thang một chiều không phản ánh việc T-Box bị tháo. Thay bằng tính toán: có thiết bị hiện tại từ telematics, đã nhận dữ liệu từ telemetry.</t>
+          <t>Thời điểm xóa mềm: bản ghi không còn thuộc hệ thống, do đã rời đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ, lý do nằm trong status_reason. NULL khi còn thuộc hệ thống.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>ACTIVATED</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="n"/>
-    </row>
-    <row r="20" ht="67.5" customHeight="1">
-      <c r="A20" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>battery_capacity_kwh</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>float8</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Kiểu enum</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Giá trị cho phép</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>vehiclestatus</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVE, INACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="4" t="n"/>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>uq_vehicles_live_vin</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>vin</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>có</t>
         </is>
       </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: VH-16] Dung lượng pin danh định có thể dùng (kWh), chưa trừ suy giảm SOH; NULL nếu chưa biết (báo cáo sẽ dùng giá trị mặc định). Thay bằng dung lượng thiết kế của pin đang lắp, hoặc dung lượng danh định của dòng xe khi chưa ghi nhận pin.</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>282.0</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-01T02:00:00Z</t>
-        </is>
-      </c>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-10T07:15:00Z</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="54" customHeight="1">
-      <c r="A23" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>deleted_at</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm xóa mềm: bản ghi không còn thuộc hệ thống, do đã rời đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ, lý do nằm trong status_reason. NULL khi còn thuộc hệ thống.</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Kiểu enum</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Giá trị cho phép</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="54" customHeight="1">
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>WHERE deleted_at IS NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="27" customHeight="1">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>vehiclestatus</t>
+          <t>uq_vehicles_live_license_plate</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE, INACTIVE, MAINTENANCE (sẽ bỏ), DECOMMISSIONED (sẽ bỏ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="27" customHeight="1">
+          <t>license_plate</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>WHERE deleted_at IS NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
       <c r="A27" s="6" t="n"/>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>vehicleactivationstatus</t>
+          <t>ix_vehicles_status</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>PENDING, DEVICE_ASSIGNED, ACTIVATED</t>
-        </is>
-      </c>
-    </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" s="4" t="n"/>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="40.5" customHeight="1">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>uq_vehicles_live_vin</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>vin</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>Planned (VH-07), replaces the full unique constraint: WHERE deleted_at IS NULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="40.5" customHeight="1">
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="n"/>
+    </row>
+    <row r="28" ht="27" customHeight="1">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>ix_vehicles_organization_id</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Vehicles of one organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="4" t="n"/>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
       <c r="A31" s="6" t="n"/>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>uq_vehicles_live_license_plate</t>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>batteries</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>license_plate</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>Planned (VH-07), replaces the full unique constraint: WHERE deleted_at IS NULL</t>
+          <t>vehicle_id</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n"/>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>ix_vehicles_status</t>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>warranties</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-    </row>
-    <row r="33"/>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n"/>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>telematics</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+    </row>
     <row r="34">
-      <c r="A34" s="4" t="n"/>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
+      <c r="A34" s="6" t="n"/>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>telemetry</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="27" customHeight="1">
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>batteries</t>
+          <t>driver_vehicle_assignments</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -10059,7 +9990,7 @@
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>warranties</t>
+          <t>driving_sessions</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -10072,20 +10003,20 @@
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>telematics</t>
+          <t>trips</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
+          <t>planned_vehicle_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="27" customHeight="1">
       <c r="A38" s="6" t="n"/>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>telemetry</t>
+          <t>fleet_vehicle_memberships</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -10094,11 +10025,11 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="27" customHeight="1">
+    <row r="39">
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>driver_vehicle_assignments</t>
+          <t>charging_sessions</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -10111,7 +10042,7 @@
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>driving_sessions</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -10124,20 +10055,20 @@
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>trips</t>
+          <t>support_cases</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>planned_vehicle_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="27" customHeight="1">
+          <t>vehicle_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>fleet_vehicle_memberships</t>
+          <t>maintenance_bookings</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -10146,11 +10077,11 @@
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="27" customHeight="1">
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>charging_sessions</t>
+          <t>charging_policy_assignments</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -10163,7 +10094,7 @@
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>policy_violations</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -10176,7 +10107,7 @@
       <c r="A45" s="6" t="n"/>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>support_cases</t>
+          <t>subscriptions</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -10189,7 +10120,7 @@
       <c r="A46" s="6" t="n"/>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>maintenance_bookings</t>
+          <t>vehicle_history</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -10198,81 +10129,29 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="27" customHeight="1">
-      <c r="A47" s="6" t="n"/>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>charging_policy_assignments</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="n"/>
-      <c r="B48" s="7" t="inlineStr">
-        <is>
-          <t>policy_violations</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="n"/>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>subscriptions</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="n"/>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>vehicle_history</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A7:I23"/>
+  <autoFilter ref="A7:I19"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'vehicle_history'!A1"/>
     <hyperlink ref="F9" location="'organizations'!A1"/>
     <hyperlink ref="F13" location="'vehicle_models'!A1"/>
-    <hyperlink ref="B35" location="'batteries'!A1"/>
-    <hyperlink ref="B36" location="'warranties'!A1"/>
-    <hyperlink ref="B37" location="'telematics'!A1"/>
-    <hyperlink ref="B38" location="'telemetry'!A1"/>
-    <hyperlink ref="B39" location="'driver_vehicle_assignments'!A1"/>
-    <hyperlink ref="B40" location="'driving_sessions'!A1"/>
-    <hyperlink ref="B41" location="'trips'!A1"/>
-    <hyperlink ref="B42" location="'fleet_vehicle_memberships'!A1"/>
-    <hyperlink ref="B43" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B44" location="'notifications'!A1"/>
-    <hyperlink ref="B45" location="'support_cases'!A1"/>
-    <hyperlink ref="B46" location="'maintenance_bookings'!A1"/>
-    <hyperlink ref="B47" location="'charging_policy_assignments'!A1"/>
-    <hyperlink ref="B48" location="'policy_violations'!A1"/>
-    <hyperlink ref="B49" location="'subscriptions'!A1"/>
-    <hyperlink ref="B50" location="'vehicle_history'!A1"/>
+    <hyperlink ref="B31" location="'batteries'!A1"/>
+    <hyperlink ref="B32" location="'warranties'!A1"/>
+    <hyperlink ref="B33" location="'telematics'!A1"/>
+    <hyperlink ref="B34" location="'telemetry'!A1"/>
+    <hyperlink ref="B35" location="'driver_vehicle_assignments'!A1"/>
+    <hyperlink ref="B36" location="'driving_sessions'!A1"/>
+    <hyperlink ref="B37" location="'trips'!A1"/>
+    <hyperlink ref="B38" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="B39" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B40" location="'notifications'!A1"/>
+    <hyperlink ref="B41" location="'support_cases'!A1"/>
+    <hyperlink ref="B42" location="'maintenance_bookings'!A1"/>
+    <hyperlink ref="B43" location="'charging_policy_assignments'!A1"/>
+    <hyperlink ref="B44" location="'policy_violations'!A1"/>
+    <hyperlink ref="B45" location="'subscriptions'!A1"/>
+    <hyperlink ref="B46" location="'vehicle_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12171,7 +12050,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Danh mục dòng xe và thông số kỹ thuật (VEH-03, VH-15), dùng chung cho mọi tổ chức, do bộ phận vận hành của chúng ta quản lý. Số liệu chỉ được nhập khi đã xác nhận và có thể cập nhật sau (lịch sử lưu các giá trị trước). Chỉ xe điện: không có số liệu diesel (đường cơ sở diesel cho báo cáo carbon là tính năng riêng). Mọi dòng xe hiện tại đều là đầu kéo; cột loại thân xe sẽ được thêm khi có loại khác. Có lưu lịch sử thay đổi vì báo cáo dựa vào các số liệu này.</t>
+          <t>Danh mục dòng xe và thông số kỹ thuật (VEH-03, VH-15), dùng chung cho mọi tổ chức, do bộ phận vận hành của chúng ta quản lý. Số liệu chỉ được nhập khi đã xác nhận và có thể cập nhật sau (lịch sử lưu các giá trị trước). Chỉ xe điện: không có số liệu diesel (đường cơ sở diesel cho báo cáo carbon là tính năng riêng). Mọi dòng xe hiện tại đều là đầu kéo; cột loại thân xe sẽ được thêm khi có loại khác. Có lưu lịch sử thay đổi vì báo cáo dựa vào các số liệu này. Cho đến khi miền pin đọc được, dung lượng pin danh định của dòng xe là dung lượng pack mà báo cáo dùng (VH-20).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(telematics): build telematics, status reports and telemetry (WP1)
telematics take organization_id, IMEI and change history; the device
report table telematic_status_reports is new; vehicle_telemetry becomes
telemetry with the renamed columns and a once-written organization_id
(TX-12, TM-15).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01URvQGCMdGQH5axXbsyq4p6
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -122,10 +122,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'battery_history'!$A$7:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'warranties'!$A$7:$I$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'warranty_history'!$A$7:$I$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'telematics'!$A$7:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'telematics'!$A$7:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'telematic_history'!$A$7:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'telematic_status_reports'!$A$6:$I$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'telemetry'!$A$6:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'telemetry'!$A$6:$I$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'drivers'!$A$7:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="32" hidden="1">'driver_history'!$A$7:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="33" hidden="1">'driver_vehicle_assignments'!$A$6:$I$14</definedName>
@@ -2078,7 +2078,7 @@
         </is>
       </c>
       <c r="H37" s="6" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
@@ -2236,7 +2236,7 @@
         </is>
       </c>
       <c r="H41" s="6" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
@@ -17519,7 +17519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -17809,7 +17809,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="67.5" customHeight="1">
+    <row r="13" ht="54" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>6</v>
       </c>
@@ -17840,7 +17840,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Xe mà thiết bị đang gắn; NULL khi trong kho hoặc đã tháo. Mỗi xe gắn tối đa một thiết bị. Các xe trước nằm trong telematic_history; view được thêm khi có tính năng đầu tiên cần (DM-27). Dự kiến: khóa ngoại chuyển sang ON DELETE RESTRICT như mọi liên kết khác (hiện là SET NULL).</t>
+          <t>Xe mà thiết bị đang gắn; NULL khi trong kho hoặc đã tháo. Mỗi xe gắn tối đa một thiết bị. Các xe trước nằm trong telematic_history; view được thêm khi có tính năng đầu tiên cần (DM-27).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -17965,79 +17965,87 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="27" customHeight="1">
+    <row r="17">
       <c r="A17" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>firmware_version</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: TX-08] Firmware nhập qua API; thiết bị tự báo trong báo cáo trạng thái (telematic_status_reports).</t>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>1.4.2</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="n"/>
-    </row>
-    <row r="18" ht="54" customHeight="1">
+          <t>2026-09-01T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>telemetry_interval_seconds</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: TX-09] Chu kỳ gửi đã đẩy xuống thiết bị này; chu kỳ nay là thiết lập của tổ chức (organization_settings), còn chu kỳ thiết bị thực sự dùng nằm trong báo cáo trạng thái (telematic_status_reports).</t>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="n"/>
-    </row>
-    <row r="19" ht="40.5" customHeight="1">
+          <t>2026-09-10T07:15:00Z</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>12</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>config_pushed_at</t>
+          <t>deleted_at</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -18054,124 +18062,44 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: TX-08] Thời điểm đẩy chu kỳ lần gần nhất; việc đẩy xảy ra khi lưu thay đổi nên lấy từ changed_at của lịch sử (DM-23).</t>
+          <t>Thời điểm xóa mềm: bản ghi không còn thuộc hệ thống, do đã rời đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ, lý do nằm trong status_reason. NULL khi còn thuộc hệ thống. Các xe trước vẫn nằm trong lịch sử.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>2026-09-12T03:00:00Z</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-01T02:00:00Z</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="inlineStr">
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>🔍</t>
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
-      <c r="A21" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-10T07:15:00Z</t>
-        </is>
-      </c>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="54" customHeight="1">
-      <c r="A22" s="6" t="n">
-        <v>15</v>
-      </c>
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Kiểu enum</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Giá trị cho phép</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>deleted_at</t>
+          <t>telematicstatus</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm xóa mềm: bản ghi không còn thuộc hệ thống, do đã rời đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ, lý do nằm trong status_reason. NULL khi còn thuộc hệ thống. Các xe trước vẫn nằm trong lịch sử.</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
+          <t>ACTIVE, INACTIVE</t>
         </is>
       </c>
     </row>
@@ -18180,156 +18108,179 @@
       <c r="A24" s="4" t="n"/>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Kiểu enum</t>
+          <t>Chỉ mục (index)</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Giá trị cho phép</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="27" customHeight="1">
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>telematicstatus</t>
+          <t>ix_telematics_status</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE, INACTIVE, MAINTENANCE (sẽ bỏ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="4" t="n"/>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+    </row>
+    <row r="26" ht="27" customHeight="1">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>ix_telematics_telematic_serial</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>telematic_serial</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Unique only among devices not deleted (WHERE deleted_at IS NULL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="40.5" customHeight="1">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>uq_telematics_imei</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>imei</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Unique only among devices not deleted: WHERE imei IS NOT NULL AND deleted_at IS NULL (TX-12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="27" customHeight="1">
       <c r="A28" s="6" t="n"/>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>ix_telematics_status</t>
+          <t>uq_telematics_active_vehicle</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>vehicle_id</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E28" s="6" t="n"/>
-      <c r="F28" s="6" t="n"/>
-    </row>
-    <row r="29" ht="40.5" customHeight="1">
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>WHERE vehicle_id IS NOT NULL AND deleted_at IS NULL, one device per truck</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="27" customHeight="1">
       <c r="A29" s="6" t="n"/>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>ix_telematics_telematic_serial</t>
+          <t>ix_telematics_organization_id</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>telematic_serial</t>
+          <t>organization_id</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E29" s="6" t="n"/>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>Planned (TX-08): unique only among devices not deleted (WHERE deleted_at IS NULL)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="27" customHeight="1">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>ix_telematics_vehicle_id</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>To be removed (TX-08): the unique index below serves it</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="54" customHeight="1">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>uq_telematics_active_vehicle</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>WHERE deleted_at IS NULL; planned (TX-08): WHERE vehicle_id IS NOT NULL AND deleted_at IS NULL, one device per truck</t>
-        </is>
-      </c>
-    </row>
-    <row r="32"/>
+          <t>Devices of one organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="4" t="n"/>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n"/>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>warranties</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>telematic_id</t>
+        </is>
+      </c>
+    </row>
     <row r="33">
-      <c r="A33" s="4" t="n"/>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
+      <c r="A33" s="6" t="n"/>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>telematic_status_reports</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>telematic_id</t>
         </is>
       </c>
     </row>
@@ -18337,7 +18288,7 @@
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>warranties</t>
+          <t>telemetry</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -18350,7 +18301,7 @@
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>telematic_status_reports</t>
+          <t>telematic_history</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -18359,43 +18310,17 @@
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>telemetry</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>telematic_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>telematic_history</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>telematic_id</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A7:I22"/>
+  <autoFilter ref="A7:I19"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'telematic_history'!A1"/>
     <hyperlink ref="F11" location="'organizations'!A1"/>
     <hyperlink ref="F13" location="'vehicles'!A1"/>
-    <hyperlink ref="B34" location="'warranties'!A1"/>
-    <hyperlink ref="B35" location="'telematic_status_reports'!A1"/>
-    <hyperlink ref="B36" location="'telemetry'!A1"/>
-    <hyperlink ref="B37" location="'telematic_history'!A1"/>
+    <hyperlink ref="B32" location="'warranties'!A1"/>
+    <hyperlink ref="B33" location="'telematic_status_reports'!A1"/>
+    <hyperlink ref="B34" location="'telemetry'!A1"/>
+    <hyperlink ref="B35" location="'telematic_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20479,7 +20404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -20684,7 +20609,7 @@
       </c>
       <c r="I9" s="6" t="n"/>
     </row>
-    <row r="10" ht="27" customHeight="1">
+    <row r="10">
       <c r="A10" s="6" t="n">
         <v>4</v>
       </c>
@@ -20707,7 +20632,7 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là message_uuid, sẽ đổi tên] Mã thiết bị gán cho mỗi bản tin, dùng để phát hiện trùng.</t>
+          <t>Mã thiết bị gán cho mỗi bản tin, dùng để phát hiện trùng.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -20764,12 +20689,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>telematic_serial</t>
+          <t>vehicle_id</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -20777,32 +20702,40 @@
           <t>không</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>vehicles.vehicle_id (khi xóa: xóa theo)</t>
+        </is>
+      </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: TM-16] Serial thiết bị, chép vào dòng để phục vụ kiểm tra và gỡ lỗi.</t>
+          <t>Xe mà bản ghi mô tả.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>TBX-2409-000123</t>
+          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13" ht="27" customHeight="1">
+    <row r="13">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id</t>
+          <t>received_at</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -20810,40 +20743,32 @@
           <t>không</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>vehicles.vehicle_id (khi xóa: xóa theo)</t>
-        </is>
-      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Xe mà bản ghi mô tả.</t>
+          <t>Thời điểm backend nhận bản tin.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
+          <t>2026-09-15T08:30:02Z</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>received_at</t>
+          <t>location</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>geography(POINT,4326)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -20855,56 +20780,56 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm backend nhận bản tin.</t>
+          <t>Vị trí GPS (điểm WGS84, kinh độ trước). Không có chỉ mục không gian (luồng ghi dày đặc).</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-15T08:30:02Z</t>
+          <t>POINT(106.6297 10.8231)</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
     </row>
-    <row r="15" ht="27" customHeight="1">
+    <row r="15">
       <c r="A15" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>speed_kmh</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>geography(POINT,4326)</t>
+          <t>float8</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Vị trí GPS (điểm WGS84, kinh độ trước). Không có chỉ mục không gian (luồng ghi dày đặc).</t>
+          <t>Tốc độ (km/h).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>POINT(106.6297 10.8231)</t>
+          <t>62.5</t>
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="27" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>speed_kmh</t>
+          <t>heading_degrees</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -20921,23 +20846,23 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là speed, sẽ đổi tên] Tốc độ (km/h).</t>
+          <t>Hướng di chuyển (độ, 0-360, 0 = hướng bắc); NULL nếu không rõ.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>62.5</t>
+          <t>135.0</t>
         </is>
       </c>
       <c r="I16" s="6" t="n"/>
     </row>
-    <row r="17" ht="27" customHeight="1">
+    <row r="17">
       <c r="A17" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>heading_degrees</t>
+          <t>soc_percent</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -20947,30 +20872,30 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là heading, sẽ đổi tên] Hướng di chuyển (độ, 0-360, 0 = hướng bắc); NULL nếu không rõ.</t>
+          <t>Mức pin còn lại (SOC), % (0-100).</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>135.0</t>
+          <t>64.2</t>
         </is>
       </c>
       <c r="I17" s="6" t="n"/>
     </row>
-    <row r="18" ht="27" customHeight="1">
+    <row r="18">
       <c r="A18" s="6" t="n">
         <v>12</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>soc_percent</t>
+          <t>battery_voltage_v</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -20980,30 +20905,30 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là soc, sẽ đổi tên] Mức pin còn lại (SOC), % (0-100).</t>
+          <t>Điện áp pack pin (V).</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>64.2</t>
+          <t>612.4</t>
         </is>
       </c>
       <c r="I18" s="6" t="n"/>
     </row>
-    <row r="19" ht="27" customHeight="1">
+    <row r="19">
       <c r="A19" s="6" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>battery_voltage_v</t>
+          <t>battery_current_a</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -21020,12 +20945,12 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là battery_voltage, sẽ đổi tên] Điện áp pack pin (V).</t>
+          <t>Dòng điện pack pin (A).</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>612.4</t>
+          <t>-85.3</t>
         </is>
       </c>
       <c r="I19" s="6" t="n"/>
@@ -21036,7 +20961,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>battery_current_a</t>
+          <t>battery_temperature_celsius</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -21053,12 +20978,12 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là battery_current, sẽ đổi tên] Dòng điện pack pin (A).</t>
+          <t>Nhiệt độ pin (°C).</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>-85.3</t>
+          <t>34.5</t>
         </is>
       </c>
       <c r="I20" s="6" t="n"/>
@@ -21069,7 +20994,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>battery_temperature_celsius</t>
+          <t>soh_percent</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -21086,28 +21011,28 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là battery_temperature, sẽ đổi tên] Nhiệt độ pin (°C).</t>
+          <t>Sức khỏe pin (SOH): dung lượng còn lại so với khi mới, % (F-A3).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>34.5</t>
+          <t>97.8</t>
         </is>
       </c>
       <c r="I21" s="6" t="n"/>
     </row>
-    <row r="22" ht="27" customHeight="1">
+    <row r="22">
       <c r="A22" s="6" t="n">
         <v>16</v>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>soh_percent</t>
+          <t>cycle_count</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>float8</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -21119,28 +21044,28 @@
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Sức khỏe pin (SOH): dung lượng còn lại so với khi mới, % (F-A3).</t>
+          <t>Số chu kỳ sạc-xả tích lũy của pack pin (F-A3).</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>97.8</t>
+          <t>213</t>
         </is>
       </c>
       <c r="I22" s="6" t="n"/>
     </row>
-    <row r="23">
+    <row r="23" ht="27" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>17</v>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>cycle_count</t>
+          <t>motor_temperature_celsius</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>float8</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -21152,23 +21077,23 @@
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Số chu kỳ sạc-xả tích lũy của pack pin (F-A3).</t>
+          <t>Nhiệt độ động cơ (°C).</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24" ht="27" customHeight="1">
+    <row r="24">
       <c r="A24" s="6" t="n">
         <v>18</v>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>motor_temperature_celsius</t>
+          <t>odometer_km</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -21185,28 +21110,28 @@
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là motor_temperature, sẽ đổi tên] Nhiệt độ động cơ (°C).</t>
+          <t>Tổng quãng đường đã chạy (km).</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>48213.7</t>
         </is>
       </c>
       <c r="I24" s="6" t="n"/>
     </row>
-    <row r="25" ht="27" customHeight="1">
+    <row r="25">
       <c r="A25" s="6" t="n">
         <v>19</v>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>odometer_km</t>
+          <t>signal_dbm</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>float8</t>
+          <t>bigint</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -21218,12 +21143,12 @@
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là odometer, sẽ đổi tên] Tổng quãng đường đã chạy (km).</t>
+          <t>Cường độ sóng di động (dBm).</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>48213.7</t>
+          <t>-71</t>
         </is>
       </c>
       <c r="I25" s="6" t="n"/>
@@ -21234,12 +21159,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>signal_dbm</t>
+          <t>error_codes</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
+          <t>jsonb</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -21251,12 +21176,12 @@
       <c r="F26" s="6" t="n"/>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là signal_strength, sẽ đổi tên] Cường độ sóng di động (dBm).</t>
+          <t>Các mã lỗi đang hoạt động, dạng mảng JSON; NULL nếu không có.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>-71</t>
+          <t>["P0A80", "U0100"]</t>
         </is>
       </c>
       <c r="I26" s="6" t="n"/>
@@ -21267,7 +21192,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>error_codes</t>
+          <t>raw_payload</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -21277,35 +21202,35 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E27" s="6" t="n"/>
       <c r="F27" s="6" t="n"/>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Các mã lỗi đang hoạt động, dạng mảng JSON; NULL nếu không có.</t>
+          <t>Bản tin gốc đúng như khi nhận, để gỡ lỗi và xử lý lại.</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>["P0A80", "U0100"]</t>
+          <t>{"serial": "TBX-2409-000123", "soc": 64.2, ...}</t>
         </is>
       </c>
       <c r="I27" s="6" t="n"/>
     </row>
-    <row r="28" ht="27" customHeight="1">
+    <row r="28">
       <c r="A28" s="6" t="n">
         <v>22</v>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>raw_payload</t>
+          <t>schema_version</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>jsonb</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -21317,84 +21242,71 @@
       <c r="F28" s="6" t="n"/>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Bản tin gốc đúng như khi nhận, để gỡ lỗi và xử lý lại.</t>
+          <t>Phiên bản cấu trúc bản tin MQTT mà thiết bị dùng (F-A1).</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>{"serial": "TBX-2409-000123", "soc": 64.2, ...}</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I28" s="6" t="n"/>
     </row>
-    <row r="29">
-      <c r="A29" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>schema_version</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="4" t="n"/>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="27" customHeight="1">
+      <c r="A31" s="6" t="n"/>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>ix_telemetry_vehicle_time</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id, recorded_at DESC</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>không</t>
         </is>
       </c>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>Phiên bản cấu trúc bản tin MQTT mà thiết bị dùng (F-A1).</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="n"/>
-    </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="4" t="n"/>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="27" customHeight="1">
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
+    </row>
+    <row r="32" ht="54" customHeight="1">
       <c r="A32" s="6" t="n"/>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>ix_telemetry_vehicle_time</t>
+          <t>ix_telemetry_vehicle_received</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id, recorded_at DESC</t>
+          <t>vehicle_id, received_at DESC</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -21403,18 +21315,22 @@
         </is>
       </c>
       <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-    </row>
-    <row r="33" ht="54" customHeight="1">
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Lần cuối backend nhận dữ liệu từ xe (giám sát thiết bị F-J1/F-J3); dùng đồng hồ nhận của backend, không bị lệch giờ thiết bị làm sai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="27" customHeight="1">
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>ix_telemetry_vehicle_received</t>
+          <t>ix_telemetry_device_message_id</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>vehicle_id, received_at DESC</t>
+          <t>device_message_id</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -21423,59 +21339,35 @@
         </is>
       </c>
       <c r="E33" s="6" t="n"/>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>Lần cuối backend nhận dữ liệu từ xe (giám sát thiết bị F-J1/F-J3); dùng đồng hồ nhận của backend, không bị lệch giờ thiết bị làm sai.</t>
-        </is>
-      </c>
+      <c r="F33" s="6" t="n"/>
     </row>
     <row r="34" ht="27" customHeight="1">
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>ix_telemetry_device_message_id</t>
+          <t>uq_telemetry_telematic_recorded_at</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>device_message_id</t>
+          <t>telematic_id, recorded_at</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E34" s="6" t="n"/>
       <c r="F34" s="6" t="n"/>
     </row>
-    <row r="35" ht="27" customHeight="1">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>uq_telemetry_telematic_recorded_at</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>telematic_id, recorded_at</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="6" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A6:I29"/>
+  <autoFilter ref="A6:I28"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F9" location="'organizations'!A1"/>
     <hyperlink ref="F11" location="'telematics'!A1"/>
-    <hyperlink ref="F13" location="'vehicles'!A1"/>
+    <hyperlink ref="F12" location="'vehicles'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(charging-stations): build the stations group and the command channel (WP1)
Locations, access grants, station and connector state tables, history,
configuration snapshots and charging_station_commands are built; the OCPP
adapters write device reports to the state tables, and the gateway runs a
command loop that picks up PENDING commands (PR-16, CS-23..CS-27).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01URvQGCMdGQH5axXbsyq4p6
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -138,17 +138,17 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="41" hidden="1">'charging_locations'!$A$7:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="42" hidden="1">'charging_location_history'!$A$7:$I$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="43" hidden="1">'charging_location_access'!$A$6:$I$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="44" hidden="1">'charging_stations'!$A$8:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="44" hidden="1">'charging_stations'!$A$8:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="45" hidden="1">'charging_station_history'!$A$7:$I$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="46" hidden="1">'charging_station_state'!$A$7:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="47" hidden="1">'charging_evses'!$A$7:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="48" hidden="1">'charging_evse_history'!$A$7:$I$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="49" hidden="1">'charging_connectors'!$A$8:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="49" hidden="1">'charging_connectors'!$A$8:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="50" hidden="1">'charging_connector_history'!$A$7:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="51" hidden="1">'charging_connector_state'!$A$7:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="52" hidden="1">'charging_ocpp_messages'!$A$6:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="53" hidden="1">'charging_station_config_capture'!$A$6:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="54" hidden="1">'charging_station_config_entries'!$A$6:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="54" hidden="1">'charging_station_config_entries'!$A$6:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="55" hidden="1">'charging_station_commands'!$A$6:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="56" hidden="1">'charging_sessions'!$A$6:$I$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="57" hidden="1">'charging_session_events'!$A$6:$I$11</definedName>
@@ -2939,7 +2939,7 @@
         </is>
       </c>
       <c r="H58" s="6" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I58" s="7" t="inlineStr">
         <is>
@@ -3164,7 +3164,7 @@
         </is>
       </c>
       <c r="H63" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I63" s="7" t="inlineStr">
         <is>
@@ -3389,7 +3389,7 @@
         </is>
       </c>
       <c r="H68" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I68" s="7" t="inlineStr">
         <is>
@@ -3397,7 +3397,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="135" customHeight="1">
+    <row r="69" ht="148.5" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
           <t>38</t>
@@ -3430,7 +3430,7 @@
       </c>
       <c r="G69" s="6" t="inlineStr">
         <is>
-          <t>Mọi lệnh chúng ta gửi tới trụ sạc và câu trả lời (STN-10, CS-20): ai yêu cầu, vì sao, liên quan phiên sạc nào, và các kết quả không để lại bản tin trong nhật ký thô (chưa gửi, hết thời gian chờ). Gửi lệnh là khả năng của cổng OCPP nên bảng thuộc miền charging_stations, không thuộc charging_sessions. Ghi khi tạo lệnh và cập nhật một lần khi có trả lời; không có lịch sử thay đổi, không xóa mềm. Phần lớn câu trả lời chỉ là chấp nhận hay từ chối; kết quả thật đến sau bằng bản tin riêng. Bảng lệnh cho T-Box (telematic_commands, deferred.md 55) sẽ dùng cùng dạng. Ràng buộc kiểm tra (CS-20): lệnh NOT_SENT không có ocpp_message_id; lệnh đã có kết quả (không PENDING, không NOT_SENT) phải có answered_at.</t>
+          <t>Mọi lệnh chúng ta gửi tới trụ sạc và câu trả lời (STN-10, CS-20): ai yêu cầu, vì sao, liên quan phiên sạc nào, và các kết quả không để lại bản tin trong nhật ký thô (chưa gửi, hết thời gian chờ). Gửi lệnh là khả năng của cổng OCPP nên bảng thuộc miền charging_stations, không thuộc charging_sessions. Ghi khi tạo lệnh và cập nhật một lần khi có trả lời; không có lịch sử thay đổi, không xóa mềm. Bảng cũng là kênh tới cổng OCPP (PR-16, CS-24): dòng xếp hàng chưa có ocpp_message_id sẽ được cổng OCPP đang giữ kết nối của trụ nhận. Phần lớn câu trả lời chỉ là chấp nhận hay từ chối; kết quả thật đến sau bằng bản tin riêng. Bảng lệnh cho T-Box (telematic_commands, deferred.md 55) sẽ dùng cùng dạng. Ràng buộc kiểm tra (CS-20): lệnh NOT_SENT không có ocpp_message_id; lệnh đã có kết quả (không PENDING, không NOT_SENT) phải có answered_at.</t>
         </is>
       </c>
       <c r="H69" s="6" t="n">
@@ -31236,7 +31236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -31537,84 +31537,92 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="27" customHeight="1">
+    <row r="14" ht="54" customHeight="1">
       <c r="A14" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>display_name</t>
+          <t>max_power_kw</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>varchar(200)</t>
+          <t>numeric(6,2)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: CS-09] Tên trạm hiển thị cho tài xế; nay là display_name của trạm, còn trụ có physical_reference.</t>
+          <t>Tổng công suất của trụ (kW), chia cho các súng (trụ 240 kW hai súng cấp khoảng 120 kW mỗi súng khi cả hai cùng sạc); NULL nếu chưa biết. Công suất và chuẩn đầu sạc theo từng súng nằm ở súng sạc (deferred.md 80).</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Trạm sạc G3 Bình Dương</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="n"/>
-    </row>
-    <row r="15" ht="27" customHeight="1">
+          <t>240.00</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="67.5" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>geography(POINT,4326)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: CS-09] Vị trí GPS; nay là charging_locations.coordinates.</t>
+          <t>Do con người đặt (DM-25). ACTIVE: đang phục vụ. INACTIVE: ngừng phục vụ, ví dụ đang sửa chữa; lý do cho biết trường hợp nào. Trụ rời hệ thống được chuyển sang INACTIVE và xóa mềm. Trụ online hay không được tính từ charging_station_state.last_seen_at.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>POINT(106.6519 10.9804)</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="n"/>
-    </row>
-    <row r="16" ht="67.5" customHeight="1">
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>max_power_kw</t>
+          <t>status_reason</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>numeric(6,2)</t>
+          <t>varchar(200)</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -31626,12 +31634,12 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là power_rating_kw, sẽ đổi tên] Tổng công suất của trụ (kW), chia cho các súng (trụ 240 kW hai súng cấp khoảng 120 kW mỗi súng khi cả hai cùng sạc); NULL nếu chưa biết. Công suất và chuẩn đầu sạc theo từng súng nằm ở súng sạc (deferred.md 80).</t>
+          <t>Lý do của trạng thái hiện tại; NULL khi ACTIVE.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>240.00</t>
+          <t>Hỏng mô-đun công suất, chờ linh kiện</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -31646,95 +31654,103 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>connector_standard</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: CS-11] Chuẩn đầu sạc; chuyển sang từng súng sạc.</t>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>CCS2</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="n"/>
-    </row>
-    <row r="18" ht="27" customHeight="1">
+          <t>2026-09-01T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40.5" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>operating_hours</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>varchar(100)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: CS-11] Giờ hoạt động dạng văn bản; trạm luôn mở 24/7.</t>
+          <t>Thời điểm con người sửa bản ghi gần nhất (UTC); báo cáo của thiết bị ghi vào charging_station_state và không làm thay đổi cột này.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>24/7</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="n"/>
-    </row>
-    <row r="19" ht="67.5" customHeight="1">
+          <t>2026-09-10T07:15:00Z</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40.5" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>deleted_at</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Do con người đặt (DM-25). ACTIVE: đang phục vụ. INACTIVE: ngừng phục vụ, ví dụ đang sửa chữa; lý do cho biết trường hợp nào. Trụ rời hệ thống được chuyển sang INACTIVE và xóa mềm. Trụ online hay không được tính từ charging_station_state.last_seen_at.</t>
+          <t>Thời điểm xóa mềm: trụ không còn thuộc hệ thống, do đã tháo đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ, lý do nằm trong status_reason. NULL khi còn thuộc hệ thống.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
@@ -31743,154 +31759,81 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>status_reason</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>varchar(200)</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>Lý do của trạng thái hiện tại; NULL khi ACTIVE.</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>Hỏng mô-đun công suất, chờ linh kiện</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>maintenance_status</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>chargingstationmaintenancestatus</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="27" customHeight="1">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>ix_charging_stations_deleted_at</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>deleted_at</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>không</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] Trạng thái bảo trì; thay bằng status ACTIVE / INACTIVE kèm lý do.</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>OPERATIONAL</t>
-        </is>
-      </c>
-      <c r="I21" s="6" t="n"/>
-    </row>
-    <row r="22" ht="27" customHeight="1">
-      <c r="A22" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>ocpp_protocol_version</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>varchar(20)</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
         </is>
       </c>
       <c r="E22" s="6" t="n"/>
       <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] Phiên bản OCPP của kết nối gần nhất; chuyển sang charging_station_state.</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>ocpp1.6</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="n"/>
     </row>
     <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="6" t="n">
-        <v>15</v>
-      </c>
+      <c r="A23" s="6" t="n"/>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>vendor</t>
+          <t>ix_charging_stations_location_id</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>varchar(100)</t>
+          <t>location_id</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] Hãng trụ sạc; chuyển sang charging_station_state.</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>Willdigits</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="n"/>
-    </row>
-    <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="6" t="n">
-        <v>16</v>
-      </c>
+    </row>
+    <row r="24" ht="40.5" customHeight="1">
+      <c r="A24" s="6" t="n"/>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>uq_charging_stations_live_registered_serial_number</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>varchar(100)</t>
+          <t>registered_serial_number</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -31899,684 +31842,131 @@
         </is>
       </c>
       <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="n"/>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] Model trụ sạc; chuyển sang charging_station_state.</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>WD-DC480</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="n"/>
-    </row>
-    <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>serial_number</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>varchar(100)</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] Số serial; chuyển sang charging_station_state.</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>WD2409001234</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="n"/>
-    </row>
-    <row r="26" ht="27" customHeight="1">
-      <c r="A26" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>firmware_version</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>varchar(100)</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] Firmware; chuyển sang charging_station_state.</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>V2.3.7</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="n"/>
-    </row>
-    <row r="27" ht="27" customHeight="1">
-      <c r="A27" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>last_boot_at</t>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>WHERE deleted_at IS NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="4" t="n"/>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>warranties</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] BootNotification gần nhất; chuyển sang charging_station_state.</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-14T22:00:05Z</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="n"/>
-    </row>
-    <row r="28" ht="27" customHeight="1">
-      <c r="A28" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>last_seen_at</t>
+          <t>station_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>charging_station_state</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] Bản tin gần nhất; chuyển sang charging_station_state.</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-15T08:29:58Z</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="n"/>
-    </row>
-    <row r="29" ht="27" customHeight="1">
-      <c r="A29" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>charger_status</t>
+          <t>station_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>charging_evses</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>chargingconnectorstatus</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] Trạng thái cả trụ (connector 0); chuyển sang charging_station_state.</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="n"/>
-    </row>
-    <row r="30" ht="27" customHeight="1">
-      <c r="A30" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>charger_status_updated_at</t>
+          <t>station_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n"/>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>charging_ocpp_messages</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] Thời điểm báo trạng thái đó; chuyển sang charging_station_state.</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-15T08:10:00Z</t>
-        </is>
-      </c>
-      <c r="I30" s="6" t="n"/>
+          <t>station_id</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="27" customHeight="1">
-      <c r="A31" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>charger_error_code</t>
+      <c r="A31" s="6" t="n"/>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>charging_station_commands</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] Mã lỗi của cả trụ; chuyển sang charging_station_state.</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>NoError</t>
-        </is>
-      </c>
-      <c r="I31" s="6" t="n"/>
-    </row>
-    <row r="32" ht="27" customHeight="1">
-      <c r="A32" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>charger_vendor_error_code</t>
+          <t>station_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n"/>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>charging_sessions</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>varchar(100)</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-11] Mã lỗi riêng của hãng cho cả trụ; chuyển sang charging_station_state.</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>E0000</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="n"/>
+          <t>station_id</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>created_at</t>
+      <c r="A33" s="6" t="n"/>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>charging_station_history</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-01T02:00:00Z</t>
-        </is>
-      </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="40.5" customHeight="1">
-      <c r="A34" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm con người sửa bản ghi gần nhất (UTC); báo cáo của thiết bị ghi vào charging_station_state và không làm thay đổi cột này.</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-10T07:15:00Z</t>
-        </is>
-      </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="40.5" customHeight="1">
-      <c r="A35" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>deleted_at</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="6" t="n"/>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm xóa mềm: trụ không còn thuộc hệ thống, do đã tháo đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ, lý do nằm trong status_reason. NULL khi còn thuộc hệ thống.</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="36"/>
-    <row r="37">
-      <c r="A37" s="4" t="n"/>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Kiểu enum</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Giá trị cho phép</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="40.5" customHeight="1">
-      <c r="A38" s="6" t="n"/>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>chargingstationmaintenancestatus</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>OPERATIONAL, UNDER_MAINTENANCE, OUT_OF_SERVICE</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="81" customHeight="1">
-      <c r="A39" s="6" t="n"/>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>chargingconnectorstatus</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>Available, Occupied, Reserved, Unavailable, Faulted, Preparing, Charging, SuspendedEV, SuspendedEVSE, Finishing</t>
-        </is>
-      </c>
-    </row>
-    <row r="40"/>
-    <row r="41">
-      <c r="A41" s="4" t="n"/>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="27" customHeight="1">
-      <c r="A42" s="6" t="n"/>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>ix_charging_stations_location</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="n"/>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>GIST; replaced by ix_charging_locations_coordinates (CS-09)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="27" customHeight="1">
-      <c r="A43" s="6" t="n"/>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>ix_charging_stations_deleted_at</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>deleted_at</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="n"/>
-      <c r="F43" s="6" t="n"/>
-    </row>
-    <row r="44" ht="27" customHeight="1">
-      <c r="A44" s="6" t="n"/>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>ix_charging_stations_location_id</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="inlineStr">
-        <is>
-          <t>location_id</t>
-        </is>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="n"/>
-      <c r="F44" s="6" t="inlineStr">
-        <is>
-          <t>Planned (CS-09)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="40.5" customHeight="1">
-      <c r="A45" s="6" t="n"/>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>uq_charging_stations_live_registered_serial_number</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="inlineStr">
-        <is>
-          <t>registered_serial_number</t>
-        </is>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="n"/>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>Planned (CS-14): WHERE deleted_at IS NULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="46"/>
-    <row r="47">
-      <c r="A47" s="4" t="n"/>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="n"/>
-      <c r="B48" s="7" t="inlineStr">
-        <is>
-          <t>warranties</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="inlineStr">
-        <is>
           <t>station_id</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="6" t="n"/>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>charging_station_state</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>station_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="n"/>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>charging_evses</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>station_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="6" t="n"/>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>charging_ocpp_messages</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>station_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="27" customHeight="1">
-      <c r="A52" s="6" t="n"/>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>charging_station_configuration_entries</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>station_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="27" customHeight="1">
-      <c r="A53" s="6" t="n"/>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>charging_station_commands</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>station_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="n"/>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>charging_sessions</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>station_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="6" t="n"/>
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>charging_station_history</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>station_id</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A8:I35"/>
+  <autoFilter ref="A8:I19"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'charging_station_history'!A1"/>
     <hyperlink ref="A6" location="'charging_station_state'!A1"/>
     <hyperlink ref="F10" location="'charging_locations'!A1"/>
-    <hyperlink ref="B48" location="'warranties'!A1"/>
-    <hyperlink ref="B49" location="'charging_station_state'!A1"/>
-    <hyperlink ref="B50" location="'charging_evses'!A1"/>
-    <hyperlink ref="B51" location="'charging_ocpp_messages'!A1"/>
-    <hyperlink ref="B52" location="'charging_station_config_entries'!A1"/>
-    <hyperlink ref="B53" location="'charging_station_commands'!A1"/>
-    <hyperlink ref="B54" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B55" location="'charging_station_history'!A1"/>
+    <hyperlink ref="B27" location="'warranties'!A1"/>
+    <hyperlink ref="B28" location="'charging_station_state'!A1"/>
+    <hyperlink ref="B29" location="'charging_evses'!A1"/>
+    <hyperlink ref="B30" location="'charging_ocpp_messages'!A1"/>
+    <hyperlink ref="B31" location="'charging_station_commands'!A1"/>
+    <hyperlink ref="B32" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B33" location="'charging_station_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -34304,7 +33694,7 @@
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Planned (CS-16): WHERE deleted_at IS NULL</t>
+          <t>WHERE deleted_at IS NULL</t>
         </is>
       </c>
     </row>
@@ -35646,7 +35036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -36017,38 +35407,42 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="27" customHeight="1">
+    <row r="16">
       <c r="A16" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>chargingconnectorstatus</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: CS-17] Trạng thái trực tiếp; chuyển sang charging_connector_state.</t>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Charging</t>
-        </is>
-      </c>
-      <c r="I16" s="6" t="n"/>
+          <t>2026-09-01T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="27" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -36056,7 +35450,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>status_updated_at</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -36066,35 +35460,39 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: CS-17] Thời điểm báo trạng thái; chuyển sang charging_connector_state.</t>
+          <t>Thời điểm con người sửa bản ghi gần nhất (UTC); báo cáo trạng thái ghi vào charging_connector_state.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-15T08:31:00Z</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="n"/>
-    </row>
-    <row r="18" ht="27" customHeight="1">
+          <t>2026-09-10T07:15:00Z</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>error_code</t>
+          <t>deleted_at</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -36106,94 +35504,55 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: CS-17] Mã lỗi theo báo cáo gần nhất; chuyển sang charging_connector_state.</t>
+          <t>Thời điểm xóa mềm: súng không còn thuộc hệ thống, do đã tháo đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ. NULL khi còn thuộc hệ thống. Súng ngừng phục vụ qua trạng thái của EVSE.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>NoError</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="n"/>
-    </row>
-    <row r="19" ht="27" customHeight="1">
-      <c r="A19" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>vendor_error_code</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>varchar(100)</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-17] Mã lỗi riêng của hãng; chuyển sang charging_connector_state.</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>E0000</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="n"/>
-    </row>
-    <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>status_info</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>varchar(50)</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-17] Thông tin văn bản tự do; chuyển sang charging_connector_state.</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>Cable locked</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="n">
-        <v>13</v>
-      </c>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>🔍</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="27" customHeight="1">
+      <c r="A21" s="6" t="n"/>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>ix_charging_connectors_evse_deleted</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>evse_id, deleted_at</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -36203,251 +35562,90 @@
       </c>
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-01T02:00:00Z</t>
-        </is>
-      </c>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
     </row>
     <row r="22" ht="27" customHeight="1">
-      <c r="A22" s="6" t="n">
-        <v>14</v>
-      </c>
+      <c r="A22" s="6" t="n"/>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>uq_charging_connectors_evse_ocpp_id</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>evse_id, ocpp_connector_id</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E22" s="6" t="n"/>
       <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm con người sửa bản ghi gần nhất (UTC); báo cáo trạng thái ghi vào charging_connector_state.</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-10T07:15:00Z</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="54" customHeight="1">
-      <c r="A23" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>deleted_at</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm xóa mềm: súng không còn thuộc hệ thống, do đã tháo đi hoặc nhập nhầm (DM-25); mọi dữ liệu vẫn được giữ. NULL khi còn thuộc hệ thống. Súng ngừng phục vụ qua trạng thái của EVSE.</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>🔍</t>
-        </is>
-      </c>
-    </row>
-    <row r="24"/>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="4" t="n"/>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
-      <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Kiểu enum</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Giá trị cho phép</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="81" customHeight="1">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>charging_connector_state</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>connector_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
       <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>chargingconnectorstatus</t>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>charging_sessions</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Available, Occupied, Reserved, Unavailable, Faulted, Preparing, Charging, SuspendedEV, SuspendedEVSE, Finishing</t>
-        </is>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="4" t="n"/>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="27" customHeight="1">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>ix_charging_connectors_evse_deleted</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>evse_id, deleted_at</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="6" t="n"/>
-    </row>
-    <row r="30" ht="27" customHeight="1">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>uq_charging_connectors_evse_ocpp_id</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>evse_id, ocpp_connector_id</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-    </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" s="4" t="n"/>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>charging_connector_state</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
           <t>connector_id</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="n"/>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>charging_sessions</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
+    <row r="27" ht="27" customHeight="1">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>charging_connector_history</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>connector_id</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="27" customHeight="1">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>charging_connector_history</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>connector_id</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A8:I23"/>
+  <autoFilter ref="A8:I18"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="A5" location="'charging_connector_history'!A1"/>
     <hyperlink ref="A6" location="'charging_connector_state'!A1"/>
     <hyperlink ref="F10" location="'charging_evses'!A1"/>
-    <hyperlink ref="B33" location="'charging_connector_state'!A1"/>
-    <hyperlink ref="B34" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B35" location="'charging_connector_history'!A1"/>
+    <hyperlink ref="B25" location="'charging_connector_state'!A1"/>
+    <hyperlink ref="B26" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B27" location="'charging_connector_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -37883,7 +37081,7 @@
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Planned (CS-18): the message viewer filtering by type (STN-15)</t>
+          <t>the message viewer filtering by type (STN-15)</t>
         </is>
       </c>
     </row>
@@ -37907,7 +37105,7 @@
       <c r="E22" s="6" t="n"/>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Planned (CS-18): pairing a request with its answer</t>
+          <t>pairing a request with its answer</t>
         </is>
       </c>
     </row>
@@ -37927,7 +37125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -38309,11 +37507,39 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="27" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>charging_station_configuration_entries</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>capture_id</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A6:I13"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F8" location="'charging_station_commands'!A1"/>
+    <hyperlink ref="B19" location="'charging_station_config_entries'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -38325,7 +37551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -38458,7 +37684,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>station_id</t>
+          <t>capture_id</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -38478,50 +37704,50 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>charging_stations.station_id (khi xóa: chặn xóa)</t>
+          <t>charging_station_configuration_captures.capture_id (khi xóa: chặn xóa)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: CS-19] Trụ sạc; nay đọc qua lệnh của lần chụp (CS-21).</t>
+          <t>Lần chụp chứa giá trị này.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>4b9d6f3a-2e8c-4a1b-9d5e-7f0c3a8b2d88</t>
+          <t>00000008-5a6b-4c7d-8e9f-0a1b2c3d4e5f</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>capture_id</t>
+          <t>component_name</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Lần chụp chứa giá trị này.</t>
+          <t>Thành phần OCPP 2.0.1, ví dụ OCPPCommCtrlr, EVSE, Connector; NULL với 1.6J (chỉ có khóa).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>00000008-5a6b-4c7d-8e9f-0a1b2c3d4e5f</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I9" s="6" t="n"/>
@@ -38532,45 +37758,45 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>captured_at</t>
+          <t>component_instance</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>[Sẽ bỏ: CS-19] Thời điểm nhận câu trả lời; nay nằm ở lần chụp.</t>
+          <t>Bản thể của thành phần khi có nhiều (2.0.1); NULL nếu không.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>2026-09-14T22:00:10Z</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I10" s="6" t="n"/>
     </row>
-    <row r="11" ht="27" customHeight="1">
+    <row r="11">
       <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>component_name</t>
+          <t>ocpp_evse_id</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -38582,7 +37808,7 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Thành phần OCPP 2.0.1, ví dụ OCPPCommCtrlr, EVSE, Connector; NULL với 1.6J (chỉ có khóa).</t>
+          <t>EVSE chứa thành phần (2.0.1); NULL với cả trụ và với 1.6J.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -38592,18 +37818,18 @@
       </c>
       <c r="I11" s="6" t="n"/>
     </row>
-    <row r="12" ht="27" customHeight="1">
+    <row r="12">
       <c r="A12" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>component_instance</t>
+          <t>ocpp_connector_id</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -38615,7 +37841,7 @@
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Bản thể của thành phần khi có nhiều (2.0.1); NULL nếu không.</t>
+          <t>Súng chứa thành phần (2.0.1); NULL nếu không.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -38625,35 +37851,35 @@
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>ocpp_evse_id</t>
+          <t>variable_name</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>varchar(100)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>EVSE chứa thành phần (2.0.1); NULL với cả trụ và với 1.6J.</t>
+          <t>Cấu hình: khóa cấu hình của 1.6J (ví dụ HeartbeatInterval) hoặc biến của 2.0.1 trong thành phần của nó.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HeartbeatInterval</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
@@ -38664,12 +37890,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>ocpp_connector_id</t>
+          <t>variable_instance</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -38681,7 +37907,7 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Súng chứa thành phần (2.0.1); NULL nếu không.</t>
+          <t>Bản thể của biến (2.0.1); NULL nếu không.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -38691,18 +37917,18 @@
       </c>
       <c r="I14" s="6" t="n"/>
     </row>
-    <row r="15" ht="40.5" customHeight="1">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>variable_name</t>
+          <t>attribute_type</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>varchar(100)</t>
+          <t>varchar(10)</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -38714,28 +37940,28 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>[Hiện tên là config_key, sẽ đổi tên] Cấu hình: khóa cấu hình của 1.6J (ví dụ HeartbeatInterval) hoặc biến của 2.0.1 trong thành phần của nó.</t>
+          <t>Giá trị nào của cấu hình: Actual (giá trị hiện tại; luôn là Actual với 1.6J), Target, MinSet hoặc MaxSet (2.0.1).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>HeartbeatInterval</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="27" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>variable_instance</t>
+          <t>value</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -38747,23 +37973,23 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Bản thể của biến (2.0.1); NULL nếu không.</t>
+          <t>Giá trị dạng chuỗi, đúng như trụ gửi; NULL nếu trụ không gửi (ví dụ cấu hình chỉ-ghi).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>60</t>
         </is>
       </c>
       <c r="I16" s="6" t="n"/>
     </row>
-    <row r="17" ht="27" customHeight="1">
+    <row r="17" ht="54" customHeight="1">
       <c r="A17" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>attribute_type</t>
+          <t>mutability</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -38780,193 +38006,70 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Giá trị nào của cấu hình: Actual (giá trị hiện tại; luôn là Actual với 1.6J), Target, MinSet hoặc MaxSet (2.0.1).</t>
+          <t>Cấu hình có đổi được không: READ_ONLY (lệnh đổi bị từ chối, ví dụ NumberOfConnectors), READ_WRITE, WRITE_ONLY (2.0.1, ví dụ mật khẩu: không hiện giá trị). Với 1.6J readonly=true là READ_ONLY, false là READ_WRITE.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Actual</t>
+          <t>READ_WRITE</t>
         </is>
       </c>
       <c r="I17" s="6" t="n"/>
     </row>
-    <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="94.5" customHeight="1">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>uq_charging_config_entries_capture_setting</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>capture_id, component_name, component_instance, ocpp_evse_id, ocpp_connector_id, variable_name, variable_instance, attribute_type</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>có</t>
         </is>
       </c>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>Giá trị dạng chuỗi, đúng như trụ gửi; NULL nếu trụ không gửi (ví dụ cấu hình chỉ-ghi).</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="n"/>
-    </row>
-    <row r="19" ht="54" customHeight="1">
-      <c r="A19" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>mutability</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>varchar(10)</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>Cấu hình có đổi được không: READ_ONLY (lệnh đổi bị từ chối, ví dụ NumberOfConnectors), READ_WRITE, WRITE_ONLY (2.0.1, ví dụ mật khẩu: không hiện giá trị). Với 1.6J readonly=true là READ_ONLY, false là READ_WRITE.</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>READ_WRITE</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="n"/>
-    </row>
-    <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>is_readonly</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>boolean</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
       <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>[Sẽ bỏ: CS-19] Trụ có báo khóa này là chỉ-đọc không; thay bằng mutability, bao cả 2.0.1.</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="n"/>
-    </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>ix_charging_config_entries_station_captured</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>station_id, captured_at</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>Replaced by ix_charging_config_captures_station_captured (CS-19)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="94.5" customHeight="1">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>uq_charging_config_entries_capture_setting</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>capture_id, component_name, component_instance, ocpp_evse_id, ocpp_connector_id, variable_name, variable_instance, attribute_type</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Planned (CS-19): NULLS NOT DISTINCT; one value per setting and attribute in a snapshot</t>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>NULLS NOT DISTINCT; one value per setting and attribute in a snapshot</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I20"/>
+  <autoFilter ref="A6:I17"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F8" location="'charging_stations'!A1"/>
+    <hyperlink ref="F8" location="'charging_station_config_capture'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -39016,7 +38119,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Mọi lệnh chúng ta gửi tới trụ sạc và câu trả lời (STN-10, CS-20): ai yêu cầu, vì sao, liên quan phiên sạc nào, và các kết quả không để lại bản tin trong nhật ký thô (chưa gửi, hết thời gian chờ). Gửi lệnh là khả năng của cổng OCPP nên bảng thuộc miền charging_stations, không thuộc charging_sessions. Ghi khi tạo lệnh và cập nhật một lần khi có trả lời; không có lịch sử thay đổi, không xóa mềm. Phần lớn câu trả lời chỉ là chấp nhận hay từ chối; kết quả thật đến sau bằng bản tin riêng. Bảng lệnh cho T-Box (telematic_commands, deferred.md 55) sẽ dùng cùng dạng. Ràng buộc kiểm tra (CS-20): lệnh NOT_SENT không có ocpp_message_id; lệnh đã có kết quả (không PENDING, không NOT_SENT) phải có answered_at.</t>
+          <t>Mọi lệnh chúng ta gửi tới trụ sạc và câu trả lời (STN-10, CS-20): ai yêu cầu, vì sao, liên quan phiên sạc nào, và các kết quả không để lại bản tin trong nhật ký thô (chưa gửi, hết thời gian chờ). Gửi lệnh là khả năng của cổng OCPP nên bảng thuộc miền charging_stations, không thuộc charging_sessions. Ghi khi tạo lệnh và cập nhật một lần khi có trả lời; không có lịch sử thay đổi, không xóa mềm. Bảng cũng là kênh tới cổng OCPP (PR-16, CS-24): dòng xếp hàng chưa có ocpp_message_id sẽ được cổng OCPP đang giữ kết nối của trụ nhận. Phần lớn câu trả lời chỉ là chấp nhận hay từ chối; kết quả thật đến sau bằng bản tin riêng. Bảng lệnh cho T-Box (telematic_commands, deferred.md 55) sẽ dùng cùng dạng. Ràng buộc kiểm tra (CS-20): lệnh NOT_SENT không có ocpp_message_id; lệnh đã có kết quả (không PENDING, không NOT_SENT) phải có answered_at.</t>
         </is>
       </c>
     </row>
@@ -39424,7 +38527,7 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Mã bản tin của khung đã gửi; dùng để tìm khung đó và câu trả lời của trụ trong charging_ocpp_messages (CS-18). NULL khi chưa gửi gì.</t>
+          <t>Mã bản tin của khung đã gửi; dùng để tìm khung đó và câu trả lời của trụ trong charging_ocpp_messages (CS-18). NULL khi lệnh còn xếp hàng hoặc chưa gửi gì.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -39434,7 +38537,7 @@
       </c>
       <c r="I16" s="6" t="n"/>
     </row>
-    <row r="17" ht="81" customHeight="1">
+    <row r="17" ht="94.5" customHeight="1">
       <c r="A17" s="6" t="n">
         <v>11</v>
       </c>
@@ -39457,7 +38560,7 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Kết quả quan sát được, cùng một dạng (không có cột lý do vì là quan sát, không phải quyết định). PENDING: đã gửi, đang chờ trả lời. ACCEPTED / REJECTED: trụ chấp nhận hoặc từ chối. ERROR: trụ trả lời bằng lỗi OCPP. TIMEOUT: không có trả lời trong thời gian cấu hình. NOT_SENT: trụ không kết nối.</t>
+          <t>Kết quả quan sát được, cùng một dạng (không có cột lý do vì là quan sát, không phải quyết định). PENDING: đã xếp hàng chờ cổng OCPP (chưa có ocpp_message_id) hoặc đã gửi và đang chờ trả lời (CS-24). ACCEPTED / REJECTED: trụ chấp nhận hoặc từ chối. ERROR: trụ trả lời bằng lỗi OCPP. TIMEOUT: không có trả lời trong thời gian cấu hình. NOT_SENT: trụ không kết nối.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">

</xml_diff>

<commit_message>
feat(notifications): add recipient routing, channel settings, delivery and inbox (WP10)
Table-driven recipient routing per notification type, organization push
and e-mail switches with history, push/e-mail delivery behind logging
fake providers, seen/read inbox state, and the TRIP_ASSIGNED alert
(NT-15..NT-17, deferred.md 100).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01URvQGCMdGQH5axXbsyq4p6
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -40409,7 +40409,7 @@
       </c>
       <c r="I8" s="6" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
@@ -40432,7 +40432,7 @@
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Loại sự kiện đã phát sinh thông báo.</t>
+          <t>Loại sự kiện đã phát sinh thông báo (TRIP_ASSIGNED, NT-15: quản lý đã lên chuyến cho tài xế).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -40728,7 +40728,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="148.5" customHeight="1">
+    <row r="20" ht="162" customHeight="1">
       <c r="A20" s="6" t="n"/>
       <c r="B20" s="6" t="inlineStr">
         <is>
@@ -40737,7 +40737,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>BATTERY_ALERT, ANOMALY_ALERT, SOH_ALERT, DEVICE_OFFLINE_ALERT, SOS_ALERT, GEOFENCE_ALERT, NO_DRIVER_CHECK_IN_ALERT, OUTSIDE_DRIVER_CHECK_IN, NO_TRIP_STARTED, LOW_WALLET_BALANCE, TOP_UP_RECEIVED, CHARGING_RECEIPT</t>
+          <t>BATTERY_ALERT, ANOMALY_ALERT, SOH_ALERT, DEVICE_OFFLINE_ALERT, SOS_ALERT, GEOFENCE_ALERT, NO_DRIVER_CHECK_IN_ALERT, OUTSIDE_DRIVER_CHECK_IN, NO_TRIP_STARTED, TRIP_ASSIGNED, LOW_WALLET_BALANCE, TOP_UP_RECEIVED, CHARGING_RECEIPT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ocpp): outlet-only meter totals, safe multipliers, station fixed at handshake, claimed_at command timeout, command validation (RV-BL5, RV-CS4, RV-CS5, RV-CS6, RV-CS8, RV-CS9, RV-CS10, RV-CS11, RV-CS12)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01URvQGCMdGQH5axXbsyq4p6
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -148,7 +148,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="52" hidden="1">'charging_ocpp_messages'!$A$6:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="53" hidden="1">'charging_station_config_capture'!$A$6:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="54" hidden="1">'charging_station_config_entries'!$A$6:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="55" hidden="1">'charging_station_commands'!$A$6:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="55" hidden="1">'charging_station_commands'!$A$6:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="56" hidden="1">'charging_sessions'!$A$6:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="57" hidden="1">'charging_session_measurements'!$A$6:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="58" hidden="1">'notifications'!$A$6:$I$17</definedName>
@@ -3432,7 +3432,7 @@
         </is>
       </c>
       <c r="H69" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I69" s="7" t="inlineStr">
         <is>
@@ -38030,7 +38030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -38486,84 +38486,84 @@
       </c>
       <c r="I16" s="6" t="n"/>
     </row>
-    <row r="17" ht="94.5" customHeight="1">
+    <row r="17" ht="81" customHeight="1">
       <c r="A17" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>outcome</t>
+          <t>claimed_at</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Kết quả quan sát được, cùng một dạng (không có cột lý do vì là quan sát, không phải quyết định). PENDING: đã xếp hàng chờ cổng OCPP (chưa có ocpp_message_id) hoặc đã gửi và đang chờ trả lời (CS-24). ACCEPTED / REJECTED: trụ chấp nhận hoặc từ chối. ERROR: trụ trả lời bằng lỗi OCPP. TIMEOUT: không có trả lời trong thời gian cấu hình. NOT_SENT: trụ không kết nối.</t>
+          <t>Thời điểm cổng OCPP nhận lệnh và chuẩn bị gửi, theo đồng hồ máy chủ của chúng ta (RV-CS6); NULL khi lệnh còn trong hàng đợi và với lệnh không gửi gì. Thời gian chờ câu trả lời tính từ đây, không tính từ requested_at, nên lệnh phải chờ đường truyền rảnh không bị đóng là hết thời gian trước khi được gửi.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>ACCEPTED</t>
+          <t>2026-09-15T08:29:11Z</t>
         </is>
       </c>
       <c r="I17" s="6" t="n"/>
     </row>
-    <row r="18" ht="54" customHeight="1">
+    <row r="18" ht="94.5" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>12</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>response_status</t>
+          <t>outcome</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>varchar(30)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Câu trả lời của trụ, đúng như gửi, có thể chi tiết hơn chấp nhận hay từ chối: Scheduled, RebootRequired, UnlockFailed, NotSupported, hoặc một mã lỗi như NotImplemented. NULL khi không có trả lời.</t>
+          <t>Kết quả quan sát được, cùng một dạng (không có cột lý do vì là quan sát, không phải quyết định). PENDING: đã xếp hàng chờ cổng OCPP (chưa có ocpp_message_id) hoặc đã gửi và đang chờ trả lời (CS-24). ACCEPTED / REJECTED: trụ chấp nhận hoặc từ chối. ERROR: trụ trả lời bằng lỗi OCPP. TIMEOUT: không có trả lời trong thời gian cấu hình. NOT_SENT: trụ không kết nối.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Accepted</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="I18" s="6" t="n"/>
     </row>
-    <row r="19" ht="27" customHeight="1">
+    <row r="19" ht="54" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>answered_at</t>
+          <t>response_status</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>varchar(30)</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -38575,62 +38575,71 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
+          <t>Câu trả lời của trụ, đúng như gửi, có thể chi tiết hơn chấp nhận hay từ chối: Scheduled, RebootRequired, UnlockFailed, NotSupported, hoặc một mã lỗi như NotImplemented. NULL khi không có trả lời.</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="27" customHeight="1">
+      <c r="A20" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>answered_at</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
           <t>Thời điểm ghi nhận câu trả lời hoặc hết thời gian chờ; NULL khi PENDING hoặc NOT_SENT.</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>2026-09-15T08:29:12Z</t>
         </is>
       </c>
-      <c r="I19" s="6" t="n"/>
-    </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="I20" s="6" t="n"/>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="27" customHeight="1">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>ix_charging_station_commands_station_requested</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>station_id, requested_at</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>A charger's commands, newest first (STN-10)</t>
         </is>
       </c>
     </row>
@@ -38638,12 +38647,12 @@
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>ix_charging_station_commands_session_id</t>
+          <t>ix_charging_station_commands_station_requested</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>session_id</t>
+          <t>station_id, requested_at</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -38654,46 +38663,70 @@
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="inlineStr">
         <is>
+          <t>A charger's commands, newest first (STN-10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="27" customHeight="1">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>ix_charging_station_commands_session_id</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>session_id</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
           <t>A session's remote start and stop</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="inlineStr">
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="4" t="n"/>
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Được tham chiếu bởi bảng</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Cột</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="27" customHeight="1">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="7" t="inlineStr">
+    <row r="27" ht="27" customHeight="1">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>charging_station_configuration_captures</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>command_id</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I19"/>
+  <autoFilter ref="A6:I20"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F8" location="'charging_stations'!A1"/>
     <hyperlink ref="F9" location="'charging_evses'!A1"/>
     <hyperlink ref="F10" location="'charging_sessions'!A1"/>
     <hyperlink ref="F13" location="'users'!A1"/>
-    <hyperlink ref="B26" location="'charging_station_config_capture'!A1"/>
+    <hyperlink ref="B27" location="'charging_station_config_capture'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(identity): invitation limits and masking, sign-up on invited numbers, phone normalization, password-guarded phone change, shared Reason type, membership-end hooks on lock, session lifetime (RV-ID2, RV-ID3, RV-ID5, RV-ID6, RV-ID8, RV-AS8, RV-ID9, RV-ID10, RV-ID11, RV-ID12)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01URvQGCMdGQH5axXbsyq4p6
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -103,7 +103,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'membership_history'!$A$7:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'user_credentials'!$A$6:$I$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'user_sessions'!$A$6:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'one_time_codes'!$A$6:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'one_time_codes'!$A$6:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'user_consents'!$A$6:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'legal_documents'!$A$6:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'user_role_assignments'!$A$6:$I$14</definedName>
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="H16" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
@@ -5986,7 +5986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6113,7 +6113,7 @@
       </c>
       <c r="I7" s="6" t="n"/>
     </row>
-    <row r="8" ht="67.5" customHeight="1">
+    <row r="8" ht="94.5" customHeight="1">
       <c r="A8" s="6" t="n">
         <v>2</v>
       </c>
@@ -6136,7 +6136,7 @@
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Mã dùng cho việc gì. INVITE: người được mời đặt mật khẩu. SIGN_UP: khách vãng lai xác minh số điện thoại trước khi tạo tài khoản. PASSWORD_RESET: quên mật khẩu. PHONE_CHANGE: xác minh số điện thoại mới. Giá trị: INVITE | SIGN_UP | PASSWORD_RESET | PHONE_CHANGE.</t>
+          <t>Mã dùng cho việc gì. INVITE: người được mời đặt mật khẩu. SIGN_UP: khách vãng lai xác minh số điện thoại trước khi tạo tài khoản. PASSWORD_RESET: quên mật khẩu. PHONE_CHANGE: xác minh số điện thoại mới. Giá trị: INVITE | INVITE_NOTICE | SIGN_UP | PASSWORD_RESET | PHONE_CHANGE. INVITE_NOTICE ghi lại tin nhắn thông báo gửi tới tài khoản đã có (không gửi mã; dòng này chỉ phục vụ giới hạn gửi).</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -6294,35 +6294,43 @@
       </c>
       <c r="I12" s="6" t="n"/>
     </row>
-    <row r="13" ht="27" customHeight="1">
+    <row r="13" ht="40.5" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>organization_id</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>organizations.organization_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm gửi mã; dùng cho thời gian chờ gửi lại và giới hạn theo số điện thoại.</t>
+          <t>Tổ chức mà lời mời thuộc về (INVITE và INVITE_NOTICE); NULL với các mục đích khác. Chấp nhận lời mời bằng mã chỉ kích hoạt tư cách thành viên trong tổ chức này.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>2026-09-01T02:00:00Z</t>
+          <t>00000010-5a6b-4c7d-8e9f-0a1b2c3d4e5f</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
@@ -6333,7 +6341,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>expires_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -6350,28 +6358,28 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm mã hết hiệu lực (ví dụ 10 phút với OTP, 72 giờ với đường dẫn mời).</t>
+          <t>Thời điểm gửi mã; dùng cho thời gian chờ gửi lại và giới hạn theo số điện thoại.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-04T02:00:00Z</t>
+          <t>2026-09-01T02:00:00Z</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
     </row>
-    <row r="15" ht="40.5" customHeight="1">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>failed_attempt_count</t>
+          <t>expires_at</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -6383,104 +6391,138 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Số lần nhập sai đối với mã này; bắt đầu từ 0. Tới 5 lần thì mã hết hiệu lực và người dùng phải xin mã mới (lại tính vào giới hạn gửi), nên không thể dò ra mã 6 chữ số.</t>
+          <t>Thời điểm mã hết hiệu lực (ví dụ 10 phút với OTP, 72 giờ với đường dẫn mời).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2026-09-04T02:00:00Z</t>
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
     </row>
-    <row r="16" ht="27" customHeight="1">
+    <row r="16" ht="40.5" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>used_at</t>
+          <t>failed_attempt_count</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
+          <t>Số lần nhập sai đối với mã này; bắt đầu từ 0. Tới 5 lần thì mã hết hiệu lực và người dùng phải xin mã mới (lại tính vào giới hạn gửi), nên không thể dò ra mã 6 chữ số.</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="17" ht="27" customHeight="1">
+      <c r="A17" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>used_at</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
           <t>Thời điểm mã được dùng; NULL khi chưa dùng. Mỗi mã chỉ dùng được một lần.</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>NULL</t>
         </is>
       </c>
-      <c r="I16" s="6" t="n"/>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="I17" s="6" t="n"/>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Chỉ mục (index)</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Các cột</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Duy nhất</t>
         </is>
       </c>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="27" customHeight="1">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="inlineStr">
+    <row r="20" ht="27" customHeight="1">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>ix_one_time_codes_phone_time</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>phone_number, created_at</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>không</t>
         </is>
       </c>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Resend cooldown and per-phone rate limit</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:I16"/>
+  <autoFilter ref="A6:I17"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F9" location="'users'!A1"/>
     <hyperlink ref="F12" location="'users'!A1"/>
+    <hyperlink ref="F13" location="'organizations'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10783,7 +10825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11475,7 +11517,7 @@
       <c r="A29" s="6" t="n"/>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>user_consents</t>
+          <t>one_time_codes</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -11488,7 +11530,7 @@
       <c r="A30" s="6" t="n"/>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>user_role_assignments</t>
+          <t>user_consents</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -11501,7 +11543,7 @@
       <c r="A31" s="6" t="n"/>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>access_audit_logs</t>
+          <t>user_role_assignments</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -11514,7 +11556,7 @@
       <c r="A32" s="6" t="n"/>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>organization_settings</t>
+          <t>access_audit_logs</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -11527,7 +11569,7 @@
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>vehicles</t>
+          <t>organization_settings</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -11540,7 +11582,7 @@
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>batteries</t>
+          <t>vehicles</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -11553,7 +11595,7 @@
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>telematics</t>
+          <t>batteries</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -11566,7 +11608,7 @@
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>telemetry</t>
+          <t>telematics</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -11579,7 +11621,7 @@
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>driving_sessions</t>
+          <t>telemetry</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -11592,7 +11634,7 @@
       <c r="A38" s="6" t="n"/>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>trips</t>
+          <t>driving_sessions</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -11605,7 +11647,7 @@
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>fleets</t>
+          <t>trips</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -11618,7 +11660,7 @@
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>geofences</t>
+          <t>fleets</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -11631,7 +11673,7 @@
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>charging_locations</t>
+          <t>geofences</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -11640,29 +11682,29 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="27" customHeight="1">
+    <row r="42">
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>charging_location_access</t>
+          <t>charging_locations</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>allowed_organization_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
+          <t>organization_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="27" customHeight="1">
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>charging_sessions</t>
+          <t>charging_location_access</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>organization_id</t>
+          <t>allowed_organization_id</t>
         </is>
       </c>
     </row>
@@ -11670,7 +11712,7 @@
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>charging_sessions</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -11679,11 +11721,11 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="27" customHeight="1">
+    <row r="45">
       <c r="A45" s="6" t="n"/>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>organization_notification_settings</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -11692,11 +11734,11 @@
         </is>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="27" customHeight="1">
       <c r="A46" s="6" t="n"/>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>support_cases</t>
+          <t>organization_notification_settings</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -11709,7 +11751,7 @@
       <c r="A47" s="6" t="n"/>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>repair_partners</t>
+          <t>support_cases</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -11722,7 +11764,7 @@
       <c r="A48" s="6" t="n"/>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>maintenance_bookings</t>
+          <t>repair_partners</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -11731,11 +11773,11 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="27" customHeight="1">
+    <row r="49">
       <c r="A49" s="6" t="n"/>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>charging_policy_assignments</t>
+          <t>maintenance_bookings</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -11744,11 +11786,11 @@
         </is>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="27" customHeight="1">
       <c r="A50" s="6" t="n"/>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>policy_violations</t>
+          <t>charging_policy_assignments</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -11761,7 +11803,7 @@
       <c r="A51" s="6" t="n"/>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>tariffs</t>
+          <t>policy_violations</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -11774,7 +11816,7 @@
       <c r="A52" s="6" t="n"/>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>tariffs</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -11787,7 +11829,7 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>invoice_lines</t>
+          <t>invoices</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -11800,7 +11842,7 @@
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>subscriptions</t>
+          <t>invoice_lines</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -11813,7 +11855,7 @@
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>driver_scores</t>
+          <t>subscriptions</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -11826,10 +11868,23 @@
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="inlineStr">
         <is>
+          <t>driver_scores</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n"/>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
           <t>organization_history</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>organization_id</t>
         </is>
@@ -11844,34 +11899,35 @@
     <hyperlink ref="B26" location="'user_sessions'!A1"/>
     <hyperlink ref="B27" location="'memberships'!A1"/>
     <hyperlink ref="B28" location="'user_state'!A1"/>
-    <hyperlink ref="B29" location="'user_consents'!A1"/>
-    <hyperlink ref="B30" location="'user_role_assignments'!A1"/>
-    <hyperlink ref="B31" location="'access_audit_logs'!A1"/>
-    <hyperlink ref="B32" location="'organization_settings'!A1"/>
-    <hyperlink ref="B33" location="'vehicles'!A1"/>
-    <hyperlink ref="B34" location="'batteries'!A1"/>
-    <hyperlink ref="B35" location="'telematics'!A1"/>
-    <hyperlink ref="B36" location="'telemetry'!A1"/>
-    <hyperlink ref="B37" location="'driving_sessions'!A1"/>
-    <hyperlink ref="B38" location="'trips'!A1"/>
-    <hyperlink ref="B39" location="'fleets'!A1"/>
-    <hyperlink ref="B40" location="'geofences'!A1"/>
-    <hyperlink ref="B41" location="'charging_locations'!A1"/>
-    <hyperlink ref="B42" location="'charging_location_access'!A1"/>
-    <hyperlink ref="B43" location="'charging_sessions'!A1"/>
-    <hyperlink ref="B44" location="'notifications'!A1"/>
-    <hyperlink ref="B45" location="'organization_notification_setti'!A1"/>
-    <hyperlink ref="B46" location="'support_cases'!A1"/>
-    <hyperlink ref="B47" location="'repair_partners'!A1"/>
-    <hyperlink ref="B48" location="'maintenance_bookings'!A1"/>
-    <hyperlink ref="B49" location="'charging_policy_assignments'!A1"/>
-    <hyperlink ref="B50" location="'policy_violations'!A1"/>
-    <hyperlink ref="B51" location="'tariffs'!A1"/>
-    <hyperlink ref="B52" location="'invoices'!A1"/>
-    <hyperlink ref="B53" location="'invoice_lines'!A1"/>
-    <hyperlink ref="B54" location="'subscriptions'!A1"/>
-    <hyperlink ref="B55" location="'driver_scores'!A1"/>
-    <hyperlink ref="B56" location="'organization_history'!A1"/>
+    <hyperlink ref="B29" location="'one_time_codes'!A1"/>
+    <hyperlink ref="B30" location="'user_consents'!A1"/>
+    <hyperlink ref="B31" location="'user_role_assignments'!A1"/>
+    <hyperlink ref="B32" location="'access_audit_logs'!A1"/>
+    <hyperlink ref="B33" location="'organization_settings'!A1"/>
+    <hyperlink ref="B34" location="'vehicles'!A1"/>
+    <hyperlink ref="B35" location="'batteries'!A1"/>
+    <hyperlink ref="B36" location="'telematics'!A1"/>
+    <hyperlink ref="B37" location="'telemetry'!A1"/>
+    <hyperlink ref="B38" location="'driving_sessions'!A1"/>
+    <hyperlink ref="B39" location="'trips'!A1"/>
+    <hyperlink ref="B40" location="'fleets'!A1"/>
+    <hyperlink ref="B41" location="'geofences'!A1"/>
+    <hyperlink ref="B42" location="'charging_locations'!A1"/>
+    <hyperlink ref="B43" location="'charging_location_access'!A1"/>
+    <hyperlink ref="B44" location="'charging_sessions'!A1"/>
+    <hyperlink ref="B45" location="'notifications'!A1"/>
+    <hyperlink ref="B46" location="'organization_notification_setti'!A1"/>
+    <hyperlink ref="B47" location="'support_cases'!A1"/>
+    <hyperlink ref="B48" location="'repair_partners'!A1"/>
+    <hyperlink ref="B49" location="'maintenance_bookings'!A1"/>
+    <hyperlink ref="B50" location="'charging_policy_assignments'!A1"/>
+    <hyperlink ref="B51" location="'policy_violations'!A1"/>
+    <hyperlink ref="B52" location="'tariffs'!A1"/>
+    <hyperlink ref="B53" location="'invoices'!A1"/>
+    <hyperlink ref="B54" location="'invoice_lines'!A1"/>
+    <hyperlink ref="B55" location="'subscriptions'!A1"/>
+    <hyperlink ref="B56" location="'driver_scores'!A1"/>
+    <hyperlink ref="B57" location="'organization_history'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(assets): case-insensitive VIN, plate and serial, row locks on transfer and install, owner and date checks, generic conflicts, finite numbers (RV-AS1 to RV-AS7, RV-AS9, RV-AS10)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01URvQGCMdGQH5axXbsyq4p6
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -9756,7 +9756,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="54" customHeight="1">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6" t="inlineStr">
         <is>
@@ -9765,7 +9765,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>vin</t>
+          <t>upper(vin)</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -9776,11 +9776,11 @@
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>WHERE deleted_at IS NULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="27" customHeight="1">
+          <t>WHERE deleted_at IS NULL; case-insensitive (RV-AS6): the value is also stored trimmed and upper-case by the request schemas</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="54" customHeight="1">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="6" t="inlineStr">
         <is>
@@ -9789,7 +9789,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>license_plate</t>
+          <t>upper(license_plate)</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -9800,7 +9800,7 @@
       <c r="E26" s="6" t="n"/>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>WHERE deleted_at IS NULL</t>
+          <t>WHERE deleted_at IS NULL; case-insensitive (RV-AS6): the value is also stored trimmed and upper-case by the request schemas</t>
         </is>
       </c>
     </row>
@@ -14928,7 +14928,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="27" customHeight="1">
+    <row r="23" ht="54" customHeight="1">
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="6" t="inlineStr">
         <is>
@@ -14937,7 +14937,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>serial_number</t>
+          <t>upper(serial_number)</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -14948,7 +14948,7 @@
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>WHERE deleted_at IS NULL</t>
+          <t>WHERE deleted_at IS NULL; case-insensitive (RV-AS6): the value is also stored trimmed and upper-case by the request schemas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record the backend hardening batch (IS-12, ID-53, BL-29, DM-30, FL-14..FL-16)
Decision log entries for each hardening decision, with FL-15 (rows with no
truck under the fleet limit) awaiting the owner's confirmation; FLT-03 is
done on the backend; the rules (domain boundaries, database history rule,
environment), architecture.md and both planners follow the code; the
domain-model generator no longer describes the removed 'Unspecified
change' fallback.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/domain-model/domain-model.xlsx
+++ b/docs/design/domain-model/domain-model.xlsx
@@ -9051,7 +9051,7 @@
       </c>
       <c r="I15" s="6" t="n"/>
     </row>
-    <row r="16" ht="54" customHeight="1">
+    <row r="16" ht="40.5" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>9</v>
       </c>
@@ -9074,7 +9074,7 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -10702,7 +10702,7 @@
       </c>
       <c r="I22" s="6" t="n"/>
     </row>
-    <row r="23" ht="54" customHeight="1">
+    <row r="23" ht="40.5" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>16</v>
       </c>
@@ -10725,7 +10725,7 @@
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -13059,7 +13059,7 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="54" customHeight="1">
+    <row r="21" ht="40.5" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
@@ -13082,7 +13082,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -14205,7 +14205,7 @@
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20" ht="54" customHeight="1">
+    <row r="20" ht="40.5" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
@@ -14228,7 +14228,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -15682,7 +15682,7 @@
       </c>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24" ht="54" customHeight="1">
+    <row r="24" ht="40.5" customHeight="1">
       <c r="A24" s="6" t="n">
         <v>17</v>
       </c>
@@ -15705,7 +15705,7 @@
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
@@ -17350,7 +17350,7 @@
       </c>
       <c r="I25" s="6" t="n"/>
     </row>
-    <row r="26" ht="54" customHeight="1">
+    <row r="26" ht="40.5" customHeight="1">
       <c r="A26" s="6" t="n">
         <v>19</v>
       </c>
@@ -17373,7 +17373,7 @@
       <c r="F26" s="6" t="n"/>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
@@ -18871,7 +18871,7 @@
       </c>
       <c r="I22" s="6" t="n"/>
     </row>
-    <row r="23" ht="54" customHeight="1">
+    <row r="23" ht="40.5" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>16</v>
       </c>
@@ -18894,7 +18894,7 @@
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -19639,7 +19639,7 @@
       </c>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24" ht="54" customHeight="1">
+    <row r="24" ht="40.5" customHeight="1">
       <c r="A24" s="6" t="n">
         <v>17</v>
       </c>
@@ -19662,7 +19662,7 @@
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
@@ -22504,7 +22504,7 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="54" customHeight="1">
+    <row r="21" ht="40.5" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
@@ -22527,7 +22527,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -25396,7 +25396,7 @@
       </c>
       <c r="I33" s="6" t="n"/>
     </row>
-    <row r="34" ht="54" customHeight="1">
+    <row r="34" ht="40.5" customHeight="1">
       <c r="A34" s="6" t="n">
         <v>27</v>
       </c>
@@ -25419,7 +25419,7 @@
       <c r="F34" s="6" t="n"/>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
@@ -26594,7 +26594,7 @@
       </c>
       <c r="I18" s="6" t="n"/>
     </row>
-    <row r="19" ht="54" customHeight="1">
+    <row r="19" ht="40.5" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>12</v>
       </c>
@@ -26617,7 +26617,7 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -30630,7 +30630,7 @@
       </c>
       <c r="I21" s="6" t="n"/>
     </row>
-    <row r="22" ht="54" customHeight="1">
+    <row r="22" ht="40.5" customHeight="1">
       <c r="A22" s="6" t="n">
         <v>15</v>
       </c>
@@ -30653,7 +30653,7 @@
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -32562,7 +32562,7 @@
       </c>
       <c r="I21" s="6" t="n"/>
     </row>
-    <row r="22" ht="54" customHeight="1">
+    <row r="22" ht="40.5" customHeight="1">
       <c r="A22" s="6" t="n">
         <v>15</v>
       </c>
@@ -32585,7 +32585,7 @@
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -34303,7 +34303,7 @@
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20" ht="54" customHeight="1">
+    <row r="20" ht="40.5" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
@@ -34326,7 +34326,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -34945,7 +34945,7 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="54" customHeight="1">
+    <row r="21" ht="40.5" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
@@ -34968,7 +34968,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -36208,7 +36208,7 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="54" customHeight="1">
+    <row r="21" ht="40.5" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
@@ -36231,7 +36231,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -42605,7 +42605,7 @@
       </c>
       <c r="I17" s="6" t="n"/>
     </row>
-    <row r="18" ht="54" customHeight="1">
+    <row r="18" ht="40.5" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>11</v>
       </c>
@@ -42628,7 +42628,7 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -47938,7 +47938,7 @@
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
-    <row r="20" ht="54" customHeight="1">
+    <row r="20" ht="40.5" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
@@ -47961,7 +47961,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -50026,7 +50026,7 @@
       </c>
       <c r="I24" s="6" t="n"/>
     </row>
-    <row r="25" ht="54" customHeight="1">
+    <row r="25" ht="40.5" customHeight="1">
       <c r="A25" s="6" t="n">
         <v>18</v>
       </c>
@@ -50049,7 +50049,7 @@
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -51831,7 +51831,7 @@
       </c>
       <c r="I18" s="6" t="n"/>
     </row>
-    <row r="19" ht="54" customHeight="1">
+    <row r="19" ht="40.5" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>12</v>
       </c>
@@ -51854,7 +51854,7 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -53517,7 +53517,7 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
-    <row r="21" ht="54" customHeight="1">
+    <row r="21" ht="40.5" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
@@ -53540,7 +53540,7 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Nếu ứng dụng không đặt, trigger ghi 'Unspecified change' (DM-29).</t>
+          <t>Lý do thay đổi dòng, do ứng dụng đặt cho giao dịch: người dùng nhập với quyết định quản trị, văn bản cố định với thao tác thường lệ. Cập nhật không có lý do sẽ bị từ chối.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">

</xml_diff>